<commit_message>
vault backup: 2026-06-09 14:18:40
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C00B95-DFE5-46E3-8FD0-EAB2DF77F0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664414AC-3491-47C3-8C12-D7E898FE868F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -883,6 +883,10 @@
     <xf numFmtId="176" fontId="7" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -898,15 +902,53 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="216">
+  <dxfs count="219">
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF9C0006"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF9C6500"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF006100"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3684,13 +3726,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3710,13 +3752,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="17"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
@@ -3741,7 +3783,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="12">
-        <f t="shared" ref="E6:E24" si="0">IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),D6/C6,"")</f>
+        <f t="shared" ref="E6:E31" si="0">IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),D6/C6,"")</f>
         <v>1</v>
       </c>
     </row>
@@ -3926,7 +3968,7 @@
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="20" t="str">
+      <c r="E17" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -3938,7 +3980,7 @@
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="20" t="str">
+      <c r="E18" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -3950,7 +3992,7 @@
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="20" t="str">
+      <c r="E19" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -3962,7 +4004,7 @@
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="20" t="str">
+      <c r="E20" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -3974,7 +4016,7 @@
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="20" t="str">
+      <c r="E21" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -3986,7 +4028,7 @@
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="20" t="str">
+      <c r="E22" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -3998,7 +4040,7 @@
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="20" t="str">
+      <c r="E23" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -4010,7 +4052,7 @@
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
-      <c r="E24" s="20" t="str">
+      <c r="E24" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -4022,9 +4064,9 @@
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="21"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="14"/>
+    </row>
+    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>28</v>
       </c>
@@ -4037,12 +4079,12 @@
       <c r="D26" s="2">
         <v>5</v>
       </c>
-      <c r="E26" s="20">
-        <f t="shared" ref="E26:E31" si="1">IF(AND(C26&lt;&gt;"",D26&lt;&gt;""),D26/C26,"")</f>
+      <c r="E26" s="12">
+        <f t="shared" si="0"/>
         <v>0.45454545454545453</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>29</v>
       </c>
@@ -4055,12 +4097,12 @@
       <c r="D27" s="2">
         <v>15</v>
       </c>
-      <c r="E27" s="20">
-        <f t="shared" si="1"/>
+      <c r="E27" s="12">
+        <f t="shared" si="0"/>
         <v>0.78947368421052633</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>30</v>
       </c>
@@ -4073,12 +4115,12 @@
       <c r="D28" s="2">
         <v>13</v>
       </c>
-      <c r="E28" s="20">
-        <f t="shared" si="1"/>
+      <c r="E28" s="12">
+        <f t="shared" si="0"/>
         <v>0.8666666666666667</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>31</v>
       </c>
@@ -4091,32 +4133,32 @@
       <c r="D29" s="2">
         <v>11</v>
       </c>
-      <c r="E29" s="20">
-        <f t="shared" si="1"/>
+      <c r="E29" s="12">
+        <f t="shared" si="0"/>
         <v>0.6470588235294118</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>32</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>33</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="20" t="str">
-        <f t="shared" si="1"/>
+      <c r="E31" s="12" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -4127,7 +4169,7 @@
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="21"/>
+      <c r="E32" s="14"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
@@ -4136,8 +4178,8 @@
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="20" t="str">
-        <f t="shared" ref="E33:E38" si="2">IF(AND(C33&lt;&gt;"",D33&lt;&gt;""),D33/C33,"")</f>
+      <c r="E33" s="13" t="str">
+        <f t="shared" ref="E33:E38" si="1">IF(AND(C33&lt;&gt;"",D33&lt;&gt;""),D33/C33,"")</f>
         <v/>
       </c>
     </row>
@@ -4148,8 +4190,8 @@
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
-      <c r="E34" s="20" t="str">
-        <f t="shared" si="2"/>
+      <c r="E34" s="13" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4160,8 +4202,8 @@
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
-      <c r="E35" s="20" t="str">
-        <f t="shared" si="2"/>
+      <c r="E35" s="13" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4172,8 +4214,8 @@
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
-      <c r="E36" s="20" t="str">
-        <f t="shared" si="2"/>
+      <c r="E36" s="13" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4184,8 +4226,8 @@
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
-      <c r="E37" s="20" t="str">
-        <f t="shared" si="2"/>
+      <c r="E37" s="13" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4196,8 +4238,8 @@
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="20" t="str">
-        <f t="shared" si="2"/>
+      <c r="E38" s="13" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4220,13 +4262,13 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="15"/>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="17"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
@@ -4245,7 +4287,7 @@
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2" t="str">
-        <f t="shared" ref="E43:E60" si="3">IF(AND(C43&lt;&gt;"",D43&lt;&gt;""),D43/C43,"")</f>
+        <f t="shared" ref="E43:E60" si="2">IF(AND(C43&lt;&gt;"",D43&lt;&gt;""),D43/C43,"")</f>
         <v/>
       </c>
     </row>
@@ -4257,7 +4299,7 @@
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4269,7 +4311,7 @@
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4281,7 +4323,7 @@
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4293,7 +4335,7 @@
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4305,7 +4347,7 @@
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4317,7 +4359,7 @@
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4329,7 +4371,7 @@
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4341,7 +4383,7 @@
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4353,7 +4395,7 @@
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4365,7 +4407,7 @@
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4377,7 +4419,7 @@
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4389,7 +4431,7 @@
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4401,7 +4443,7 @@
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4413,7 +4455,7 @@
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4425,7 +4467,7 @@
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4437,7 +4479,7 @@
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4449,7 +4491,7 @@
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4472,13 +4514,13 @@
       </c>
     </row>
     <row r="63" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="13" t="s">
+      <c r="A63" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="15"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="17"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
@@ -4497,7 +4539,7 @@
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2" t="str">
-        <f t="shared" ref="E65:E73" si="4">IF(AND(C65&lt;&gt;"",D65&lt;&gt;""),D65/C65,"")</f>
+        <f t="shared" ref="E65:E73" si="3">IF(AND(C65&lt;&gt;"",D65&lt;&gt;""),D65/C65,"")</f>
         <v/>
       </c>
     </row>
@@ -4509,7 +4551,7 @@
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4521,7 +4563,7 @@
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4533,7 +4575,7 @@
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4545,7 +4587,7 @@
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
       <c r="E69" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4557,7 +4599,7 @@
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
       <c r="E70" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4569,7 +4611,7 @@
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
       <c r="E71" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4581,7 +4623,7 @@
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
       <c r="E72" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4593,7 +4635,7 @@
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
       <c r="E73" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4614,7 +4656,7 @@
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2" t="str">
-        <f t="shared" ref="E75:E83" si="5">IF(AND(C75&lt;&gt;"",D75&lt;&gt;""),D75/C75,"")</f>
+        <f t="shared" ref="E75:E83" si="4">IF(AND(C75&lt;&gt;"",D75&lt;&gt;""),D75/C75,"")</f>
         <v/>
       </c>
     </row>
@@ -4626,7 +4668,7 @@
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4638,7 +4680,7 @@
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4650,7 +4692,7 @@
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4662,7 +4704,7 @@
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4674,7 +4716,7 @@
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4686,7 +4728,7 @@
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4698,7 +4740,7 @@
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -4710,18 +4752,18 @@
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="84" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="13" t="s">
+      <c r="A84" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B84" s="14"/>
-      <c r="C84" s="14"/>
-      <c r="D84" s="14"/>
-      <c r="E84" s="15"/>
+      <c r="B84" s="16"/>
+      <c r="C84" s="16"/>
+      <c r="D84" s="16"/>
+      <c r="E84" s="17"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
@@ -4898,134 +4940,134 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E16">
-    <cfRule type="cellIs" dxfId="215" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="214" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="213" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="218" priority="4" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="217" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="216" priority="6" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17:E24">
-    <cfRule type="cellIs" dxfId="212" priority="4" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="211" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="210" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="215" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="214" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="213" priority="9" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E34:E38">
+    <cfRule type="cellIs" dxfId="209" priority="82" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="208" priority="83" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="207" priority="84" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E40">
+    <cfRule type="cellIs" dxfId="206" priority="214" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="205" priority="215" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="204" priority="216" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E43:E60">
+    <cfRule type="cellIs" dxfId="203" priority="97" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="202" priority="98" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="201" priority="99" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E64:E73">
+    <cfRule type="cellIs" dxfId="200" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="199" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="198" priority="153" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E76:E83">
+    <cfRule type="cellIs" dxfId="197" priority="178" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="196" priority="179" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="195" priority="180" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E85:E88">
+    <cfRule type="cellIs" dxfId="194" priority="202" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="193" priority="203" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="192" priority="204" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E91">
+    <cfRule type="cellIs" dxfId="191" priority="223" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="190" priority="224" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="189" priority="225" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E94">
+    <cfRule type="cellIs" dxfId="188" priority="220" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="187" priority="221" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="186" priority="222" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26:E31">
-    <cfRule type="cellIs" dxfId="209" priority="61" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="208" priority="62" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="63" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E34:E38">
-    <cfRule type="cellIs" dxfId="206" priority="79" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="205" priority="80" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="204" priority="81" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E40">
-    <cfRule type="cellIs" dxfId="203" priority="211" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="202" priority="212" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="201" priority="213" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E43:E60">
-    <cfRule type="cellIs" dxfId="200" priority="94" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="199" priority="95" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="198" priority="96" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E64:E73">
-    <cfRule type="cellIs" dxfId="197" priority="148" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="149" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="195" priority="150" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E76:E83">
-    <cfRule type="cellIs" dxfId="194" priority="175" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="193" priority="176" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="177" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E85:E88">
-    <cfRule type="cellIs" dxfId="191" priority="199" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="190" priority="200" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="201" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E91">
-    <cfRule type="cellIs" dxfId="188" priority="220" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="221" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="186" priority="222" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E94">
-    <cfRule type="cellIs" dxfId="185" priority="217" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="218" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="219" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5049,32 +5091,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="17"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -5650,146 +5692,146 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E11">
-    <cfRule type="cellIs" dxfId="182" priority="4" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="185" priority="4" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="184" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="183" priority="6" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E16">
-    <cfRule type="cellIs" dxfId="179" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="178" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="177" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="182" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="181" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="180" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:E19">
-    <cfRule type="cellIs" dxfId="176" priority="37" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="38" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="39" operator="lessThan">
+    <cfRule type="cellIs" dxfId="179" priority="37" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="178" priority="38" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="177" priority="39" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E23">
-    <cfRule type="cellIs" dxfId="173" priority="43" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="44" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="171" priority="45" operator="lessThan">
+    <cfRule type="cellIs" dxfId="176" priority="43" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="175" priority="44" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="174" priority="45" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25:E28">
-    <cfRule type="cellIs" dxfId="170" priority="52" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="169" priority="53" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="168" priority="54" operator="lessThan">
+    <cfRule type="cellIs" dxfId="173" priority="52" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="172" priority="53" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="171" priority="54" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30">
-    <cfRule type="cellIs" dxfId="167" priority="64" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="65" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="66" operator="lessThan">
+    <cfRule type="cellIs" dxfId="170" priority="64" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="169" priority="65" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="168" priority="66" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I11">
-    <cfRule type="cellIs" dxfId="164" priority="67" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="163" priority="68" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="162" priority="69" operator="lessThan">
+    <cfRule type="cellIs" dxfId="167" priority="67" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="166" priority="68" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="165" priority="69" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I16">
-    <cfRule type="cellIs" dxfId="161" priority="85" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="86" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="159" priority="87" operator="lessThan">
+    <cfRule type="cellIs" dxfId="164" priority="85" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="163" priority="86" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="162" priority="87" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I18:I19">
-    <cfRule type="cellIs" dxfId="158" priority="97" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="98" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="156" priority="99" operator="lessThan">
+    <cfRule type="cellIs" dxfId="161" priority="97" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="160" priority="98" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="159" priority="99" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21:I23">
-    <cfRule type="cellIs" dxfId="155" priority="103" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="104" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="153" priority="105" operator="lessThan">
+    <cfRule type="cellIs" dxfId="158" priority="103" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="157" priority="104" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="156" priority="105" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I25:I28">
-    <cfRule type="cellIs" dxfId="152" priority="112" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="113" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="114" operator="lessThan">
+    <cfRule type="cellIs" dxfId="155" priority="112" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="154" priority="113" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="153" priority="114" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I30">
-    <cfRule type="cellIs" dxfId="149" priority="124" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="148" priority="125" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="126" operator="lessThan">
+    <cfRule type="cellIs" dxfId="152" priority="124" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="151" priority="125" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="150" priority="126" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5813,32 +5855,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="17"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -6744,206 +6786,206 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E8">
-    <cfRule type="cellIs" dxfId="146" priority="22" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="23" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="24" operator="lessThan">
+    <cfRule type="cellIs" dxfId="149" priority="22" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="148" priority="23" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="147" priority="24" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E12">
-    <cfRule type="cellIs" dxfId="143" priority="19" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="20" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="21" operator="lessThan">
+    <cfRule type="cellIs" dxfId="146" priority="19" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="145" priority="20" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="144" priority="21" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14:E19">
-    <cfRule type="cellIs" dxfId="140" priority="16" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="17" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="143" priority="16" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="142" priority="17" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="141" priority="18" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E24">
-    <cfRule type="cellIs" dxfId="137" priority="10" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="11" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="12" operator="lessThan">
+    <cfRule type="cellIs" dxfId="140" priority="10" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="139" priority="11" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="12" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26:E32">
-    <cfRule type="cellIs" dxfId="134" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="137" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="135" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34:E35">
-    <cfRule type="cellIs" dxfId="131" priority="4" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="134" priority="4" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="6" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E37:E39">
-    <cfRule type="cellIs" dxfId="128" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="3" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="131" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="3" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="129" priority="1" operator="greaterThanOrEqual">
       <formula>0.9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E40">
-    <cfRule type="cellIs" dxfId="125" priority="100" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="101" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="102" operator="lessThan">
+    <cfRule type="cellIs" dxfId="128" priority="100" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="127" priority="101" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="126" priority="102" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E42">
-    <cfRule type="cellIs" dxfId="122" priority="112" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="113" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="114" operator="lessThan">
+    <cfRule type="cellIs" dxfId="125" priority="112" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="113" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="114" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I8">
-    <cfRule type="cellIs" dxfId="119" priority="115" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="116" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="117" operator="lessThan">
+    <cfRule type="cellIs" dxfId="122" priority="115" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="121" priority="116" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="117" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:I12">
-    <cfRule type="cellIs" dxfId="116" priority="124" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="125" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="126" operator="lessThan">
+    <cfRule type="cellIs" dxfId="119" priority="124" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="125" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="117" priority="126" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I14:I19">
-    <cfRule type="cellIs" dxfId="113" priority="133" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="134" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="135" operator="lessThan">
+    <cfRule type="cellIs" dxfId="116" priority="133" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="134" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="114" priority="135" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21:I24">
-    <cfRule type="cellIs" dxfId="110" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="113" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="112" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26:I32">
-    <cfRule type="cellIs" dxfId="107" priority="163" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="164" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="165" operator="lessThan">
+    <cfRule type="cellIs" dxfId="110" priority="163" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="164" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="108" priority="165" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I34:I35">
-    <cfRule type="cellIs" dxfId="104" priority="184" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="185" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="186" operator="lessThan">
+    <cfRule type="cellIs" dxfId="107" priority="184" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="185" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="186" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I37:I40">
-    <cfRule type="cellIs" dxfId="101" priority="190" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="191" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="99" priority="192" operator="lessThan">
+    <cfRule type="cellIs" dxfId="104" priority="190" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="191" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="192" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I42">
-    <cfRule type="cellIs" dxfId="98" priority="202" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="203" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="204" operator="lessThan">
+    <cfRule type="cellIs" dxfId="101" priority="202" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="203" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="99" priority="204" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6967,32 +7009,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="17"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -7827,218 +7869,218 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E7">
-    <cfRule type="cellIs" dxfId="95" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="98" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="96" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E11">
-    <cfRule type="cellIs" dxfId="92" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="95" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="94" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="93" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E16">
-    <cfRule type="cellIs" dxfId="89" priority="16" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="17" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="92" priority="16" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="91" priority="17" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="90" priority="18" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:E19">
-    <cfRule type="cellIs" dxfId="86" priority="28" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="29" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="30" operator="lessThan">
+    <cfRule type="cellIs" dxfId="89" priority="28" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="88" priority="29" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="87" priority="30" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E25">
-    <cfRule type="cellIs" dxfId="83" priority="34" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="35" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="36" operator="lessThan">
+    <cfRule type="cellIs" dxfId="86" priority="34" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="85" priority="35" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="84" priority="36" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27:E30">
-    <cfRule type="cellIs" dxfId="80" priority="49" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="50" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="51" operator="lessThan">
+    <cfRule type="cellIs" dxfId="83" priority="49" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="82" priority="50" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="81" priority="51" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32:E36">
-    <cfRule type="cellIs" dxfId="77" priority="61" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="62" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="63" operator="lessThan">
+    <cfRule type="cellIs" dxfId="80" priority="61" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="79" priority="62" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="78" priority="63" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E38:E45">
-    <cfRule type="cellIs" dxfId="74" priority="76" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="77" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="78" operator="lessThan">
+    <cfRule type="cellIs" dxfId="77" priority="76" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="77" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="75" priority="78" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E47">
-    <cfRule type="cellIs" dxfId="71" priority="100" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="101" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="102" operator="lessThan">
+    <cfRule type="cellIs" dxfId="74" priority="100" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="101" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="102" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I7">
-    <cfRule type="cellIs" dxfId="68" priority="103" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="104" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="105" operator="lessThan">
+    <cfRule type="cellIs" dxfId="71" priority="103" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="70" priority="104" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="69" priority="105" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:I11">
-    <cfRule type="cellIs" dxfId="65" priority="109" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="110" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="111" operator="lessThan">
+    <cfRule type="cellIs" dxfId="68" priority="109" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="67" priority="110" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="111" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I16">
-    <cfRule type="cellIs" dxfId="62" priority="118" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="119" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="120" operator="lessThan">
+    <cfRule type="cellIs" dxfId="65" priority="118" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="119" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="63" priority="120" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I18:I19">
-    <cfRule type="cellIs" dxfId="59" priority="130" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="131" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="132" operator="lessThan">
+    <cfRule type="cellIs" dxfId="62" priority="130" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="131" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="60" priority="132" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21:I25">
-    <cfRule type="cellIs" dxfId="56" priority="136" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="137" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="138" operator="lessThan">
+    <cfRule type="cellIs" dxfId="59" priority="136" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="58" priority="137" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="57" priority="138" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I27:I30">
-    <cfRule type="cellIs" dxfId="53" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="56" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="54" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I32:I36">
-    <cfRule type="cellIs" dxfId="50" priority="163" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="164" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="165" operator="lessThan">
+    <cfRule type="cellIs" dxfId="53" priority="163" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="164" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="51" priority="165" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I38:I45">
-    <cfRule type="cellIs" dxfId="47" priority="178" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="179" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="180" operator="lessThan">
+    <cfRule type="cellIs" dxfId="50" priority="178" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="179" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="180" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I47">
-    <cfRule type="cellIs" dxfId="44" priority="202" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="203" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="204" operator="lessThan">
+    <cfRule type="cellIs" dxfId="47" priority="202" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="203" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="204" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8062,32 +8104,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="17"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -8816,170 +8858,170 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E7">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E11">
-    <cfRule type="cellIs" dxfId="38" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="41" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="39" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E20">
-    <cfRule type="cellIs" dxfId="35" priority="16" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="17" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="38" priority="16" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="17" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="18" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E22:E28">
-    <cfRule type="cellIs" dxfId="32" priority="40" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="41" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="42" operator="lessThan">
+    <cfRule type="cellIs" dxfId="35" priority="40" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="41" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="42" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30:E32">
-    <cfRule type="cellIs" dxfId="29" priority="61" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="62" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="63" operator="lessThan">
+    <cfRule type="cellIs" dxfId="32" priority="61" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="62" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="63" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34:E39">
-    <cfRule type="cellIs" dxfId="26" priority="70" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="71" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="72" operator="lessThan">
+    <cfRule type="cellIs" dxfId="29" priority="70" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="71" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="72" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E41">
-    <cfRule type="cellIs" dxfId="23" priority="88" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="89" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="90" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="88" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="89" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="90" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I7">
-    <cfRule type="cellIs" dxfId="20" priority="91" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="92" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="93" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="91" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="92" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="93" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:I11">
-    <cfRule type="cellIs" dxfId="17" priority="97" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="98" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="99" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="97" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="98" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="99" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I20">
-    <cfRule type="cellIs" dxfId="14" priority="106" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="107" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="108" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="106" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="107" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="108" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I22:I28">
-    <cfRule type="cellIs" dxfId="11" priority="130" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="131" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="132" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="130" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="131" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="132" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I30:I32">
-    <cfRule type="cellIs" dxfId="8" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I34:I39">
-    <cfRule type="cellIs" dxfId="5" priority="160" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="161" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="162" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="160" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="161" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="162" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I41">
-    <cfRule type="cellIs" dxfId="2" priority="178" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="179" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="180" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="178" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="179" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="180" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
vault backup: 2026-06-10 14:21:32
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664414AC-3491-47C3-8C12-D7E898FE868F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D8D9D1-51AA-419A-8815-DD5A09980CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -906,7 +906,7 @@
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="219">
+  <dxfs count="225">
     <dxf>
       <font>
         <b/>
@@ -951,7 +951,10 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <sz val="10.5"/>
         <color rgb="FF9C0006"/>
+        <name val="微软雅黑"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -962,1376 +965,15 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF9C6500"/>
+        <name val="微软雅黑"/>
       </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2381,6 +1023,1420 @@
       <font>
         <b/>
         <sz val="10.5"/>
+        <color rgb="FF006100"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF006100"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
         <color rgb="FF9C0006"/>
         <name val="微软雅黑"/>
       </font>
@@ -2409,6 +2465,34 @@
       <font>
         <b/>
         <sz val="10.5"/>
+        <color rgb="FF9C0006"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF9C6500"/>
+        <name val="微软雅黑"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="10.5"/>
         <color rgb="FF006100"/>
         <name val="微软雅黑"/>
       </font>
@@ -3309,7 +3393,10 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <sz val="10.5"/>
         <color rgb="FF9C0006"/>
+        <name val="微软雅黑"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -3320,7 +3407,10 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <b/>
+        <sz val="10.5"/>
+        <color rgb="FF9C6500"/>
+        <name val="微软雅黑"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -3331,7 +3421,10 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <sz val="10.5"/>
         <color rgb="FF006100"/>
+        <name val="微软雅黑"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -4940,134 +5033,134 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E16">
-    <cfRule type="cellIs" dxfId="218" priority="4" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="217" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="216" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="224" priority="4" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="223" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="222" priority="6" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17:E24">
-    <cfRule type="cellIs" dxfId="215" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="214" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="213" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="221" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="220" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="219" priority="9" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26:E31">
+    <cfRule type="cellIs" dxfId="218" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="217" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="216" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34:E38">
-    <cfRule type="cellIs" dxfId="209" priority="82" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="208" priority="83" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="84" operator="lessThan">
+    <cfRule type="cellIs" dxfId="215" priority="82" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="214" priority="83" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="213" priority="84" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E40">
-    <cfRule type="cellIs" dxfId="206" priority="214" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="205" priority="215" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="204" priority="216" operator="lessThan">
+    <cfRule type="cellIs" dxfId="212" priority="214" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="211" priority="215" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="210" priority="216" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E43:E60">
-    <cfRule type="cellIs" dxfId="203" priority="97" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="202" priority="98" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="201" priority="99" operator="lessThan">
+    <cfRule type="cellIs" dxfId="209" priority="97" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="208" priority="98" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="207" priority="99" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E64:E73">
-    <cfRule type="cellIs" dxfId="200" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="199" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="198" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="206" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="205" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="204" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E76:E83">
-    <cfRule type="cellIs" dxfId="197" priority="178" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="179" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="195" priority="180" operator="lessThan">
+    <cfRule type="cellIs" dxfId="203" priority="178" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="202" priority="179" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="201" priority="180" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E85:E88">
-    <cfRule type="cellIs" dxfId="194" priority="202" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="193" priority="203" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="204" operator="lessThan">
+    <cfRule type="cellIs" dxfId="200" priority="202" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="199" priority="203" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="198" priority="204" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E91">
-    <cfRule type="cellIs" dxfId="191" priority="223" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="190" priority="224" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="225" operator="lessThan">
+    <cfRule type="cellIs" dxfId="197" priority="223" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="196" priority="224" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="195" priority="225" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E94">
-    <cfRule type="cellIs" dxfId="188" priority="220" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="221" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="186" priority="222" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E26:E31">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="194" priority="220" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="193" priority="221" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="192" priority="222" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5434,16 +5527,22 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2" t="str">
-        <f>IF(AND(C18&lt;&gt;"",D18&lt;&gt;""),D18/C18,"")</f>
-        <v/>
+      <c r="B18" s="11">
+        <v>609</v>
+      </c>
+      <c r="C18" s="11">
+        <v>72</v>
+      </c>
+      <c r="D18" s="11">
+        <v>51</v>
+      </c>
+      <c r="E18" s="12">
+        <f t="shared" ref="E18:E19" si="2">IF(AND(C18&lt;&gt;"",D18&lt;&gt;""),D18/C18,"")</f>
+        <v>0.70833333333333337</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="2"/>
@@ -5453,15 +5552,15 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="str">
-        <f>IF(AND(C19&lt;&gt;"",D19&lt;&gt;""),D19/C19,"")</f>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="12" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F19" s="9"/>
@@ -5485,15 +5584,15 @@
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2" t="str">
-        <f>IF(AND(C21&lt;&gt;"",D21&lt;&gt;""),D21/C21,"")</f>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="12" t="str">
+        <f t="shared" ref="E21:E23" si="3">IF(AND(C21&lt;&gt;"",D21&lt;&gt;""),D21/C21,"")</f>
         <v/>
       </c>
       <c r="F21" s="9"/>
@@ -5504,15 +5603,15 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2" t="str">
-        <f>IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),D22/C22,"")</f>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="12" t="str">
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F22" s="9"/>
@@ -5523,15 +5622,15 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2" t="str">
-        <f>IF(AND(C23&lt;&gt;"",D23&lt;&gt;""),D23/C23,"")</f>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12" t="str">
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F23" s="9"/>
@@ -5555,15 +5654,15 @@
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2" t="str">
-        <f>IF(AND(C25&lt;&gt;"",D25&lt;&gt;""),D25/C25,"")</f>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12" t="str">
+        <f t="shared" ref="E25:E27" si="4">IF(AND(C25&lt;&gt;"",D25&lt;&gt;""),D25/C25,"")</f>
         <v/>
       </c>
       <c r="F25" s="9"/>
@@ -5574,15 +5673,15 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2" t="str">
-        <f>IF(AND(C26&lt;&gt;"",D26&lt;&gt;""),D26/C26,"")</f>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12" t="str">
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F26" s="9"/>
@@ -5593,15 +5692,15 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2" t="str">
-        <f>IF(AND(C27&lt;&gt;"",D27&lt;&gt;""),D27/C27,"")</f>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12" t="str">
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F27" s="9"/>
@@ -5619,15 +5718,15 @@
       <c r="B28" s="8"/>
       <c r="C28" s="8">
         <f>SUM(C5:C27)</f>
-        <v>361</v>
+        <v>433</v>
       </c>
       <c r="D28" s="8">
         <f>SUM(D5:D27)</f>
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="E28" s="8">
         <f>IF(C28&gt;0, D28/C28,"")</f>
-        <v>0.75900277008310246</v>
+        <v>0.75057736720554269</v>
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="8">
@@ -5650,15 +5749,15 @@
       <c r="B30" s="5"/>
       <c r="C30" s="5">
         <f>C28+G28</f>
-        <v>361</v>
+        <v>433</v>
       </c>
       <c r="D30" s="5">
         <f>D28+H28</f>
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="E30" s="5">
         <f>IF(C30&gt;0, D30/C30,"")</f>
-        <v>0.75900277008310246</v>
+        <v>0.75057736720554269</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -5692,146 +5791,158 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E11">
-    <cfRule type="cellIs" dxfId="185" priority="4" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="191" priority="13" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="190" priority="14" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="189" priority="15" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E16">
-    <cfRule type="cellIs" dxfId="182" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="188" priority="10" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="187" priority="11" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="186" priority="12" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28">
+    <cfRule type="cellIs" dxfId="179" priority="61" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="178" priority="62" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="177" priority="63" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E30">
+    <cfRule type="cellIs" dxfId="176" priority="73" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="175" priority="74" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="174" priority="75" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:I11">
+    <cfRule type="cellIs" dxfId="173" priority="76" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="172" priority="77" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="171" priority="78" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I13:I16">
+    <cfRule type="cellIs" dxfId="170" priority="94" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="169" priority="95" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="168" priority="96" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I18:I19">
+    <cfRule type="cellIs" dxfId="167" priority="106" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="166" priority="107" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="165" priority="108" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I21:I23">
+    <cfRule type="cellIs" dxfId="164" priority="112" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="163" priority="113" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="162" priority="114" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I25:I28">
+    <cfRule type="cellIs" dxfId="161" priority="121" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="160" priority="122" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="159" priority="123" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I30">
+    <cfRule type="cellIs" dxfId="158" priority="133" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="157" priority="134" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="156" priority="135" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:E19">
-    <cfRule type="cellIs" dxfId="179" priority="37" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="178" priority="38" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="177" priority="39" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E23">
-    <cfRule type="cellIs" dxfId="176" priority="43" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="44" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="45" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E25:E28">
-    <cfRule type="cellIs" dxfId="173" priority="52" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="53" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="171" priority="54" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E30">
-    <cfRule type="cellIs" dxfId="170" priority="64" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="169" priority="65" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="168" priority="66" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I11">
-    <cfRule type="cellIs" dxfId="167" priority="67" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="68" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="69" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I13:I16">
-    <cfRule type="cellIs" dxfId="164" priority="85" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="163" priority="86" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="162" priority="87" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I18:I19">
-    <cfRule type="cellIs" dxfId="161" priority="97" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="98" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="159" priority="99" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I21:I23">
-    <cfRule type="cellIs" dxfId="158" priority="103" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="104" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="156" priority="105" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I25:I28">
-    <cfRule type="cellIs" dxfId="155" priority="112" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="113" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="153" priority="114" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I30">
-    <cfRule type="cellIs" dxfId="152" priority="124" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="125" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="126" operator="lessThan">
+  <conditionalFormatting sqref="E25:E27">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6786,206 +6897,206 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E8">
-    <cfRule type="cellIs" dxfId="149" priority="22" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="148" priority="23" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="24" operator="lessThan">
+    <cfRule type="cellIs" dxfId="155" priority="22" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="154" priority="23" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="153" priority="24" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E12">
-    <cfRule type="cellIs" dxfId="146" priority="19" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="20" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="21" operator="lessThan">
+    <cfRule type="cellIs" dxfId="152" priority="19" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="151" priority="20" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="150" priority="21" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14:E19">
-    <cfRule type="cellIs" dxfId="143" priority="16" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="17" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="149" priority="16" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="148" priority="17" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="147" priority="18" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E24">
-    <cfRule type="cellIs" dxfId="140" priority="10" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="11" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="12" operator="lessThan">
+    <cfRule type="cellIs" dxfId="146" priority="10" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="145" priority="11" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="144" priority="12" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26:E32">
-    <cfRule type="cellIs" dxfId="137" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="143" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="142" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="141" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34:E35">
-    <cfRule type="cellIs" dxfId="134" priority="4" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="140" priority="4" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="139" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="6" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E37:E39">
-    <cfRule type="cellIs" dxfId="131" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="3" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="137" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="3" operator="lessThan">
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="135" priority="1" operator="greaterThanOrEqual">
       <formula>0.9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E40">
-    <cfRule type="cellIs" dxfId="128" priority="100" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="101" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="102" operator="lessThan">
+    <cfRule type="cellIs" dxfId="134" priority="100" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="101" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="102" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E42">
-    <cfRule type="cellIs" dxfId="125" priority="112" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="113" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="114" operator="lessThan">
+    <cfRule type="cellIs" dxfId="131" priority="112" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="113" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="129" priority="114" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I8">
-    <cfRule type="cellIs" dxfId="122" priority="115" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="116" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="117" operator="lessThan">
+    <cfRule type="cellIs" dxfId="128" priority="115" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="127" priority="116" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="126" priority="117" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:I12">
-    <cfRule type="cellIs" dxfId="119" priority="124" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="125" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="126" operator="lessThan">
+    <cfRule type="cellIs" dxfId="125" priority="124" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="125" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="126" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I14:I19">
-    <cfRule type="cellIs" dxfId="116" priority="133" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="134" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="135" operator="lessThan">
+    <cfRule type="cellIs" dxfId="122" priority="133" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="121" priority="134" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="135" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21:I24">
-    <cfRule type="cellIs" dxfId="113" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="119" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="117" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26:I32">
-    <cfRule type="cellIs" dxfId="110" priority="163" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="164" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="165" operator="lessThan">
+    <cfRule type="cellIs" dxfId="116" priority="163" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="164" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="114" priority="165" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I34:I35">
-    <cfRule type="cellIs" dxfId="107" priority="184" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="185" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="186" operator="lessThan">
+    <cfRule type="cellIs" dxfId="113" priority="184" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="112" priority="185" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="186" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I37:I40">
-    <cfRule type="cellIs" dxfId="104" priority="190" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="191" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="192" operator="lessThan">
+    <cfRule type="cellIs" dxfId="110" priority="190" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="191" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="108" priority="192" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I42">
-    <cfRule type="cellIs" dxfId="101" priority="202" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="203" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="99" priority="204" operator="lessThan">
+    <cfRule type="cellIs" dxfId="107" priority="202" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="203" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="204" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7869,218 +7980,218 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E7">
-    <cfRule type="cellIs" dxfId="98" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="104" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E11">
-    <cfRule type="cellIs" dxfId="95" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="101" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="99" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E16">
-    <cfRule type="cellIs" dxfId="92" priority="16" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="17" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="98" priority="16" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="17" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="96" priority="18" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:E19">
-    <cfRule type="cellIs" dxfId="89" priority="28" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="29" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="30" operator="lessThan">
+    <cfRule type="cellIs" dxfId="95" priority="28" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="94" priority="29" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="93" priority="30" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E25">
-    <cfRule type="cellIs" dxfId="86" priority="34" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="35" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="36" operator="lessThan">
+    <cfRule type="cellIs" dxfId="92" priority="34" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="91" priority="35" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="90" priority="36" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27:E30">
-    <cfRule type="cellIs" dxfId="83" priority="49" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="50" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="51" operator="lessThan">
+    <cfRule type="cellIs" dxfId="89" priority="49" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="88" priority="50" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="87" priority="51" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32:E36">
-    <cfRule type="cellIs" dxfId="80" priority="61" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="62" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="63" operator="lessThan">
+    <cfRule type="cellIs" dxfId="86" priority="61" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="85" priority="62" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="84" priority="63" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E38:E45">
-    <cfRule type="cellIs" dxfId="77" priority="76" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="77" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="78" operator="lessThan">
+    <cfRule type="cellIs" dxfId="83" priority="76" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="82" priority="77" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="81" priority="78" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E47">
-    <cfRule type="cellIs" dxfId="74" priority="100" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="101" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="102" operator="lessThan">
+    <cfRule type="cellIs" dxfId="80" priority="100" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="79" priority="101" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="78" priority="102" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I7">
-    <cfRule type="cellIs" dxfId="71" priority="103" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="104" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="105" operator="lessThan">
+    <cfRule type="cellIs" dxfId="77" priority="103" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="104" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="75" priority="105" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:I11">
-    <cfRule type="cellIs" dxfId="68" priority="109" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="110" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="111" operator="lessThan">
+    <cfRule type="cellIs" dxfId="74" priority="109" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="110" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="111" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I16">
-    <cfRule type="cellIs" dxfId="65" priority="118" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="119" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="120" operator="lessThan">
+    <cfRule type="cellIs" dxfId="71" priority="118" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="70" priority="119" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="69" priority="120" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I18:I19">
-    <cfRule type="cellIs" dxfId="62" priority="130" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="131" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="132" operator="lessThan">
+    <cfRule type="cellIs" dxfId="68" priority="130" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="67" priority="131" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="132" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21:I25">
-    <cfRule type="cellIs" dxfId="59" priority="136" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="137" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="138" operator="lessThan">
+    <cfRule type="cellIs" dxfId="65" priority="136" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="137" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="63" priority="138" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I27:I30">
-    <cfRule type="cellIs" dxfId="56" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="62" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="60" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I32:I36">
-    <cfRule type="cellIs" dxfId="53" priority="163" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="164" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="165" operator="lessThan">
+    <cfRule type="cellIs" dxfId="59" priority="163" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="58" priority="164" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="57" priority="165" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I38:I45">
-    <cfRule type="cellIs" dxfId="50" priority="178" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="179" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="180" operator="lessThan">
+    <cfRule type="cellIs" dxfId="56" priority="178" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="179" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="54" priority="180" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I47">
-    <cfRule type="cellIs" dxfId="47" priority="202" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="203" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="204" operator="lessThan">
+    <cfRule type="cellIs" dxfId="53" priority="202" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="203" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="51" priority="204" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8858,170 +8969,170 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E6:E7">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="3" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E11">
-    <cfRule type="cellIs" dxfId="41" priority="7" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="8" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="47" priority="7" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="8" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="9" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E20">
-    <cfRule type="cellIs" dxfId="38" priority="16" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="17" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="18" operator="lessThan">
+    <cfRule type="cellIs" dxfId="44" priority="16" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="17" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="18" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E22:E28">
-    <cfRule type="cellIs" dxfId="35" priority="40" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="41" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="42" operator="lessThan">
+    <cfRule type="cellIs" dxfId="41" priority="40" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="41" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="39" priority="42" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30:E32">
-    <cfRule type="cellIs" dxfId="32" priority="61" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="62" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="63" operator="lessThan">
+    <cfRule type="cellIs" dxfId="38" priority="61" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="62" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="63" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34:E39">
-    <cfRule type="cellIs" dxfId="29" priority="70" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="71" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="72" operator="lessThan">
+    <cfRule type="cellIs" dxfId="35" priority="70" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="71" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="72" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E41">
-    <cfRule type="cellIs" dxfId="26" priority="88" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="89" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="90" operator="lessThan">
+    <cfRule type="cellIs" dxfId="32" priority="88" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="89" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="90" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I7">
-    <cfRule type="cellIs" dxfId="23" priority="91" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="92" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="93" operator="lessThan">
+    <cfRule type="cellIs" dxfId="29" priority="91" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="92" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="93" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:I11">
-    <cfRule type="cellIs" dxfId="20" priority="97" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="98" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="99" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="97" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="98" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="99" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I20">
-    <cfRule type="cellIs" dxfId="17" priority="106" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="107" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="108" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="106" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="107" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="108" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I22:I28">
-    <cfRule type="cellIs" dxfId="14" priority="130" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="131" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="132" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="130" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="131" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="132" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I30:I32">
-    <cfRule type="cellIs" dxfId="11" priority="151" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="152" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="153" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="151" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="152" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="153" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I34:I39">
-    <cfRule type="cellIs" dxfId="8" priority="160" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="161" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="162" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="160" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="161" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="162" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I41">
-    <cfRule type="cellIs" dxfId="5" priority="178" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="179" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="180" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="178" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="179" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="180" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
vault backup: 2026-06-14 17:40:09
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601BC7EA-EEAF-4FDC-81F5-4D2692614903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB53537F-D1A4-4727-A8A2-C91102FC54B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -577,214 +577,215 @@
     <t>8.7 外部排序</t>
   </si>
   <si>
+    <t>1.1 计算机发展历程</t>
+  </si>
+  <si>
+    <t>1.2 计算机系统层次结构</t>
+  </si>
+  <si>
+    <t>1.3 计算机的性能指标</t>
+  </si>
+  <si>
+    <t>第2章 数据的表示和运算</t>
+  </si>
+  <si>
+    <t>2.1 数制与编码</t>
+  </si>
+  <si>
+    <t>2.2 运算方法和运算电路</t>
+  </si>
+  <si>
+    <t>2.3 浮点数的表示与运算</t>
+  </si>
+  <si>
+    <t>第3章 存储系统</t>
+  </si>
+  <si>
+    <t>3.1 存储器概述</t>
+  </si>
+  <si>
+    <t>3.2 主存储器</t>
+  </si>
+  <si>
+    <t>3.3 主存储器与CPU的连接</t>
+  </si>
+  <si>
+    <t>3.4 外部存储器</t>
+  </si>
+  <si>
+    <t>3.5 高速缓冲存储器</t>
+  </si>
+  <si>
+    <t>3.6 虚拟存储器</t>
+  </si>
+  <si>
+    <t>第4章 指令系统</t>
+  </si>
+  <si>
+    <t>4.1 指令系统</t>
+  </si>
+  <si>
+    <t>4.2 寻址方式</t>
+  </si>
+  <si>
+    <t>4.3 程序的机器级代码表示</t>
+  </si>
+  <si>
+    <t>4.4 CISC和RISC的基本概念</t>
+  </si>
+  <si>
+    <t>第5章 中央处理器</t>
+  </si>
+  <si>
+    <t>5.1 CPU的功能和基本结构</t>
+  </si>
+  <si>
+    <t>5.2 指令执行过程</t>
+  </si>
+  <si>
+    <t>5.3 数据通路的功能和基本结构</t>
+  </si>
+  <si>
+    <t>5.4 控制器的功能和工作原理</t>
+  </si>
+  <si>
+    <t>5.5 异常和中断机制</t>
+  </si>
+  <si>
+    <t>5.6 指令流水线</t>
+  </si>
+  <si>
+    <t>5.7 多处理器的基本概念</t>
+  </si>
+  <si>
+    <t>第6章 总线</t>
+  </si>
+  <si>
+    <t>6.1 总线概述</t>
+  </si>
+  <si>
+    <t>6.2 总线事务和定时</t>
+  </si>
+  <si>
+    <t>第7章 输入/输出系统</t>
+  </si>
+  <si>
+    <t>7.1 I/O系统基本概念</t>
+  </si>
+  <si>
+    <t>7.2 I/O接口</t>
+  </si>
+  <si>
+    <t>7.3 I/O方式</t>
+  </si>
+  <si>
+    <t>王道计算机网络 课后习题正确率记录</t>
+  </si>
+  <si>
+    <t>第1章 计算机网络体系结构</t>
+  </si>
+  <si>
+    <t>1.1 计算机网络概述</t>
+  </si>
+  <si>
+    <t>1.2 计算机网络体系结构与参考模型</t>
+  </si>
+  <si>
+    <t>第2章 物理层</t>
+  </si>
+  <si>
+    <t>2.1 通信基础</t>
+  </si>
+  <si>
+    <t>2.2 传输介质</t>
+  </si>
+  <si>
+    <t>2.3 物理层设备</t>
+  </si>
+  <si>
+    <t>第3章 数据链路层</t>
+  </si>
+  <si>
+    <t>3.1 数据链路层的功能</t>
+  </si>
+  <si>
+    <t>3.2 组帧</t>
+  </si>
+  <si>
+    <t>3.3 差错控制</t>
+  </si>
+  <si>
+    <t>3.4 流量控制与可靠传输机制</t>
+  </si>
+  <si>
+    <t>3.5 介质访问控制</t>
+  </si>
+  <si>
+    <t>3.6 局域网</t>
+  </si>
+  <si>
+    <t>3.7 广域网</t>
+  </si>
+  <si>
+    <t>3.8 数据链路层设备</t>
+  </si>
+  <si>
+    <t>第4章 网络层</t>
+  </si>
+  <si>
+    <t>4.1 网络层的功能</t>
+  </si>
+  <si>
+    <t>4.2 IPv4</t>
+  </si>
+  <si>
+    <t>4.3 IPv6</t>
+  </si>
+  <si>
+    <t>4.4 路由算法与路由协议</t>
+  </si>
+  <si>
+    <t>4.5 IP多播</t>
+  </si>
+  <si>
+    <t>4.6 移动IP</t>
+  </si>
+  <si>
+    <t>4.7 网络层设备</t>
+  </si>
+  <si>
+    <t>第5章 传输层</t>
+  </si>
+  <si>
+    <t>5.1 传输层提供的服务</t>
+  </si>
+  <si>
+    <t>5.2 UDP</t>
+  </si>
+  <si>
+    <t>5.3 TCP</t>
+  </si>
+  <si>
+    <t>第6章 应用层</t>
+  </si>
+  <si>
+    <t>6.1 网络应用模型</t>
+  </si>
+  <si>
+    <t>6.2 域名系统</t>
+  </si>
+  <si>
+    <t>6.3 文件传输协议</t>
+  </si>
+  <si>
+    <t>6.4 电子邮件</t>
+  </si>
+  <si>
+    <t>6.5 万维网</t>
+  </si>
+  <si>
     <t>王道计算机组成原理 课后习题正确率记录</t>
-  </si>
-  <si>
-    <t>1.1 计算机发展历程</t>
-  </si>
-  <si>
-    <t>1.2 计算机系统层次结构</t>
-  </si>
-  <si>
-    <t>1.3 计算机的性能指标</t>
-  </si>
-  <si>
-    <t>第2章 数据的表示和运算</t>
-  </si>
-  <si>
-    <t>2.1 数制与编码</t>
-  </si>
-  <si>
-    <t>2.2 运算方法和运算电路</t>
-  </si>
-  <si>
-    <t>2.3 浮点数的表示与运算</t>
-  </si>
-  <si>
-    <t>第3章 存储系统</t>
-  </si>
-  <si>
-    <t>3.1 存储器概述</t>
-  </si>
-  <si>
-    <t>3.2 主存储器</t>
-  </si>
-  <si>
-    <t>3.3 主存储器与CPU的连接</t>
-  </si>
-  <si>
-    <t>3.4 外部存储器</t>
-  </si>
-  <si>
-    <t>3.5 高速缓冲存储器</t>
-  </si>
-  <si>
-    <t>3.6 虚拟存储器</t>
-  </si>
-  <si>
-    <t>第4章 指令系统</t>
-  </si>
-  <si>
-    <t>4.1 指令系统</t>
-  </si>
-  <si>
-    <t>4.2 寻址方式</t>
-  </si>
-  <si>
-    <t>4.3 程序的机器级代码表示</t>
-  </si>
-  <si>
-    <t>4.4 CISC和RISC的基本概念</t>
-  </si>
-  <si>
-    <t>第5章 中央处理器</t>
-  </si>
-  <si>
-    <t>5.1 CPU的功能和基本结构</t>
-  </si>
-  <si>
-    <t>5.2 指令执行过程</t>
-  </si>
-  <si>
-    <t>5.3 数据通路的功能和基本结构</t>
-  </si>
-  <si>
-    <t>5.4 控制器的功能和工作原理</t>
-  </si>
-  <si>
-    <t>5.5 异常和中断机制</t>
-  </si>
-  <si>
-    <t>5.6 指令流水线</t>
-  </si>
-  <si>
-    <t>5.7 多处理器的基本概念</t>
-  </si>
-  <si>
-    <t>第6章 总线</t>
-  </si>
-  <si>
-    <t>6.1 总线概述</t>
-  </si>
-  <si>
-    <t>6.2 总线事务和定时</t>
-  </si>
-  <si>
-    <t>第7章 输入/输出系统</t>
-  </si>
-  <si>
-    <t>7.1 I/O系统基本概念</t>
-  </si>
-  <si>
-    <t>7.2 I/O接口</t>
-  </si>
-  <si>
-    <t>7.3 I/O方式</t>
-  </si>
-  <si>
-    <t>王道计算机网络 课后习题正确率记录</t>
-  </si>
-  <si>
-    <t>第1章 计算机网络体系结构</t>
-  </si>
-  <si>
-    <t>1.1 计算机网络概述</t>
-  </si>
-  <si>
-    <t>1.2 计算机网络体系结构与参考模型</t>
-  </si>
-  <si>
-    <t>第2章 物理层</t>
-  </si>
-  <si>
-    <t>2.1 通信基础</t>
-  </si>
-  <si>
-    <t>2.2 传输介质</t>
-  </si>
-  <si>
-    <t>2.3 物理层设备</t>
-  </si>
-  <si>
-    <t>第3章 数据链路层</t>
-  </si>
-  <si>
-    <t>3.1 数据链路层的功能</t>
-  </si>
-  <si>
-    <t>3.2 组帧</t>
-  </si>
-  <si>
-    <t>3.3 差错控制</t>
-  </si>
-  <si>
-    <t>3.4 流量控制与可靠传输机制</t>
-  </si>
-  <si>
-    <t>3.5 介质访问控制</t>
-  </si>
-  <si>
-    <t>3.6 局域网</t>
-  </si>
-  <si>
-    <t>3.7 广域网</t>
-  </si>
-  <si>
-    <t>3.8 数据链路层设备</t>
-  </si>
-  <si>
-    <t>第4章 网络层</t>
-  </si>
-  <si>
-    <t>4.1 网络层的功能</t>
-  </si>
-  <si>
-    <t>4.2 IPv4</t>
-  </si>
-  <si>
-    <t>4.3 IPv6</t>
-  </si>
-  <si>
-    <t>4.4 路由算法与路由协议</t>
-  </si>
-  <si>
-    <t>4.5 IP多播</t>
-  </si>
-  <si>
-    <t>4.6 移动IP</t>
-  </si>
-  <si>
-    <t>4.7 网络层设备</t>
-  </si>
-  <si>
-    <t>第5章 传输层</t>
-  </si>
-  <si>
-    <t>5.1 传输层提供的服务</t>
-  </si>
-  <si>
-    <t>5.2 UDP</t>
-  </si>
-  <si>
-    <t>5.3 TCP</t>
-  </si>
-  <si>
-    <t>第6章 应用层</t>
-  </si>
-  <si>
-    <t>6.1 网络应用模型</t>
-  </si>
-  <si>
-    <t>6.2 域名系统</t>
-  </si>
-  <si>
-    <t>6.3 文件传输协议</t>
-  </si>
-  <si>
-    <t>6.4 电子邮件</t>
-  </si>
-  <si>
-    <t>6.5 万维网</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -794,7 +795,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -895,6 +896,13 @@
     <font>
       <sz val="11"/>
       <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -1080,7 +1088,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1201,6 +1209,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -11588,8 +11599,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
-        <v>179</v>
+      <c r="A1" s="50" t="s">
+        <v>248</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -11735,7 +11746,7 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B6" s="27">
         <v>507</v>
@@ -11801,7 +11812,7 @@
     </row>
     <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B7" s="27">
         <v>507</v>
@@ -11867,7 +11878,7 @@
     </row>
     <row r="8" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B8" s="27">
         <v>508</v>
@@ -11933,7 +11944,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
@@ -11959,7 +11970,7 @@
     </row>
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B10" s="27">
         <v>509</v>
@@ -12025,7 +12036,7 @@
     </row>
     <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B11" s="27">
         <v>510</v>
@@ -12091,7 +12102,7 @@
     </row>
     <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B12" s="27">
         <v>512</v>
@@ -12157,7 +12168,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B13" s="23"/>
       <c r="C13" s="23"/>
@@ -12183,7 +12194,7 @@
     </row>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B14" s="27">
         <v>513</v>
@@ -12249,7 +12260,7 @@
     </row>
     <row r="15" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B15" s="27">
         <v>514</v>
@@ -12315,7 +12326,7 @@
     </row>
     <row r="16" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B16" s="27">
         <v>515</v>
@@ -12381,7 +12392,7 @@
     </row>
     <row r="17" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B17" s="27">
         <v>516</v>
@@ -12447,7 +12458,7 @@
     </row>
     <row r="18" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B18" s="27">
         <v>516</v>
@@ -12513,7 +12524,7 @@
     </row>
     <row r="19" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B19" s="27">
         <v>517</v>
@@ -12579,7 +12590,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B20" s="23"/>
       <c r="C20" s="23"/>
@@ -12605,7 +12616,7 @@
     </row>
     <row r="21" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B21" s="27">
         <v>518</v>
@@ -12671,7 +12682,7 @@
     </row>
     <row r="22" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B22" s="27">
         <v>518</v>
@@ -12737,7 +12748,7 @@
     </row>
     <row r="23" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B23" s="27">
         <v>519</v>
@@ -12799,7 +12810,7 @@
     </row>
     <row r="24" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B24" s="27">
         <v>520</v>
@@ -12865,7 +12876,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -12891,7 +12902,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B26" s="27">
         <v>521</v>
@@ -12957,7 +12968,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B27" s="27">
         <v>521</v>
@@ -13023,7 +13034,7 @@
     </row>
     <row r="28" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B28" s="27">
         <v>522</v>
@@ -13089,7 +13100,7 @@
     </row>
     <row r="29" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B29" s="27">
         <v>523</v>
@@ -13155,7 +13166,7 @@
     </row>
     <row r="30" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B30" s="27">
         <v>524</v>
@@ -13221,7 +13232,7 @@
     </row>
     <row r="31" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B31" s="27">
         <v>525</v>
@@ -13287,7 +13298,7 @@
     </row>
     <row r="32" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B32" s="27">
         <v>525</v>
@@ -13353,7 +13364,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B33" s="23"/>
       <c r="C33" s="23"/>
@@ -13379,7 +13390,7 @@
     </row>
     <row r="34" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B34" s="27">
         <v>526</v>
@@ -13445,7 +13456,7 @@
     </row>
     <row r="35" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="26" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B35" s="27">
         <v>526</v>
@@ -13511,7 +13522,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="25" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B36" s="23"/>
       <c r="C36" s="23"/>
@@ -13537,7 +13548,7 @@
     </row>
     <row r="37" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B37" s="27">
         <v>526</v>
@@ -13603,7 +13614,7 @@
     </row>
     <row r="38" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B38" s="27">
         <v>527</v>
@@ -13669,7 +13680,7 @@
     </row>
     <row r="39" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="26" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B39" s="27">
         <v>528</v>
@@ -15701,7 +15712,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -15821,7 +15832,7 @@
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B5" s="23"/>
       <c r="C5" s="23"/>
@@ -15847,7 +15858,7 @@
     </row>
     <row r="6" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
@@ -15903,7 +15914,7 @@
     </row>
     <row r="7" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B7" s="27"/>
       <c r="C7" s="27"/>
@@ -15959,7 +15970,7 @@
     </row>
     <row r="8" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
@@ -15985,7 +15996,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B9" s="27"/>
       <c r="C9" s="27"/>
@@ -16041,7 +16052,7 @@
     </row>
     <row r="10" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
@@ -16097,7 +16108,7 @@
     </row>
     <row r="11" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B11" s="27"/>
       <c r="C11" s="27"/>
@@ -16153,7 +16164,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="23"/>
@@ -16179,7 +16190,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="27"/>
@@ -16235,7 +16246,7 @@
     </row>
     <row r="14" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
@@ -16291,7 +16302,7 @@
     </row>
     <row r="15" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -16347,7 +16358,7 @@
     </row>
     <row r="16" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B16" s="27"/>
       <c r="C16" s="27"/>
@@ -16403,7 +16414,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="27"/>
@@ -16459,7 +16470,7 @@
     </row>
     <row r="18" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="27"/>
@@ -16515,7 +16526,7 @@
     </row>
     <row r="19" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="27"/>
@@ -16571,7 +16582,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
@@ -16627,7 +16638,7 @@
     </row>
     <row r="21" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="23"/>
@@ -16653,7 +16664,7 @@
     </row>
     <row r="22" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
@@ -16709,7 +16720,7 @@
     </row>
     <row r="23" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B23" s="27"/>
       <c r="C23" s="27"/>
@@ -16765,7 +16776,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B24" s="27"/>
       <c r="C24" s="27"/>
@@ -16821,7 +16832,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
@@ -16877,7 +16888,7 @@
     </row>
     <row r="26" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
@@ -16933,7 +16944,7 @@
     </row>
     <row r="27" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B27" s="27"/>
       <c r="C27" s="27"/>
@@ -16989,7 +17000,7 @@
     </row>
     <row r="28" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B28" s="27"/>
       <c r="C28" s="27"/>
@@ -17045,7 +17056,7 @@
     </row>
     <row r="29" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B29" s="23"/>
       <c r="C29" s="23"/>
@@ -17071,7 +17082,7 @@
     </row>
     <row r="30" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -17127,7 +17138,7 @@
     </row>
     <row r="31" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B31" s="27"/>
       <c r="C31" s="27"/>
@@ -17183,7 +17194,7 @@
     </row>
     <row r="32" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B32" s="27"/>
       <c r="C32" s="27"/>
@@ -17239,7 +17250,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B33" s="23"/>
       <c r="C33" s="23"/>
@@ -17265,7 +17276,7 @@
     </row>
     <row r="34" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B34" s="27"/>
       <c r="C34" s="27"/>
@@ -17321,7 +17332,7 @@
     </row>
     <row r="35" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="26" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B35" s="27"/>
       <c r="C35" s="27"/>
@@ -17377,7 +17388,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="26" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B36" s="27"/>
       <c r="C36" s="27"/>
@@ -17433,7 +17444,7 @@
     </row>
     <row r="37" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="26" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B37" s="27"/>
       <c r="C37" s="27"/>
@@ -17489,7 +17500,7 @@
     </row>
     <row r="38" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-18 22:31:34
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D604357E-BFC2-40AA-B49F-886213ED7CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D462556C-0851-423B-A4D8-B496C94096E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="263">
   <si>
     <t>高等数学辅导讲义严选题 习题正确率记录</t>
   </si>
@@ -830,10 +830,6 @@
   </si>
   <si>
     <t>未完成</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>等第二章 物理层后记录</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -8409,36 +8405,50 @@
       <c r="A5" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34" t="str">
+      <c r="B5" s="34">
+        <v>618</v>
+      </c>
+      <c r="C5" s="34">
+        <v>18</v>
+      </c>
+      <c r="D5" s="34">
+        <v>14</v>
+      </c>
+      <c r="E5" s="34">
         <f t="shared" ref="E5:E14" si="0">IF(AND(C5&lt;&gt;"",D5&lt;&gt;""),D5/C5,"")</f>
-        <v/>
-      </c>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34" t="str">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="F5" s="34">
+        <v>8</v>
+      </c>
+      <c r="G5" s="34">
+        <v>8</v>
+      </c>
+      <c r="H5" s="34">
         <f t="shared" ref="H5:H14" si="1">IF(AND(F5&lt;&gt;"",G5&lt;&gt;""),G5/F5,"")</f>
-        <v/>
-      </c>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34" t="str">
+        <v>1</v>
+      </c>
+      <c r="I5" s="34">
+        <v>23</v>
+      </c>
+      <c r="J5" s="34">
+        <v>21</v>
+      </c>
+      <c r="K5" s="34">
         <f t="shared" ref="K5:K14" si="2">IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),J5/I5,"")</f>
-        <v/>
+        <v>0.91304347826086951</v>
       </c>
       <c r="L5" s="34">
         <f t="shared" ref="L5:L13" si="3">C5+F5+I5</f>
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="M5" s="34">
         <f t="shared" ref="M5:M13" si="4">D5+G5+J5</f>
-        <v>0</v>
-      </c>
-      <c r="N5" s="34" t="e">
+        <v>43</v>
+      </c>
+      <c r="N5" s="34">
         <f t="shared" ref="N5:N14" si="5">IF(AND(L5&lt;&gt;"",M5&lt;&gt;""),M5/L5,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.87755102040816324</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -8736,51 +8746,51 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="37" t="e">
+        <v>14</v>
+      </c>
+      <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="37" t="e">
+        <v>8</v>
+      </c>
+      <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J14" s="37">
         <f>SUM(J5:J13)</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="37" t="e">
+        <v>21</v>
+      </c>
+      <c r="K14" s="37">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.91304347826086951</v>
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>0</v>
-      </c>
-      <c r="N14" s="37" t="e">
+        <v>43</v>
+      </c>
+      <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.87755102040816324</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -8791,51 +8801,51 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="40" t="e">
+        <v>14</v>
+      </c>
+      <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="40" t="e">
+        <v>8</v>
+      </c>
+      <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J16" s="40">
         <f>J14</f>
-        <v>0</v>
-      </c>
-      <c r="K16" s="40" t="e">
+        <v>21</v>
+      </c>
+      <c r="K16" s="40">
         <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),J16/I16,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.91304347826086951</v>
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="40" t="e">
+        <v>43</v>
+      </c>
+      <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.87755102040816324</v>
       </c>
     </row>
   </sheetData>
@@ -9049,26 +9059,28 @@
       <c r="A6" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="4">
+        <v>618</v>
+      </c>
       <c r="C6" s="4">
         <v>15</v>
       </c>
       <c r="D6" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" ref="E6:E15" si="0">IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),D6/C6,"")</f>
-        <v>0.8</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="F6" s="4">
         <v>22</v>
       </c>
       <c r="G6" s="4">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H6" s="4">
         <f t="shared" ref="H6:H15" si="1">IF(AND(F6&lt;&gt;"",G6&lt;&gt;""),G6/F6,"")</f>
-        <v>0.63636363636363635</v>
+        <v>0.95454545454545459</v>
       </c>
       <c r="I6" s="4">
         <f t="shared" ref="I6:I14" si="2">C6+F6</f>
@@ -9076,11 +9088,11 @@
       </c>
       <c r="J6" s="4">
         <f t="shared" ref="J6:J14" si="3">D6+G6</f>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K6" s="4">
         <f t="shared" ref="K6:K15" si="4">IF(AND(I6&lt;&gt;"",J6&lt;&gt;""),J6/I6,"")</f>
-        <v>0.70270270270270274</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9334,11 +9346,11 @@
       </c>
       <c r="D15" s="7">
         <f>SUM(D6:D14)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="F15" s="7">
         <f>SUM(F6:F14)</f>
@@ -9346,11 +9358,11 @@
       </c>
       <c r="G15" s="7">
         <f>SUM(G6:G14)</f>
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H15" s="7">
         <f t="shared" si="1"/>
-        <v>0.63636363636363635</v>
+        <v>0.95454545454545459</v>
       </c>
       <c r="I15" s="7">
         <f>SUM(I6:I14)</f>
@@ -9358,11 +9370,11 @@
       </c>
       <c r="J15" s="7">
         <f>SUM(J6:J14)</f>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="4"/>
-        <v>0.70270270270270274</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9912,11 +9924,11 @@
       </c>
       <c r="D36" s="10">
         <f>D15+D24+D35</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E36" s="10">
         <f t="shared" si="9"/>
-        <v>0.8</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="F36" s="10">
         <f>F15+F24+F35</f>
@@ -9924,11 +9936,11 @@
       </c>
       <c r="G36" s="10">
         <f>G15+G24+G35</f>
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H36" s="10">
         <f t="shared" si="10"/>
-        <v>0.63636363636363635</v>
+        <v>0.95454545454545459</v>
       </c>
       <c r="I36" s="10">
         <f>I15+I24+I35</f>
@@ -9936,11 +9948,11 @@
       </c>
       <c r="J36" s="10">
         <f>J15+J24+J35</f>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>0.70270270270270274</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10054,19 +10066,21 @@
       </c>
       <c r="B44" s="4">
         <f t="shared" ref="B44:B52" si="13">B6</f>
-        <v>0</v>
+        <v>618</v>
       </c>
       <c r="C44" s="4">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D44" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E44" s="4">
         <f t="shared" ref="E44:E53" si="14">IF(AND(C44&lt;&gt;"",D44&lt;&gt;""),D44/C44,"")</f>
-        <v>0.625</v>
-      </c>
-      <c r="F44" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="F44" s="4">
+        <v>12</v>
+      </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4" t="str">
         <f t="shared" ref="H44:H53" si="15">IF(AND(F44&lt;&gt;"",G44&lt;&gt;""),G44/F44,"")</f>
@@ -10080,15 +10094,15 @@
       </c>
       <c r="L44" s="4">
         <f t="shared" ref="L44:L52" si="17">C44+F44+I44</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M44" s="4">
         <f t="shared" ref="M44:M52" si="18">D44+G44+J44</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N44" s="4">
         <f t="shared" ref="N44:N53" si="19">IF(AND(L44&lt;&gt;"",M44&lt;&gt;""),M44/L44,"")</f>
-        <v>0.625</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -10410,27 +10424,27 @@
       <c r="B53" s="6"/>
       <c r="C53" s="7">
         <f>SUM(C44:C52)</f>
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D53" s="7">
         <f>SUM(D44:D52)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E53" s="7">
         <f t="shared" si="14"/>
-        <v>0.625</v>
+        <v>1</v>
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G53" s="7">
         <f>SUM(G44:G52)</f>
         <v>0</v>
       </c>
-      <c r="H53" s="7" t="e">
+      <c r="H53" s="7">
         <f t="shared" si="15"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I53" s="7">
         <f>SUM(I44:I52)</f>
@@ -10446,15 +10460,15 @@
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.625</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -11156,27 +11170,27 @@
       <c r="B74" s="9"/>
       <c r="C74" s="10">
         <f>C53+C62+C73</f>
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D74" s="10">
         <f>D53+D62+D73</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E74" s="10">
         <f t="shared" si="27"/>
-        <v>0.625</v>
+        <v>1</v>
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G74" s="10">
         <f>G53+G62+G73</f>
         <v>0</v>
       </c>
-      <c r="H74" s="10" t="e">
+      <c r="H74" s="10">
         <f t="shared" si="28"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I74" s="10">
         <f>I53+I62+I73</f>
@@ -11192,15 +11206,15 @@
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.625</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11294,7 +11308,7 @@
       </c>
       <c r="B82" s="4">
         <f t="shared" ref="B82:B90" si="32">B6</f>
-        <v>0</v>
+        <v>618</v>
       </c>
       <c r="C82" s="4">
         <f t="shared" ref="C82:C90" si="33">I6</f>
@@ -11302,35 +11316,35 @@
       </c>
       <c r="D82" s="4">
         <f t="shared" ref="D82:D90" si="34">J6</f>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E82" s="4">
         <f t="shared" ref="E82:E91" si="35">IF(AND(C82&lt;&gt;"",D82&lt;&gt;""),D82/C82,"")</f>
-        <v>0.70270270270270274</v>
+        <v>0.94594594594594594</v>
       </c>
       <c r="F82" s="4">
         <f t="shared" ref="F82:F90" si="36">L44</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G82" s="4">
         <f t="shared" ref="G82:G90" si="37">M44</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H82" s="4">
         <f t="shared" ref="H82:H91" si="38">IF(AND(F82&lt;&gt;"",G82&lt;&gt;""),G82/F82,"")</f>
-        <v>0.625</v>
+        <v>0.29411764705882354</v>
       </c>
       <c r="I82" s="4">
         <f t="shared" ref="I82:I90" si="39">C82+F82</f>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J82" s="4">
         <f t="shared" ref="J82:J90" si="40">D82+G82</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K82" s="4">
         <f t="shared" ref="K82:K91" si="41">IF(AND(I82&lt;&gt;"",J82&lt;&gt;""),J82/I82,"")</f>
-        <v>0.67924528301886788</v>
+        <v>0.7407407407407407</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -11704,35 +11718,35 @@
       </c>
       <c r="D91" s="7">
         <f>SUM(D82:D90)</f>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E91" s="7">
         <f t="shared" si="35"/>
-        <v>0.70270270270270274</v>
+        <v>0.94594594594594594</v>
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.625</v>
+        <v>0.29411764705882354</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.67924528301886788</v>
+        <v>0.7407407407407407</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12492,35 +12506,35 @@
       </c>
       <c r="D112" s="10">
         <f>D91+D100+D111</f>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E112" s="10">
         <f t="shared" si="51"/>
-        <v>0.70270270270270274</v>
+        <v>0.94594594594594594</v>
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.625</v>
+        <v>0.29411764705882354</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.67924528301886788</v>
+        <v>0.7407407407407407</v>
       </c>
     </row>
   </sheetData>
@@ -21266,23 +21280,27 @@
         <v>227</v>
       </c>
       <c r="B6" s="15">
-        <v>16</v>
+        <v>616</v>
       </c>
       <c r="C6" s="15">
         <v>17</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15" t="str">
+      <c r="D6" s="15">
+        <v>14</v>
+      </c>
+      <c r="E6" s="15">
         <f>IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),D6/C6,"")</f>
-        <v/>
+        <v>0.82352941176470584</v>
       </c>
       <c r="F6" s="15">
         <v>5</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15" t="str">
+      <c r="G6" s="15">
+        <v>4</v>
+      </c>
+      <c r="H6" s="15">
         <f>IF(AND(F6&lt;&gt;"",G6&lt;&gt;""),G6/F6,"")</f>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="I6" s="15">
         <f>C6-F6</f>
@@ -21290,15 +21308,13 @@
       </c>
       <c r="J6" s="15">
         <f>D6-G6</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K6" s="15">
         <f>IF(AND(I6&lt;&gt;"",J6&lt;&gt;""),J6/I6,"")</f>
-        <v>0</v>
-      </c>
-      <c r="L6" s="11" t="s">
-        <v>263</v>
-      </c>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L6" s="11"/>
       <c r="M6" s="15"/>
       <c r="N6" s="15"/>
       <c r="O6" s="15"/>
@@ -21329,30 +21345,40 @@
       <c r="A7" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15" t="str">
+      <c r="B7" s="15">
+        <v>617</v>
+      </c>
+      <c r="C7" s="15">
+        <v>38</v>
+      </c>
+      <c r="D7" s="15">
+        <v>30</v>
+      </c>
+      <c r="E7" s="15">
         <f>IF(AND(C7&lt;&gt;"",D7&lt;&gt;""),D7/C7,"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15" t="str">
+        <v>0.78947368421052633</v>
+      </c>
+      <c r="F7" s="15">
+        <v>10</v>
+      </c>
+      <c r="G7" s="15">
+        <v>8</v>
+      </c>
+      <c r="H7" s="15">
         <f>IF(AND(F7&lt;&gt;"",G7&lt;&gt;""),G7/F7,"")</f>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="I7" s="15">
         <f>C7-F7</f>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J7" s="15">
         <f>D7-G7</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="15" t="e">
+        <v>22</v>
+      </c>
+      <c r="K7" s="15">
         <f>IF(AND(I7&lt;&gt;"",J7&lt;&gt;""),J7/I7,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="L7" s="11"/>
       <c r="M7" s="15"/>
@@ -21411,30 +21437,40 @@
       <c r="A9" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15" t="str">
+      <c r="B9" s="15">
+        <v>618</v>
+      </c>
+      <c r="C9" s="15">
+        <v>28</v>
+      </c>
+      <c r="D9" s="15">
+        <v>21</v>
+      </c>
+      <c r="E9" s="15">
         <f>IF(AND(C9&lt;&gt;"",D9&lt;&gt;""),D9/C9,"")</f>
-        <v/>
-      </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15" t="str">
+        <v>0.75</v>
+      </c>
+      <c r="F9" s="15">
+        <v>11</v>
+      </c>
+      <c r="G9" s="15">
+        <v>10</v>
+      </c>
+      <c r="H9" s="15">
         <f>IF(AND(F9&lt;&gt;"",G9&lt;&gt;""),G9/F9,"")</f>
-        <v/>
+        <v>0.90909090909090906</v>
       </c>
       <c r="I9" s="15">
         <f t="shared" ref="I9:J11" si="0">C9-F9</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K9" s="15" t="e">
+        <v>11</v>
+      </c>
+      <c r="K9" s="15">
         <f>IF(AND(I9&lt;&gt;"",J9&lt;&gt;""),J9/I9,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="L9" s="11"/>
       <c r="M9" s="15"/>
@@ -21467,30 +21503,40 @@
       <c r="A10" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15" t="str">
+      <c r="B10" s="15">
+        <v>618</v>
+      </c>
+      <c r="C10" s="15">
+        <v>12</v>
+      </c>
+      <c r="D10" s="15">
+        <v>10</v>
+      </c>
+      <c r="E10" s="15">
         <f>IF(AND(C10&lt;&gt;"",D10&lt;&gt;""),D10/C10,"")</f>
-        <v/>
-      </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15" t="str">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F10" s="15">
+        <v>2</v>
+      </c>
+      <c r="G10" s="15">
+        <v>2</v>
+      </c>
+      <c r="H10" s="15">
         <f>IF(AND(F10&lt;&gt;"",G10&lt;&gt;""),G10/F10,"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J10" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K10" s="15" t="e">
+        <v>8</v>
+      </c>
+      <c r="K10" s="15">
         <f>IF(AND(I10&lt;&gt;"",J10&lt;&gt;""),J10/I10,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.8</v>
       </c>
       <c r="L10" s="11"/>
       <c r="M10" s="15"/>
@@ -21523,30 +21569,40 @@
       <c r="A11" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15" t="str">
+      <c r="B11" s="15">
+        <v>618</v>
+      </c>
+      <c r="C11" s="15">
+        <v>9</v>
+      </c>
+      <c r="D11" s="15">
+        <v>9</v>
+      </c>
+      <c r="E11" s="15">
         <f>IF(AND(C11&lt;&gt;"",D11&lt;&gt;""),D11/C11,"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F11" s="15">
+        <v>0</v>
+      </c>
+      <c r="G11" s="15">
+        <v>0</v>
+      </c>
+      <c r="H11" s="15" t="e">
         <f>IF(AND(F11&lt;&gt;"",G11&lt;&gt;""),G11/F11,"")</f>
-        <v/>
+        <v>#DIV/0!</v>
       </c>
       <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J11" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K11" s="15" t="e">
+        <v>9</v>
+      </c>
+      <c r="K11" s="15">
         <f>IF(AND(I11&lt;&gt;"",J11&lt;&gt;""),J11/I11,"")</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="L11" s="11"/>
       <c r="M11" s="15"/>
@@ -22974,39 +23030,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.80769230769230771</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>0.78947368421052633</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23055,39 +23111,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0</v>
+        <v>0.80769230769230771</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0</v>
+        <v>0.78947368421052633</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-19 14:43:20
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D462556C-0851-423B-A4D8-B496C94096E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE981BE-AE38-4529-BEF8-9952F3A65384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
     <sheet name="武忠祥高数严选题" sheetId="8" r:id="rId2"/>
-    <sheet name="李林880专题" sheetId="3" r:id="rId3"/>
+    <sheet name="李林880" sheetId="3" r:id="rId3"/>
     <sheet name="王道数据结构" sheetId="4" r:id="rId4"/>
     <sheet name="王道计组" sheetId="5" r:id="rId5"/>
     <sheet name="王道操作系统" sheetId="6" r:id="rId6"/>
@@ -293,9 +293,6 @@
     <t>总计</t>
   </si>
   <si>
-    <t>李林880专题 （选择&amp;填空）习题正确率记录</t>
-  </si>
-  <si>
     <t>时间</t>
   </si>
   <si>
@@ -830,6 +827,10 @@
   </si>
   <si>
     <t>未完成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>李林880 （选择&amp;填空）习题正确率记录</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1249,16 +1250,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1283,22 +1293,13 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7066,7 +7067,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="55" t="s">
         <v>19</v>
       </c>
       <c r="B1" s="46"/>
@@ -7093,7 +7094,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="54" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="48"/>
@@ -7604,7 +7605,7 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="51" t="s">
+      <c r="A41" s="54" t="s">
         <v>58</v>
       </c>
       <c r="B41" s="48"/>
@@ -8091,7 +8092,7 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="51" t="s">
+      <c r="A83" s="54" t="s">
         <v>76</v>
       </c>
       <c r="B83" s="48"/>
@@ -8315,7 +8316,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="46"/>
@@ -8336,26 +8337,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="54" t="s">
+      <c r="C3" s="57" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="46"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="58" t="s">
+      <c r="E3" s="58"/>
+      <c r="F3" s="61" t="s">
         <v>2</v>
       </c>
       <c r="G3" s="46"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="57" t="s">
+      <c r="H3" s="58"/>
+      <c r="I3" s="60" t="s">
         <v>3</v>
       </c>
       <c r="J3" s="46"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="56" t="s">
+      <c r="K3" s="58"/>
+      <c r="L3" s="59" t="s">
         <v>4</v>
       </c>
       <c r="M3" s="46"/>
-      <c r="N3" s="55"/>
+      <c r="N3" s="58"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -8971,8 +8972,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
-        <v>84</v>
+      <c r="A1" s="65" t="s">
+        <v>262</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -8989,17 +8990,17 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="63" t="s">
+      <c r="C3" s="52" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="48"/>
       <c r="E3" s="49"/>
-      <c r="F3" s="61" t="s">
+      <c r="F3" s="50" t="s">
         <v>76</v>
       </c>
       <c r="G3" s="48"/>
       <c r="H3" s="49"/>
-      <c r="I3" s="62" t="s">
+      <c r="I3" s="51" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="48"/>
@@ -9010,7 +9011,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>6</v>
@@ -9041,7 +9042,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="47" t="s">
         <v>23</v>
       </c>
       <c r="B5" s="48"/>
@@ -9057,7 +9058,7 @@
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="4">
         <v>618</v>
@@ -9097,7 +9098,7 @@
     </row>
     <row r="7" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -9127,7 +9128,7 @@
     </row>
     <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -9157,7 +9158,7 @@
     </row>
     <row r="9" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -9187,7 +9188,7 @@
     </row>
     <row r="10" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -9217,7 +9218,7 @@
     </row>
     <row r="11" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -9247,7 +9248,7 @@
     </row>
     <row r="12" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -9277,7 +9278,7 @@
     </row>
     <row r="13" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -9307,7 +9308,7 @@
     </row>
     <row r="14" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -9337,7 +9338,7 @@
     </row>
     <row r="15" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7">
@@ -9379,7 +9380,7 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="60" t="s">
+      <c r="A17" s="47" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="48"/>
@@ -9395,7 +9396,7 @@
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -9425,7 +9426,7 @@
     </row>
     <row r="19" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -9455,7 +9456,7 @@
     </row>
     <row r="20" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -9485,7 +9486,7 @@
     </row>
     <row r="21" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -9515,7 +9516,7 @@
     </row>
     <row r="22" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -9545,7 +9546,7 @@
     </row>
     <row r="23" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9575,7 +9576,7 @@
     </row>
     <row r="24" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7">
@@ -9617,7 +9618,7 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="60" t="s">
+      <c r="A26" s="47" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="48"/>
@@ -9633,7 +9634,7 @@
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -9663,7 +9664,7 @@
     </row>
     <row r="28" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9693,7 +9694,7 @@
     </row>
     <row r="29" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -9723,7 +9724,7 @@
     </row>
     <row r="30" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -9753,7 +9754,7 @@
     </row>
     <row r="31" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -9783,7 +9784,7 @@
     </row>
     <row r="32" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -9813,7 +9814,7 @@
     </row>
     <row r="33" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -9843,7 +9844,7 @@
     </row>
     <row r="34" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -9873,7 +9874,7 @@
     </row>
     <row r="35" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7">
@@ -9915,7 +9916,7 @@
     </row>
     <row r="36" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="10">
@@ -9956,8 +9957,8 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="59" t="s">
-        <v>113</v>
+      <c r="A39" s="45" t="s">
+        <v>112</v>
       </c>
       <c r="B39" s="46"/>
       <c r="C39" s="46"/>
@@ -9977,22 +9978,22 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="63" t="s">
+      <c r="C41" s="52" t="s">
         <v>22</v>
       </c>
       <c r="D41" s="48"/>
       <c r="E41" s="49"/>
-      <c r="F41" s="61" t="s">
+      <c r="F41" s="50" t="s">
         <v>76</v>
       </c>
       <c r="G41" s="48"/>
       <c r="H41" s="49"/>
-      <c r="I41" s="64" t="s">
-        <v>114</v>
+      <c r="I41" s="53" t="s">
+        <v>113</v>
       </c>
       <c r="J41" s="48"/>
       <c r="K41" s="49"/>
-      <c r="L41" s="62" t="s">
+      <c r="L41" s="51" t="s">
         <v>4</v>
       </c>
       <c r="M41" s="48"/>
@@ -10003,7 +10004,7 @@
         <v>5</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>6</v>
@@ -10043,7 +10044,7 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="60" t="s">
+      <c r="A43" s="47" t="s">
         <v>23</v>
       </c>
       <c r="B43" s="48"/>
@@ -10062,7 +10063,7 @@
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B44" s="4">
         <f t="shared" ref="B44:B52" si="13">B6</f>
@@ -10081,33 +10082,39 @@
       <c r="F44" s="4">
         <v>12</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4" t="str">
+      <c r="G44" s="4">
+        <v>6</v>
+      </c>
+      <c r="H44" s="4">
         <f t="shared" ref="H44:H53" si="15">IF(AND(F44&lt;&gt;"",G44&lt;&gt;""),G44/F44,"")</f>
-        <v/>
-      </c>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="I44" s="4">
+        <v>2</v>
+      </c>
+      <c r="J44" s="4">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4">
         <f t="shared" ref="K44:K53" si="16">IF(AND(I44&lt;&gt;"",J44&lt;&gt;""),J44/I44,"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L44" s="4">
         <f t="shared" ref="L44:L52" si="17">C44+F44+I44</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M44" s="4">
         <f t="shared" ref="M44:M52" si="18">D44+G44+J44</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N44" s="4">
         <f t="shared" ref="N44:N53" si="19">IF(AND(L44&lt;&gt;"",M44&lt;&gt;""),M44/L44,"")</f>
-        <v>0.29411764705882354</v>
+        <v>0.57894736842105265</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B45" s="4">
         <f t="shared" si="13"/>
@@ -10146,7 +10153,7 @@
     </row>
     <row r="46" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B46" s="4">
         <f t="shared" si="13"/>
@@ -10185,7 +10192,7 @@
     </row>
     <row r="47" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B47" s="4">
         <f t="shared" si="13"/>
@@ -10224,7 +10231,7 @@
     </row>
     <row r="48" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B48" s="4">
         <f t="shared" si="13"/>
@@ -10263,7 +10270,7 @@
     </row>
     <row r="49" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B49" s="4">
         <f t="shared" si="13"/>
@@ -10302,7 +10309,7 @@
     </row>
     <row r="50" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B50" s="4">
         <f t="shared" si="13"/>
@@ -10341,7 +10348,7 @@
     </row>
     <row r="51" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" s="4">
         <f t="shared" si="13"/>
@@ -10380,7 +10387,7 @@
     </row>
     <row r="52" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B52" s="4">
         <f t="shared" si="13"/>
@@ -10419,7 +10426,7 @@
     </row>
     <row r="53" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7">
@@ -10440,40 +10447,40 @@
       </c>
       <c r="G53" s="7">
         <f>SUM(G44:G52)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H53" s="7">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I53" s="7">
         <f>SUM(I44:I52)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J53" s="7">
         <f>SUM(J44:J52)</f>
         <v>0</v>
       </c>
-      <c r="K53" s="7" t="e">
+      <c r="K53" s="7">
         <f t="shared" si="16"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.29411764705882354</v>
+        <v>0.57894736842105265</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="60" t="s">
+      <c r="A55" s="47" t="s">
         <v>43</v>
       </c>
       <c r="B55" s="48"/>
@@ -10492,7 +10499,7 @@
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B56" s="4">
         <f t="shared" ref="B56:B61" si="20">B18</f>
@@ -10531,7 +10538,7 @@
     </row>
     <row r="57" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B57" s="4">
         <f t="shared" si="20"/>
@@ -10570,7 +10577,7 @@
     </row>
     <row r="58" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B58" s="4">
         <f t="shared" si="20"/>
@@ -10609,7 +10616,7 @@
     </row>
     <row r="59" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B59" s="4">
         <f t="shared" si="20"/>
@@ -10648,7 +10655,7 @@
     </row>
     <row r="60" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B60" s="4">
         <f t="shared" si="20"/>
@@ -10687,7 +10694,7 @@
     </row>
     <row r="61" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B61" s="4">
         <f t="shared" si="20"/>
@@ -10726,7 +10733,7 @@
     </row>
     <row r="62" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7">
@@ -10780,7 +10787,7 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="60" t="s">
+      <c r="A64" s="47" t="s">
         <v>50</v>
       </c>
       <c r="B64" s="48"/>
@@ -10799,7 +10806,7 @@
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B65" s="4">
         <f t="shared" ref="B65:B72" si="26">B27</f>
@@ -10838,7 +10845,7 @@
     </row>
     <row r="66" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B66" s="4">
         <f t="shared" si="26"/>
@@ -10877,7 +10884,7 @@
     </row>
     <row r="67" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B67" s="4">
         <f t="shared" si="26"/>
@@ -10916,7 +10923,7 @@
     </row>
     <row r="68" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B68" s="4">
         <f t="shared" si="26"/>
@@ -10955,7 +10962,7 @@
     </row>
     <row r="69" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B69" s="4">
         <f t="shared" si="26"/>
@@ -10994,7 +11001,7 @@
     </row>
     <row r="70" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B70" s="4">
         <f t="shared" si="26"/>
@@ -11033,7 +11040,7 @@
     </row>
     <row r="71" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B71" s="4">
         <f t="shared" si="26"/>
@@ -11072,7 +11079,7 @@
     </row>
     <row r="72" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B72" s="4">
         <f t="shared" si="26"/>
@@ -11111,7 +11118,7 @@
     </row>
     <row r="73" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7">
@@ -11165,7 +11172,7 @@
     </row>
     <row r="74" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B74" s="9"/>
       <c r="C74" s="10">
@@ -11186,40 +11193,40 @@
       </c>
       <c r="G74" s="10">
         <f>G53+G62+G73</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H74" s="10">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I74" s="10">
         <f>I53+I62+I73</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J74" s="10">
         <f>J53+J62+J73</f>
         <v>0</v>
       </c>
-      <c r="K74" s="10" t="e">
+      <c r="K74" s="10">
         <f t="shared" si="29"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.29411764705882354</v>
+        <v>0.57894736842105265</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="59" t="s">
-        <v>115</v>
+      <c r="A77" s="45" t="s">
+        <v>114</v>
       </c>
       <c r="B77" s="46"/>
       <c r="C77" s="46"/>
@@ -11236,17 +11243,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="63" t="s">
-        <v>116</v>
+      <c r="C79" s="52" t="s">
+        <v>115</v>
       </c>
       <c r="D79" s="48"/>
       <c r="E79" s="49"/>
-      <c r="F79" s="61" t="s">
-        <v>113</v>
+      <c r="F79" s="50" t="s">
+        <v>112</v>
       </c>
       <c r="G79" s="48"/>
       <c r="H79" s="49"/>
-      <c r="I79" s="62" t="s">
+      <c r="I79" s="51" t="s">
         <v>83</v>
       </c>
       <c r="J79" s="48"/>
@@ -11257,7 +11264,7 @@
         <v>5</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>6</v>
@@ -11288,7 +11295,7 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="60" t="s">
+      <c r="A81" s="47" t="s">
         <v>23</v>
       </c>
       <c r="B81" s="48"/>
@@ -11304,7 +11311,7 @@
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B82" s="4">
         <f t="shared" ref="B82:B90" si="32">B6</f>
@@ -11324,32 +11331,32 @@
       </c>
       <c r="F82" s="4">
         <f t="shared" ref="F82:F90" si="36">L44</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G82" s="4">
         <f t="shared" ref="G82:G90" si="37">M44</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H82" s="4">
         <f t="shared" ref="H82:H91" si="38">IF(AND(F82&lt;&gt;"",G82&lt;&gt;""),G82/F82,"")</f>
-        <v>0.29411764705882354</v>
+        <v>0.57894736842105265</v>
       </c>
       <c r="I82" s="4">
         <f t="shared" ref="I82:I90" si="39">C82+F82</f>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J82" s="4">
         <f t="shared" ref="J82:J90" si="40">D82+G82</f>
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K82" s="4">
         <f t="shared" ref="K82:K91" si="41">IF(AND(I82&lt;&gt;"",J82&lt;&gt;""),J82/I82,"")</f>
-        <v>0.7407407407407407</v>
+        <v>0.8214285714285714</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B83" s="4">
         <f t="shared" si="32"/>
@@ -11394,7 +11401,7 @@
     </row>
     <row r="84" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B84" s="4">
         <f t="shared" si="32"/>
@@ -11439,7 +11446,7 @@
     </row>
     <row r="85" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B85" s="4">
         <f t="shared" si="32"/>
@@ -11484,7 +11491,7 @@
     </row>
     <row r="86" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B86" s="4">
         <f t="shared" si="32"/>
@@ -11529,7 +11536,7 @@
     </row>
     <row r="87" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B87" s="4">
         <f t="shared" si="32"/>
@@ -11574,7 +11581,7 @@
     </row>
     <row r="88" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B88" s="4">
         <f t="shared" si="32"/>
@@ -11619,7 +11626,7 @@
     </row>
     <row r="89" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B89" s="4">
         <f t="shared" si="32"/>
@@ -11664,7 +11671,7 @@
     </row>
     <row r="90" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B90" s="4">
         <f t="shared" si="32"/>
@@ -11709,7 +11716,7 @@
     </row>
     <row r="91" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7">
@@ -11726,32 +11733,32 @@
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.29411764705882354</v>
+        <v>0.57894736842105265</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.7407407407407407</v>
+        <v>0.8214285714285714</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="60" t="s">
+      <c r="A93" s="47" t="s">
         <v>43</v>
       </c>
       <c r="B93" s="48"/>
@@ -11767,7 +11774,7 @@
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B94" s="4">
         <f t="shared" ref="B94:B99" si="42">B18</f>
@@ -11812,7 +11819,7 @@
     </row>
     <row r="95" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B95" s="4">
         <f t="shared" si="42"/>
@@ -11857,7 +11864,7 @@
     </row>
     <row r="96" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B96" s="4">
         <f t="shared" si="42"/>
@@ -11902,7 +11909,7 @@
     </row>
     <row r="97" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B97" s="4">
         <f t="shared" si="42"/>
@@ -11947,7 +11954,7 @@
     </row>
     <row r="98" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B98" s="4">
         <f t="shared" si="42"/>
@@ -11992,7 +11999,7 @@
     </row>
     <row r="99" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B99" s="4">
         <f t="shared" si="42"/>
@@ -12037,7 +12044,7 @@
     </row>
     <row r="100" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7">
@@ -12079,7 +12086,7 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="60" t="s">
+      <c r="A102" s="47" t="s">
         <v>50</v>
       </c>
       <c r="B102" s="48"/>
@@ -12095,7 +12102,7 @@
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B103" s="4">
         <f t="shared" ref="B103:B110" si="49">B27</f>
@@ -12140,7 +12147,7 @@
     </row>
     <row r="104" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B104" s="4">
         <f t="shared" si="49"/>
@@ -12185,7 +12192,7 @@
     </row>
     <row r="105" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B105" s="4">
         <f t="shared" si="49"/>
@@ -12230,7 +12237,7 @@
     </row>
     <row r="106" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B106" s="4">
         <f t="shared" si="49"/>
@@ -12275,7 +12282,7 @@
     </row>
     <row r="107" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B107" s="4">
         <f t="shared" si="49"/>
@@ -12320,7 +12327,7 @@
     </row>
     <row r="108" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B108" s="4">
         <f t="shared" si="49"/>
@@ -12365,7 +12372,7 @@
     </row>
     <row r="109" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B109" s="4">
         <f t="shared" si="49"/>
@@ -12410,7 +12417,7 @@
     </row>
     <row r="110" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B110" s="4">
         <f t="shared" si="49"/>
@@ -12455,7 +12462,7 @@
     </row>
     <row r="111" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7">
@@ -12497,7 +12504,7 @@
     </row>
     <row r="112" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B112" s="9"/>
       <c r="C112" s="10">
@@ -12514,27 +12521,27 @@
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.29411764705882354</v>
+        <v>0.57894736842105265</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.7407407407407407</v>
+        <v>0.8214285714285714</v>
       </c>
     </row>
   </sheetData>
@@ -12954,8 +12961,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
-        <v>117</v>
+      <c r="A1" s="62" t="s">
+        <v>116</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -12981,8 +12988,8 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
-        <v>118</v>
+      <c r="A3" s="64" t="s">
+        <v>117</v>
       </c>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
@@ -12995,8 +13002,8 @@
       <c r="J3" s="48"/>
       <c r="K3" s="49"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="47" t="s">
-        <v>119</v>
+      <c r="M3" s="63" t="s">
+        <v>118</v>
       </c>
       <c r="N3" s="48"/>
       <c r="O3" s="48"/>
@@ -13010,7 +13017,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>20</v>
@@ -13025,22 +13032,22 @@
         <v>8</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>126</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>20</v>
@@ -13055,27 +13062,27 @@
         <v>8</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -13101,7 +13108,7 @@
     </row>
     <row r="6" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B6" s="15">
         <v>415</v>
@@ -13167,7 +13174,7 @@
     </row>
     <row r="7" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B7" s="15">
         <v>416</v>
@@ -13233,7 +13240,7 @@
     </row>
     <row r="8" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -13259,7 +13266,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B9" s="15">
         <v>417</v>
@@ -13325,7 +13332,7 @@
     </row>
     <row r="10" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B10" s="15">
         <v>418</v>
@@ -13391,7 +13398,7 @@
     </row>
     <row r="11" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B11" s="15">
         <v>419</v>
@@ -13457,7 +13464,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -13483,7 +13490,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B13" s="15">
         <v>420</v>
@@ -13549,7 +13556,7 @@
     </row>
     <row r="14" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B14" s="15">
         <v>421</v>
@@ -13615,7 +13622,7 @@
     </row>
     <row r="15" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B15" s="15">
         <v>422</v>
@@ -13681,7 +13688,7 @@
     </row>
     <row r="16" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B16" s="15">
         <v>423</v>
@@ -13747,7 +13754,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -13773,7 +13780,7 @@
     </row>
     <row r="18" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B18" s="15">
         <v>424</v>
@@ -13839,7 +13846,7 @@
     </row>
     <row r="19" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B19" s="15">
         <v>424</v>
@@ -13905,7 +13912,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -13931,7 +13938,7 @@
     </row>
     <row r="21" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B21" s="15">
         <v>425</v>
@@ -13997,7 +14004,7 @@
     </row>
     <row r="22" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B22" s="15">
         <v>425</v>
@@ -14063,7 +14070,7 @@
     </row>
     <row r="23" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B23" s="15">
         <v>426</v>
@@ -14129,7 +14136,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B24" s="15">
         <v>427</v>
@@ -14195,7 +14202,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B25" s="15">
         <v>428</v>
@@ -14261,7 +14268,7 @@
     </row>
     <row r="26" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
@@ -14287,7 +14294,7 @@
     </row>
     <row r="27" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B27" s="15">
         <v>429</v>
@@ -14353,7 +14360,7 @@
     </row>
     <row r="28" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B28" s="15">
         <v>430</v>
@@ -14419,7 +14426,7 @@
     </row>
     <row r="29" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B29" s="15">
         <v>501</v>
@@ -14485,7 +14492,7 @@
     </row>
     <row r="30" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B30" s="15">
         <v>502</v>
@@ -14551,7 +14558,7 @@
     </row>
     <row r="31" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
@@ -14577,7 +14584,7 @@
     </row>
     <row r="32" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B32" s="15">
         <v>503</v>
@@ -14643,7 +14650,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B33" s="15">
         <v>503</v>
@@ -14709,7 +14716,7 @@
     </row>
     <row r="34" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="42" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B34" s="15">
         <v>503</v>
@@ -14747,7 +14754,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="L34" s="43" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="M34" s="15"/>
       <c r="N34" s="15"/>
@@ -14777,7 +14784,7 @@
     </row>
     <row r="35" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B35" s="15">
         <v>504</v>
@@ -14843,7 +14850,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B36" s="15">
         <v>504</v>
@@ -14909,7 +14916,7 @@
     </row>
     <row r="37" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
@@ -14935,7 +14942,7 @@
     </row>
     <row r="38" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B38" s="15">
         <v>505</v>
@@ -15001,7 +15008,7 @@
     </row>
     <row r="39" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B39" s="15">
         <v>505</v>
@@ -15067,7 +15074,7 @@
     </row>
     <row r="40" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B40" s="15">
         <v>505</v>
@@ -15133,7 +15140,7 @@
     </row>
     <row r="41" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B41" s="15">
         <v>505</v>
@@ -15199,7 +15206,7 @@
     </row>
     <row r="42" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B42" s="15">
         <v>506</v>
@@ -15265,7 +15272,7 @@
     </row>
     <row r="43" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B43" s="15">
         <v>506</v>
@@ -15295,7 +15302,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="L43" s="44" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M43" s="15"/>
       <c r="N43" s="15"/>
@@ -15325,7 +15332,7 @@
     </row>
     <row r="44" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B44" s="15">
         <v>506</v>
@@ -15355,7 +15362,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="L44" s="44" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M44" s="15"/>
       <c r="N44" s="15"/>
@@ -16201,7 +16208,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="65" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -16227,8 +16234,8 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
-        <v>118</v>
+      <c r="A3" s="64" t="s">
+        <v>117</v>
       </c>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
@@ -16241,8 +16248,8 @@
       <c r="J3" s="48"/>
       <c r="K3" s="49"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="47" t="s">
-        <v>119</v>
+      <c r="M3" s="63" t="s">
+        <v>118</v>
       </c>
       <c r="N3" s="48"/>
       <c r="O3" s="48"/>
@@ -16256,7 +16263,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>20</v>
@@ -16271,22 +16278,22 @@
         <v>8</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>126</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>20</v>
@@ -16301,27 +16308,27 @@
         <v>8</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -16347,7 +16354,7 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B6" s="15">
         <v>507</v>
@@ -16413,7 +16420,7 @@
     </row>
     <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B7" s="15">
         <v>507</v>
@@ -16479,7 +16486,7 @@
     </row>
     <row r="8" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B8" s="15">
         <v>508</v>
@@ -16545,7 +16552,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -16571,7 +16578,7 @@
     </row>
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B10" s="15">
         <v>509</v>
@@ -16637,7 +16644,7 @@
     </row>
     <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B11" s="15">
         <v>510</v>
@@ -16703,7 +16710,7 @@
     </row>
     <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B12" s="15">
         <v>512</v>
@@ -16769,7 +16776,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -16795,7 +16802,7 @@
     </row>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B14" s="15">
         <v>513</v>
@@ -16861,7 +16868,7 @@
     </row>
     <row r="15" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B15" s="15">
         <v>514</v>
@@ -16927,7 +16934,7 @@
     </row>
     <row r="16" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B16" s="15">
         <v>515</v>
@@ -16993,7 +17000,7 @@
     </row>
     <row r="17" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B17" s="15">
         <v>516</v>
@@ -17059,7 +17066,7 @@
     </row>
     <row r="18" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B18" s="15">
         <v>516</v>
@@ -17125,7 +17132,7 @@
     </row>
     <row r="19" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B19" s="15">
         <v>517</v>
@@ -17191,7 +17198,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -17217,7 +17224,7 @@
     </row>
     <row r="21" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B21" s="15">
         <v>518</v>
@@ -17283,7 +17290,7 @@
     </row>
     <row r="22" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B22" s="15">
         <v>518</v>
@@ -17349,7 +17356,7 @@
     </row>
     <row r="23" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B23" s="15">
         <v>519</v>
@@ -17383,7 +17390,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="L23" s="44" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M23" s="15"/>
       <c r="N23" s="15"/>
@@ -17413,7 +17420,7 @@
     </row>
     <row r="24" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B24" s="15">
         <v>520</v>
@@ -17479,7 +17486,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -17505,7 +17512,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B26" s="15">
         <v>521</v>
@@ -17571,7 +17578,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B27" s="15">
         <v>521</v>
@@ -17637,7 +17644,7 @@
     </row>
     <row r="28" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B28" s="15">
         <v>522</v>
@@ -17703,7 +17710,7 @@
     </row>
     <row r="29" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B29" s="15">
         <v>523</v>
@@ -17769,7 +17776,7 @@
     </row>
     <row r="30" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B30" s="15">
         <v>524</v>
@@ -17835,7 +17842,7 @@
     </row>
     <row r="31" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B31" s="15">
         <v>525</v>
@@ -17901,7 +17908,7 @@
     </row>
     <row r="32" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B32" s="15">
         <v>525</v>
@@ -17967,7 +17974,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -17993,7 +18000,7 @@
     </row>
     <row r="34" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B34" s="15">
         <v>526</v>
@@ -18059,7 +18066,7 @@
     </row>
     <row r="35" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B35" s="15">
         <v>526</v>
@@ -18125,7 +18132,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -18151,7 +18158,7 @@
     </row>
     <row r="37" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B37" s="15">
         <v>526</v>
@@ -18217,7 +18224,7 @@
     </row>
     <row r="38" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B38" s="15">
         <v>527</v>
@@ -18283,7 +18290,7 @@
     </row>
     <row r="39" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B39" s="15">
         <v>528</v>
@@ -19092,8 +19099,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
-        <v>202</v>
+      <c r="A1" s="62" t="s">
+        <v>201</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -19119,8 +19126,8 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
-        <v>118</v>
+      <c r="A3" s="64" t="s">
+        <v>117</v>
       </c>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
@@ -19133,8 +19140,8 @@
       <c r="J3" s="48"/>
       <c r="K3" s="49"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="47" t="s">
-        <v>119</v>
+      <c r="M3" s="63" t="s">
+        <v>118</v>
       </c>
       <c r="N3" s="48"/>
       <c r="O3" s="48"/>
@@ -19148,7 +19155,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>20</v>
@@ -19163,22 +19170,22 @@
         <v>8</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>126</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>20</v>
@@ -19193,27 +19200,27 @@
         <v>8</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -19239,7 +19246,7 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B6" s="15">
         <v>530</v>
@@ -19305,7 +19312,7 @@
     </row>
     <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B7" s="15">
         <v>530</v>
@@ -19371,7 +19378,7 @@
     </row>
     <row r="8" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B8" s="15">
         <v>530</v>
@@ -19437,7 +19444,7 @@
     </row>
     <row r="9" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B9" s="15">
         <v>531</v>
@@ -19503,7 +19510,7 @@
     </row>
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B10" s="15">
         <v>531</v>
@@ -19569,7 +19576,7 @@
     </row>
     <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B11" s="15">
         <v>531</v>
@@ -19635,7 +19642,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -19661,7 +19668,7 @@
     </row>
     <row r="13" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B13" s="15">
         <v>601</v>
@@ -19727,7 +19734,7 @@
     </row>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B14" s="15">
         <v>602</v>
@@ -19793,7 +19800,7 @@
     </row>
     <row r="15" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B15" s="15">
         <v>606</v>
@@ -19859,7 +19866,7 @@
     </row>
     <row r="16" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B16" s="15">
         <v>607</v>
@@ -19925,7 +19932,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -19951,7 +19958,7 @@
     </row>
     <row r="18" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B18" s="15">
         <v>609</v>
@@ -20017,7 +20024,7 @@
     </row>
     <row r="19" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B19" s="15">
         <v>610</v>
@@ -20083,7 +20090,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -20109,7 +20116,7 @@
     </row>
     <row r="21" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B21" s="15">
         <v>611</v>
@@ -20175,7 +20182,7 @@
     </row>
     <row r="22" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B22" s="15">
         <v>614</v>
@@ -20241,7 +20248,7 @@
     </row>
     <row r="23" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B23" s="15">
         <v>614</v>
@@ -20307,7 +20314,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
@@ -20333,7 +20340,7 @@
     </row>
     <row r="25" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B25" s="15">
         <v>614</v>
@@ -20399,7 +20406,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B26" s="15">
         <v>615</v>
@@ -20465,7 +20472,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B27" s="15">
         <v>615</v>
@@ -21130,8 +21137,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
-        <v>225</v>
+      <c r="A1" s="62" t="s">
+        <v>224</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -21157,8 +21164,8 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
-        <v>118</v>
+      <c r="A3" s="64" t="s">
+        <v>117</v>
       </c>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
@@ -21171,8 +21178,8 @@
       <c r="J3" s="48"/>
       <c r="K3" s="49"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="47" t="s">
-        <v>119</v>
+      <c r="M3" s="63" t="s">
+        <v>118</v>
       </c>
       <c r="N3" s="48"/>
       <c r="O3" s="48"/>
@@ -21186,7 +21193,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>20</v>
@@ -21201,22 +21208,22 @@
         <v>8</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>126</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>20</v>
@@ -21231,27 +21238,27 @@
         <v>8</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -21277,7 +21284,7 @@
     </row>
     <row r="6" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B6" s="15">
         <v>616</v>
@@ -21343,7 +21350,7 @@
     </row>
     <row r="7" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B7" s="15">
         <v>617</v>
@@ -21409,7 +21416,7 @@
     </row>
     <row r="8" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -21435,7 +21442,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B9" s="15">
         <v>618</v>
@@ -21501,7 +21508,7 @@
     </row>
     <row r="10" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B10" s="15">
         <v>618</v>
@@ -21567,7 +21574,7 @@
     </row>
     <row r="11" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B11" s="15">
         <v>618</v>
@@ -21633,7 +21640,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -21659,7 +21666,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
@@ -21715,7 +21722,7 @@
     </row>
     <row r="14" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
@@ -21771,7 +21778,7 @@
     </row>
     <row r="15" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
@@ -21827,7 +21834,7 @@
     </row>
     <row r="16" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
@@ -21883,7 +21890,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -21939,7 +21946,7 @@
     </row>
     <row r="18" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
@@ -21995,7 +22002,7 @@
     </row>
     <row r="19" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -22051,7 +22058,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -22107,7 +22114,7 @@
     </row>
     <row r="21" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -22133,7 +22140,7 @@
     </row>
     <row r="22" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -22189,7 +22196,7 @@
     </row>
     <row r="23" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -22245,7 +22252,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -22301,7 +22308,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -22357,7 +22364,7 @@
     </row>
     <row r="26" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -22413,7 +22420,7 @@
     </row>
     <row r="27" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -22469,7 +22476,7 @@
     </row>
     <row r="28" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -22525,7 +22532,7 @@
     </row>
     <row r="29" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -22551,7 +22558,7 @@
     </row>
     <row r="30" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
@@ -22607,7 +22614,7 @@
     </row>
     <row r="31" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -22663,7 +22670,7 @@
     </row>
     <row r="32" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -22719,7 +22726,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -22745,7 +22752,7 @@
     </row>
     <row r="34" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
@@ -22801,7 +22808,7 @@
     </row>
     <row r="35" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -22857,7 +22864,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
@@ -22913,7 +22920,7 @@
     </row>
     <row r="37" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>
@@ -22969,7 +22976,7 @@
     </row>
     <row r="38" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-20 19:42:16
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FF6858-418B-46C2-B3EE-8E0957E38028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2502D9-047E-4C3A-A580-858D85DB98B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1436,14 +1436,14 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1469,16 +1469,16 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1487,7 +1487,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1507,6 +1507,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FFFFEB9C"/>
         </patternFill>
@@ -1531,6 +1539,22 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
@@ -1579,6 +1603,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FFFFEB9C"/>
         </patternFill>
@@ -1611,6 +1643,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
@@ -1619,6 +1659,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
@@ -1645,54 +1693,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -9406,7 +9406,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="67" t="s">
         <v>127</v>
       </c>
       <c r="B1" s="55"/>
@@ -9429,12 +9429,12 @@
       </c>
       <c r="D3" s="59"/>
       <c r="E3" s="60"/>
-      <c r="F3" s="68" t="s">
+      <c r="F3" s="70" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="59"/>
       <c r="H3" s="60"/>
-      <c r="I3" s="70" t="s">
+      <c r="I3" s="69" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="59"/>
@@ -9476,7 +9476,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="68" t="s">
         <v>53</v>
       </c>
       <c r="B5" s="59"/>
@@ -9814,7 +9814,7 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="67" t="s">
+      <c r="A17" s="68" t="s">
         <v>73</v>
       </c>
       <c r="B17" s="59"/>
@@ -10052,7 +10052,7 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="67" t="s">
+      <c r="A26" s="68" t="s">
         <v>80</v>
       </c>
       <c r="B26" s="59"/>
@@ -10391,7 +10391,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="69" t="s">
+      <c r="A39" s="73" t="s">
         <v>156</v>
       </c>
       <c r="B39" s="55"/>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="D41" s="59"/>
       <c r="E41" s="60"/>
-      <c r="F41" s="68" t="s">
+      <c r="F41" s="70" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="59"/>
@@ -10427,7 +10427,7 @@
       </c>
       <c r="J41" s="59"/>
       <c r="K41" s="60"/>
-      <c r="L41" s="70" t="s">
+      <c r="L41" s="69" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="59"/>
@@ -10478,7 +10478,7 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="67" t="s">
+      <c r="A43" s="68" t="s">
         <v>53</v>
       </c>
       <c r="B43" s="59"/>
@@ -10914,7 +10914,7 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="67" t="s">
+      <c r="A55" s="68" t="s">
         <v>73</v>
       </c>
       <c r="B55" s="59"/>
@@ -11221,7 +11221,7 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="67" t="s">
+      <c r="A64" s="68" t="s">
         <v>80</v>
       </c>
       <c r="B64" s="59"/>
@@ -11659,7 +11659,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="69" t="s">
+      <c r="A77" s="73" t="s">
         <v>158</v>
       </c>
       <c r="B77" s="55"/>
@@ -11682,12 +11682,12 @@
       </c>
       <c r="D79" s="59"/>
       <c r="E79" s="60"/>
-      <c r="F79" s="68" t="s">
+      <c r="F79" s="70" t="s">
         <v>156</v>
       </c>
       <c r="G79" s="59"/>
       <c r="H79" s="60"/>
-      <c r="I79" s="70" t="s">
+      <c r="I79" s="69" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="59"/>
@@ -11729,7 +11729,7 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="67" t="s">
+      <c r="A81" s="68" t="s">
         <v>53</v>
       </c>
       <c r="B81" s="59"/>
@@ -12192,7 +12192,7 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="67" t="s">
+      <c r="A93" s="68" t="s">
         <v>73</v>
       </c>
       <c r="B93" s="59"/>
@@ -12520,7 +12520,7 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="67" t="s">
+      <c r="A102" s="68" t="s">
         <v>80</v>
       </c>
       <c r="B102" s="59"/>
@@ -12980,6 +12980,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -12996,12 +13002,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -16641,7 +16641,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="67" t="s">
         <v>212</v>
       </c>
       <c r="B1" s="55"/>
@@ -22300,7 +22300,9 @@
       <c r="A16" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="B16" s="15"/>
+      <c r="B16" s="15">
+        <v>620</v>
+      </c>
       <c r="C16" s="15"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15" t="str">
@@ -24154,6 +24156,9 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.39997558519241921"/>
+  </sheetPr>
   <dimension ref="A1:X23"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
@@ -24169,7 +24174,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24199,35 +24204,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="57" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="56" t="s">
+      <c r="G3" s="57" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="56" t="s">
+      <c r="L3" s="57" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="56" t="s">
+      <c r="Q3" s="57" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="54" t="s">
+      <c r="V3" s="56" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>
@@ -25491,11 +25496,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K21">
-    <cfRule type="cellIs" dxfId="23" priority="11" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="10" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="23" priority="10" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="11" operator="between">
+      <formula>0.8</formula>
       <formula>0.9</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="21" priority="12" operator="lessThan">
@@ -25530,24 +25535,24 @@
     <cfRule type="cellIs" dxfId="14" priority="25" operator="greaterThanOrEqual">
       <formula>0.9</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="27" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="26" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
+    <cfRule type="cellIs" dxfId="13" priority="26" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="27" operator="lessThan">
+      <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U5:U21">
-    <cfRule type="cellIs" dxfId="11" priority="30" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="28" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="29" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
+    <cfRule type="cellIs" dxfId="11" priority="28" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="29" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="30" operator="lessThan">
+      <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U23">
@@ -25575,15 +25580,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X23">
-    <cfRule type="cellIs" dxfId="2" priority="45" operator="lessThan">
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="43" operator="greaterThanOrEqual">
-      <formula>0.9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="44" operator="between">
-      <formula>0.8</formula>
-      <formula>0.9</formula>
+    <cfRule type="cellIs" dxfId="2" priority="43" operator="greaterThanOrEqual">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="44" operator="between">
+      <formula>0.8</formula>
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="45" operator="lessThan">
+      <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-21 11:47:32
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2502D9-047E-4C3A-A580-858D85DB98B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642F5922-017B-4145-AD3E-47993928C4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1436,21 +1436,21 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1490,13 +1490,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7528,13 +7528,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="60" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="58"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8039,13 +8039,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="59"/>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="B41" s="57"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8526,13 +8526,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="58" t="s">
+      <c r="A83" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="59"/>
-      <c r="C83" s="59"/>
-      <c r="D83" s="59"/>
-      <c r="E83" s="60"/>
+      <c r="B83" s="57"/>
+      <c r="C83" s="57"/>
+      <c r="D83" s="57"/>
+      <c r="E83" s="58"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8774,23 +8774,23 @@
       <c r="C3" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
       <c r="F3" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="59"/>
-      <c r="N3" s="60"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="58"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9427,18 +9427,18 @@
       <c r="C3" s="72" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
       <c r="F3" s="70" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9479,16 +9479,16 @@
       <c r="A5" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="60"/>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9817,16 +9817,16 @@
       <c r="A17" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="60"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="58"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10055,16 +10055,16 @@
       <c r="A26" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="60"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="58"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10415,23 +10415,23 @@
       <c r="C41" s="72" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
       <c r="F41" s="70" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="59"/>
-      <c r="H41" s="60"/>
+      <c r="G41" s="57"/>
+      <c r="H41" s="58"/>
       <c r="I41" s="71" t="s">
         <v>157</v>
       </c>
-      <c r="J41" s="59"/>
-      <c r="K41" s="60"/>
+      <c r="J41" s="57"/>
+      <c r="K41" s="58"/>
       <c r="L41" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="59"/>
-      <c r="N41" s="60"/>
+      <c r="M41" s="57"/>
+      <c r="N41" s="58"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10481,19 +10481,19 @@
       <c r="A43" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="59"/>
-      <c r="C43" s="59"/>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="59"/>
-      <c r="I43" s="59"/>
-      <c r="J43" s="59"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="60"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="57"/>
+      <c r="J43" s="57"/>
+      <c r="K43" s="57"/>
+      <c r="L43" s="57"/>
+      <c r="M43" s="57"/>
+      <c r="N43" s="58"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10917,19 +10917,19 @@
       <c r="A55" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="59"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="F55" s="59"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="59"/>
-      <c r="I55" s="59"/>
-      <c r="J55" s="59"/>
-      <c r="K55" s="59"/>
-      <c r="L55" s="59"/>
-      <c r="M55" s="59"/>
-      <c r="N55" s="60"/>
+      <c r="B55" s="57"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="57"/>
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="57"/>
+      <c r="I55" s="57"/>
+      <c r="J55" s="57"/>
+      <c r="K55" s="57"/>
+      <c r="L55" s="57"/>
+      <c r="M55" s="57"/>
+      <c r="N55" s="58"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11224,19 +11224,19 @@
       <c r="A64" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="59"/>
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-      <c r="F64" s="59"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="59"/>
-      <c r="I64" s="59"/>
-      <c r="J64" s="59"/>
-      <c r="K64" s="59"/>
-      <c r="L64" s="59"/>
-      <c r="M64" s="59"/>
-      <c r="N64" s="60"/>
+      <c r="B64" s="57"/>
+      <c r="C64" s="57"/>
+      <c r="D64" s="57"/>
+      <c r="E64" s="57"/>
+      <c r="F64" s="57"/>
+      <c r="G64" s="57"/>
+      <c r="H64" s="57"/>
+      <c r="I64" s="57"/>
+      <c r="J64" s="57"/>
+      <c r="K64" s="57"/>
+      <c r="L64" s="57"/>
+      <c r="M64" s="57"/>
+      <c r="N64" s="58"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11680,18 +11680,18 @@
       <c r="C79" s="72" t="s">
         <v>159</v>
       </c>
-      <c r="D79" s="59"/>
-      <c r="E79" s="60"/>
+      <c r="D79" s="57"/>
+      <c r="E79" s="58"/>
       <c r="F79" s="70" t="s">
         <v>156</v>
       </c>
-      <c r="G79" s="59"/>
-      <c r="H79" s="60"/>
+      <c r="G79" s="57"/>
+      <c r="H79" s="58"/>
       <c r="I79" s="69" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="59"/>
-      <c r="K79" s="60"/>
+      <c r="J79" s="57"/>
+      <c r="K79" s="58"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11732,16 +11732,16 @@
       <c r="A81" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="59"/>
-      <c r="C81" s="59"/>
-      <c r="D81" s="59"/>
-      <c r="E81" s="59"/>
-      <c r="F81" s="59"/>
-      <c r="G81" s="59"/>
-      <c r="H81" s="59"/>
-      <c r="I81" s="59"/>
-      <c r="J81" s="59"/>
-      <c r="K81" s="60"/>
+      <c r="B81" s="57"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12195,16 +12195,16 @@
       <c r="A93" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="59"/>
-      <c r="C93" s="59"/>
-      <c r="D93" s="59"/>
-      <c r="E93" s="59"/>
-      <c r="F93" s="59"/>
-      <c r="G93" s="59"/>
-      <c r="H93" s="59"/>
-      <c r="I93" s="59"/>
-      <c r="J93" s="59"/>
-      <c r="K93" s="60"/>
+      <c r="B93" s="57"/>
+      <c r="C93" s="57"/>
+      <c r="D93" s="57"/>
+      <c r="E93" s="57"/>
+      <c r="F93" s="57"/>
+      <c r="G93" s="57"/>
+      <c r="H93" s="57"/>
+      <c r="I93" s="57"/>
+      <c r="J93" s="57"/>
+      <c r="K93" s="58"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12523,16 +12523,16 @@
       <c r="A102" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="59"/>
-      <c r="C102" s="59"/>
-      <c r="D102" s="59"/>
-      <c r="E102" s="59"/>
-      <c r="F102" s="59"/>
-      <c r="G102" s="59"/>
-      <c r="H102" s="59"/>
-      <c r="I102" s="59"/>
-      <c r="J102" s="59"/>
-      <c r="K102" s="60"/>
+      <c r="B102" s="57"/>
+      <c r="C102" s="57"/>
+      <c r="D102" s="57"/>
+      <c r="E102" s="57"/>
+      <c r="F102" s="57"/>
+      <c r="G102" s="57"/>
+      <c r="H102" s="57"/>
+      <c r="I102" s="57"/>
+      <c r="J102" s="57"/>
+      <c r="K102" s="58"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13395,7 +13395,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>160</v>
       </c>
       <c r="B1" s="55"/>
@@ -13422,32 +13422,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16668,32 +16668,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19533,7 +19533,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>248</v>
       </c>
       <c r="B1" s="55"/>
@@ -19560,32 +19560,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21571,7 +21571,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>271</v>
       </c>
       <c r="B1" s="55"/>
@@ -21598,32 +21598,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -22303,29 +22303,37 @@
       <c r="B16" s="15">
         <v>620</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15" t="str">
+      <c r="C16" s="15">
+        <v>31</v>
+      </c>
+      <c r="D16" s="15">
+        <v>28</v>
+      </c>
+      <c r="E16" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15" t="str">
+        <v>0.90322580645161288</v>
+      </c>
+      <c r="F16" s="15">
+        <v>10</v>
+      </c>
+      <c r="G16" s="15">
+        <v>8</v>
+      </c>
+      <c r="H16" s="15">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="I16" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J16" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="K16" s="15" t="e">
+        <v>20</v>
+      </c>
+      <c r="K16" s="15">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.95238095238095233</v>
       </c>
       <c r="L16" s="11"/>
       <c r="M16" s="15"/>
@@ -22424,7 +22432,7 @@
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
       <c r="H18" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(AND(F18&lt;&gt;"",G18&lt;&gt;""),G18/F18,"")</f>
         <v/>
       </c>
       <c r="I18" s="15">
@@ -22432,7 +22440,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="15">
-        <f t="shared" si="4"/>
+        <f>D18-G18</f>
         <v>0</v>
       </c>
       <c r="K18" s="15" t="e">
@@ -22480,7 +22488,7 @@
       <c r="F19" s="15"/>
       <c r="G19" s="15"/>
       <c r="H19" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(AND(F19&lt;&gt;"",G19&lt;&gt;""),G19/F19,"")</f>
         <v/>
       </c>
       <c r="I19" s="15">
@@ -22488,7 +22496,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="15">
-        <f t="shared" si="4"/>
+        <f>D19-G19</f>
         <v>0</v>
       </c>
       <c r="K19" s="15" t="e">
@@ -23503,39 +23511,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>96</v>
+        <v>124</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.8</v>
+        <v>0.82119205298013243</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.87096774193548387</v>
+        <v>0.85365853658536583</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.7752808988764045</v>
+        <v>0.80909090909090908</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23584,39 +23592,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>96</v>
+        <v>124</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.8</v>
+        <v>0.82119205298013243</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.87096774193548387</v>
+        <v>0.85365853658536583</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.7752808988764045</v>
+        <v>0.80909090909090908</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
@@ -24174,7 +24182,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24204,35 +24212,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="76" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="76" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="57" t="s">
+      <c r="L3" s="76" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="57" t="s">
+      <c r="Q3" s="76" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="56" t="s">
+      <c r="V3" s="75" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-21 16:52:22
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642F5922-017B-4145-AD3E-47993928C4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A52CDD89-50C7-4D31-BE25-350CD2E630F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1469,25 +1469,25 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9406,7 +9406,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="72" t="s">
         <v>127</v>
       </c>
       <c r="B1" s="55"/>
@@ -9424,17 +9424,17 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="72" t="s">
+      <c r="C3" s="67" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="57"/>
       <c r="E3" s="58"/>
-      <c r="F3" s="70" t="s">
+      <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="57"/>
       <c r="H3" s="58"/>
-      <c r="I3" s="69" t="s">
+      <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="57"/>
@@ -10391,7 +10391,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="70" t="s">
         <v>156</v>
       </c>
       <c r="B39" s="55"/>
@@ -10412,22 +10412,22 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="72" t="s">
+      <c r="C41" s="67" t="s">
         <v>52</v>
       </c>
       <c r="D41" s="57"/>
       <c r="E41" s="58"/>
-      <c r="F41" s="70" t="s">
+      <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="57"/>
       <c r="H41" s="58"/>
-      <c r="I41" s="71" t="s">
+      <c r="I41" s="73" t="s">
         <v>157</v>
       </c>
       <c r="J41" s="57"/>
       <c r="K41" s="58"/>
-      <c r="L41" s="69" t="s">
+      <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="57"/>
@@ -11659,7 +11659,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="73" t="s">
+      <c r="A77" s="70" t="s">
         <v>158</v>
       </c>
       <c r="B77" s="55"/>
@@ -11677,17 +11677,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="72" t="s">
+      <c r="C79" s="67" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="57"/>
       <c r="E79" s="58"/>
-      <c r="F79" s="70" t="s">
+      <c r="F79" s="69" t="s">
         <v>156</v>
       </c>
       <c r="G79" s="57"/>
       <c r="H79" s="58"/>
-      <c r="I79" s="69" t="s">
+      <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="57"/>
@@ -12980,12 +12980,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13002,6 +12996,12 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -16641,7 +16641,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="72" t="s">
         <v>212</v>
       </c>
       <c r="B1" s="55"/>
@@ -22366,30 +22366,40 @@
       <c r="A17" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15" t="str">
+      <c r="B17" s="15">
+        <v>621</v>
+      </c>
+      <c r="C17" s="15">
+        <v>21</v>
+      </c>
+      <c r="D17" s="15">
+        <v>21</v>
+      </c>
+      <c r="E17" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F17" s="15">
+        <v>2</v>
+      </c>
+      <c r="G17" s="15">
+        <v>2</v>
+      </c>
+      <c r="H17" s="15">
         <f t="shared" si="3"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I17" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="K17" s="15" t="e">
+        <v>19</v>
+      </c>
+      <c r="K17" s="15">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="L17" s="11"/>
       <c r="M17" s="15"/>
@@ -23511,39 +23521,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.82119205298013243</v>
+        <v>0.84302325581395354</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.85365853658536583</v>
+        <v>0.86046511627906974</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.80909090909090908</v>
+        <v>0.83720930232558144</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23592,39 +23602,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.82119205298013243</v>
+        <v>0.84302325581395354</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.85365853658536583</v>
+        <v>0.86046511627906974</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.80909090909090908</v>
+        <v>0.83720930232558144</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-22 17:10:29
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A52CDD89-50C7-4D31-BE25-350CD2E630F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6856F19-2CF2-4B49-A2A4-1DCD57165205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1436,21 +1436,21 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1490,13 +1490,13 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7528,13 +7528,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="60"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8039,13 +8039,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="60" t="s">
+      <c r="A41" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="57"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8526,13 +8526,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="60" t="s">
+      <c r="A83" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="57"/>
-      <c r="C83" s="57"/>
-      <c r="D83" s="57"/>
-      <c r="E83" s="58"/>
+      <c r="B83" s="59"/>
+      <c r="C83" s="59"/>
+      <c r="D83" s="59"/>
+      <c r="E83" s="60"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8774,23 +8774,23 @@
       <c r="C3" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
       <c r="I3" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="58"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="60"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9427,18 +9427,18 @@
       <c r="C3" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
       <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9479,16 +9479,16 @@
       <c r="A5" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9817,16 +9817,16 @@
       <c r="A17" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="57"/>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="58"/>
+      <c r="B17" s="59"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="60"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10055,16 +10055,16 @@
       <c r="A26" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="57"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="58"/>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="60"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10415,23 +10415,23 @@
       <c r="C41" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
       <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="57"/>
-      <c r="H41" s="58"/>
+      <c r="G41" s="59"/>
+      <c r="H41" s="60"/>
       <c r="I41" s="73" t="s">
         <v>157</v>
       </c>
-      <c r="J41" s="57"/>
-      <c r="K41" s="58"/>
+      <c r="J41" s="59"/>
+      <c r="K41" s="60"/>
       <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="57"/>
-      <c r="N41" s="58"/>
+      <c r="M41" s="59"/>
+      <c r="N41" s="60"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10481,19 +10481,19 @@
       <c r="A43" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="57"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="57"/>
-      <c r="N43" s="58"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
+      <c r="H43" s="59"/>
+      <c r="I43" s="59"/>
+      <c r="J43" s="59"/>
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
+      <c r="M43" s="59"/>
+      <c r="N43" s="60"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10917,19 +10917,19 @@
       <c r="A55" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="57"/>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="57"/>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
-      <c r="I55" s="57"/>
-      <c r="J55" s="57"/>
-      <c r="K55" s="57"/>
-      <c r="L55" s="57"/>
-      <c r="M55" s="57"/>
-      <c r="N55" s="58"/>
+      <c r="B55" s="59"/>
+      <c r="C55" s="59"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="59"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="59"/>
+      <c r="K55" s="59"/>
+      <c r="L55" s="59"/>
+      <c r="M55" s="59"/>
+      <c r="N55" s="60"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11224,19 +11224,19 @@
       <c r="A64" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="57"/>
-      <c r="H64" s="57"/>
-      <c r="I64" s="57"/>
-      <c r="J64" s="57"/>
-      <c r="K64" s="57"/>
-      <c r="L64" s="57"/>
-      <c r="M64" s="57"/>
-      <c r="N64" s="58"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="59"/>
+      <c r="D64" s="59"/>
+      <c r="E64" s="59"/>
+      <c r="F64" s="59"/>
+      <c r="G64" s="59"/>
+      <c r="H64" s="59"/>
+      <c r="I64" s="59"/>
+      <c r="J64" s="59"/>
+      <c r="K64" s="59"/>
+      <c r="L64" s="59"/>
+      <c r="M64" s="59"/>
+      <c r="N64" s="60"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11680,18 +11680,18 @@
       <c r="C79" s="67" t="s">
         <v>159</v>
       </c>
-      <c r="D79" s="57"/>
-      <c r="E79" s="58"/>
+      <c r="D79" s="59"/>
+      <c r="E79" s="60"/>
       <c r="F79" s="69" t="s">
         <v>156</v>
       </c>
-      <c r="G79" s="57"/>
-      <c r="H79" s="58"/>
+      <c r="G79" s="59"/>
+      <c r="H79" s="60"/>
       <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="57"/>
-      <c r="K79" s="58"/>
+      <c r="J79" s="59"/>
+      <c r="K79" s="60"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11732,16 +11732,16 @@
       <c r="A81" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="57"/>
-      <c r="C81" s="57"/>
-      <c r="D81" s="57"/>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="57"/>
-      <c r="J81" s="57"/>
-      <c r="K81" s="58"/>
+      <c r="B81" s="59"/>
+      <c r="C81" s="59"/>
+      <c r="D81" s="59"/>
+      <c r="E81" s="59"/>
+      <c r="F81" s="59"/>
+      <c r="G81" s="59"/>
+      <c r="H81" s="59"/>
+      <c r="I81" s="59"/>
+      <c r="J81" s="59"/>
+      <c r="K81" s="60"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12195,16 +12195,16 @@
       <c r="A93" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="57"/>
-      <c r="C93" s="57"/>
-      <c r="D93" s="57"/>
-      <c r="E93" s="57"/>
-      <c r="F93" s="57"/>
-      <c r="G93" s="57"/>
-      <c r="H93" s="57"/>
-      <c r="I93" s="57"/>
-      <c r="J93" s="57"/>
-      <c r="K93" s="58"/>
+      <c r="B93" s="59"/>
+      <c r="C93" s="59"/>
+      <c r="D93" s="59"/>
+      <c r="E93" s="59"/>
+      <c r="F93" s="59"/>
+      <c r="G93" s="59"/>
+      <c r="H93" s="59"/>
+      <c r="I93" s="59"/>
+      <c r="J93" s="59"/>
+      <c r="K93" s="60"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12523,16 +12523,16 @@
       <c r="A102" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="57"/>
-      <c r="C102" s="57"/>
-      <c r="D102" s="57"/>
-      <c r="E102" s="57"/>
-      <c r="F102" s="57"/>
-      <c r="G102" s="57"/>
-      <c r="H102" s="57"/>
-      <c r="I102" s="57"/>
-      <c r="J102" s="57"/>
-      <c r="K102" s="58"/>
+      <c r="B102" s="59"/>
+      <c r="C102" s="59"/>
+      <c r="D102" s="59"/>
+      <c r="E102" s="59"/>
+      <c r="F102" s="59"/>
+      <c r="G102" s="59"/>
+      <c r="H102" s="59"/>
+      <c r="I102" s="59"/>
+      <c r="J102" s="59"/>
+      <c r="K102" s="60"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13395,7 +13395,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>160</v>
       </c>
       <c r="B1" s="55"/>
@@ -13422,32 +13422,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16668,32 +16668,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19533,7 +19533,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>248</v>
       </c>
       <c r="B1" s="55"/>
@@ -19560,32 +19560,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21571,7 +21571,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>271</v>
       </c>
       <c r="B1" s="55"/>
@@ -21598,32 +21598,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -22432,7 +22432,9 @@
       <c r="A18" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="B18" s="15"/>
+      <c r="B18" s="15">
+        <v>622</v>
+      </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="15" t="str">
@@ -24192,7 +24194,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24222,35 +24224,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="57" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="76" t="s">
+      <c r="G3" s="57" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="76" t="s">
+      <c r="L3" s="57" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="76" t="s">
+      <c r="Q3" s="57" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="75" t="s">
+      <c r="V3" s="56" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>
@@ -24682,15 +24684,21 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q9" s="48"/>
-      <c r="R9" s="48"/>
+      <c r="Q9" s="48">
+        <v>6.21</v>
+      </c>
+      <c r="R9" s="48">
+        <v>20</v>
+      </c>
       <c r="S9" s="48">
         <v>5</v>
       </c>
-      <c r="T9" s="48"/>
-      <c r="U9" s="48" t="str">
+      <c r="T9" s="48">
+        <v>2</v>
+      </c>
+      <c r="U9" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="V9" s="48">
         <f t="shared" si="4"/>
@@ -24698,11 +24706,11 @@
       </c>
       <c r="W9" s="48">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="X9" s="48">
         <f t="shared" si="6"/>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25386,11 +25394,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>2.5000000000000001E-2</v>
+        <v>0.05</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25398,11 +25406,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>5.6250000000000001E-2</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25460,11 +25468,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>2.5000000000000001E-2</v>
+        <v>0.05</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -25472,11 +25480,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>5.6250000000000001E-2</v>
+        <v>6.25E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-06-23 15:54:15
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6856F19-2CF2-4B49-A2A4-1DCD57165205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998E818E-94EC-4F71-AF87-7EFB1337A1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1436,21 +1436,21 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1490,13 +1490,13 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7528,13 +7528,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="60" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="58"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8039,13 +8039,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="59"/>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="B41" s="57"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8526,13 +8526,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="58" t="s">
+      <c r="A83" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="59"/>
-      <c r="C83" s="59"/>
-      <c r="D83" s="59"/>
-      <c r="E83" s="60"/>
+      <c r="B83" s="57"/>
+      <c r="C83" s="57"/>
+      <c r="D83" s="57"/>
+      <c r="E83" s="58"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8774,23 +8774,23 @@
       <c r="C3" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
       <c r="F3" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="59"/>
-      <c r="N3" s="60"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="58"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9427,18 +9427,18 @@
       <c r="C3" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
       <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9479,16 +9479,16 @@
       <c r="A5" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="60"/>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9817,16 +9817,16 @@
       <c r="A17" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="60"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="58"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10055,16 +10055,16 @@
       <c r="A26" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="60"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="58"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10415,23 +10415,23 @@
       <c r="C41" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
       <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="59"/>
-      <c r="H41" s="60"/>
+      <c r="G41" s="57"/>
+      <c r="H41" s="58"/>
       <c r="I41" s="73" t="s">
         <v>157</v>
       </c>
-      <c r="J41" s="59"/>
-      <c r="K41" s="60"/>
+      <c r="J41" s="57"/>
+      <c r="K41" s="58"/>
       <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="59"/>
-      <c r="N41" s="60"/>
+      <c r="M41" s="57"/>
+      <c r="N41" s="58"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10481,19 +10481,19 @@
       <c r="A43" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="59"/>
-      <c r="C43" s="59"/>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="59"/>
-      <c r="I43" s="59"/>
-      <c r="J43" s="59"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="60"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="57"/>
+      <c r="J43" s="57"/>
+      <c r="K43" s="57"/>
+      <c r="L43" s="57"/>
+      <c r="M43" s="57"/>
+      <c r="N43" s="58"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10917,19 +10917,19 @@
       <c r="A55" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="59"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="F55" s="59"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="59"/>
-      <c r="I55" s="59"/>
-      <c r="J55" s="59"/>
-      <c r="K55" s="59"/>
-      <c r="L55" s="59"/>
-      <c r="M55" s="59"/>
-      <c r="N55" s="60"/>
+      <c r="B55" s="57"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="57"/>
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="57"/>
+      <c r="I55" s="57"/>
+      <c r="J55" s="57"/>
+      <c r="K55" s="57"/>
+      <c r="L55" s="57"/>
+      <c r="M55" s="57"/>
+      <c r="N55" s="58"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11224,19 +11224,19 @@
       <c r="A64" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="59"/>
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-      <c r="F64" s="59"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="59"/>
-      <c r="I64" s="59"/>
-      <c r="J64" s="59"/>
-      <c r="K64" s="59"/>
-      <c r="L64" s="59"/>
-      <c r="M64" s="59"/>
-      <c r="N64" s="60"/>
+      <c r="B64" s="57"/>
+      <c r="C64" s="57"/>
+      <c r="D64" s="57"/>
+      <c r="E64" s="57"/>
+      <c r="F64" s="57"/>
+      <c r="G64" s="57"/>
+      <c r="H64" s="57"/>
+      <c r="I64" s="57"/>
+      <c r="J64" s="57"/>
+      <c r="K64" s="57"/>
+      <c r="L64" s="57"/>
+      <c r="M64" s="57"/>
+      <c r="N64" s="58"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11680,18 +11680,18 @@
       <c r="C79" s="67" t="s">
         <v>159</v>
       </c>
-      <c r="D79" s="59"/>
-      <c r="E79" s="60"/>
+      <c r="D79" s="57"/>
+      <c r="E79" s="58"/>
       <c r="F79" s="69" t="s">
         <v>156</v>
       </c>
-      <c r="G79" s="59"/>
-      <c r="H79" s="60"/>
+      <c r="G79" s="57"/>
+      <c r="H79" s="58"/>
       <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="59"/>
-      <c r="K79" s="60"/>
+      <c r="J79" s="57"/>
+      <c r="K79" s="58"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11732,16 +11732,16 @@
       <c r="A81" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="59"/>
-      <c r="C81" s="59"/>
-      <c r="D81" s="59"/>
-      <c r="E81" s="59"/>
-      <c r="F81" s="59"/>
-      <c r="G81" s="59"/>
-      <c r="H81" s="59"/>
-      <c r="I81" s="59"/>
-      <c r="J81" s="59"/>
-      <c r="K81" s="60"/>
+      <c r="B81" s="57"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12195,16 +12195,16 @@
       <c r="A93" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="59"/>
-      <c r="C93" s="59"/>
-      <c r="D93" s="59"/>
-      <c r="E93" s="59"/>
-      <c r="F93" s="59"/>
-      <c r="G93" s="59"/>
-      <c r="H93" s="59"/>
-      <c r="I93" s="59"/>
-      <c r="J93" s="59"/>
-      <c r="K93" s="60"/>
+      <c r="B93" s="57"/>
+      <c r="C93" s="57"/>
+      <c r="D93" s="57"/>
+      <c r="E93" s="57"/>
+      <c r="F93" s="57"/>
+      <c r="G93" s="57"/>
+      <c r="H93" s="57"/>
+      <c r="I93" s="57"/>
+      <c r="J93" s="57"/>
+      <c r="K93" s="58"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12523,16 +12523,16 @@
       <c r="A102" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="59"/>
-      <c r="C102" s="59"/>
-      <c r="D102" s="59"/>
-      <c r="E102" s="59"/>
-      <c r="F102" s="59"/>
-      <c r="G102" s="59"/>
-      <c r="H102" s="59"/>
-      <c r="I102" s="59"/>
-      <c r="J102" s="59"/>
-      <c r="K102" s="60"/>
+      <c r="B102" s="57"/>
+      <c r="C102" s="57"/>
+      <c r="D102" s="57"/>
+      <c r="E102" s="57"/>
+      <c r="F102" s="57"/>
+      <c r="G102" s="57"/>
+      <c r="H102" s="57"/>
+      <c r="I102" s="57"/>
+      <c r="J102" s="57"/>
+      <c r="K102" s="58"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13395,7 +13395,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>160</v>
       </c>
       <c r="B1" s="55"/>
@@ -13422,32 +13422,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16668,32 +16668,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19533,7 +19533,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>248</v>
       </c>
       <c r="B1" s="55"/>
@@ -19560,32 +19560,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21571,7 +21571,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>271</v>
       </c>
       <c r="B1" s="55"/>
@@ -21598,32 +21598,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -22435,29 +22435,37 @@
       <c r="B18" s="15">
         <v>622</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15" t="str">
+      <c r="C18" s="15">
+        <v>49</v>
+      </c>
+      <c r="D18" s="15">
+        <v>36</v>
+      </c>
+      <c r="E18" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15" t="str">
+        <v>0.73469387755102045</v>
+      </c>
+      <c r="F18" s="15">
+        <v>13</v>
+      </c>
+      <c r="G18" s="15">
+        <v>11</v>
+      </c>
+      <c r="H18" s="15">
         <f>IF(AND(F18&lt;&gt;"",G18&lt;&gt;""),G18/F18,"")</f>
-        <v/>
+        <v>0.84615384615384615</v>
       </c>
       <c r="I18" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J18" s="15">
         <f>D18-G18</f>
-        <v>0</v>
-      </c>
-      <c r="K18" s="15" t="e">
+        <v>25</v>
+      </c>
+      <c r="K18" s="15">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.69444444444444442</v>
       </c>
       <c r="L18" s="11"/>
       <c r="M18" s="15"/>
@@ -22490,30 +22498,40 @@
       <c r="A19" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15" t="str">
+      <c r="B19" s="15">
+        <v>623</v>
+      </c>
+      <c r="C19" s="15">
+        <v>12</v>
+      </c>
+      <c r="D19" s="15">
+        <v>11</v>
+      </c>
+      <c r="E19" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15" t="str">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F19" s="15">
+        <v>0</v>
+      </c>
+      <c r="G19" s="15">
+        <v>0</v>
+      </c>
+      <c r="H19" s="15" t="e">
         <f>IF(AND(F19&lt;&gt;"",G19&lt;&gt;""),G19/F19,"")</f>
-        <v/>
+        <v>#DIV/0!</v>
       </c>
       <c r="I19" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J19" s="15">
         <f>D19-G19</f>
-        <v>0</v>
-      </c>
-      <c r="K19" s="15" t="e">
+        <v>11</v>
+      </c>
+      <c r="K19" s="15">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="15"/>
@@ -22546,30 +22564,40 @@
       <c r="A20" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15" t="str">
+      <c r="B20" s="15">
+        <v>623</v>
+      </c>
+      <c r="C20" s="15">
+        <v>23</v>
+      </c>
+      <c r="D20" s="15">
+        <v>17</v>
+      </c>
+      <c r="E20" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15" t="str">
+        <v>0.73913043478260865</v>
+      </c>
+      <c r="F20" s="15">
+        <v>5</v>
+      </c>
+      <c r="G20" s="15">
+        <v>2</v>
+      </c>
+      <c r="H20" s="15">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="I20" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="K20" s="15" t="e">
+        <v>15</v>
+      </c>
+      <c r="K20" s="15">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="L20" s="11"/>
       <c r="M20" s="15"/>
@@ -23523,39 +23551,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>172</v>
+        <v>256</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>145</v>
+        <v>209</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.84302325581395354</v>
+        <v>0.81640625</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.86046511627906974</v>
+        <v>0.81967213114754101</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>129</v>
+        <v>195</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>108</v>
+        <v>159</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.83720930232558144</v>
+        <v>0.81538461538461537</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23604,39 +23632,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>172</v>
+        <v>256</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>145</v>
+        <v>209</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.84302325581395354</v>
+        <v>0.81640625</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.86046511627906974</v>
+        <v>0.81967213114754101</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>129</v>
+        <v>195</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>108</v>
+        <v>159</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.83720930232558144</v>
+        <v>0.81538461538461537</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
@@ -24194,7 +24222,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24224,35 +24252,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="76" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="76" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="57" t="s">
+      <c r="L3" s="76" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="57" t="s">
+      <c r="Q3" s="76" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="56" t="s">
+      <c r="V3" s="75" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-25 20:33:13
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998E818E-94EC-4F71-AF87-7EFB1337A1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25E65FD-ACCF-4829-BF0F-671B52A6811B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -390,581 +390,582 @@
     <t>选择题</t>
   </si>
   <si>
+    <t>问答题</t>
+  </si>
+  <si>
+    <t>第一章 函数 极限 连续</t>
+  </si>
+  <si>
+    <t>第二章 一元函数微分学</t>
+  </si>
+  <si>
+    <t>第三章 一元函数积分学</t>
+  </si>
+  <si>
+    <t>第四章 常微分方程</t>
+  </si>
+  <si>
+    <t>第五章 多元函数微分学</t>
+  </si>
+  <si>
+    <t>第六章 二重积分</t>
+  </si>
+  <si>
+    <t>第七章 无穷级数 (仅数学一、三)</t>
+  </si>
+  <si>
+    <t>第八章 向量代数与空间解析几何及多元微分学在几何上的应用 (仅数学一)</t>
+  </si>
+  <si>
+    <t>第九章 多元函数积分学及其应用 (仅数学一)</t>
+  </si>
+  <si>
+    <t>李林880 （选择&amp;填空）习题正确率记录</t>
+  </si>
+  <si>
+    <t>时间</t>
+  </si>
+  <si>
+    <t>第一章 函数、极限、连续</t>
+  </si>
+  <si>
+    <t>第二章 一元函数微分学及其应用</t>
+  </si>
+  <si>
+    <t>第三章 一元函数积分学及其应用</t>
+  </si>
+  <si>
+    <t>第四章 空间解析几何</t>
+  </si>
+  <si>
+    <t>第五章 多元函数微分学及其应用</t>
+  </si>
+  <si>
+    <t>第六章 重积分及其应用</t>
+  </si>
+  <si>
+    <t>第七章 微分方程及其应用</t>
+  </si>
+  <si>
+    <t>第八章 无穷级数</t>
+  </si>
+  <si>
+    <t>第九章 曲线积分与曲面积分</t>
+  </si>
+  <si>
+    <t>高等数学 合计</t>
+  </si>
+  <si>
+    <t>第十章 行列式</t>
+  </si>
+  <si>
+    <t>第十一章 矩阵</t>
+  </si>
+  <si>
+    <t>第十二章 向量</t>
+  </si>
+  <si>
+    <t>第十三章 线性方程组</t>
+  </si>
+  <si>
+    <t>第十四章 相似矩阵</t>
+  </si>
+  <si>
+    <t>第十五章 二次型</t>
+  </si>
+  <si>
+    <t>线性代数 合计</t>
+  </si>
+  <si>
+    <t>第十六章 随机事件及其概率</t>
+  </si>
+  <si>
+    <t>第十七章 随机变量及其分布</t>
+  </si>
+  <si>
+    <t>第十八章 多维随机变量及其分布</t>
+  </si>
+  <si>
+    <t>第十九章 随机变量的数字特征</t>
+  </si>
+  <si>
+    <t>第二十章 大数定律与中心极限定理</t>
+  </si>
+  <si>
+    <t>第二十一章 数理统计的基本概念</t>
+  </si>
+  <si>
+    <t>第二十二章 参数估计</t>
+  </si>
+  <si>
+    <t>第二十三章 假设检验</t>
+  </si>
+  <si>
+    <t>概率论与数理统计 合计</t>
+  </si>
+  <si>
+    <t>总 计</t>
+  </si>
+  <si>
+    <t>解答区</t>
+  </si>
+  <si>
+    <t>扩展篇</t>
+  </si>
+  <si>
+    <t>选填+解答总计区</t>
+  </si>
+  <si>
+    <t>选填区</t>
+  </si>
+  <si>
+    <t>王道数据结构 课后习题正确率记录</t>
+  </si>
+  <si>
+    <t>一 刷</t>
+  </si>
+  <si>
+    <t>二 刷</t>
+  </si>
+  <si>
+    <t>小节</t>
+  </si>
+  <si>
+    <t>真题总</t>
+  </si>
+  <si>
+    <t>真题正</t>
+  </si>
+  <si>
+    <t>真题率</t>
+  </si>
+  <si>
+    <t>自编总</t>
+  </si>
+  <si>
+    <t>自编正</t>
+  </si>
+  <si>
+    <t>自编率</t>
+  </si>
+  <si>
+    <t>第1章 绪论</t>
+  </si>
+  <si>
+    <t>1.1 数据结构的基本概念</t>
+  </si>
+  <si>
+    <t>1.2 算法和算法评价</t>
+  </si>
+  <si>
+    <t>第2章 线性表</t>
+  </si>
+  <si>
+    <t>2.1 线性表的定义和基本操作</t>
+  </si>
+  <si>
+    <t>2.2 线性表的顺序表示</t>
+  </si>
+  <si>
+    <t>2.3 线性表的链式表示</t>
+  </si>
+  <si>
+    <t>第3章 栈、队列和数组</t>
+  </si>
+  <si>
+    <t>3.1 栈</t>
+  </si>
+  <si>
+    <t>3.2 队列</t>
+  </si>
+  <si>
+    <t>3.3 栈和队列的应用</t>
+  </si>
+  <si>
+    <t>3.4 数组和特殊矩阵</t>
+  </si>
+  <si>
+    <t>第4章 串</t>
+  </si>
+  <si>
+    <t>4.1 串的定义和实现</t>
+  </si>
+  <si>
+    <t>4.2 串的模式匹配</t>
+  </si>
+  <si>
+    <t>第5章 树与二叉树</t>
+  </si>
+  <si>
+    <t>5.1 树的基本概念</t>
+  </si>
+  <si>
+    <t>5.2 二叉树的概念</t>
+  </si>
+  <si>
+    <t>5.3 二叉树的遍历和线索二叉树</t>
+  </si>
+  <si>
+    <t>5.4 树、森林</t>
+  </si>
+  <si>
+    <t>5.5 树与二叉树的应用</t>
+  </si>
+  <si>
+    <t>第6章 图</t>
+  </si>
+  <si>
+    <t>6.1 图的基本概念</t>
+  </si>
+  <si>
+    <t>6.2 图的存储及基本操作</t>
+  </si>
+  <si>
+    <t>6.3 图的遍历</t>
+  </si>
+  <si>
+    <t>6.4 图的应用</t>
+  </si>
+  <si>
+    <t>第7章 查找</t>
+  </si>
+  <si>
+    <t>7.1 查找的基本概念</t>
+  </si>
+  <si>
+    <t>7.2 顺序查找和折半查找</t>
+  </si>
+  <si>
+    <t>7.3 树形查找</t>
+  </si>
+  <si>
+    <t>未包含红黑树</t>
+  </si>
+  <si>
+    <t>7.4 B树和B+树</t>
+  </si>
+  <si>
+    <t>7.5 散列(Hash)表</t>
+  </si>
+  <si>
+    <t>第8章 排序</t>
+  </si>
+  <si>
+    <t>8.1 排序的基本概念</t>
+  </si>
+  <si>
+    <t>8.2 插入排序</t>
+  </si>
+  <si>
+    <t>8.3 交换排序</t>
+  </si>
+  <si>
+    <t>8.4 选择排序</t>
+  </si>
+  <si>
+    <t>8.5 归并排序、基数排序和计数排序</t>
+  </si>
+  <si>
+    <t>8.6 各种内部排序算法的比较及应用</t>
+  </si>
+  <si>
+    <t>未完成</t>
+  </si>
+  <si>
+    <t>8.7 外部排序</t>
+  </si>
+  <si>
+    <t>王道计算机组成原理 课后习题正确率记录</t>
+  </si>
+  <si>
+    <t>第1章 计算机系统概述</t>
+  </si>
+  <si>
+    <t>1.1 计算机发展历程</t>
+  </si>
+  <si>
+    <t>1.2 计算机系统层次结构</t>
+  </si>
+  <si>
+    <t>1.3 计算机的性能指标</t>
+  </si>
+  <si>
+    <t>第2章 数据的表示和运算</t>
+  </si>
+  <si>
+    <t>2.1 数制与编码</t>
+  </si>
+  <si>
+    <t>2.2 运算方法和运算电路</t>
+  </si>
+  <si>
+    <t>2.3 浮点数的表示与运算</t>
+  </si>
+  <si>
+    <t>第3章 存储系统</t>
+  </si>
+  <si>
+    <t>3.1 存储器概述</t>
+  </si>
+  <si>
+    <t>3.2 主存储器</t>
+  </si>
+  <si>
+    <t>3.3 主存储器与CPU的连接</t>
+  </si>
+  <si>
+    <t>3.4 外部存储器</t>
+  </si>
+  <si>
+    <t>3.5 高速缓冲存储器</t>
+  </si>
+  <si>
+    <t>3.6 虚拟存储器</t>
+  </si>
+  <si>
+    <t>第4章 指令系统</t>
+  </si>
+  <si>
+    <t>4.1 指令系统</t>
+  </si>
+  <si>
+    <t>4.2 寻址方式</t>
+  </si>
+  <si>
+    <t>4.3 程序的机器级代码表示</t>
+  </si>
+  <si>
+    <t>4.4 CISC和RISC的基本概念</t>
+  </si>
+  <si>
+    <t>第5章 中央处理器</t>
+  </si>
+  <si>
+    <t>5.1 CPU的功能和基本结构</t>
+  </si>
+  <si>
+    <t>5.2 指令执行过程</t>
+  </si>
+  <si>
+    <t>5.3 数据通路的功能和基本结构</t>
+  </si>
+  <si>
+    <t>5.4 控制器的功能和工作原理</t>
+  </si>
+  <si>
+    <t>5.5 异常和中断机制</t>
+  </si>
+  <si>
+    <t>5.6 指令流水线</t>
+  </si>
+  <si>
+    <t>5.7 多处理器的基本概念</t>
+  </si>
+  <si>
+    <t>第6章 总线</t>
+  </si>
+  <si>
+    <t>6.1 总线概述</t>
+  </si>
+  <si>
+    <t>6.2 总线事务和定时</t>
+  </si>
+  <si>
+    <t>第7章 输入/输出系统</t>
+  </si>
+  <si>
+    <t>7.1 I/O系统基本概念</t>
+  </si>
+  <si>
+    <t>7.2 I/O接口</t>
+  </si>
+  <si>
+    <t>7.3 I/O方式</t>
+  </si>
+  <si>
+    <t>王道操作系统 课后习题正确率记录</t>
+  </si>
+  <si>
+    <t>1.1 操作系统的基本概念</t>
+  </si>
+  <si>
+    <t>1.2 操作系统发展历程</t>
+  </si>
+  <si>
+    <t>1.3 操作系统的运行环境</t>
+  </si>
+  <si>
+    <t>1.4 操作系统结构</t>
+  </si>
+  <si>
+    <t>1.5 操作系统引导</t>
+  </si>
+  <si>
+    <t>1.6 虚拟机</t>
+  </si>
+  <si>
+    <t>第2章 进程与线程</t>
+  </si>
+  <si>
+    <t>2.1 进程与线程简介</t>
+  </si>
+  <si>
+    <t>2.2 CPU调度</t>
+  </si>
+  <si>
+    <t>2.3 同步与互斥</t>
+  </si>
+  <si>
+    <t>2.4 死锁</t>
+  </si>
+  <si>
+    <t>第3章 内存管理</t>
+  </si>
+  <si>
+    <t>3.1 内存管理概念</t>
+  </si>
+  <si>
+    <t>3.2 虚拟内存管理</t>
+  </si>
+  <si>
+    <t>第4章 文件管理</t>
+  </si>
+  <si>
+    <t>4.1 文件系统基础</t>
+  </si>
+  <si>
+    <t>4.2 目录与文件</t>
+  </si>
+  <si>
+    <t>4.3 文件系统</t>
+  </si>
+  <si>
+    <t>第5章 输入/输出管理</t>
+  </si>
+  <si>
+    <t>5.1 I/O管理概述</t>
+  </si>
+  <si>
+    <t>5.2 设备独立性软件</t>
+  </si>
+  <si>
+    <t>5.3 磁盘和固态硬盘</t>
+  </si>
+  <si>
+    <t>王道计算机网络 课后习题正确率记录</t>
+  </si>
+  <si>
+    <t>第1章 计算机网络体系结构</t>
+  </si>
+  <si>
+    <t>1.1 计算机网络概述</t>
+  </si>
+  <si>
+    <t>1.2 计算机网络体系结构与参考模型</t>
+  </si>
+  <si>
+    <t>第2章 物理层</t>
+  </si>
+  <si>
+    <t>2.1 通信基础</t>
+  </si>
+  <si>
+    <t>2.2 传输介质</t>
+  </si>
+  <si>
+    <t>2.3 物理层设备</t>
+  </si>
+  <si>
+    <t>第3章 数据链路层</t>
+  </si>
+  <si>
+    <t>3.1 数据链路层的功能</t>
+  </si>
+  <si>
+    <t>3.2 组帧</t>
+  </si>
+  <si>
+    <t>3.3 差错控制</t>
+  </si>
+  <si>
+    <t>3.4 流量控制与可靠传输机制</t>
+  </si>
+  <si>
+    <t>3.5 介质访问控制</t>
+  </si>
+  <si>
+    <t>3.6 局域网</t>
+  </si>
+  <si>
+    <t>3.7 广域网</t>
+  </si>
+  <si>
+    <t>3.8 数据链路层设备</t>
+  </si>
+  <si>
+    <t>第4章 网络层</t>
+  </si>
+  <si>
+    <t>4.1 网络层的功能</t>
+  </si>
+  <si>
+    <t>4.2 IPv4</t>
+  </si>
+  <si>
+    <t>4.3 IPv6</t>
+  </si>
+  <si>
+    <t>4.4 路由算法与路由协议</t>
+  </si>
+  <si>
+    <t>4.5 IP多播</t>
+  </si>
+  <si>
+    <t>4.6 移动IP</t>
+  </si>
+  <si>
+    <t>4.7 网络层设备</t>
+  </si>
+  <si>
+    <t>第5章 传输层</t>
+  </si>
+  <si>
+    <t>5.1 传输层提供的服务</t>
+  </si>
+  <si>
+    <t>5.2 UDP</t>
+  </si>
+  <si>
+    <t>5.3 TCP</t>
+  </si>
+  <si>
+    <t>第6章 应用层</t>
+  </si>
+  <si>
+    <t>6.1 网络应用模型</t>
+  </si>
+  <si>
+    <t>6.2 域名系统</t>
+  </si>
+  <si>
+    <t>6.3 文件传输协议</t>
+  </si>
+  <si>
+    <t>6.4 电子邮件</t>
+  </si>
+  <si>
+    <t>6.5 万维网</t>
+  </si>
+  <si>
     <t>填空题</t>
-  </si>
-  <si>
-    <t>问答题</t>
-  </si>
-  <si>
-    <t>第一章 函数 极限 连续</t>
-  </si>
-  <si>
-    <t>第二章 一元函数微分学</t>
-  </si>
-  <si>
-    <t>第三章 一元函数积分学</t>
-  </si>
-  <si>
-    <t>第四章 常微分方程</t>
-  </si>
-  <si>
-    <t>第五章 多元函数微分学</t>
-  </si>
-  <si>
-    <t>第六章 二重积分</t>
-  </si>
-  <si>
-    <t>第七章 无穷级数 (仅数学一、三)</t>
-  </si>
-  <si>
-    <t>第八章 向量代数与空间解析几何及多元微分学在几何上的应用 (仅数学一)</t>
-  </si>
-  <si>
-    <t>第九章 多元函数积分学及其应用 (仅数学一)</t>
-  </si>
-  <si>
-    <t>李林880 （选择&amp;填空）习题正确率记录</t>
-  </si>
-  <si>
-    <t>时间</t>
-  </si>
-  <si>
-    <t>第一章 函数、极限、连续</t>
-  </si>
-  <si>
-    <t>第二章 一元函数微分学及其应用</t>
-  </si>
-  <si>
-    <t>第三章 一元函数积分学及其应用</t>
-  </si>
-  <si>
-    <t>第四章 空间解析几何</t>
-  </si>
-  <si>
-    <t>第五章 多元函数微分学及其应用</t>
-  </si>
-  <si>
-    <t>第六章 重积分及其应用</t>
-  </si>
-  <si>
-    <t>第七章 微分方程及其应用</t>
-  </si>
-  <si>
-    <t>第八章 无穷级数</t>
-  </si>
-  <si>
-    <t>第九章 曲线积分与曲面积分</t>
-  </si>
-  <si>
-    <t>高等数学 合计</t>
-  </si>
-  <si>
-    <t>第十章 行列式</t>
-  </si>
-  <si>
-    <t>第十一章 矩阵</t>
-  </si>
-  <si>
-    <t>第十二章 向量</t>
-  </si>
-  <si>
-    <t>第十三章 线性方程组</t>
-  </si>
-  <si>
-    <t>第十四章 相似矩阵</t>
-  </si>
-  <si>
-    <t>第十五章 二次型</t>
-  </si>
-  <si>
-    <t>线性代数 合计</t>
-  </si>
-  <si>
-    <t>第十六章 随机事件及其概率</t>
-  </si>
-  <si>
-    <t>第十七章 随机变量及其分布</t>
-  </si>
-  <si>
-    <t>第十八章 多维随机变量及其分布</t>
-  </si>
-  <si>
-    <t>第十九章 随机变量的数字特征</t>
-  </si>
-  <si>
-    <t>第二十章 大数定律与中心极限定理</t>
-  </si>
-  <si>
-    <t>第二十一章 数理统计的基本概念</t>
-  </si>
-  <si>
-    <t>第二十二章 参数估计</t>
-  </si>
-  <si>
-    <t>第二十三章 假设检验</t>
-  </si>
-  <si>
-    <t>概率论与数理统计 合计</t>
-  </si>
-  <si>
-    <t>总 计</t>
-  </si>
-  <si>
-    <t>解答区</t>
-  </si>
-  <si>
-    <t>扩展篇</t>
-  </si>
-  <si>
-    <t>选填+解答总计区</t>
-  </si>
-  <si>
-    <t>选填区</t>
-  </si>
-  <si>
-    <t>王道数据结构 课后习题正确率记录</t>
-  </si>
-  <si>
-    <t>一 刷</t>
-  </si>
-  <si>
-    <t>二 刷</t>
-  </si>
-  <si>
-    <t>小节</t>
-  </si>
-  <si>
-    <t>真题总</t>
-  </si>
-  <si>
-    <t>真题正</t>
-  </si>
-  <si>
-    <t>真题率</t>
-  </si>
-  <si>
-    <t>自编总</t>
-  </si>
-  <si>
-    <t>自编正</t>
-  </si>
-  <si>
-    <t>自编率</t>
-  </si>
-  <si>
-    <t>第1章 绪论</t>
-  </si>
-  <si>
-    <t>1.1 数据结构的基本概念</t>
-  </si>
-  <si>
-    <t>1.2 算法和算法评价</t>
-  </si>
-  <si>
-    <t>第2章 线性表</t>
-  </si>
-  <si>
-    <t>2.1 线性表的定义和基本操作</t>
-  </si>
-  <si>
-    <t>2.2 线性表的顺序表示</t>
-  </si>
-  <si>
-    <t>2.3 线性表的链式表示</t>
-  </si>
-  <si>
-    <t>第3章 栈、队列和数组</t>
-  </si>
-  <si>
-    <t>3.1 栈</t>
-  </si>
-  <si>
-    <t>3.2 队列</t>
-  </si>
-  <si>
-    <t>3.3 栈和队列的应用</t>
-  </si>
-  <si>
-    <t>3.4 数组和特殊矩阵</t>
-  </si>
-  <si>
-    <t>第4章 串</t>
-  </si>
-  <si>
-    <t>4.1 串的定义和实现</t>
-  </si>
-  <si>
-    <t>4.2 串的模式匹配</t>
-  </si>
-  <si>
-    <t>第5章 树与二叉树</t>
-  </si>
-  <si>
-    <t>5.1 树的基本概念</t>
-  </si>
-  <si>
-    <t>5.2 二叉树的概念</t>
-  </si>
-  <si>
-    <t>5.3 二叉树的遍历和线索二叉树</t>
-  </si>
-  <si>
-    <t>5.4 树、森林</t>
-  </si>
-  <si>
-    <t>5.5 树与二叉树的应用</t>
-  </si>
-  <si>
-    <t>第6章 图</t>
-  </si>
-  <si>
-    <t>6.1 图的基本概念</t>
-  </si>
-  <si>
-    <t>6.2 图的存储及基本操作</t>
-  </si>
-  <si>
-    <t>6.3 图的遍历</t>
-  </si>
-  <si>
-    <t>6.4 图的应用</t>
-  </si>
-  <si>
-    <t>第7章 查找</t>
-  </si>
-  <si>
-    <t>7.1 查找的基本概念</t>
-  </si>
-  <si>
-    <t>7.2 顺序查找和折半查找</t>
-  </si>
-  <si>
-    <t>7.3 树形查找</t>
-  </si>
-  <si>
-    <t>未包含红黑树</t>
-  </si>
-  <si>
-    <t>7.4 B树和B+树</t>
-  </si>
-  <si>
-    <t>7.5 散列(Hash)表</t>
-  </si>
-  <si>
-    <t>第8章 排序</t>
-  </si>
-  <si>
-    <t>8.1 排序的基本概念</t>
-  </si>
-  <si>
-    <t>8.2 插入排序</t>
-  </si>
-  <si>
-    <t>8.3 交换排序</t>
-  </si>
-  <si>
-    <t>8.4 选择排序</t>
-  </si>
-  <si>
-    <t>8.5 归并排序、基数排序和计数排序</t>
-  </si>
-  <si>
-    <t>8.6 各种内部排序算法的比较及应用</t>
-  </si>
-  <si>
-    <t>未完成</t>
-  </si>
-  <si>
-    <t>8.7 外部排序</t>
-  </si>
-  <si>
-    <t>王道计算机组成原理 课后习题正确率记录</t>
-  </si>
-  <si>
-    <t>第1章 计算机系统概述</t>
-  </si>
-  <si>
-    <t>1.1 计算机发展历程</t>
-  </si>
-  <si>
-    <t>1.2 计算机系统层次结构</t>
-  </si>
-  <si>
-    <t>1.3 计算机的性能指标</t>
-  </si>
-  <si>
-    <t>第2章 数据的表示和运算</t>
-  </si>
-  <si>
-    <t>2.1 数制与编码</t>
-  </si>
-  <si>
-    <t>2.2 运算方法和运算电路</t>
-  </si>
-  <si>
-    <t>2.3 浮点数的表示与运算</t>
-  </si>
-  <si>
-    <t>第3章 存储系统</t>
-  </si>
-  <si>
-    <t>3.1 存储器概述</t>
-  </si>
-  <si>
-    <t>3.2 主存储器</t>
-  </si>
-  <si>
-    <t>3.3 主存储器与CPU的连接</t>
-  </si>
-  <si>
-    <t>3.4 外部存储器</t>
-  </si>
-  <si>
-    <t>3.5 高速缓冲存储器</t>
-  </si>
-  <si>
-    <t>3.6 虚拟存储器</t>
-  </si>
-  <si>
-    <t>第4章 指令系统</t>
-  </si>
-  <si>
-    <t>4.1 指令系统</t>
-  </si>
-  <si>
-    <t>4.2 寻址方式</t>
-  </si>
-  <si>
-    <t>4.3 程序的机器级代码表示</t>
-  </si>
-  <si>
-    <t>4.4 CISC和RISC的基本概念</t>
-  </si>
-  <si>
-    <t>第5章 中央处理器</t>
-  </si>
-  <si>
-    <t>5.1 CPU的功能和基本结构</t>
-  </si>
-  <si>
-    <t>5.2 指令执行过程</t>
-  </si>
-  <si>
-    <t>5.3 数据通路的功能和基本结构</t>
-  </si>
-  <si>
-    <t>5.4 控制器的功能和工作原理</t>
-  </si>
-  <si>
-    <t>5.5 异常和中断机制</t>
-  </si>
-  <si>
-    <t>5.6 指令流水线</t>
-  </si>
-  <si>
-    <t>5.7 多处理器的基本概念</t>
-  </si>
-  <si>
-    <t>第6章 总线</t>
-  </si>
-  <si>
-    <t>6.1 总线概述</t>
-  </si>
-  <si>
-    <t>6.2 总线事务和定时</t>
-  </si>
-  <si>
-    <t>第7章 输入/输出系统</t>
-  </si>
-  <si>
-    <t>7.1 I/O系统基本概念</t>
-  </si>
-  <si>
-    <t>7.2 I/O接口</t>
-  </si>
-  <si>
-    <t>7.3 I/O方式</t>
-  </si>
-  <si>
-    <t>王道操作系统 课后习题正确率记录</t>
-  </si>
-  <si>
-    <t>1.1 操作系统的基本概念</t>
-  </si>
-  <si>
-    <t>1.2 操作系统发展历程</t>
-  </si>
-  <si>
-    <t>1.3 操作系统的运行环境</t>
-  </si>
-  <si>
-    <t>1.4 操作系统结构</t>
-  </si>
-  <si>
-    <t>1.5 操作系统引导</t>
-  </si>
-  <si>
-    <t>1.6 虚拟机</t>
-  </si>
-  <si>
-    <t>第2章 进程与线程</t>
-  </si>
-  <si>
-    <t>2.1 进程与线程简介</t>
-  </si>
-  <si>
-    <t>2.2 CPU调度</t>
-  </si>
-  <si>
-    <t>2.3 同步与互斥</t>
-  </si>
-  <si>
-    <t>2.4 死锁</t>
-  </si>
-  <si>
-    <t>第3章 内存管理</t>
-  </si>
-  <si>
-    <t>3.1 内存管理概念</t>
-  </si>
-  <si>
-    <t>3.2 虚拟内存管理</t>
-  </si>
-  <si>
-    <t>第4章 文件管理</t>
-  </si>
-  <si>
-    <t>4.1 文件系统基础</t>
-  </si>
-  <si>
-    <t>4.2 目录与文件</t>
-  </si>
-  <si>
-    <t>4.3 文件系统</t>
-  </si>
-  <si>
-    <t>第5章 输入/输出管理</t>
-  </si>
-  <si>
-    <t>5.1 I/O管理概述</t>
-  </si>
-  <si>
-    <t>5.2 设备独立性软件</t>
-  </si>
-  <si>
-    <t>5.3 磁盘和固态硬盘</t>
-  </si>
-  <si>
-    <t>王道计算机网络 课后习题正确率记录</t>
-  </si>
-  <si>
-    <t>第1章 计算机网络体系结构</t>
-  </si>
-  <si>
-    <t>1.1 计算机网络概述</t>
-  </si>
-  <si>
-    <t>1.2 计算机网络体系结构与参考模型</t>
-  </si>
-  <si>
-    <t>第2章 物理层</t>
-  </si>
-  <si>
-    <t>2.1 通信基础</t>
-  </si>
-  <si>
-    <t>2.2 传输介质</t>
-  </si>
-  <si>
-    <t>2.3 物理层设备</t>
-  </si>
-  <si>
-    <t>第3章 数据链路层</t>
-  </si>
-  <si>
-    <t>3.1 数据链路层的功能</t>
-  </si>
-  <si>
-    <t>3.2 组帧</t>
-  </si>
-  <si>
-    <t>3.3 差错控制</t>
-  </si>
-  <si>
-    <t>3.4 流量控制与可靠传输机制</t>
-  </si>
-  <si>
-    <t>3.5 介质访问控制</t>
-  </si>
-  <si>
-    <t>3.6 局域网</t>
-  </si>
-  <si>
-    <t>3.7 广域网</t>
-  </si>
-  <si>
-    <t>3.8 数据链路层设备</t>
-  </si>
-  <si>
-    <t>第4章 网络层</t>
-  </si>
-  <si>
-    <t>4.1 网络层的功能</t>
-  </si>
-  <si>
-    <t>4.2 IPv4</t>
-  </si>
-  <si>
-    <t>4.3 IPv6</t>
-  </si>
-  <si>
-    <t>4.4 路由算法与路由协议</t>
-  </si>
-  <si>
-    <t>4.5 IP多播</t>
-  </si>
-  <si>
-    <t>4.6 移动IP</t>
-  </si>
-  <si>
-    <t>4.7 网络层设备</t>
-  </si>
-  <si>
-    <t>第5章 传输层</t>
-  </si>
-  <si>
-    <t>5.1 传输层提供的服务</t>
-  </si>
-  <si>
-    <t>5.2 UDP</t>
-  </si>
-  <si>
-    <t>5.3 TCP</t>
-  </si>
-  <si>
-    <t>第6章 应用层</t>
-  </si>
-  <si>
-    <t>6.1 网络应用模型</t>
-  </si>
-  <si>
-    <t>6.2 域名系统</t>
-  </si>
-  <si>
-    <t>6.3 文件传输协议</t>
-  </si>
-  <si>
-    <t>6.4 电子邮件</t>
-  </si>
-  <si>
-    <t>6.5 万维网</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1110,6 +1111,13 @@
     <font>
       <sz val="11"/>
       <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -1466,28 +1474,28 @@
     <xf numFmtId="0" fontId="16" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -8777,12 +8785,12 @@
       <c r="D3" s="57"/>
       <c r="E3" s="58"/>
       <c r="F3" s="66" t="s">
-        <v>116</v>
+        <v>305</v>
       </c>
       <c r="G3" s="57"/>
       <c r="H3" s="58"/>
       <c r="I3" s="65" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J3" s="57"/>
       <c r="K3" s="58"/>
@@ -8838,7 +8846,7 @@
     </row>
     <row r="5" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B5" s="34">
         <v>618</v>
@@ -8888,43 +8896,57 @@
     </row>
     <row r="6" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="B6" s="34"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34" t="str">
+        <v>118</v>
+      </c>
+      <c r="B6" s="34">
+        <v>624</v>
+      </c>
+      <c r="C6" s="34">
+        <v>17</v>
+      </c>
+      <c r="D6" s="34">
+        <v>14</v>
+      </c>
+      <c r="E6" s="34">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34" t="str">
+        <v>0.82352941176470584</v>
+      </c>
+      <c r="F6" s="34">
+        <v>11</v>
+      </c>
+      <c r="G6" s="34">
+        <v>10</v>
+      </c>
+      <c r="H6" s="34">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34" t="str">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="I6" s="34">
+        <v>26</v>
+      </c>
+      <c r="J6" s="34">
+        <v>15</v>
+      </c>
+      <c r="K6" s="34">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.57692307692307687</v>
       </c>
       <c r="L6" s="34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="M6" s="34">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N6" s="34" t="e">
+        <v>39</v>
+      </c>
+      <c r="N6" s="34">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.72222222222222221</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B7" s="34"/>
       <c r="C7" s="34"/>
@@ -8960,7 +8982,7 @@
     </row>
     <row r="8" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B8" s="34"/>
       <c r="C8" s="34"/>
@@ -8996,7 +9018,7 @@
     </row>
     <row r="9" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="34"/>
@@ -9032,7 +9054,7 @@
     </row>
     <row r="10" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B10" s="34"/>
       <c r="C10" s="34"/>
@@ -9068,7 +9090,7 @@
     </row>
     <row r="11" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B11" s="34"/>
       <c r="C11" s="34"/>
@@ -9104,7 +9126,7 @@
     </row>
     <row r="12" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B12" s="34"/>
       <c r="C12" s="34"/>
@@ -9140,7 +9162,7 @@
     </row>
     <row r="13" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B13" s="34"/>
       <c r="C13" s="34"/>
@@ -9181,51 +9203,51 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>0.77777777777777779</v>
+        <v>0.8</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.94736842105263153</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="J14" s="37">
         <f>SUM(J5:J13)</f>
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="K14" s="37">
         <f t="shared" si="2"/>
-        <v>0.91304347826086951</v>
+        <v>0.73469387755102045</v>
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.87755102040816324</v>
+        <v>0.79611650485436891</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9236,51 +9258,51 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>0.77777777777777779</v>
+        <v>0.8</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>1</v>
+        <v>0.94736842105263153</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="J16" s="40">
         <f>J14</f>
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="K16" s="40">
         <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),J16/I16,"")</f>
-        <v>0.91304347826086951</v>
+        <v>0.73469387755102045</v>
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.87755102040816324</v>
+        <v>0.79611650485436891</v>
       </c>
     </row>
   </sheetData>
@@ -9406,8 +9428,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
-        <v>127</v>
+      <c r="A1" s="67" t="s">
+        <v>126</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -9424,17 +9446,17 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="72" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="57"/>
       <c r="E3" s="58"/>
-      <c r="F3" s="69" t="s">
+      <c r="F3" s="70" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="57"/>
       <c r="H3" s="58"/>
-      <c r="I3" s="71" t="s">
+      <c r="I3" s="69" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="57"/>
@@ -9445,7 +9467,7 @@
         <v>50</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>9</v>
@@ -9492,7 +9514,7 @@
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B6" s="4">
         <v>618</v>
@@ -9532,7 +9554,7 @@
     </row>
     <row r="7" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -9562,7 +9584,7 @@
     </row>
     <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -9592,7 +9614,7 @@
     </row>
     <row r="9" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -9622,7 +9644,7 @@
     </row>
     <row r="10" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -9652,7 +9674,7 @@
     </row>
     <row r="11" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -9682,7 +9704,7 @@
     </row>
     <row r="12" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -9712,7 +9734,7 @@
     </row>
     <row r="13" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -9742,7 +9764,7 @@
     </row>
     <row r="14" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -9772,7 +9794,7 @@
     </row>
     <row r="15" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7">
@@ -9830,7 +9852,7 @@
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -9860,7 +9882,7 @@
     </row>
     <row r="19" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -9890,7 +9912,7 @@
     </row>
     <row r="20" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -9920,7 +9942,7 @@
     </row>
     <row r="21" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -9950,7 +9972,7 @@
     </row>
     <row r="22" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -9980,7 +10002,7 @@
     </row>
     <row r="23" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -10010,7 +10032,7 @@
     </row>
     <row r="24" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7">
@@ -10068,7 +10090,7 @@
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -10098,7 +10120,7 @@
     </row>
     <row r="28" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -10128,7 +10150,7 @@
     </row>
     <row r="29" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -10158,7 +10180,7 @@
     </row>
     <row r="30" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -10188,7 +10210,7 @@
     </row>
     <row r="31" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -10218,7 +10240,7 @@
     </row>
     <row r="32" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -10248,7 +10270,7 @@
     </row>
     <row r="33" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -10278,7 +10300,7 @@
     </row>
     <row r="34" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -10308,7 +10330,7 @@
     </row>
     <row r="35" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7">
@@ -10350,7 +10372,7 @@
     </row>
     <row r="36" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="10">
@@ -10391,8 +10413,8 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="70" t="s">
-        <v>156</v>
+      <c r="A39" s="73" t="s">
+        <v>155</v>
       </c>
       <c r="B39" s="55"/>
       <c r="C39" s="55"/>
@@ -10412,22 +10434,22 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="67" t="s">
+      <c r="C41" s="72" t="s">
         <v>52</v>
       </c>
       <c r="D41" s="57"/>
       <c r="E41" s="58"/>
-      <c r="F41" s="69" t="s">
+      <c r="F41" s="70" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="57"/>
       <c r="H41" s="58"/>
-      <c r="I41" s="73" t="s">
-        <v>157</v>
+      <c r="I41" s="71" t="s">
+        <v>156</v>
       </c>
       <c r="J41" s="57"/>
       <c r="K41" s="58"/>
-      <c r="L41" s="71" t="s">
+      <c r="L41" s="69" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="57"/>
@@ -10438,7 +10460,7 @@
         <v>50</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>9</v>
@@ -10497,7 +10519,7 @@
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B44" s="4">
         <f t="shared" ref="B44:B52" si="13">B6</f>
@@ -10548,7 +10570,7 @@
     </row>
     <row r="45" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B45" s="4">
         <f t="shared" si="13"/>
@@ -10587,7 +10609,7 @@
     </row>
     <row r="46" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B46" s="4">
         <f t="shared" si="13"/>
@@ -10626,7 +10648,7 @@
     </row>
     <row r="47" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B47" s="4">
         <f t="shared" si="13"/>
@@ -10665,7 +10687,7 @@
     </row>
     <row r="48" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B48" s="4">
         <f t="shared" si="13"/>
@@ -10704,7 +10726,7 @@
     </row>
     <row r="49" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B49" s="4">
         <f t="shared" si="13"/>
@@ -10743,7 +10765,7 @@
     </row>
     <row r="50" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B50" s="4">
         <f t="shared" si="13"/>
@@ -10782,7 +10804,7 @@
     </row>
     <row r="51" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B51" s="4">
         <f t="shared" si="13"/>
@@ -10821,7 +10843,7 @@
     </row>
     <row r="52" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B52" s="4">
         <f t="shared" si="13"/>
@@ -10860,7 +10882,7 @@
     </row>
     <row r="53" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7">
@@ -10933,7 +10955,7 @@
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B56" s="4">
         <f t="shared" ref="B56:B61" si="20">B18</f>
@@ -10972,7 +10994,7 @@
     </row>
     <row r="57" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B57" s="4">
         <f t="shared" si="20"/>
@@ -11011,7 +11033,7 @@
     </row>
     <row r="58" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B58" s="4">
         <f t="shared" si="20"/>
@@ -11050,7 +11072,7 @@
     </row>
     <row r="59" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B59" s="4">
         <f t="shared" si="20"/>
@@ -11089,7 +11111,7 @@
     </row>
     <row r="60" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B60" s="4">
         <f t="shared" si="20"/>
@@ -11128,7 +11150,7 @@
     </row>
     <row r="61" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B61" s="4">
         <f t="shared" si="20"/>
@@ -11167,7 +11189,7 @@
     </row>
     <row r="62" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7">
@@ -11240,7 +11262,7 @@
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B65" s="4">
         <f t="shared" ref="B65:B72" si="26">B27</f>
@@ -11279,7 +11301,7 @@
     </row>
     <row r="66" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B66" s="4">
         <f t="shared" si="26"/>
@@ -11318,7 +11340,7 @@
     </row>
     <row r="67" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B67" s="4">
         <f t="shared" si="26"/>
@@ -11357,7 +11379,7 @@
     </row>
     <row r="68" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B68" s="4">
         <f t="shared" si="26"/>
@@ -11396,7 +11418,7 @@
     </row>
     <row r="69" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B69" s="4">
         <f t="shared" si="26"/>
@@ -11435,7 +11457,7 @@
     </row>
     <row r="70" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B70" s="4">
         <f t="shared" si="26"/>
@@ -11474,7 +11496,7 @@
     </row>
     <row r="71" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B71" s="4">
         <f t="shared" si="26"/>
@@ -11513,7 +11535,7 @@
     </row>
     <row r="72" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B72" s="4">
         <f t="shared" si="26"/>
@@ -11552,7 +11574,7 @@
     </row>
     <row r="73" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7">
@@ -11606,7 +11628,7 @@
     </row>
     <row r="74" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B74" s="9"/>
       <c r="C74" s="10">
@@ -11659,8 +11681,8 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="70" t="s">
-        <v>158</v>
+      <c r="A77" s="73" t="s">
+        <v>157</v>
       </c>
       <c r="B77" s="55"/>
       <c r="C77" s="55"/>
@@ -11677,17 +11699,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="67" t="s">
-        <v>159</v>
+      <c r="C79" s="72" t="s">
+        <v>158</v>
       </c>
       <c r="D79" s="57"/>
       <c r="E79" s="58"/>
-      <c r="F79" s="69" t="s">
-        <v>156</v>
+      <c r="F79" s="70" t="s">
+        <v>155</v>
       </c>
       <c r="G79" s="57"/>
       <c r="H79" s="58"/>
-      <c r="I79" s="71" t="s">
+      <c r="I79" s="69" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="57"/>
@@ -11698,7 +11720,7 @@
         <v>50</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>9</v>
@@ -11745,7 +11767,7 @@
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B82" s="4">
         <f t="shared" ref="B82:B90" si="32">B6</f>
@@ -11790,7 +11812,7 @@
     </row>
     <row r="83" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B83" s="4">
         <f t="shared" si="32"/>
@@ -11835,7 +11857,7 @@
     </row>
     <row r="84" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B84" s="4">
         <f t="shared" si="32"/>
@@ -11880,7 +11902,7 @@
     </row>
     <row r="85" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B85" s="4">
         <f t="shared" si="32"/>
@@ -11925,7 +11947,7 @@
     </row>
     <row r="86" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B86" s="4">
         <f t="shared" si="32"/>
@@ -11970,7 +11992,7 @@
     </row>
     <row r="87" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B87" s="4">
         <f t="shared" si="32"/>
@@ -12015,7 +12037,7 @@
     </row>
     <row r="88" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B88" s="4">
         <f t="shared" si="32"/>
@@ -12060,7 +12082,7 @@
     </row>
     <row r="89" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B89" s="4">
         <f t="shared" si="32"/>
@@ -12105,7 +12127,7 @@
     </row>
     <row r="90" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B90" s="4">
         <f t="shared" si="32"/>
@@ -12150,7 +12172,7 @@
     </row>
     <row r="91" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7">
@@ -12208,7 +12230,7 @@
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B94" s="4">
         <f t="shared" ref="B94:B99" si="42">B18</f>
@@ -12253,7 +12275,7 @@
     </row>
     <row r="95" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B95" s="4">
         <f t="shared" si="42"/>
@@ -12298,7 +12320,7 @@
     </row>
     <row r="96" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B96" s="4">
         <f t="shared" si="42"/>
@@ -12343,7 +12365,7 @@
     </row>
     <row r="97" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B97" s="4">
         <f t="shared" si="42"/>
@@ -12388,7 +12410,7 @@
     </row>
     <row r="98" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B98" s="4">
         <f t="shared" si="42"/>
@@ -12433,7 +12455,7 @@
     </row>
     <row r="99" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B99" s="4">
         <f t="shared" si="42"/>
@@ -12478,7 +12500,7 @@
     </row>
     <row r="100" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7">
@@ -12536,7 +12558,7 @@
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B103" s="4">
         <f t="shared" ref="B103:B110" si="49">B27</f>
@@ -12581,7 +12603,7 @@
     </row>
     <row r="104" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B104" s="4">
         <f t="shared" si="49"/>
@@ -12626,7 +12648,7 @@
     </row>
     <row r="105" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B105" s="4">
         <f t="shared" si="49"/>
@@ -12671,7 +12693,7 @@
     </row>
     <row r="106" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B106" s="4">
         <f t="shared" si="49"/>
@@ -12716,7 +12738,7 @@
     </row>
     <row r="107" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B107" s="4">
         <f t="shared" si="49"/>
@@ -12761,7 +12783,7 @@
     </row>
     <row r="108" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B108" s="4">
         <f t="shared" si="49"/>
@@ -12806,7 +12828,7 @@
     </row>
     <row r="109" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B109" s="4">
         <f t="shared" si="49"/>
@@ -12851,7 +12873,7 @@
     </row>
     <row r="110" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B110" s="4">
         <f t="shared" si="49"/>
@@ -12896,7 +12918,7 @@
     </row>
     <row r="111" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7">
@@ -12938,7 +12960,7 @@
     </row>
     <row r="112" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B112" s="9"/>
       <c r="C112" s="10">
@@ -12980,6 +13002,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -12996,12 +13024,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13396,7 +13418,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -13423,7 +13445,7 @@
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="59" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" s="57"/>
       <c r="C3" s="57"/>
@@ -13437,7 +13459,7 @@
       <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N3" s="57"/>
       <c r="O3" s="57"/>
@@ -13451,7 +13473,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>7</v>
@@ -13466,22 +13488,22 @@
         <v>11</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>169</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>7</v>
@@ -13496,27 +13518,27 @@
         <v>11</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -13542,7 +13564,7 @@
     </row>
     <row r="6" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B6" s="15">
         <v>415</v>
@@ -13608,7 +13630,7 @@
     </row>
     <row r="7" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B7" s="15">
         <v>416</v>
@@ -13674,7 +13696,7 @@
     </row>
     <row r="8" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -13700,7 +13722,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B9" s="15">
         <v>417</v>
@@ -13766,7 +13788,7 @@
     </row>
     <row r="10" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B10" s="15">
         <v>418</v>
@@ -13832,7 +13854,7 @@
     </row>
     <row r="11" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B11" s="15">
         <v>419</v>
@@ -13898,7 +13920,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -13924,7 +13946,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B13" s="15">
         <v>420</v>
@@ -13990,7 +14012,7 @@
     </row>
     <row r="14" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B14" s="15">
         <v>421</v>
@@ -14056,7 +14078,7 @@
     </row>
     <row r="15" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B15" s="15">
         <v>422</v>
@@ -14122,7 +14144,7 @@
     </row>
     <row r="16" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B16" s="15">
         <v>423</v>
@@ -14188,7 +14210,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -14214,7 +14236,7 @@
     </row>
     <row r="18" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B18" s="15">
         <v>424</v>
@@ -14280,7 +14302,7 @@
     </row>
     <row r="19" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B19" s="15">
         <v>424</v>
@@ -14346,7 +14368,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -14372,7 +14394,7 @@
     </row>
     <row r="21" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B21" s="15">
         <v>425</v>
@@ -14438,7 +14460,7 @@
     </row>
     <row r="22" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B22" s="15">
         <v>425</v>
@@ -14504,7 +14526,7 @@
     </row>
     <row r="23" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B23" s="15">
         <v>426</v>
@@ -14570,7 +14592,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B24" s="15">
         <v>427</v>
@@ -14636,7 +14658,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B25" s="15">
         <v>428</v>
@@ -14702,7 +14724,7 @@
     </row>
     <row r="26" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
@@ -14728,7 +14750,7 @@
     </row>
     <row r="27" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B27" s="15">
         <v>429</v>
@@ -14794,7 +14816,7 @@
     </row>
     <row r="28" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B28" s="15">
         <v>430</v>
@@ -14860,7 +14882,7 @@
     </row>
     <row r="29" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B29" s="15">
         <v>501</v>
@@ -14926,7 +14948,7 @@
     </row>
     <row r="30" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B30" s="15">
         <v>502</v>
@@ -14992,7 +15014,7 @@
     </row>
     <row r="31" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
@@ -15018,7 +15040,7 @@
     </row>
     <row r="32" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B32" s="15">
         <v>503</v>
@@ -15084,7 +15106,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B33" s="15">
         <v>503</v>
@@ -15150,7 +15172,7 @@
     </row>
     <row r="34" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="42" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B34" s="15">
         <v>503</v>
@@ -15188,7 +15210,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="L34" s="43" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M34" s="15"/>
       <c r="N34" s="15"/>
@@ -15218,7 +15240,7 @@
     </row>
     <row r="35" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B35" s="15">
         <v>504</v>
@@ -15284,7 +15306,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B36" s="15">
         <v>504</v>
@@ -15350,7 +15372,7 @@
     </row>
     <row r="37" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
@@ -15376,7 +15398,7 @@
     </row>
     <row r="38" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B38" s="15">
         <v>505</v>
@@ -15442,7 +15464,7 @@
     </row>
     <row r="39" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B39" s="15">
         <v>505</v>
@@ -15508,7 +15530,7 @@
     </row>
     <row r="40" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B40" s="15">
         <v>505</v>
@@ -15574,7 +15596,7 @@
     </row>
     <row r="41" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B41" s="15">
         <v>505</v>
@@ -15640,7 +15662,7 @@
     </row>
     <row r="42" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B42" s="15">
         <v>506</v>
@@ -15706,7 +15728,7 @@
     </row>
     <row r="43" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B43" s="15">
         <v>506</v>
@@ -15736,7 +15758,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="L43" s="44" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M43" s="15"/>
       <c r="N43" s="15"/>
@@ -15766,7 +15788,7 @@
     </row>
     <row r="44" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B44" s="15">
         <v>506</v>
@@ -15796,7 +15818,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="L44" s="44" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M44" s="15"/>
       <c r="N44" s="15"/>
@@ -16641,8 +16663,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
-        <v>212</v>
+      <c r="A1" s="67" t="s">
+        <v>211</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -16669,7 +16691,7 @@
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="59" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" s="57"/>
       <c r="C3" s="57"/>
@@ -16683,7 +16705,7 @@
       <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N3" s="57"/>
       <c r="O3" s="57"/>
@@ -16697,7 +16719,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>7</v>
@@ -16712,22 +16734,22 @@
         <v>11</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>169</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>7</v>
@@ -16742,27 +16764,27 @@
         <v>11</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -16788,7 +16810,7 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B6" s="15">
         <v>507</v>
@@ -16854,7 +16876,7 @@
     </row>
     <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B7" s="15">
         <v>507</v>
@@ -16920,7 +16942,7 @@
     </row>
     <row r="8" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B8" s="15">
         <v>508</v>
@@ -16986,7 +17008,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -17012,7 +17034,7 @@
     </row>
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B10" s="15">
         <v>509</v>
@@ -17078,7 +17100,7 @@
     </row>
     <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B11" s="15">
         <v>510</v>
@@ -17144,7 +17166,7 @@
     </row>
     <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B12" s="15">
         <v>512</v>
@@ -17210,7 +17232,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -17236,7 +17258,7 @@
     </row>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B14" s="15">
         <v>513</v>
@@ -17302,7 +17324,7 @@
     </row>
     <row r="15" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B15" s="15">
         <v>514</v>
@@ -17368,7 +17390,7 @@
     </row>
     <row r="16" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B16" s="15">
         <v>515</v>
@@ -17434,7 +17456,7 @@
     </row>
     <row r="17" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B17" s="15">
         <v>516</v>
@@ -17500,7 +17522,7 @@
     </row>
     <row r="18" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B18" s="15">
         <v>516</v>
@@ -17566,7 +17588,7 @@
     </row>
     <row r="19" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B19" s="15">
         <v>517</v>
@@ -17632,7 +17654,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -17658,7 +17680,7 @@
     </row>
     <row r="21" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B21" s="15">
         <v>518</v>
@@ -17724,7 +17746,7 @@
     </row>
     <row r="22" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B22" s="15">
         <v>518</v>
@@ -17790,7 +17812,7 @@
     </row>
     <row r="23" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B23" s="15">
         <v>519</v>
@@ -17824,7 +17846,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="L23" s="44" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M23" s="15"/>
       <c r="N23" s="15"/>
@@ -17854,7 +17876,7 @@
     </row>
     <row r="24" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B24" s="15">
         <v>520</v>
@@ -17920,7 +17942,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -17946,7 +17968,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B26" s="15">
         <v>521</v>
@@ -18012,7 +18034,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B27" s="15">
         <v>521</v>
@@ -18078,7 +18100,7 @@
     </row>
     <row r="28" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B28" s="15">
         <v>522</v>
@@ -18144,7 +18166,7 @@
     </row>
     <row r="29" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B29" s="15">
         <v>523</v>
@@ -18210,7 +18232,7 @@
     </row>
     <row r="30" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B30" s="15">
         <v>524</v>
@@ -18276,7 +18298,7 @@
     </row>
     <row r="31" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B31" s="15">
         <v>525</v>
@@ -18342,7 +18364,7 @@
     </row>
     <row r="32" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B32" s="15">
         <v>525</v>
@@ -18408,7 +18430,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -18434,7 +18456,7 @@
     </row>
     <row r="34" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B34" s="15">
         <v>526</v>
@@ -18500,7 +18522,7 @@
     </row>
     <row r="35" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B35" s="15">
         <v>526</v>
@@ -18566,7 +18588,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -18592,7 +18614,7 @@
     </row>
     <row r="37" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B37" s="15">
         <v>526</v>
@@ -18658,7 +18680,7 @@
     </row>
     <row r="38" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B38" s="15">
         <v>527</v>
@@ -18724,7 +18746,7 @@
     </row>
     <row r="39" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B39" s="15">
         <v>528</v>
@@ -19534,7 +19556,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -19561,7 +19583,7 @@
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="59" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" s="57"/>
       <c r="C3" s="57"/>
@@ -19575,7 +19597,7 @@
       <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N3" s="57"/>
       <c r="O3" s="57"/>
@@ -19589,7 +19611,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>7</v>
@@ -19604,22 +19626,22 @@
         <v>11</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>169</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>7</v>
@@ -19634,27 +19656,27 @@
         <v>11</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -19680,7 +19702,7 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B6" s="15">
         <v>530</v>
@@ -19746,7 +19768,7 @@
     </row>
     <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B7" s="15">
         <v>530</v>
@@ -19812,7 +19834,7 @@
     </row>
     <row r="8" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B8" s="15">
         <v>530</v>
@@ -19878,7 +19900,7 @@
     </row>
     <row r="9" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B9" s="15">
         <v>531</v>
@@ -19944,7 +19966,7 @@
     </row>
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B10" s="15">
         <v>531</v>
@@ -20010,7 +20032,7 @@
     </row>
     <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B11" s="15">
         <v>531</v>
@@ -20076,7 +20098,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -20102,7 +20124,7 @@
     </row>
     <row r="13" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B13" s="15">
         <v>601</v>
@@ -20168,7 +20190,7 @@
     </row>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B14" s="15">
         <v>602</v>
@@ -20234,7 +20256,7 @@
     </row>
     <row r="15" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B15" s="15">
         <v>606</v>
@@ -20300,7 +20322,7 @@
     </row>
     <row r="16" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B16" s="15">
         <v>607</v>
@@ -20366,7 +20388,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -20392,7 +20414,7 @@
     </row>
     <row r="18" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B18" s="15">
         <v>609</v>
@@ -20458,7 +20480,7 @@
     </row>
     <row r="19" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B19" s="15">
         <v>610</v>
@@ -20524,7 +20546,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -20550,7 +20572,7 @@
     </row>
     <row r="21" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B21" s="15">
         <v>611</v>
@@ -20616,7 +20638,7 @@
     </row>
     <row r="22" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B22" s="15">
         <v>614</v>
@@ -20682,7 +20704,7 @@
     </row>
     <row r="23" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B23" s="15">
         <v>614</v>
@@ -20748,7 +20770,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
@@ -20774,7 +20796,7 @@
     </row>
     <row r="25" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B25" s="15">
         <v>614</v>
@@ -20840,7 +20862,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B26" s="15">
         <v>615</v>
@@ -20906,7 +20928,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B27" s="15">
         <v>615</v>
@@ -21572,7 +21594,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -21599,7 +21621,7 @@
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="59" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" s="57"/>
       <c r="C3" s="57"/>
@@ -21613,7 +21635,7 @@
       <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N3" s="57"/>
       <c r="O3" s="57"/>
@@ -21627,7 +21649,7 @@
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>7</v>
@@ -21642,22 +21664,22 @@
         <v>11</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>169</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>7</v>
@@ -21672,27 +21694,27 @@
         <v>11</v>
       </c>
       <c r="Q4" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="R4" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -21718,7 +21740,7 @@
     </row>
     <row r="6" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B6" s="15">
         <v>616</v>
@@ -21784,7 +21806,7 @@
     </row>
     <row r="7" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B7" s="15">
         <v>617</v>
@@ -21850,7 +21872,7 @@
     </row>
     <row r="8" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -21876,7 +21898,7 @@
     </row>
     <row r="9" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B9" s="15">
         <v>618</v>
@@ -21942,7 +21964,7 @@
     </row>
     <row r="10" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B10" s="15">
         <v>618</v>
@@ -22008,7 +22030,7 @@
     </row>
     <row r="11" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B11" s="15">
         <v>618</v>
@@ -22074,7 +22096,7 @@
     </row>
     <row r="12" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -22100,7 +22122,7 @@
     </row>
     <row r="13" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B13" s="15">
         <v>619</v>
@@ -22166,7 +22188,7 @@
     </row>
     <row r="14" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B14" s="15">
         <v>619</v>
@@ -22232,7 +22254,7 @@
     </row>
     <row r="15" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B15" s="15">
         <v>619</v>
@@ -22298,7 +22320,7 @@
     </row>
     <row r="16" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B16" s="15">
         <v>620</v>
@@ -22364,7 +22386,7 @@
     </row>
     <row r="17" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B17" s="15">
         <v>621</v>
@@ -22430,7 +22452,7 @@
     </row>
     <row r="18" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B18" s="15">
         <v>622</v>
@@ -22496,7 +22518,7 @@
     </row>
     <row r="19" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B19" s="15">
         <v>623</v>
@@ -22562,7 +22584,7 @@
     </row>
     <row r="20" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B20" s="15">
         <v>623</v>
@@ -22628,7 +22650,7 @@
     </row>
     <row r="21" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -22654,32 +22676,42 @@
     </row>
     <row r="22" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>289</v>
-      </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15" t="str">
+        <v>288</v>
+      </c>
+      <c r="B22" s="15">
+        <v>624</v>
+      </c>
+      <c r="C22" s="15">
+        <v>21</v>
+      </c>
+      <c r="D22" s="15">
+        <v>16</v>
+      </c>
+      <c r="E22" s="15">
         <f t="shared" ref="E22:E28" si="10">IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),D22/C22,"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15" t="str">
+        <v>0.76190476190476186</v>
+      </c>
+      <c r="F22" s="15">
+        <v>3</v>
+      </c>
+      <c r="G22" s="15">
+        <v>3</v>
+      </c>
+      <c r="H22" s="15">
         <f t="shared" ref="H22:H28" si="11">IF(AND(F22&lt;&gt;"",G22&lt;&gt;""),G22/F22,"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I22" s="15">
         <f t="shared" ref="I22:J28" si="12">C22-F22</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J22" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K22" s="15" t="e">
+        <v>13</v>
+      </c>
+      <c r="K22" s="15">
         <f t="shared" ref="K22:K28" si="13">IF(AND(I22&lt;&gt;"",J22&lt;&gt;""),J22/I22,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.72222222222222221</v>
       </c>
       <c r="L22" s="11"/>
       <c r="M22" s="15"/>
@@ -22710,7 +22742,7 @@
     </row>
     <row r="23" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -22766,7 +22798,7 @@
     </row>
     <row r="24" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -22822,7 +22854,7 @@
     </row>
     <row r="25" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -22878,7 +22910,7 @@
     </row>
     <row r="26" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -22934,7 +22966,7 @@
     </row>
     <row r="27" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -22990,7 +23022,7 @@
     </row>
     <row r="28" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -23046,7 +23078,7 @@
     </row>
     <row r="29" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -23072,7 +23104,7 @@
     </row>
     <row r="30" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
@@ -23128,7 +23160,7 @@
     </row>
     <row r="31" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -23184,7 +23216,7 @@
     </row>
     <row r="32" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -23240,7 +23272,7 @@
     </row>
     <row r="33" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -23266,7 +23298,7 @@
     </row>
     <row r="34" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
@@ -23322,7 +23354,7 @@
     </row>
     <row r="35" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -23378,7 +23410,7 @@
     </row>
     <row r="36" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
@@ -23434,7 +23466,7 @@
     </row>
     <row r="37" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>
@@ -23490,7 +23522,7 @@
     </row>
     <row r="38" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
@@ -23551,39 +23583,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.81640625</v>
+        <v>0.81227436823104693</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.81967213114754101</v>
+        <v>0.828125</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>195</v>
+        <v>213</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.81538461538461537</v>
+        <v>0.80751173708920188</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23632,39 +23664,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.81640625</v>
+        <v>0.81227436823104693</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.81967213114754101</v>
+        <v>0.828125</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>195</v>
+        <v>213</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.81538461538461537</v>
+        <v>0.80751173708920188</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
@@ -24745,25 +24777,37 @@
       <c r="A10" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
+      <c r="B10" s="48">
+        <v>6.23</v>
+      </c>
+      <c r="C10" s="48">
+        <v>17</v>
+      </c>
       <c r="D10" s="48">
         <v>5</v>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48" t="str">
+      <c r="E10" s="48">
+        <v>2</v>
+      </c>
+      <c r="F10" s="48">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
+        <v>0.4</v>
+      </c>
+      <c r="G10" s="48">
+        <v>6.25</v>
+      </c>
+      <c r="H10" s="48">
+        <v>28</v>
+      </c>
       <c r="I10" s="48">
         <v>5</v>
       </c>
-      <c r="J10" s="48"/>
-      <c r="K10" s="48" t="str">
+      <c r="J10" s="48">
+        <v>3</v>
+      </c>
+      <c r="K10" s="48">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="L10" s="48"/>
       <c r="M10" s="48"/>
@@ -24791,11 +24835,11 @@
       </c>
       <c r="W10" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X10" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25380,11 +25424,11 @@
       </c>
       <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" si="0"/>
-        <v>2.5000000000000001E-2</v>
+        <v>0.05</v>
       </c>
       <c r="G21" s="50"/>
       <c r="H21" s="50"/>
@@ -25394,11 +25438,11 @@
       </c>
       <c r="J21" s="46">
         <f>SUM(J5:J20)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K21" s="46">
         <f t="shared" si="1"/>
-        <v>7.4999999999999997E-2</v>
+        <v>0.1125</v>
       </c>
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
@@ -25434,11 +25478,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>6.25E-2</v>
+        <v>7.8125E-2</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25454,11 +25498,11 @@
       </c>
       <c r="E23" s="53">
         <f>E21</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F23" s="53">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23/D23,"")</f>
-        <v>2.5000000000000001E-2</v>
+        <v>0.05</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -25468,11 +25512,11 @@
       </c>
       <c r="J23" s="53">
         <f>J21</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K23" s="53">
         <f>IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),J23/I23,"")</f>
-        <v>7.4999999999999997E-2</v>
+        <v>0.1125</v>
       </c>
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
@@ -25508,11 +25552,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>6.25E-2</v>
+        <v>7.8125E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-06-26 10:04:13
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25E65FD-ACCF-4829-BF0F-671B52A6811B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51BA39C-AB44-49E9-BC00-759574EEF8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1444,21 +1444,21 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1477,34 +1477,34 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7536,13 +7536,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="60"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8047,13 +8047,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="60" t="s">
+      <c r="A41" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="57"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8534,13 +8534,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="60" t="s">
+      <c r="A83" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="57"/>
-      <c r="C83" s="57"/>
-      <c r="D83" s="57"/>
-      <c r="E83" s="58"/>
+      <c r="B83" s="59"/>
+      <c r="C83" s="59"/>
+      <c r="D83" s="59"/>
+      <c r="E83" s="60"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8782,23 +8782,23 @@
       <c r="C3" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="66" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
       <c r="I3" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="58"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="60"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9428,7 +9428,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="72" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="55"/>
@@ -9446,21 +9446,21 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="72" t="s">
+      <c r="C3" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="70" t="s">
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="69" t="s">
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9501,16 +9501,16 @@
       <c r="A5" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9839,16 +9839,16 @@
       <c r="A17" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="57"/>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="58"/>
+      <c r="B17" s="59"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="60"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10077,16 +10077,16 @@
       <c r="A26" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="57"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="58"/>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="60"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10413,7 +10413,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="70" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="55"/>
@@ -10434,26 +10434,26 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="72" t="s">
+      <c r="C41" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
-      <c r="F41" s="70" t="s">
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
+      <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="57"/>
-      <c r="H41" s="58"/>
-      <c r="I41" s="71" t="s">
+      <c r="G41" s="59"/>
+      <c r="H41" s="60"/>
+      <c r="I41" s="73" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="57"/>
-      <c r="K41" s="58"/>
-      <c r="L41" s="69" t="s">
+      <c r="J41" s="59"/>
+      <c r="K41" s="60"/>
+      <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="57"/>
-      <c r="N41" s="58"/>
+      <c r="M41" s="59"/>
+      <c r="N41" s="60"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10503,19 +10503,19 @@
       <c r="A43" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="57"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="57"/>
-      <c r="N43" s="58"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
+      <c r="H43" s="59"/>
+      <c r="I43" s="59"/>
+      <c r="J43" s="59"/>
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
+      <c r="M43" s="59"/>
+      <c r="N43" s="60"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10573,22 +10573,31 @@
         <v>129</v>
       </c>
       <c r="B45" s="4">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4" t="str">
+        <v>625</v>
+      </c>
+      <c r="C45" s="4">
+        <v>17</v>
+      </c>
+      <c r="D45" s="4">
+        <v>16</v>
+      </c>
+      <c r="E45" s="4">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4" t="str">
+        <v>0.94117647058823528</v>
+      </c>
+      <c r="F45" s="4">
+        <v>17</v>
+      </c>
+      <c r="G45" s="4">
+        <v>13</v>
+      </c>
+      <c r="H45" s="4">
         <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="I45" s="4"/>
+        <v>0.76470588235294112</v>
+      </c>
+      <c r="I45" s="4">
+        <v>19</v>
+      </c>
       <c r="J45" s="4"/>
       <c r="K45" s="4" t="str">
         <f t="shared" si="16"/>
@@ -10596,15 +10605,15 @@
       </c>
       <c r="L45" s="4">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="M45" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="N45" s="4" t="e">
+        <v>29</v>
+      </c>
+      <c r="N45" s="4">
         <f t="shared" si="19"/>
-        <v>#DIV/0!</v>
+        <v>0.54716981132075471</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -10887,31 +10896,31 @@
       <c r="B53" s="6"/>
       <c r="C53" s="7">
         <f>SUM(C44:C52)</f>
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="D53" s="7">
         <f>SUM(D44:D52)</f>
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E53" s="7">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0.95454545454545459</v>
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="G53" s="7">
         <f>SUM(G44:G52)</f>
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H53" s="7">
         <f t="shared" si="15"/>
-        <v>0.5</v>
+        <v>0.65517241379310343</v>
       </c>
       <c r="I53" s="7">
         <f>SUM(I44:I52)</f>
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="J53" s="7">
         <f>SUM(J44:J52)</f>
@@ -10923,15 +10932,15 @@
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.57894736842105265</v>
+        <v>0.55555555555555558</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -10939,19 +10948,19 @@
       <c r="A55" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="57"/>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="57"/>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
-      <c r="I55" s="57"/>
-      <c r="J55" s="57"/>
-      <c r="K55" s="57"/>
-      <c r="L55" s="57"/>
-      <c r="M55" s="57"/>
-      <c r="N55" s="58"/>
+      <c r="B55" s="59"/>
+      <c r="C55" s="59"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="59"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="59"/>
+      <c r="K55" s="59"/>
+      <c r="L55" s="59"/>
+      <c r="M55" s="59"/>
+      <c r="N55" s="60"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11246,19 +11255,19 @@
       <c r="A64" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="57"/>
-      <c r="H64" s="57"/>
-      <c r="I64" s="57"/>
-      <c r="J64" s="57"/>
-      <c r="K64" s="57"/>
-      <c r="L64" s="57"/>
-      <c r="M64" s="57"/>
-      <c r="N64" s="58"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="59"/>
+      <c r="D64" s="59"/>
+      <c r="E64" s="59"/>
+      <c r="F64" s="59"/>
+      <c r="G64" s="59"/>
+      <c r="H64" s="59"/>
+      <c r="I64" s="59"/>
+      <c r="J64" s="59"/>
+      <c r="K64" s="59"/>
+      <c r="L64" s="59"/>
+      <c r="M64" s="59"/>
+      <c r="N64" s="60"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11633,31 +11642,31 @@
       <c r="B74" s="9"/>
       <c r="C74" s="10">
         <f>C53+C62+C73</f>
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="D74" s="10">
         <f>D53+D62+D73</f>
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E74" s="10">
         <f t="shared" si="27"/>
-        <v>1</v>
+        <v>0.95454545454545459</v>
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="G74" s="10">
         <f>G53+G62+G73</f>
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H74" s="10">
         <f t="shared" si="28"/>
-        <v>0.5</v>
+        <v>0.65517241379310343</v>
       </c>
       <c r="I74" s="10">
         <f>I53+I62+I73</f>
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="J74" s="10">
         <f>J53+J62+J73</f>
@@ -11669,19 +11678,19 @@
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.57894736842105265</v>
+        <v>0.55555555555555558</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="73" t="s">
+      <c r="A77" s="70" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="55"/>
@@ -11699,21 +11708,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="72" t="s">
+      <c r="C79" s="67" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="57"/>
-      <c r="E79" s="58"/>
-      <c r="F79" s="70" t="s">
+      <c r="D79" s="59"/>
+      <c r="E79" s="60"/>
+      <c r="F79" s="69" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="57"/>
-      <c r="H79" s="58"/>
-      <c r="I79" s="69" t="s">
+      <c r="G79" s="59"/>
+      <c r="H79" s="60"/>
+      <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="57"/>
-      <c r="K79" s="58"/>
+      <c r="J79" s="59"/>
+      <c r="K79" s="60"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11754,16 +11763,16 @@
       <c r="A81" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="57"/>
-      <c r="C81" s="57"/>
-      <c r="D81" s="57"/>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="57"/>
-      <c r="J81" s="57"/>
-      <c r="K81" s="58"/>
+      <c r="B81" s="59"/>
+      <c r="C81" s="59"/>
+      <c r="D81" s="59"/>
+      <c r="E81" s="59"/>
+      <c r="F81" s="59"/>
+      <c r="G81" s="59"/>
+      <c r="H81" s="59"/>
+      <c r="I81" s="59"/>
+      <c r="J81" s="59"/>
+      <c r="K81" s="60"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -11832,27 +11841,27 @@
       </c>
       <c r="F83" s="4">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G83" s="4">
         <f t="shared" si="37"/>
-        <v>0</v>
-      </c>
-      <c r="H83" s="4" t="e">
+        <v>29</v>
+      </c>
+      <c r="H83" s="4">
         <f t="shared" si="38"/>
-        <v>#DIV/0!</v>
+        <v>0.54716981132075471</v>
       </c>
       <c r="I83" s="4">
         <f t="shared" si="39"/>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="J83" s="4">
         <f t="shared" si="40"/>
-        <v>0</v>
-      </c>
-      <c r="K83" s="4" t="e">
+        <v>29</v>
+      </c>
+      <c r="K83" s="4">
         <f t="shared" si="41"/>
-        <v>#DIV/0!</v>
+        <v>0.54716981132075471</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12189,27 +12198,27 @@
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.57894736842105265</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.8214285714285714</v>
+        <v>0.68807339449541283</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12217,16 +12226,16 @@
       <c r="A93" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="57"/>
-      <c r="C93" s="57"/>
-      <c r="D93" s="57"/>
-      <c r="E93" s="57"/>
-      <c r="F93" s="57"/>
-      <c r="G93" s="57"/>
-      <c r="H93" s="57"/>
-      <c r="I93" s="57"/>
-      <c r="J93" s="57"/>
-      <c r="K93" s="58"/>
+      <c r="B93" s="59"/>
+      <c r="C93" s="59"/>
+      <c r="D93" s="59"/>
+      <c r="E93" s="59"/>
+      <c r="F93" s="59"/>
+      <c r="G93" s="59"/>
+      <c r="H93" s="59"/>
+      <c r="I93" s="59"/>
+      <c r="J93" s="59"/>
+      <c r="K93" s="60"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12545,16 +12554,16 @@
       <c r="A102" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="57"/>
-      <c r="C102" s="57"/>
-      <c r="D102" s="57"/>
-      <c r="E102" s="57"/>
-      <c r="F102" s="57"/>
-      <c r="G102" s="57"/>
-      <c r="H102" s="57"/>
-      <c r="I102" s="57"/>
-      <c r="J102" s="57"/>
-      <c r="K102" s="58"/>
+      <c r="B102" s="59"/>
+      <c r="C102" s="59"/>
+      <c r="D102" s="59"/>
+      <c r="E102" s="59"/>
+      <c r="F102" s="59"/>
+      <c r="G102" s="59"/>
+      <c r="H102" s="59"/>
+      <c r="I102" s="59"/>
+      <c r="J102" s="59"/>
+      <c r="K102" s="60"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -12977,37 +12986,31 @@
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.57894736842105265</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.8214285714285714</v>
+        <v>0.68807339449541283</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13024,6 +13027,12 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13417,7 +13426,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="55"/>
@@ -13444,32 +13453,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16663,7 +16672,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="72" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="55"/>
@@ -16690,32 +16699,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19555,7 +19564,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="55"/>
@@ -19582,32 +19591,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21593,7 +21602,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="55"/>
@@ -21620,32 +21629,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24254,7 +24263,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24284,35 +24293,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="57" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="76" t="s">
+      <c r="G3" s="57" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="76" t="s">
+      <c r="L3" s="57" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="76" t="s">
+      <c r="Q3" s="57" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="75" t="s">
+      <c r="V3" s="56" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-26 22:33:28
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51BA39C-AB44-49E9-BC00-759574EEF8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749A5A13-8345-44CF-A973-40EF18BAA05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1444,21 +1444,33 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1477,27 +1489,6 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1505,6 +1496,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7509,7 +7509,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="65" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="55"/>
@@ -7536,13 +7536,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="58"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8047,13 +8047,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="59"/>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="B41" s="57"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8534,13 +8534,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="58" t="s">
+      <c r="A83" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="59"/>
-      <c r="C83" s="59"/>
-      <c r="D83" s="59"/>
-      <c r="E83" s="60"/>
+      <c r="B83" s="57"/>
+      <c r="C83" s="57"/>
+      <c r="D83" s="57"/>
+      <c r="E83" s="58"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8758,7 +8758,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="66" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="55"/>
@@ -8779,26 +8779,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="63" t="s">
+      <c r="C3" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="70" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="65" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="69" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="64" t="s">
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="59"/>
-      <c r="N3" s="60"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="58"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9428,7 +9428,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="54" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="55"/>
@@ -9446,21 +9446,21 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="69" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="71" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9498,19 +9498,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="60"/>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9556,12 +9556,18 @@
       <c r="A7" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4" t="str">
+      <c r="B7" s="4">
+        <v>626</v>
+      </c>
+      <c r="C7" s="4">
+        <v>34</v>
+      </c>
+      <c r="D7" s="4">
+        <v>29</v>
+      </c>
+      <c r="E7" s="4">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.8529411764705882</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -9571,15 +9577,15 @@
       </c>
       <c r="I7" s="4">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="J7" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K7" s="4" t="e">
+        <v>29</v>
+      </c>
+      <c r="K7" s="4">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0.8529411764705882</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9799,15 +9805,15 @@
       <c r="B15" s="6"/>
       <c r="C15" s="7">
         <f>SUM(C6:C14)</f>
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="D15" s="7">
         <f>SUM(D6:D14)</f>
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>0.93333333333333335</v>
+        <v>0.87755102040816324</v>
       </c>
       <c r="F15" s="7">
         <f>SUM(F6:F14)</f>
@@ -9823,32 +9829,32 @@
       </c>
       <c r="I15" s="7">
         <f>SUM(I6:I14)</f>
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="J15" s="7">
         <f>SUM(J6:J14)</f>
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="4"/>
-        <v>0.94594594594594594</v>
+        <v>0.90140845070422537</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="68" t="s">
+      <c r="A17" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="60"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="58"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10074,19 +10080,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="68" t="s">
+      <c r="A26" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="60"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="58"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10377,15 +10383,15 @@
       <c r="B36" s="9"/>
       <c r="C36" s="10">
         <f>C15+C24+C35</f>
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="D36" s="10">
         <f>D15+D24+D35</f>
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="E36" s="10">
         <f t="shared" si="9"/>
-        <v>0.93333333333333335</v>
+        <v>0.87755102040816324</v>
       </c>
       <c r="F36" s="10">
         <f>F15+F24+F35</f>
@@ -10401,19 +10407,19 @@
       </c>
       <c r="I36" s="10">
         <f>I15+I24+I35</f>
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="J36" s="10">
         <f>J15+J24+J35</f>
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>0.94594594594594594</v>
+        <v>0.90140845070422537</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="70" t="s">
+      <c r="A39" s="63" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="55"/>
@@ -10434,26 +10440,26 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="67" t="s">
+      <c r="C41" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="69" t="s">
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="59"/>
-      <c r="H41" s="60"/>
-      <c r="I41" s="73" t="s">
+      <c r="G41" s="57"/>
+      <c r="H41" s="58"/>
+      <c r="I41" s="61" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="59"/>
-      <c r="K41" s="60"/>
-      <c r="L41" s="71" t="s">
+      <c r="J41" s="57"/>
+      <c r="K41" s="58"/>
+      <c r="L41" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="59"/>
-      <c r="N41" s="60"/>
+      <c r="M41" s="57"/>
+      <c r="N41" s="58"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10500,22 +10506,22 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="68" t="s">
+      <c r="A43" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="59"/>
-      <c r="C43" s="59"/>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="59"/>
-      <c r="I43" s="59"/>
-      <c r="J43" s="59"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="60"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="57"/>
+      <c r="J43" s="57"/>
+      <c r="K43" s="57"/>
+      <c r="L43" s="57"/>
+      <c r="M43" s="57"/>
+      <c r="N43" s="58"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10576,28 +10582,22 @@
         <v>625</v>
       </c>
       <c r="C45" s="4">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D45" s="4">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E45" s="4">
         <f t="shared" si="14"/>
-        <v>0.94117647058823528</v>
-      </c>
-      <c r="F45" s="4">
-        <v>17</v>
-      </c>
-      <c r="G45" s="4">
-        <v>13</v>
-      </c>
-      <c r="H45" s="4">
+        <v>0.63157894736842102</v>
+      </c>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>0.76470588235294112</v>
-      </c>
-      <c r="I45" s="4">
-        <v>19</v>
-      </c>
+        <v/>
+      </c>
+      <c r="I45" s="4"/>
       <c r="J45" s="4"/>
       <c r="K45" s="4" t="str">
         <f t="shared" si="16"/>
@@ -10605,15 +10605,15 @@
       </c>
       <c r="L45" s="4">
         <f t="shared" si="17"/>
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="M45" s="4">
         <f t="shared" si="18"/>
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="N45" s="4">
         <f t="shared" si="19"/>
-        <v>0.54716981132075471</v>
+        <v>0.63157894736842102</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -10896,31 +10896,31 @@
       <c r="B53" s="6"/>
       <c r="C53" s="7">
         <f>SUM(C44:C52)</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D53" s="7">
         <f>SUM(D44:D52)</f>
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E53" s="7">
         <f t="shared" si="14"/>
-        <v>0.95454545454545459</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G53" s="7">
         <f>SUM(G44:G52)</f>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H53" s="7">
         <f t="shared" si="15"/>
-        <v>0.65517241379310343</v>
+        <v>0.5</v>
       </c>
       <c r="I53" s="7">
         <f>SUM(I44:I52)</f>
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="J53" s="7">
         <f>SUM(J44:J52)</f>
@@ -10932,35 +10932,35 @@
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.55555555555555558</v>
+        <v>0.60526315789473684</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="68" t="s">
+      <c r="A55" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="59"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="F55" s="59"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="59"/>
-      <c r="I55" s="59"/>
-      <c r="J55" s="59"/>
-      <c r="K55" s="59"/>
-      <c r="L55" s="59"/>
-      <c r="M55" s="59"/>
-      <c r="N55" s="60"/>
+      <c r="B55" s="57"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="57"/>
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="57"/>
+      <c r="I55" s="57"/>
+      <c r="J55" s="57"/>
+      <c r="K55" s="57"/>
+      <c r="L55" s="57"/>
+      <c r="M55" s="57"/>
+      <c r="N55" s="58"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11252,22 +11252,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="68" t="s">
+      <c r="A64" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="59"/>
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-      <c r="F64" s="59"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="59"/>
-      <c r="I64" s="59"/>
-      <c r="J64" s="59"/>
-      <c r="K64" s="59"/>
-      <c r="L64" s="59"/>
-      <c r="M64" s="59"/>
-      <c r="N64" s="60"/>
+      <c r="B64" s="57"/>
+      <c r="C64" s="57"/>
+      <c r="D64" s="57"/>
+      <c r="E64" s="57"/>
+      <c r="F64" s="57"/>
+      <c r="G64" s="57"/>
+      <c r="H64" s="57"/>
+      <c r="I64" s="57"/>
+      <c r="J64" s="57"/>
+      <c r="K64" s="57"/>
+      <c r="L64" s="57"/>
+      <c r="M64" s="57"/>
+      <c r="N64" s="58"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11642,31 +11642,31 @@
       <c r="B74" s="9"/>
       <c r="C74" s="10">
         <f>C53+C62+C73</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D74" s="10">
         <f>D53+D62+D73</f>
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E74" s="10">
         <f t="shared" si="27"/>
-        <v>0.95454545454545459</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G74" s="10">
         <f>G53+G62+G73</f>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H74" s="10">
         <f t="shared" si="28"/>
-        <v>0.65517241379310343</v>
+        <v>0.5</v>
       </c>
       <c r="I74" s="10">
         <f>I53+I62+I73</f>
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="J74" s="10">
         <f>J53+J62+J73</f>
@@ -11678,19 +11678,19 @@
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.55555555555555558</v>
+        <v>0.60526315789473684</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="70" t="s">
+      <c r="A77" s="63" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="55"/>
@@ -11708,21 +11708,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="67" t="s">
+      <c r="C79" s="62" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="59"/>
-      <c r="E79" s="60"/>
-      <c r="F79" s="69" t="s">
+      <c r="D79" s="57"/>
+      <c r="E79" s="58"/>
+      <c r="F79" s="60" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="59"/>
-      <c r="H79" s="60"/>
-      <c r="I79" s="71" t="s">
+      <c r="G79" s="57"/>
+      <c r="H79" s="58"/>
+      <c r="I79" s="59" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="59"/>
-      <c r="K79" s="60"/>
+      <c r="J79" s="57"/>
+      <c r="K79" s="58"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11760,19 +11760,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="68" t="s">
+      <c r="A81" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="59"/>
-      <c r="C81" s="59"/>
-      <c r="D81" s="59"/>
-      <c r="E81" s="59"/>
-      <c r="F81" s="59"/>
-      <c r="G81" s="59"/>
-      <c r="H81" s="59"/>
-      <c r="I81" s="59"/>
-      <c r="J81" s="59"/>
-      <c r="K81" s="60"/>
+      <c r="B81" s="57"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -11825,31 +11825,31 @@
       </c>
       <c r="B83" s="4">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>626</v>
       </c>
       <c r="C83" s="4">
         <f t="shared" si="33"/>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="D83" s="4">
         <f t="shared" si="34"/>
-        <v>0</v>
-      </c>
-      <c r="E83" s="4" t="e">
+        <v>29</v>
+      </c>
+      <c r="E83" s="4">
         <f t="shared" si="35"/>
-        <v>#DIV/0!</v>
+        <v>0.8529411764705882</v>
       </c>
       <c r="F83" s="4">
         <f t="shared" si="36"/>
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="G83" s="4">
         <f t="shared" si="37"/>
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="H83" s="4">
         <f t="shared" si="38"/>
-        <v>0.54716981132075471</v>
+        <v>0.63157894736842102</v>
       </c>
       <c r="I83" s="4">
         <f t="shared" si="39"/>
@@ -11857,11 +11857,11 @@
       </c>
       <c r="J83" s="4">
         <f t="shared" si="40"/>
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="K83" s="4">
         <f t="shared" si="41"/>
-        <v>0.54716981132075471</v>
+        <v>0.77358490566037741</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12186,27 +12186,27 @@
       <c r="B91" s="6"/>
       <c r="C91" s="7">
         <f>SUM(C82:C90)</f>
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="D91" s="7">
         <f>SUM(D82:D90)</f>
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="E91" s="7">
         <f t="shared" si="35"/>
-        <v>0.94594594594594594</v>
+        <v>0.90140845070422537</v>
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.55555555555555558</v>
+        <v>0.60526315789473684</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
@@ -12214,28 +12214,28 @@
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.68807339449541283</v>
+        <v>0.79816513761467889</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="68" t="s">
+      <c r="A93" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="59"/>
-      <c r="C93" s="59"/>
-      <c r="D93" s="59"/>
-      <c r="E93" s="59"/>
-      <c r="F93" s="59"/>
-      <c r="G93" s="59"/>
-      <c r="H93" s="59"/>
-      <c r="I93" s="59"/>
-      <c r="J93" s="59"/>
-      <c r="K93" s="60"/>
+      <c r="B93" s="57"/>
+      <c r="C93" s="57"/>
+      <c r="D93" s="57"/>
+      <c r="E93" s="57"/>
+      <c r="F93" s="57"/>
+      <c r="G93" s="57"/>
+      <c r="H93" s="57"/>
+      <c r="I93" s="57"/>
+      <c r="J93" s="57"/>
+      <c r="K93" s="58"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12551,19 +12551,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="68" t="s">
+      <c r="A102" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="59"/>
-      <c r="C102" s="59"/>
-      <c r="D102" s="59"/>
-      <c r="E102" s="59"/>
-      <c r="F102" s="59"/>
-      <c r="G102" s="59"/>
-      <c r="H102" s="59"/>
-      <c r="I102" s="59"/>
-      <c r="J102" s="59"/>
-      <c r="K102" s="60"/>
+      <c r="B102" s="57"/>
+      <c r="C102" s="57"/>
+      <c r="D102" s="57"/>
+      <c r="E102" s="57"/>
+      <c r="F102" s="57"/>
+      <c r="G102" s="57"/>
+      <c r="H102" s="57"/>
+      <c r="I102" s="57"/>
+      <c r="J102" s="57"/>
+      <c r="K102" s="58"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -12974,27 +12974,27 @@
       <c r="B112" s="9"/>
       <c r="C112" s="10">
         <f>C91+C100+C111</f>
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="D112" s="10">
         <f>D91+D100+D111</f>
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="E112" s="10">
         <f t="shared" si="51"/>
-        <v>0.94594594594594594</v>
+        <v>0.90140845070422537</v>
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.55555555555555558</v>
+        <v>0.60526315789473684</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
@@ -13002,15 +13002,21 @@
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.68807339449541283</v>
+        <v>0.79816513761467889</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13027,12 +13033,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13426,7 +13426,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="71" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="55"/>
@@ -13453,32 +13453,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="73" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16672,7 +16672,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="54" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="55"/>
@@ -16699,32 +16699,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="73" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19564,7 +19564,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="71" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="55"/>
@@ -19591,32 +19591,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="73" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21602,7 +21602,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="71" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="55"/>
@@ -21629,32 +21629,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="73" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24263,7 +24263,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24293,35 +24293,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="76" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="76" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="57" t="s">
+      <c r="L3" s="76" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="57" t="s">
+      <c r="Q3" s="76" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="56" t="s">
+      <c r="V3" s="75" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-28 09:30:42
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749A5A13-8345-44CF-A973-40EF18BAA05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29DC31A0-3D86-498A-AB94-C94A56218CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -9569,23 +9569,27 @@
         <f t="shared" si="0"/>
         <v>0.8529411764705882</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4" t="str">
+      <c r="F7" s="4">
+        <v>35</v>
+      </c>
+      <c r="G7" s="4">
+        <v>30</v>
+      </c>
+      <c r="H7" s="4">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I7" s="4">
         <f t="shared" si="2"/>
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="J7" s="4">
         <f t="shared" si="3"/>
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="K7" s="4">
         <f t="shared" si="4"/>
-        <v>0.8529411764705882</v>
+        <v>0.85507246376811596</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9817,27 +9821,27 @@
       </c>
       <c r="F15" s="7">
         <f>SUM(F6:F14)</f>
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="G15" s="7">
         <f>SUM(G6:G14)</f>
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H15" s="7">
         <f t="shared" si="1"/>
-        <v>0.95454545454545459</v>
+        <v>0.89473684210526316</v>
       </c>
       <c r="I15" s="7">
         <f>SUM(I6:I14)</f>
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="J15" s="7">
         <f>SUM(J6:J14)</f>
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="4"/>
-        <v>0.90140845070422537</v>
+        <v>0.8867924528301887</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -10395,27 +10399,27 @@
       </c>
       <c r="F36" s="10">
         <f>F15+F24+F35</f>
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="G36" s="10">
         <f>G15+G24+G35</f>
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H36" s="10">
         <f t="shared" si="10"/>
-        <v>0.95454545454545459</v>
+        <v>0.89473684210526316</v>
       </c>
       <c r="I36" s="10">
         <f>I15+I24+I35</f>
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="J36" s="10">
         <f>J15+J24+J35</f>
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>0.90140845070422537</v>
+        <v>0.8867924528301887</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11829,15 +11833,15 @@
       </c>
       <c r="C83" s="4">
         <f t="shared" si="33"/>
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="D83" s="4">
         <f t="shared" si="34"/>
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="E83" s="4">
         <f t="shared" si="35"/>
-        <v>0.8529411764705882</v>
+        <v>0.85507246376811596</v>
       </c>
       <c r="F83" s="4">
         <f t="shared" si="36"/>
@@ -11853,15 +11857,15 @@
       </c>
       <c r="I83" s="4">
         <f t="shared" si="39"/>
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="J83" s="4">
         <f t="shared" si="40"/>
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="K83" s="4">
         <f t="shared" si="41"/>
-        <v>0.77358490566037741</v>
+        <v>0.80681818181818177</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12186,15 +12190,15 @@
       <c r="B91" s="6"/>
       <c r="C91" s="7">
         <f>SUM(C82:C90)</f>
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="D91" s="7">
         <f>SUM(D82:D90)</f>
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="E91" s="7">
         <f t="shared" si="35"/>
-        <v>0.90140845070422537</v>
+        <v>0.8867924528301887</v>
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
@@ -12210,15 +12214,15 @@
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.79816513761467889</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12974,15 +12978,15 @@
       <c r="B112" s="9"/>
       <c r="C112" s="10">
         <f>C91+C100+C111</f>
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="D112" s="10">
         <f>D91+D100+D111</f>
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="E112" s="10">
         <f t="shared" si="51"/>
-        <v>0.90140845070422537</v>
+        <v>0.8867924528301887</v>
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
@@ -12998,15 +13002,15 @@
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.79816513761467889</v>
+        <v>0.8125</v>
       </c>
     </row>
   </sheetData>
@@ -22753,30 +22757,40 @@
       <c r="A23" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15" t="str">
+      <c r="B23" s="15">
+        <v>627</v>
+      </c>
+      <c r="C23" s="15">
+        <v>72</v>
+      </c>
+      <c r="D23" s="15">
+        <v>56</v>
+      </c>
+      <c r="E23" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15" t="str">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="F23" s="15">
+        <v>23</v>
+      </c>
+      <c r="G23" s="15">
+        <v>18</v>
+      </c>
+      <c r="H23" s="15">
         <f t="shared" si="11"/>
-        <v/>
+        <v>0.78260869565217395</v>
       </c>
       <c r="I23" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="J23" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K23" s="15" t="e">
+        <v>38</v>
+      </c>
+      <c r="K23" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
+        <v>0.77551020408163263</v>
       </c>
       <c r="L23" s="11"/>
       <c r="M23" s="15"/>
@@ -23592,39 +23606,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>277</v>
+        <v>349</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>225</v>
+        <v>281</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.81227436823104693</v>
+        <v>0.80515759312320911</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.828125</v>
+        <v>0.81609195402298851</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>213</v>
+        <v>262</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>172</v>
+        <v>210</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.80751173708920188</v>
+        <v>0.80152671755725191</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23673,39 +23687,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>277</v>
+        <v>349</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>225</v>
+        <v>281</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.81227436823104693</v>
+        <v>0.80515759312320911</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.828125</v>
+        <v>0.81609195402298851</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>213</v>
+        <v>262</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>172</v>
+        <v>210</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.80751173708920188</v>
+        <v>0.80152671755725191</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-30 16:51:44
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E182BC50-5042-42CD-A249-C0DE6A84CCC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71CDD83-5D28-4AC8-A1F7-6187DF0521F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1477,25 +1477,25 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9428,7 +9428,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="67" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="55"/>
@@ -9446,17 +9446,17 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="72" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="57"/>
       <c r="E3" s="58"/>
-      <c r="F3" s="69" t="s">
+      <c r="F3" s="70" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="57"/>
       <c r="H3" s="58"/>
-      <c r="I3" s="71" t="s">
+      <c r="I3" s="69" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="57"/>
@@ -10423,7 +10423,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="70" t="s">
+      <c r="A39" s="73" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="55"/>
@@ -10444,22 +10444,22 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="67" t="s">
+      <c r="C41" s="72" t="s">
         <v>52</v>
       </c>
       <c r="D41" s="57"/>
       <c r="E41" s="58"/>
-      <c r="F41" s="69" t="s">
+      <c r="F41" s="70" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="57"/>
       <c r="H41" s="58"/>
-      <c r="I41" s="73" t="s">
+      <c r="I41" s="71" t="s">
         <v>156</v>
       </c>
       <c r="J41" s="57"/>
       <c r="K41" s="58"/>
-      <c r="L41" s="71" t="s">
+      <c r="L41" s="69" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="57"/>
@@ -11702,7 +11702,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="70" t="s">
+      <c r="A77" s="73" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="55"/>
@@ -11720,17 +11720,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="67" t="s">
+      <c r="C79" s="72" t="s">
         <v>158</v>
       </c>
       <c r="D79" s="57"/>
       <c r="E79" s="58"/>
-      <c r="F79" s="69" t="s">
+      <c r="F79" s="70" t="s">
         <v>155</v>
       </c>
       <c r="G79" s="57"/>
       <c r="H79" s="58"/>
-      <c r="I79" s="71" t="s">
+      <c r="I79" s="69" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="57"/>
@@ -13023,6 +13023,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13039,12 +13045,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -16684,7 +16684,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="67" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="55"/>
@@ -22897,30 +22897,40 @@
       <c r="A25" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15" t="str">
+      <c r="B25" s="15">
+        <v>629</v>
+      </c>
+      <c r="C25" s="15">
+        <v>27</v>
+      </c>
+      <c r="D25" s="15">
+        <v>20</v>
+      </c>
+      <c r="E25" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15" t="str">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="F25" s="15">
+        <v>4</v>
+      </c>
+      <c r="G25" s="15">
+        <v>3</v>
+      </c>
+      <c r="H25" s="15">
         <f t="shared" si="11"/>
-        <v/>
+        <v>0.75</v>
       </c>
       <c r="I25" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J25" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K25" s="15" t="e">
+        <v>17</v>
+      </c>
+      <c r="K25" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
+        <v>0.73913043478260865</v>
       </c>
       <c r="L25" s="11"/>
       <c r="M25" s="15"/>
@@ -22953,30 +22963,40 @@
       <c r="A26" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15" t="str">
+      <c r="B26" s="15">
+        <v>630</v>
+      </c>
+      <c r="C26" s="15">
+        <v>4</v>
+      </c>
+      <c r="D26" s="15">
+        <v>4</v>
+      </c>
+      <c r="E26" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F26" s="15">
+        <v>0</v>
+      </c>
+      <c r="G26" s="15">
+        <v>0</v>
+      </c>
+      <c r="H26" s="15" t="e">
         <f t="shared" si="11"/>
-        <v/>
+        <v>#DIV/0!</v>
       </c>
       <c r="I26" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J26" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K26" s="15" t="e">
+        <v>4</v>
+      </c>
+      <c r="K26" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="L26" s="11"/>
       <c r="M26" s="15"/>
@@ -23009,30 +23029,40 @@
       <c r="A27" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15" t="str">
+      <c r="B27" s="15">
+        <v>630</v>
+      </c>
+      <c r="C27" s="15">
+        <v>3</v>
+      </c>
+      <c r="D27" s="15">
+        <v>3</v>
+      </c>
+      <c r="E27" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F27" s="15">
+        <v>0</v>
+      </c>
+      <c r="G27" s="15">
+        <v>0</v>
+      </c>
+      <c r="H27" s="15" t="e">
         <f t="shared" si="11"/>
-        <v/>
+        <v>#DIV/0!</v>
       </c>
       <c r="I27" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J27" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K27" s="15" t="e">
+        <v>3</v>
+      </c>
+      <c r="K27" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="L27" s="11"/>
       <c r="M27" s="15"/>
@@ -23065,30 +23095,40 @@
       <c r="A28" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15" t="str">
+      <c r="B28" s="15">
+        <v>630</v>
+      </c>
+      <c r="C28" s="15">
+        <v>21</v>
+      </c>
+      <c r="D28" s="15">
+        <v>18</v>
+      </c>
+      <c r="E28" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15" t="str">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="F28" s="15">
+        <v>3</v>
+      </c>
+      <c r="G28" s="15">
+        <v>2</v>
+      </c>
+      <c r="H28" s="15">
         <f t="shared" si="11"/>
-        <v/>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I28" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J28" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K28" s="15" t="e">
+        <v>16</v>
+      </c>
+      <c r="K28" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="L28" s="11"/>
       <c r="M28" s="15"/>
@@ -23624,39 +23664,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>356</v>
+        <v>411</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>287</v>
+        <v>332</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.8061797752808989</v>
+        <v>0.80778588807785889</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.81818181818181823</v>
+        <v>0.81052631578947365</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>268</v>
+        <v>316</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>215</v>
+        <v>255</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.80223880597014929</v>
+        <v>0.80696202531645567</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23705,39 +23745,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>356</v>
+        <v>411</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>287</v>
+        <v>332</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.8061797752808989</v>
+        <v>0.80778588807785889</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.81818181818181823</v>
+        <v>0.81052631578947365</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>268</v>
+        <v>316</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>215</v>
+        <v>255</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.80223880597014929</v>
+        <v>0.80696202531645567</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-30 22:10:05
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71CDD83-5D28-4AC8-A1F7-6187DF0521F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681ED759-4D1C-4900-BA70-73B82D2DBE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1477,25 +1477,25 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9428,7 +9428,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="72" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="55"/>
@@ -9446,17 +9446,17 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="72" t="s">
+      <c r="C3" s="67" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="57"/>
       <c r="E3" s="58"/>
-      <c r="F3" s="70" t="s">
+      <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="57"/>
       <c r="H3" s="58"/>
-      <c r="I3" s="69" t="s">
+      <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="57"/>
@@ -10423,7 +10423,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="70" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="55"/>
@@ -10444,22 +10444,22 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="72" t="s">
+      <c r="C41" s="67" t="s">
         <v>52</v>
       </c>
       <c r="D41" s="57"/>
       <c r="E41" s="58"/>
-      <c r="F41" s="70" t="s">
+      <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="57"/>
       <c r="H41" s="58"/>
-      <c r="I41" s="71" t="s">
+      <c r="I41" s="73" t="s">
         <v>156</v>
       </c>
       <c r="J41" s="57"/>
       <c r="K41" s="58"/>
-      <c r="L41" s="69" t="s">
+      <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="57"/>
@@ -11702,7 +11702,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="73" t="s">
+      <c r="A77" s="70" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="55"/>
@@ -11720,17 +11720,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="72" t="s">
+      <c r="C79" s="67" t="s">
         <v>158</v>
       </c>
       <c r="D79" s="57"/>
       <c r="E79" s="58"/>
-      <c r="F79" s="70" t="s">
+      <c r="F79" s="69" t="s">
         <v>155</v>
       </c>
       <c r="G79" s="57"/>
       <c r="H79" s="58"/>
-      <c r="I79" s="69" t="s">
+      <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="57"/>
@@ -13023,12 +13023,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13045,6 +13039,12 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -16684,7 +16684,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="72" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="55"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-01 17:47:57
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681ED759-4D1C-4900-BA70-73B82D2DBE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A88AF6-5D4C-43D1-A6D7-9D9A810DD07F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -23187,30 +23187,40 @@
       <c r="A30" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15" t="str">
+      <c r="B30" s="15">
+        <v>701</v>
+      </c>
+      <c r="C30" s="15">
+        <v>10</v>
+      </c>
+      <c r="D30" s="15">
+        <v>9</v>
+      </c>
+      <c r="E30" s="15">
         <f>IF(AND(C30&lt;&gt;"",D30&lt;&gt;""),D30/C30,"")</f>
-        <v/>
-      </c>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15" t="str">
+        <v>0.9</v>
+      </c>
+      <c r="F30" s="15">
+        <v>0</v>
+      </c>
+      <c r="G30" s="15">
+        <v>0</v>
+      </c>
+      <c r="H30" s="15" t="e">
         <f>IF(AND(F30&lt;&gt;"",G30&lt;&gt;""),G30/F30,"")</f>
-        <v/>
+        <v>#DIV/0!</v>
       </c>
       <c r="I30" s="15">
         <f t="shared" ref="I30:J32" si="18">C30-F30</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J30" s="15">
         <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="K30" s="15" t="e">
+        <v>9</v>
+      </c>
+      <c r="K30" s="15">
         <f>IF(AND(I30&lt;&gt;"",J30&lt;&gt;""),J30/I30,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.9</v>
       </c>
       <c r="L30" s="11"/>
       <c r="M30" s="15"/>
@@ -23243,30 +23253,40 @@
       <c r="A31" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15" t="str">
+      <c r="B31" s="15">
+        <v>701</v>
+      </c>
+      <c r="C31" s="15">
+        <v>17</v>
+      </c>
+      <c r="D31" s="15">
+        <v>11</v>
+      </c>
+      <c r="E31" s="15">
         <f>IF(AND(C31&lt;&gt;"",D31&lt;&gt;""),D31/C31,"")</f>
-        <v/>
-      </c>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15" t="str">
+        <v>0.6470588235294118</v>
+      </c>
+      <c r="F31" s="15">
+        <v>4</v>
+      </c>
+      <c r="G31" s="15">
+        <v>1</v>
+      </c>
+      <c r="H31" s="15">
         <f>IF(AND(F31&lt;&gt;"",G31&lt;&gt;""),G31/F31,"")</f>
-        <v/>
+        <v>0.25</v>
       </c>
       <c r="I31" s="15">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J31" s="15">
         <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="K31" s="15" t="e">
+        <v>10</v>
+      </c>
+      <c r="K31" s="15">
         <f>IF(AND(I31&lt;&gt;"",J31&lt;&gt;""),J31/I31,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.76923076923076927</v>
       </c>
       <c r="L31" s="11"/>
       <c r="M31" s="15"/>
@@ -23664,39 +23684,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>411</v>
+        <v>438</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>332</v>
+        <v>352</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.80778588807785889</v>
+        <v>0.80365296803652964</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.81052631578947365</v>
+        <v>0.78787878787878785</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>316</v>
+        <v>339</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.80696202531645567</v>
+        <v>0.80825958702064893</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23745,39 +23765,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>411</v>
+        <v>438</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>332</v>
+        <v>352</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.80778588807785889</v>
+        <v>0.80365296803652964</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.81052631578947365</v>
+        <v>0.78787878787878785</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>316</v>
+        <v>339</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.80696202531645567</v>
+        <v>0.80825958702064893</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-03 16:35:51
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A88AF6-5D4C-43D1-A6D7-9D9A810DD07F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B03D23E9-1CDC-4BE0-B94B-140ABBA46493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1309,7 +1309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1444,21 +1444,21 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1498,13 +1498,16 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7536,13 +7539,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="60"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8047,13 +8050,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="60" t="s">
+      <c r="A41" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="57"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8534,13 +8537,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="60" t="s">
+      <c r="A83" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="57"/>
-      <c r="C83" s="57"/>
-      <c r="D83" s="57"/>
-      <c r="E83" s="58"/>
+      <c r="B83" s="59"/>
+      <c r="C83" s="59"/>
+      <c r="D83" s="59"/>
+      <c r="E83" s="60"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8782,23 +8785,23 @@
       <c r="C3" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="66" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
       <c r="I3" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="58"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="60"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -8948,20 +8951,30 @@
       <c r="A7" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="B7" s="34"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34" t="str">
+      <c r="B7" s="34">
+        <v>702</v>
+      </c>
+      <c r="C7" s="34">
+        <v>13</v>
+      </c>
+      <c r="D7" s="34">
+        <v>11</v>
+      </c>
+      <c r="E7" s="34">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34" t="str">
+        <v>0.84615384615384615</v>
+      </c>
+      <c r="F7" s="34">
+        <v>24</v>
+      </c>
+      <c r="G7" s="34">
+        <v>18</v>
+      </c>
+      <c r="H7" s="34">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I7" s="34"/>
+        <v>0.75</v>
+      </c>
+      <c r="I7" s="77"/>
       <c r="J7" s="34"/>
       <c r="K7" s="34" t="str">
         <f t="shared" si="2"/>
@@ -8969,15 +8982,15 @@
       </c>
       <c r="L7" s="34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="M7" s="34">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N7" s="34" t="e">
+        <v>29</v>
+      </c>
+      <c r="N7" s="34">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.78378378378378377</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9203,27 +9216,27 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.8125</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>0.94736842105263153</v>
+        <v>0.83720930232558144</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
@@ -9239,15 +9252,15 @@
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>103</v>
+        <v>140</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.79611650485436891</v>
+        <v>0.79285714285714282</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9258,27 +9271,27 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>0.8</v>
+        <v>0.8125</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>0.94736842105263153</v>
+        <v>0.83720930232558144</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
@@ -9294,15 +9307,15 @@
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>103</v>
+        <v>140</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.79611650485436891</v>
+        <v>0.79285714285714282</v>
       </c>
     </row>
   </sheetData>
@@ -9449,18 +9462,18 @@
       <c r="C3" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
       <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9501,16 +9514,16 @@
       <c r="A5" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9849,16 +9862,16 @@
       <c r="A17" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="57"/>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="58"/>
+      <c r="B17" s="59"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="60"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10087,16 +10100,16 @@
       <c r="A26" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="57"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="58"/>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="60"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10447,23 +10460,23 @@
       <c r="C41" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
       <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="57"/>
-      <c r="H41" s="58"/>
+      <c r="G41" s="59"/>
+      <c r="H41" s="60"/>
       <c r="I41" s="73" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="57"/>
-      <c r="K41" s="58"/>
+      <c r="J41" s="59"/>
+      <c r="K41" s="60"/>
       <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="57"/>
-      <c r="N41" s="58"/>
+      <c r="M41" s="59"/>
+      <c r="N41" s="60"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10513,19 +10526,19 @@
       <c r="A43" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="57"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="57"/>
-      <c r="N43" s="58"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
+      <c r="H43" s="59"/>
+      <c r="I43" s="59"/>
+      <c r="J43" s="59"/>
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
+      <c r="M43" s="59"/>
+      <c r="N43" s="60"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10960,19 +10973,19 @@
       <c r="A55" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="57"/>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="57"/>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
-      <c r="I55" s="57"/>
-      <c r="J55" s="57"/>
-      <c r="K55" s="57"/>
-      <c r="L55" s="57"/>
-      <c r="M55" s="57"/>
-      <c r="N55" s="58"/>
+      <c r="B55" s="59"/>
+      <c r="C55" s="59"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="59"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="59"/>
+      <c r="K55" s="59"/>
+      <c r="L55" s="59"/>
+      <c r="M55" s="59"/>
+      <c r="N55" s="60"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11267,19 +11280,19 @@
       <c r="A64" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="57"/>
-      <c r="H64" s="57"/>
-      <c r="I64" s="57"/>
-      <c r="J64" s="57"/>
-      <c r="K64" s="57"/>
-      <c r="L64" s="57"/>
-      <c r="M64" s="57"/>
-      <c r="N64" s="58"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="59"/>
+      <c r="D64" s="59"/>
+      <c r="E64" s="59"/>
+      <c r="F64" s="59"/>
+      <c r="G64" s="59"/>
+      <c r="H64" s="59"/>
+      <c r="I64" s="59"/>
+      <c r="J64" s="59"/>
+      <c r="K64" s="59"/>
+      <c r="L64" s="59"/>
+      <c r="M64" s="59"/>
+      <c r="N64" s="60"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11723,18 +11736,18 @@
       <c r="C79" s="67" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="57"/>
-      <c r="E79" s="58"/>
+      <c r="D79" s="59"/>
+      <c r="E79" s="60"/>
       <c r="F79" s="69" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="57"/>
-      <c r="H79" s="58"/>
+      <c r="G79" s="59"/>
+      <c r="H79" s="60"/>
       <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="57"/>
-      <c r="K79" s="58"/>
+      <c r="J79" s="59"/>
+      <c r="K79" s="60"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11775,16 +11788,16 @@
       <c r="A81" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="57"/>
-      <c r="C81" s="57"/>
-      <c r="D81" s="57"/>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="57"/>
-      <c r="J81" s="57"/>
-      <c r="K81" s="58"/>
+      <c r="B81" s="59"/>
+      <c r="C81" s="59"/>
+      <c r="D81" s="59"/>
+      <c r="E81" s="59"/>
+      <c r="F81" s="59"/>
+      <c r="G81" s="59"/>
+      <c r="H81" s="59"/>
+      <c r="I81" s="59"/>
+      <c r="J81" s="59"/>
+      <c r="K81" s="60"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12238,16 +12251,16 @@
       <c r="A93" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="57"/>
-      <c r="C93" s="57"/>
-      <c r="D93" s="57"/>
-      <c r="E93" s="57"/>
-      <c r="F93" s="57"/>
-      <c r="G93" s="57"/>
-      <c r="H93" s="57"/>
-      <c r="I93" s="57"/>
-      <c r="J93" s="57"/>
-      <c r="K93" s="58"/>
+      <c r="B93" s="59"/>
+      <c r="C93" s="59"/>
+      <c r="D93" s="59"/>
+      <c r="E93" s="59"/>
+      <c r="F93" s="59"/>
+      <c r="G93" s="59"/>
+      <c r="H93" s="59"/>
+      <c r="I93" s="59"/>
+      <c r="J93" s="59"/>
+      <c r="K93" s="60"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12566,16 +12579,16 @@
       <c r="A102" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="57"/>
-      <c r="C102" s="57"/>
-      <c r="D102" s="57"/>
-      <c r="E102" s="57"/>
-      <c r="F102" s="57"/>
-      <c r="G102" s="57"/>
-      <c r="H102" s="57"/>
-      <c r="I102" s="57"/>
-      <c r="J102" s="57"/>
-      <c r="K102" s="58"/>
+      <c r="B102" s="59"/>
+      <c r="C102" s="59"/>
+      <c r="D102" s="59"/>
+      <c r="E102" s="59"/>
+      <c r="F102" s="59"/>
+      <c r="G102" s="59"/>
+      <c r="H102" s="59"/>
+      <c r="I102" s="59"/>
+      <c r="J102" s="59"/>
+      <c r="K102" s="60"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13438,7 +13451,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="55"/>
@@ -13465,32 +13478,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16711,32 +16724,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19576,7 +19589,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="55"/>
@@ -19603,32 +19616,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21614,7 +21627,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="74" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="55"/>
@@ -21641,32 +21654,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="76" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="56" t="s">
+      <c r="M3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24355,7 +24368,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -24385,35 +24398,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="57" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="55"/>
       <c r="D3" s="55"/>
       <c r="E3" s="55"/>
       <c r="F3" s="55"/>
-      <c r="G3" s="76" t="s">
+      <c r="G3" s="57" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="55"/>
       <c r="I3" s="55"/>
       <c r="J3" s="55"/>
       <c r="K3" s="55"/>
-      <c r="L3" s="76" t="s">
+      <c r="L3" s="57" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="55"/>
       <c r="N3" s="55"/>
       <c r="O3" s="55"/>
       <c r="P3" s="55"/>
-      <c r="Q3" s="76" t="s">
+      <c r="Q3" s="57" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="55"/>
       <c r="S3" s="55"/>
       <c r="T3" s="55"/>
       <c r="U3" s="55"/>
-      <c r="V3" s="75" t="s">
+      <c r="V3" s="56" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="55"/>
@@ -24926,15 +24939,21 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q10" s="48"/>
-      <c r="R10" s="48"/>
+      <c r="Q10" s="48">
+        <v>7.2</v>
+      </c>
+      <c r="R10" s="48">
+        <v>15</v>
+      </c>
       <c r="S10" s="48">
         <v>5</v>
       </c>
-      <c r="T10" s="48"/>
-      <c r="U10" s="48" t="str">
+      <c r="T10" s="48">
+        <v>4</v>
+      </c>
+      <c r="U10" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="V10" s="48">
         <f t="shared" si="4"/>
@@ -24942,11 +24961,11 @@
       </c>
       <c r="W10" s="48">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="X10" s="48">
         <f t="shared" si="6"/>
-        <v>0.45</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25573,11 +25592,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25585,11 +25604,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>9.0624999999999997E-2</v>
+        <v>0.10312499999999999</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25647,11 +25666,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -25659,11 +25678,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>9.0624999999999997E-2</v>
+        <v>0.10312499999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-04 19:25:14
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B03D23E9-1CDC-4BE0-B94B-140ABBA46493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DA38D4-BF28-4B94-864C-3E06B33A01CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1444,21 +1444,36 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1477,27 +1492,6 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1507,7 +1501,13 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7512,13 +7512,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="66" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
     </row>
     <row r="2" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7539,13 +7539,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="57"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8050,13 +8050,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="59"/>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="B41" s="56"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="57"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8537,13 +8537,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="58" t="s">
+      <c r="A83" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="59"/>
-      <c r="C83" s="59"/>
-      <c r="D83" s="59"/>
-      <c r="E83" s="60"/>
+      <c r="B83" s="56"/>
+      <c r="C83" s="56"/>
+      <c r="D83" s="56"/>
+      <c r="E83" s="57"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8761,47 +8761,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
     </row>
     <row r="2" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="63" t="s">
+      <c r="C3" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="56"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="71" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="65" t="s">
+      <c r="G3" s="56"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="70" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="64" t="s">
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="59"/>
-      <c r="N3" s="60"/>
+      <c r="M3" s="56"/>
+      <c r="N3" s="57"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -8974,23 +8974,27 @@
         <f t="shared" si="1"/>
         <v>0.75</v>
       </c>
-      <c r="I7" s="77"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34" t="str">
+      <c r="I7" s="54">
+        <v>25</v>
+      </c>
+      <c r="J7" s="34">
+        <v>13</v>
+      </c>
+      <c r="K7" s="34">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.52</v>
       </c>
       <c r="L7" s="34">
         <f t="shared" si="3"/>
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="M7" s="34">
         <f t="shared" si="4"/>
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="N7" s="34">
         <f t="shared" si="5"/>
-        <v>0.78378378378378377</v>
+        <v>0.67741935483870963</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9240,27 +9244,27 @@
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="J14" s="37">
         <f>SUM(J5:J13)</f>
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="K14" s="37">
         <f t="shared" si="2"/>
-        <v>0.73469387755102045</v>
+        <v>0.66216216216216217</v>
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.79285714285714282</v>
+        <v>0.75151515151515147</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9295,27 +9299,27 @@
       </c>
       <c r="I16" s="40">
         <f>I14</f>
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="J16" s="40">
         <f>J14</f>
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="K16" s="40">
         <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),J16/I16,"")</f>
-        <v>0.73469387755102045</v>
+        <v>0.66216216216216217</v>
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.79285714285714282</v>
+        <v>0.75151515151515147</v>
       </c>
     </row>
   </sheetData>
@@ -9441,39 +9445,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="63" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
     </row>
     <row r="2" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="69" t="s">
+      <c r="D3" s="56"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="71" t="s">
+      <c r="G3" s="56"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9511,19 +9515,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="60"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="57"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9609,12 +9613,18 @@
       <c r="A8" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4" t="str">
+      <c r="B8" s="4">
+        <v>704</v>
+      </c>
+      <c r="C8" s="4">
+        <v>32</v>
+      </c>
+      <c r="D8" s="4">
+        <v>28</v>
+      </c>
+      <c r="E8" s="4">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.875</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -9624,15 +9634,15 @@
       </c>
       <c r="I8" s="4">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="J8" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K8" s="4" t="e">
+        <v>28</v>
+      </c>
+      <c r="K8" s="4">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9822,15 +9832,15 @@
       <c r="B15" s="6"/>
       <c r="C15" s="7">
         <f>SUM(C6:C14)</f>
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="D15" s="7">
         <f>SUM(D6:D14)</f>
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>0.87755102040816324</v>
+        <v>0.87654320987654322</v>
       </c>
       <c r="F15" s="7">
         <f>SUM(F6:F14)</f>
@@ -9846,32 +9856,32 @@
       </c>
       <c r="I15" s="7">
         <f>SUM(I6:I14)</f>
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="J15" s="7">
         <f>SUM(J6:J14)</f>
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="4"/>
-        <v>0.8867924528301887</v>
+        <v>0.88405797101449279</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="68" t="s">
+      <c r="A17" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="60"/>
+      <c r="B17" s="56"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="56"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="56"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="57"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10097,19 +10107,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="68" t="s">
+      <c r="A26" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="60"/>
+      <c r="B26" s="56"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="56"/>
+      <c r="G26" s="56"/>
+      <c r="H26" s="56"/>
+      <c r="I26" s="56"/>
+      <c r="J26" s="56"/>
+      <c r="K26" s="57"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10400,15 +10410,15 @@
       <c r="B36" s="9"/>
       <c r="C36" s="10">
         <f>C15+C24+C35</f>
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="D36" s="10">
         <f>D15+D24+D35</f>
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="E36" s="10">
         <f t="shared" si="9"/>
-        <v>0.87755102040816324</v>
+        <v>0.87654320987654322</v>
       </c>
       <c r="F36" s="10">
         <f>F15+F24+F35</f>
@@ -10424,59 +10434,59 @@
       </c>
       <c r="I36" s="10">
         <f>I15+I24+I35</f>
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="J36" s="10">
         <f>J15+J24+J35</f>
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>0.8867924528301887</v>
+        <v>0.88405797101449279</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="70" t="s">
+      <c r="A39" s="60" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="55"/>
-      <c r="C39" s="55"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
-      <c r="I39" s="55"/>
-      <c r="J39" s="55"/>
-      <c r="K39" s="55"/>
-      <c r="L39" s="55"/>
-      <c r="M39" s="55"/>
-      <c r="N39" s="55"/>
+      <c r="B39" s="61"/>
+      <c r="C39" s="61"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="61"/>
+      <c r="G39" s="61"/>
+      <c r="H39" s="61"/>
+      <c r="I39" s="61"/>
+      <c r="J39" s="61"/>
+      <c r="K39" s="61"/>
+      <c r="L39" s="61"/>
+      <c r="M39" s="61"/>
+      <c r="N39" s="61"/>
     </row>
     <row r="40" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="67" t="s">
+      <c r="C41" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="69" t="s">
+      <c r="D41" s="56"/>
+      <c r="E41" s="57"/>
+      <c r="F41" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="59"/>
-      <c r="H41" s="60"/>
-      <c r="I41" s="73" t="s">
+      <c r="G41" s="56"/>
+      <c r="H41" s="57"/>
+      <c r="I41" s="64" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="59"/>
-      <c r="K41" s="60"/>
-      <c r="L41" s="71" t="s">
+      <c r="J41" s="56"/>
+      <c r="K41" s="57"/>
+      <c r="L41" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="59"/>
-      <c r="N41" s="60"/>
+      <c r="M41" s="56"/>
+      <c r="N41" s="57"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10523,22 +10533,22 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="68" t="s">
+      <c r="A43" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="59"/>
-      <c r="C43" s="59"/>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="59"/>
-      <c r="I43" s="59"/>
-      <c r="J43" s="59"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="60"/>
+      <c r="B43" s="56"/>
+      <c r="C43" s="56"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="56"/>
+      <c r="H43" s="56"/>
+      <c r="I43" s="56"/>
+      <c r="J43" s="56"/>
+      <c r="K43" s="56"/>
+      <c r="L43" s="56"/>
+      <c r="M43" s="56"/>
+      <c r="N43" s="57"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10647,7 +10657,7 @@
       </c>
       <c r="B46" s="4">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>704</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -10970,22 +10980,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="68" t="s">
+      <c r="A55" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="59"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="F55" s="59"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="59"/>
-      <c r="I55" s="59"/>
-      <c r="J55" s="59"/>
-      <c r="K55" s="59"/>
-      <c r="L55" s="59"/>
-      <c r="M55" s="59"/>
-      <c r="N55" s="60"/>
+      <c r="B55" s="56"/>
+      <c r="C55" s="56"/>
+      <c r="D55" s="56"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="56"/>
+      <c r="G55" s="56"/>
+      <c r="H55" s="56"/>
+      <c r="I55" s="56"/>
+      <c r="J55" s="56"/>
+      <c r="K55" s="56"/>
+      <c r="L55" s="56"/>
+      <c r="M55" s="56"/>
+      <c r="N55" s="57"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11277,22 +11287,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="68" t="s">
+      <c r="A64" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="59"/>
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-      <c r="F64" s="59"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="59"/>
-      <c r="I64" s="59"/>
-      <c r="J64" s="59"/>
-      <c r="K64" s="59"/>
-      <c r="L64" s="59"/>
-      <c r="M64" s="59"/>
-      <c r="N64" s="60"/>
+      <c r="B64" s="56"/>
+      <c r="C64" s="56"/>
+      <c r="D64" s="56"/>
+      <c r="E64" s="56"/>
+      <c r="F64" s="56"/>
+      <c r="G64" s="56"/>
+      <c r="H64" s="56"/>
+      <c r="I64" s="56"/>
+      <c r="J64" s="56"/>
+      <c r="K64" s="56"/>
+      <c r="L64" s="56"/>
+      <c r="M64" s="56"/>
+      <c r="N64" s="57"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11715,39 +11725,39 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="70" t="s">
+      <c r="A77" s="60" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="55"/>
-      <c r="C77" s="55"/>
-      <c r="D77" s="55"/>
-      <c r="E77" s="55"/>
-      <c r="F77" s="55"/>
-      <c r="G77" s="55"/>
-      <c r="H77" s="55"/>
-      <c r="I77" s="55"/>
-      <c r="J77" s="55"/>
-      <c r="K77" s="55"/>
+      <c r="B77" s="61"/>
+      <c r="C77" s="61"/>
+      <c r="D77" s="61"/>
+      <c r="E77" s="61"/>
+      <c r="F77" s="61"/>
+      <c r="G77" s="61"/>
+      <c r="H77" s="61"/>
+      <c r="I77" s="61"/>
+      <c r="J77" s="61"/>
+      <c r="K77" s="61"/>
     </row>
     <row r="78" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="67" t="s">
+      <c r="C79" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="59"/>
-      <c r="E79" s="60"/>
-      <c r="F79" s="69" t="s">
+      <c r="D79" s="56"/>
+      <c r="E79" s="57"/>
+      <c r="F79" s="59" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="59"/>
-      <c r="H79" s="60"/>
-      <c r="I79" s="71" t="s">
+      <c r="G79" s="56"/>
+      <c r="H79" s="57"/>
+      <c r="I79" s="62" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="59"/>
-      <c r="K79" s="60"/>
+      <c r="J79" s="56"/>
+      <c r="K79" s="57"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11785,19 +11795,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="68" t="s">
+      <c r="A81" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="59"/>
-      <c r="C81" s="59"/>
-      <c r="D81" s="59"/>
-      <c r="E81" s="59"/>
-      <c r="F81" s="59"/>
-      <c r="G81" s="59"/>
-      <c r="H81" s="59"/>
-      <c r="I81" s="59"/>
-      <c r="J81" s="59"/>
-      <c r="K81" s="60"/>
+      <c r="B81" s="56"/>
+      <c r="C81" s="56"/>
+      <c r="D81" s="56"/>
+      <c r="E81" s="56"/>
+      <c r="F81" s="56"/>
+      <c r="G81" s="56"/>
+      <c r="H81" s="56"/>
+      <c r="I81" s="56"/>
+      <c r="J81" s="56"/>
+      <c r="K81" s="57"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -11895,19 +11905,19 @@
       </c>
       <c r="B84" s="4">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>704</v>
       </c>
       <c r="C84" s="4">
         <f t="shared" si="33"/>
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="D84" s="4">
         <f t="shared" si="34"/>
-        <v>0</v>
-      </c>
-      <c r="E84" s="4" t="e">
+        <v>28</v>
+      </c>
+      <c r="E84" s="4">
         <f t="shared" si="35"/>
-        <v>#DIV/0!</v>
+        <v>0.875</v>
       </c>
       <c r="F84" s="4">
         <f t="shared" si="36"/>
@@ -11923,15 +11933,15 @@
       </c>
       <c r="I84" s="4">
         <f t="shared" si="39"/>
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="J84" s="4">
         <f t="shared" si="40"/>
-        <v>0</v>
-      </c>
-      <c r="K84" s="4" t="e">
+        <v>28</v>
+      </c>
+      <c r="K84" s="4">
         <f t="shared" si="41"/>
-        <v>#DIV/0!</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12211,15 +12221,15 @@
       <c r="B91" s="6"/>
       <c r="C91" s="7">
         <f>SUM(C82:C90)</f>
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="D91" s="7">
         <f>SUM(D82:D90)</f>
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="E91" s="7">
         <f t="shared" si="35"/>
-        <v>0.8867924528301887</v>
+        <v>0.88405797101449279</v>
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
@@ -12235,32 +12245,32 @@
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>163</v>
+        <v>195</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.79141104294478526</v>
+        <v>0.80512820512820515</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="68" t="s">
+      <c r="A93" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="59"/>
-      <c r="C93" s="59"/>
-      <c r="D93" s="59"/>
-      <c r="E93" s="59"/>
-      <c r="F93" s="59"/>
-      <c r="G93" s="59"/>
-      <c r="H93" s="59"/>
-      <c r="I93" s="59"/>
-      <c r="J93" s="59"/>
-      <c r="K93" s="60"/>
+      <c r="B93" s="56"/>
+      <c r="C93" s="56"/>
+      <c r="D93" s="56"/>
+      <c r="E93" s="56"/>
+      <c r="F93" s="56"/>
+      <c r="G93" s="56"/>
+      <c r="H93" s="56"/>
+      <c r="I93" s="56"/>
+      <c r="J93" s="56"/>
+      <c r="K93" s="57"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12576,19 +12586,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="68" t="s">
+      <c r="A102" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="59"/>
-      <c r="C102" s="59"/>
-      <c r="D102" s="59"/>
-      <c r="E102" s="59"/>
-      <c r="F102" s="59"/>
-      <c r="G102" s="59"/>
-      <c r="H102" s="59"/>
-      <c r="I102" s="59"/>
-      <c r="J102" s="59"/>
-      <c r="K102" s="60"/>
+      <c r="B102" s="56"/>
+      <c r="C102" s="56"/>
+      <c r="D102" s="56"/>
+      <c r="E102" s="56"/>
+      <c r="F102" s="56"/>
+      <c r="G102" s="56"/>
+      <c r="H102" s="56"/>
+      <c r="I102" s="56"/>
+      <c r="J102" s="56"/>
+      <c r="K102" s="57"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -12999,15 +13009,15 @@
       <c r="B112" s="9"/>
       <c r="C112" s="10">
         <f>C91+C100+C111</f>
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="D112" s="10">
         <f>D91+D100+D111</f>
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="E112" s="10">
         <f t="shared" si="51"/>
-        <v>0.8867924528301887</v>
+        <v>0.88405797101449279</v>
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
@@ -13023,15 +13033,15 @@
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>163</v>
+        <v>195</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.79141104294478526</v>
+        <v>0.80512820512820515</v>
       </c>
     </row>
   </sheetData>
@@ -13451,59 +13461,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="72" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="61"/>
+      <c r="T1" s="61"/>
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="56"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="56"/>
+      <c r="Q3" s="56"/>
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="57"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16697,59 +16707,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="63" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="61"/>
+      <c r="T1" s="61"/>
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="56"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="56"/>
+      <c r="Q3" s="56"/>
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="57"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19589,59 +19599,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="72" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="61"/>
+      <c r="T1" s="61"/>
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="56"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="56"/>
+      <c r="Q3" s="56"/>
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="57"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21627,59 +21637,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="72" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="61"/>
+      <c r="T1" s="61"/>
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="75" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="56"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="56"/>
+      <c r="Q3" s="56"/>
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="57"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -23332,30 +23342,40 @@
       <c r="A32" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15" t="str">
+      <c r="B32" s="15">
+        <v>703</v>
+      </c>
+      <c r="C32" s="15">
+        <v>61</v>
+      </c>
+      <c r="D32" s="15">
+        <v>51</v>
+      </c>
+      <c r="E32" s="15">
         <f>IF(AND(C32&lt;&gt;"",D32&lt;&gt;""),D32/C32,"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="15" t="str">
+        <v>0.83606557377049184</v>
+      </c>
+      <c r="F32" s="15">
+        <v>21</v>
+      </c>
+      <c r="G32" s="15">
+        <v>18</v>
+      </c>
+      <c r="H32" s="15">
         <f>IF(AND(F32&lt;&gt;"",G32&lt;&gt;""),G32/F32,"")</f>
-        <v/>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I32" s="15">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J32" s="15">
         <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="K32" s="15" t="e">
+        <v>33</v>
+      </c>
+      <c r="K32" s="15">
         <f>IF(AND(I32&lt;&gt;"",J32&lt;&gt;""),J32/I32,"")</f>
-        <v>#DIV/0!</v>
+        <v>0.82499999999999996</v>
       </c>
       <c r="L32" s="11"/>
       <c r="M32" s="15"/>
@@ -23414,30 +23434,40 @@
       <c r="A34" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15" t="str">
+      <c r="B34" s="15">
+        <v>704</v>
+      </c>
+      <c r="C34" s="15">
+        <v>6</v>
+      </c>
+      <c r="D34" s="15">
+        <v>6</v>
+      </c>
+      <c r="E34" s="15">
         <f t="shared" ref="E34:E39" si="20">IF(AND(C34&lt;&gt;"",D34&lt;&gt;""),D34/C34,"")</f>
-        <v/>
-      </c>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F34" s="15">
+        <v>1</v>
+      </c>
+      <c r="G34" s="15">
+        <v>1</v>
+      </c>
+      <c r="H34" s="15">
         <f t="shared" ref="H34:H39" si="21">IF(AND(F34&lt;&gt;"",G34&lt;&gt;""),G34/F34,"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I34" s="15">
         <f t="shared" ref="I34:J38" si="22">C34-F34</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J34" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="K34" s="15" t="e">
+        <v>5</v>
+      </c>
+      <c r="K34" s="15">
         <f t="shared" ref="K34:K39" si="23">IF(AND(I34&lt;&gt;"",J34&lt;&gt;""),J34/I34,"")</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="L34" s="11"/>
       <c r="M34" s="15"/>
@@ -23470,30 +23500,40 @@
       <c r="A35" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15" t="str">
+      <c r="B35" s="15">
+        <v>704</v>
+      </c>
+      <c r="C35" s="15">
+        <v>14</v>
+      </c>
+      <c r="D35" s="15">
+        <v>11</v>
+      </c>
+      <c r="E35" s="15">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15" t="str">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="F35" s="15">
+        <v>4</v>
+      </c>
+      <c r="G35" s="15">
+        <v>4</v>
+      </c>
+      <c r="H35" s="15">
         <f t="shared" si="21"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I35" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J35" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="K35" s="15" t="e">
+        <v>7</v>
+      </c>
+      <c r="K35" s="15">
         <f t="shared" si="23"/>
-        <v>#DIV/0!</v>
+        <v>0.7</v>
       </c>
       <c r="L35" s="11"/>
       <c r="M35" s="15"/>
@@ -23526,30 +23566,40 @@
       <c r="A36" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15" t="str">
+      <c r="B36" s="15">
+        <v>704</v>
+      </c>
+      <c r="C36" s="15">
+        <v>11</v>
+      </c>
+      <c r="D36" s="15">
+        <v>10</v>
+      </c>
+      <c r="E36" s="15">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="15" t="str">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="F36" s="15">
+        <v>2</v>
+      </c>
+      <c r="G36" s="15">
+        <v>2</v>
+      </c>
+      <c r="H36" s="15">
         <f t="shared" si="21"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I36" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J36" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="K36" s="15" t="e">
+        <v>8</v>
+      </c>
+      <c r="K36" s="15">
         <f t="shared" si="23"/>
-        <v>#DIV/0!</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="L36" s="11"/>
       <c r="M36" s="15"/>
@@ -23697,39 +23747,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>438</v>
+        <v>530</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>352</v>
+        <v>430</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.80365296803652964</v>
+        <v>0.81132075471698117</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.78787878787878785</v>
+        <v>0.8110236220472441</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>339</v>
+        <v>403</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>274</v>
+        <v>327</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.80825958702064893</v>
+        <v>0.81141439205955335</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23778,39 +23828,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>438</v>
+        <v>530</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>352</v>
+        <v>430</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.80365296803652964</v>
+        <v>0.81132075471698117</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.78787878787878785</v>
+        <v>0.8110236220472441</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>339</v>
+        <v>403</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>274</v>
+        <v>327</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.80825958702064893</v>
+        <v>0.81141439205955335</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
@@ -24368,69 +24418,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
+      <c r="A1" s="75" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="61"/>
+      <c r="T1" s="61"/>
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
+      <c r="W1" s="61"/>
+      <c r="X1" s="61"/>
     </row>
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="57" t="s">
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="57" t="s">
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="55"/>
-      <c r="N3" s="55"/>
-      <c r="O3" s="55"/>
-      <c r="P3" s="55"/>
-      <c r="Q3" s="57" t="s">
+      <c r="M3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="55"/>
-      <c r="S3" s="55"/>
-      <c r="T3" s="55"/>
-      <c r="U3" s="55"/>
-      <c r="V3" s="56" t="s">
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="55"/>
-      <c r="X3" s="55"/>
+      <c r="W3" s="61"/>
+      <c r="X3" s="61"/>
     </row>
     <row r="4" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">

</xml_diff>

<commit_message>
vault backup: 2026-07-05 11:39:52
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DA38D4-BF28-4B94-864C-3E06B33A01CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2657B98-1432-4C0E-9878-1CE0250085DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1447,28 +1447,16 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1492,13 +1480,25 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7512,13 +7512,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
     </row>
     <row r="2" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7539,13 +7539,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="61" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="59"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8050,13 +8050,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="65" t="s">
+      <c r="A41" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="56"/>
-      <c r="C41" s="56"/>
-      <c r="D41" s="56"/>
-      <c r="E41" s="57"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="59"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8537,13 +8537,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="65" t="s">
+      <c r="A83" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="56"/>
-      <c r="C83" s="56"/>
-      <c r="D83" s="56"/>
-      <c r="E83" s="57"/>
+      <c r="B83" s="58"/>
+      <c r="C83" s="58"/>
+      <c r="D83" s="58"/>
+      <c r="E83" s="59"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8761,47 +8761,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="63" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
     </row>
     <row r="2" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="68" t="s">
+      <c r="C3" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="56"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="71" t="s">
+      <c r="D3" s="58"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="67" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="56"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="70" t="s">
+      <c r="G3" s="58"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="56"/>
-      <c r="K3" s="57"/>
-      <c r="L3" s="69" t="s">
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="56"/>
-      <c r="N3" s="57"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="59"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9445,39 +9445,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
     </row>
     <row r="2" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="56"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="59" t="s">
+      <c r="D3" s="58"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="56"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="62" t="s">
+      <c r="G3" s="58"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="56"/>
-      <c r="K3" s="57"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9515,19 +9515,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="56"/>
-      <c r="C5" s="56"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="57"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
+      <c r="J5" s="58"/>
+      <c r="K5" s="59"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9869,19 +9869,19 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="58" t="s">
+      <c r="A17" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="56"/>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="56"/>
-      <c r="J17" s="56"/>
-      <c r="K17" s="57"/>
+      <c r="B17" s="58"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="58"/>
+      <c r="K17" s="59"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10107,19 +10107,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="58" t="s">
+      <c r="A26" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="56"/>
-      <c r="C26" s="56"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="56"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="56"/>
-      <c r="H26" s="56"/>
-      <c r="I26" s="56"/>
-      <c r="J26" s="56"/>
-      <c r="K26" s="57"/>
+      <c r="B26" s="58"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="59"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10446,47 +10446,47 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="60" t="s">
+      <c r="A39" s="74" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="61"/>
-      <c r="C39" s="61"/>
-      <c r="D39" s="61"/>
-      <c r="E39" s="61"/>
-      <c r="F39" s="61"/>
-      <c r="G39" s="61"/>
-      <c r="H39" s="61"/>
-      <c r="I39" s="61"/>
-      <c r="J39" s="61"/>
-      <c r="K39" s="61"/>
-      <c r="L39" s="61"/>
-      <c r="M39" s="61"/>
-      <c r="N39" s="61"/>
+      <c r="B39" s="56"/>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="56"/>
+      <c r="K39" s="56"/>
+      <c r="L39" s="56"/>
+      <c r="M39" s="56"/>
+      <c r="N39" s="56"/>
     </row>
     <row r="40" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="55" t="s">
+      <c r="C41" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="56"/>
-      <c r="E41" s="57"/>
-      <c r="F41" s="59" t="s">
+      <c r="D41" s="58"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="56"/>
-      <c r="H41" s="57"/>
-      <c r="I41" s="64" t="s">
+      <c r="G41" s="58"/>
+      <c r="H41" s="59"/>
+      <c r="I41" s="72" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="56"/>
-      <c r="K41" s="57"/>
-      <c r="L41" s="62" t="s">
+      <c r="J41" s="58"/>
+      <c r="K41" s="59"/>
+      <c r="L41" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="56"/>
-      <c r="N41" s="57"/>
+      <c r="M41" s="58"/>
+      <c r="N41" s="59"/>
     </row>
     <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10533,22 +10533,22 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="58" t="s">
+      <c r="A43" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="56"/>
-      <c r="C43" s="56"/>
-      <c r="D43" s="56"/>
-      <c r="E43" s="56"/>
-      <c r="F43" s="56"/>
-      <c r="G43" s="56"/>
-      <c r="H43" s="56"/>
-      <c r="I43" s="56"/>
-      <c r="J43" s="56"/>
-      <c r="K43" s="56"/>
-      <c r="L43" s="56"/>
-      <c r="M43" s="56"/>
-      <c r="N43" s="57"/>
+      <c r="B43" s="58"/>
+      <c r="C43" s="58"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="58"/>
+      <c r="F43" s="58"/>
+      <c r="G43" s="58"/>
+      <c r="H43" s="58"/>
+      <c r="I43" s="58"/>
+      <c r="J43" s="58"/>
+      <c r="K43" s="58"/>
+      <c r="L43" s="58"/>
+      <c r="M43" s="58"/>
+      <c r="N43" s="59"/>
     </row>
     <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10980,22 +10980,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="58" t="s">
+      <c r="A55" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="56"/>
-      <c r="C55" s="56"/>
-      <c r="D55" s="56"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="56"/>
-      <c r="G55" s="56"/>
-      <c r="H55" s="56"/>
-      <c r="I55" s="56"/>
-      <c r="J55" s="56"/>
-      <c r="K55" s="56"/>
-      <c r="L55" s="56"/>
-      <c r="M55" s="56"/>
-      <c r="N55" s="57"/>
+      <c r="B55" s="58"/>
+      <c r="C55" s="58"/>
+      <c r="D55" s="58"/>
+      <c r="E55" s="58"/>
+      <c r="F55" s="58"/>
+      <c r="G55" s="58"/>
+      <c r="H55" s="58"/>
+      <c r="I55" s="58"/>
+      <c r="J55" s="58"/>
+      <c r="K55" s="58"/>
+      <c r="L55" s="58"/>
+      <c r="M55" s="58"/>
+      <c r="N55" s="59"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11287,22 +11287,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="58" t="s">
+      <c r="A64" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="56"/>
-      <c r="C64" s="56"/>
-      <c r="D64" s="56"/>
-      <c r="E64" s="56"/>
-      <c r="F64" s="56"/>
-      <c r="G64" s="56"/>
-      <c r="H64" s="56"/>
-      <c r="I64" s="56"/>
-      <c r="J64" s="56"/>
-      <c r="K64" s="56"/>
-      <c r="L64" s="56"/>
-      <c r="M64" s="56"/>
-      <c r="N64" s="57"/>
+      <c r="B64" s="58"/>
+      <c r="C64" s="58"/>
+      <c r="D64" s="58"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="58"/>
+      <c r="G64" s="58"/>
+      <c r="H64" s="58"/>
+      <c r="I64" s="58"/>
+      <c r="J64" s="58"/>
+      <c r="K64" s="58"/>
+      <c r="L64" s="58"/>
+      <c r="M64" s="58"/>
+      <c r="N64" s="59"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11725,39 +11725,39 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="60" t="s">
+      <c r="A77" s="74" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="61"/>
-      <c r="C77" s="61"/>
-      <c r="D77" s="61"/>
-      <c r="E77" s="61"/>
-      <c r="F77" s="61"/>
-      <c r="G77" s="61"/>
-      <c r="H77" s="61"/>
-      <c r="I77" s="61"/>
-      <c r="J77" s="61"/>
-      <c r="K77" s="61"/>
+      <c r="B77" s="56"/>
+      <c r="C77" s="56"/>
+      <c r="D77" s="56"/>
+      <c r="E77" s="56"/>
+      <c r="F77" s="56"/>
+      <c r="G77" s="56"/>
+      <c r="H77" s="56"/>
+      <c r="I77" s="56"/>
+      <c r="J77" s="56"/>
+      <c r="K77" s="56"/>
     </row>
     <row r="78" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="55" t="s">
+      <c r="C79" s="73" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="56"/>
-      <c r="E79" s="57"/>
-      <c r="F79" s="59" t="s">
+      <c r="D79" s="58"/>
+      <c r="E79" s="59"/>
+      <c r="F79" s="71" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="56"/>
-      <c r="H79" s="57"/>
-      <c r="I79" s="62" t="s">
+      <c r="G79" s="58"/>
+      <c r="H79" s="59"/>
+      <c r="I79" s="70" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="56"/>
-      <c r="K79" s="57"/>
+      <c r="J79" s="58"/>
+      <c r="K79" s="59"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11795,19 +11795,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="58" t="s">
+      <c r="A81" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="56"/>
-      <c r="C81" s="56"/>
-      <c r="D81" s="56"/>
-      <c r="E81" s="56"/>
-      <c r="F81" s="56"/>
-      <c r="G81" s="56"/>
-      <c r="H81" s="56"/>
-      <c r="I81" s="56"/>
-      <c r="J81" s="56"/>
-      <c r="K81" s="57"/>
+      <c r="B81" s="58"/>
+      <c r="C81" s="58"/>
+      <c r="D81" s="58"/>
+      <c r="E81" s="58"/>
+      <c r="F81" s="58"/>
+      <c r="G81" s="58"/>
+      <c r="H81" s="58"/>
+      <c r="I81" s="58"/>
+      <c r="J81" s="58"/>
+      <c r="K81" s="59"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12258,19 +12258,19 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="58" t="s">
+      <c r="A93" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="56"/>
-      <c r="C93" s="56"/>
-      <c r="D93" s="56"/>
-      <c r="E93" s="56"/>
-      <c r="F93" s="56"/>
-      <c r="G93" s="56"/>
-      <c r="H93" s="56"/>
-      <c r="I93" s="56"/>
-      <c r="J93" s="56"/>
-      <c r="K93" s="57"/>
+      <c r="B93" s="58"/>
+      <c r="C93" s="58"/>
+      <c r="D93" s="58"/>
+      <c r="E93" s="58"/>
+      <c r="F93" s="58"/>
+      <c r="G93" s="58"/>
+      <c r="H93" s="58"/>
+      <c r="I93" s="58"/>
+      <c r="J93" s="58"/>
+      <c r="K93" s="59"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12586,19 +12586,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="58" t="s">
+      <c r="A102" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="56"/>
-      <c r="C102" s="56"/>
-      <c r="D102" s="56"/>
-      <c r="E102" s="56"/>
-      <c r="F102" s="56"/>
-      <c r="G102" s="56"/>
-      <c r="H102" s="56"/>
-      <c r="I102" s="56"/>
-      <c r="J102" s="56"/>
-      <c r="K102" s="57"/>
+      <c r="B102" s="58"/>
+      <c r="C102" s="58"/>
+      <c r="D102" s="58"/>
+      <c r="E102" s="58"/>
+      <c r="F102" s="58"/>
+      <c r="G102" s="58"/>
+      <c r="H102" s="58"/>
+      <c r="I102" s="58"/>
+      <c r="J102" s="58"/>
+      <c r="K102" s="59"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13046,6 +13046,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13062,12 +13068,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13461,59 +13461,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="61"/>
-      <c r="T1" s="61"/>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="60" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="57" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="57"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16707,59 +16707,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="68" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="61"/>
-      <c r="T1" s="61"/>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="60" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="57" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="57"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19599,59 +19599,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="55" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="61"/>
-      <c r="T1" s="61"/>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="60" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="57" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="57"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21637,59 +21637,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="55" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="61"/>
-      <c r="T1" s="61"/>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="60" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="57" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="57"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24421,29 +24421,29 @@
       <c r="A1" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="61"/>
-      <c r="T1" s="61"/>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
-      <c r="W1" s="61"/>
-      <c r="X1" s="61"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
+      <c r="W1" s="56"/>
+      <c r="X1" s="56"/>
     </row>
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -24451,36 +24451,36 @@
       <c r="B3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
       <c r="G3" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="61"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="56"/>
       <c r="L3" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="61"/>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
+      <c r="M3" s="56"/>
+      <c r="N3" s="56"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="56"/>
       <c r="Q3" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
       <c r="V3" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="61"/>
-      <c r="X3" s="61"/>
+      <c r="W3" s="56"/>
+      <c r="X3" s="56"/>
     </row>
     <row r="4" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
@@ -25022,15 +25022,21 @@
       <c r="A11" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="48"/>
-      <c r="C11" s="48"/>
+      <c r="B11" s="48">
+        <v>7.4</v>
+      </c>
+      <c r="C11" s="48">
+        <v>15</v>
+      </c>
       <c r="D11" s="48">
         <v>5</v>
       </c>
-      <c r="E11" s="48"/>
-      <c r="F11" s="48" t="str">
+      <c r="E11" s="48">
+        <v>5</v>
+      </c>
+      <c r="F11" s="48">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="G11" s="48"/>
       <c r="H11" s="48"/>
@@ -25068,11 +25074,11 @@
       </c>
       <c r="W11" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X11" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25600,11 +25606,11 @@
       </c>
       <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.1125</v>
       </c>
       <c r="G21" s="50"/>
       <c r="H21" s="50"/>
@@ -25654,11 +25660,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.10312499999999999</v>
+        <v>0.11874999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25674,11 +25680,11 @@
       </c>
       <c r="E23" s="53">
         <f>E21</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F23" s="53">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23/D23,"")</f>
-        <v>0.05</v>
+        <v>0.1125</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -25728,11 +25734,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.10312499999999999</v>
+        <v>0.11874999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-05 17:26:04
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2657B98-1432-4C0E-9878-1CE0250085DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14D6165-6442-45A0-BC31-4A6F03DFE6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1447,16 +1447,28 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1480,25 +1492,13 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7512,7 +7512,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="66" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="56"/>
@@ -7539,7 +7539,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="61" t="s">
+      <c r="A4" s="65" t="s">
         <v>52</v>
       </c>
       <c r="B4" s="58"/>
@@ -8050,7 +8050,7 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="61" t="s">
+      <c r="A41" s="65" t="s">
         <v>88</v>
       </c>
       <c r="B41" s="58"/>
@@ -8537,7 +8537,7 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="61" t="s">
+      <c r="A83" s="65" t="s">
         <v>106</v>
       </c>
       <c r="B83" s="58"/>
@@ -8761,7 +8761,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="67" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="56"/>
@@ -8782,22 +8782,22 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="64" t="s">
+      <c r="C3" s="68" t="s">
         <v>115</v>
       </c>
       <c r="D3" s="58"/>
       <c r="E3" s="59"/>
-      <c r="F3" s="67" t="s">
+      <c r="F3" s="71" t="s">
         <v>305</v>
       </c>
       <c r="G3" s="58"/>
       <c r="H3" s="59"/>
-      <c r="I3" s="66" t="s">
+      <c r="I3" s="70" t="s">
         <v>116</v>
       </c>
       <c r="J3" s="58"/>
       <c r="K3" s="59"/>
-      <c r="L3" s="65" t="s">
+      <c r="L3" s="69" t="s">
         <v>47</v>
       </c>
       <c r="M3" s="58"/>
@@ -9445,7 +9445,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="55" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="56"/>
@@ -9463,17 +9463,17 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="73" t="s">
+      <c r="C3" s="63" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="58"/>
       <c r="E3" s="59"/>
-      <c r="F3" s="71" t="s">
+      <c r="F3" s="61" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="58"/>
       <c r="H3" s="59"/>
-      <c r="I3" s="70" t="s">
+      <c r="I3" s="60" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="58"/>
@@ -9515,7 +9515,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="57" t="s">
         <v>53</v>
       </c>
       <c r="B5" s="58"/>
@@ -9869,7 +9869,7 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="69" t="s">
+      <c r="A17" s="57" t="s">
         <v>73</v>
       </c>
       <c r="B17" s="58"/>
@@ -10107,7 +10107,7 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="69" t="s">
+      <c r="A26" s="57" t="s">
         <v>80</v>
       </c>
       <c r="B26" s="58"/>
@@ -10446,7 +10446,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="74" t="s">
+      <c r="A39" s="64" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="56"/>
@@ -10467,22 +10467,22 @@
     <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="73" t="s">
+      <c r="C41" s="63" t="s">
         <v>52</v>
       </c>
       <c r="D41" s="58"/>
       <c r="E41" s="59"/>
-      <c r="F41" s="71" t="s">
+      <c r="F41" s="61" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="58"/>
       <c r="H41" s="59"/>
-      <c r="I41" s="72" t="s">
+      <c r="I41" s="62" t="s">
         <v>156</v>
       </c>
       <c r="J41" s="58"/>
       <c r="K41" s="59"/>
-      <c r="L41" s="70" t="s">
+      <c r="L41" s="60" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="58"/>
@@ -10533,7 +10533,7 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="69" t="s">
+      <c r="A43" s="57" t="s">
         <v>53</v>
       </c>
       <c r="B43" s="58"/>
@@ -10659,11 +10659,15 @@
         <f t="shared" si="13"/>
         <v>704</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4" t="str">
+      <c r="C46" s="4">
+        <v>17</v>
+      </c>
+      <c r="D46" s="4">
+        <v>13</v>
+      </c>
+      <c r="E46" s="4">
         <f t="shared" si="14"/>
-        <v/>
+        <v>0.76470588235294112</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -10679,15 +10683,15 @@
       </c>
       <c r="L46" s="4">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="M46" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="N46" s="4" t="e">
+        <v>13</v>
+      </c>
+      <c r="N46" s="4">
         <f t="shared" si="19"/>
-        <v>#DIV/0!</v>
+        <v>0.76470588235294112</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -10931,15 +10935,15 @@
       <c r="B53" s="6"/>
       <c r="C53" s="7">
         <f>SUM(C44:C52)</f>
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="D53" s="7">
         <f>SUM(D44:D52)</f>
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E53" s="7">
         <f t="shared" si="14"/>
-        <v>0.70833333333333337</v>
+        <v>0.73170731707317072</v>
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
@@ -10967,20 +10971,20 @@
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.61403508771929827</v>
+        <v>0.64864864864864868</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="69" t="s">
+      <c r="A55" s="57" t="s">
         <v>73</v>
       </c>
       <c r="B55" s="58"/>
@@ -11287,7 +11291,7 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="69" t="s">
+      <c r="A64" s="57" t="s">
         <v>80</v>
       </c>
       <c r="B64" s="58"/>
@@ -11677,15 +11681,15 @@
       <c r="B74" s="9"/>
       <c r="C74" s="10">
         <f>C53+C62+C73</f>
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="D74" s="10">
         <f>D53+D62+D73</f>
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E74" s="10">
         <f t="shared" si="27"/>
-        <v>0.70833333333333337</v>
+        <v>0.73170731707317072</v>
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
@@ -11713,19 +11717,19 @@
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.61403508771929827</v>
+        <v>0.64864864864864868</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="74" t="s">
+      <c r="A77" s="64" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="56"/>
@@ -11743,17 +11747,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="73" t="s">
+      <c r="C79" s="63" t="s">
         <v>158</v>
       </c>
       <c r="D79" s="58"/>
       <c r="E79" s="59"/>
-      <c r="F79" s="71" t="s">
+      <c r="F79" s="61" t="s">
         <v>155</v>
       </c>
       <c r="G79" s="58"/>
       <c r="H79" s="59"/>
-      <c r="I79" s="70" t="s">
+      <c r="I79" s="60" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="58"/>
@@ -11795,7 +11799,7 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="69" t="s">
+      <c r="A81" s="57" t="s">
         <v>53</v>
       </c>
       <c r="B81" s="58"/>
@@ -11921,27 +11925,27 @@
       </c>
       <c r="F84" s="4">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G84" s="4">
         <f t="shared" si="37"/>
-        <v>0</v>
-      </c>
-      <c r="H84" s="4" t="e">
+        <v>13</v>
+      </c>
+      <c r="H84" s="4">
         <f t="shared" si="38"/>
-        <v>#DIV/0!</v>
+        <v>0.76470588235294112</v>
       </c>
       <c r="I84" s="4">
         <f t="shared" si="39"/>
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="J84" s="4">
         <f t="shared" si="40"/>
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="K84" s="4">
         <f t="shared" si="41"/>
-        <v>0.875</v>
+        <v>0.83673469387755106</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12233,32 +12237,32 @@
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.61403508771929827</v>
+        <v>0.64864864864864868</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.80512820512820515</v>
+        <v>0.80188679245283023</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="69" t="s">
+      <c r="A93" s="57" t="s">
         <v>73</v>
       </c>
       <c r="B93" s="58"/>
@@ -12586,7 +12590,7 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="69" t="s">
+      <c r="A102" s="57" t="s">
         <v>80</v>
       </c>
       <c r="B102" s="58"/>
@@ -13021,27 +13025,27 @@
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.61403508771929827</v>
+        <v>0.64864864864864868</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.80512820512820515</v>
+        <v>0.80188679245283023</v>
       </c>
     </row>
   </sheetData>
@@ -13461,7 +13465,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="72" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="56"/>
@@ -13488,7 +13492,7 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
       <c r="B3" s="58"/>
@@ -13502,7 +13506,7 @@
       <c r="J3" s="58"/>
       <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="57" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
       <c r="N3" s="58"/>
@@ -16707,7 +16711,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="55" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="56"/>
@@ -16734,7 +16738,7 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
       <c r="B3" s="58"/>
@@ -16748,7 +16752,7 @@
       <c r="J3" s="58"/>
       <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="57" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
       <c r="N3" s="58"/>
@@ -19599,7 +19603,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="72" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="56"/>
@@ -19626,7 +19630,7 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
       <c r="B3" s="58"/>
@@ -19640,7 +19644,7 @@
       <c r="J3" s="58"/>
       <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="57" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
       <c r="N3" s="58"/>
@@ -21637,7 +21641,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="72" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="56"/>
@@ -21664,7 +21668,7 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
       <c r="B3" s="58"/>
@@ -21678,7 +21682,7 @@
       <c r="J3" s="58"/>
       <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="57" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
       <c r="N3" s="58"/>
@@ -23632,30 +23636,40 @@
       <c r="A37" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15" t="str">
+      <c r="B37" s="15">
+        <v>705</v>
+      </c>
+      <c r="C37" s="15">
+        <v>12</v>
+      </c>
+      <c r="D37" s="15">
+        <v>12</v>
+      </c>
+      <c r="E37" s="15">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="F37" s="15"/>
-      <c r="G37" s="15"/>
-      <c r="H37" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F37" s="15">
+        <v>5</v>
+      </c>
+      <c r="G37" s="15">
+        <v>5</v>
+      </c>
+      <c r="H37" s="15">
         <f t="shared" si="21"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I37" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J37" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="K37" s="15" t="e">
+        <v>7</v>
+      </c>
+      <c r="K37" s="15">
         <f t="shared" si="23"/>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="L37" s="11"/>
       <c r="M37" s="15"/>
@@ -23688,30 +23702,40 @@
       <c r="A38" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15" t="str">
+      <c r="B38" s="15">
+        <v>705</v>
+      </c>
+      <c r="C38" s="15">
+        <v>19</v>
+      </c>
+      <c r="D38" s="15">
+        <v>15</v>
+      </c>
+      <c r="E38" s="15">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="15" t="str">
+        <v>0.78947368421052633</v>
+      </c>
+      <c r="F38" s="15">
+        <v>4</v>
+      </c>
+      <c r="G38" s="15">
+        <v>4</v>
+      </c>
+      <c r="H38" s="15">
         <f t="shared" si="21"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I38" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J38" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="K38" s="15" t="e">
+        <v>11</v>
+      </c>
+      <c r="K38" s="15">
         <f t="shared" si="23"/>
-        <v>#DIV/0!</v>
+        <v>0.73333333333333328</v>
       </c>
       <c r="L38" s="11"/>
       <c r="M38" s="15"/>
@@ -23747,39 +23771,39 @@
       <c r="B39" s="17"/>
       <c r="C39" s="18">
         <f>SUM(C5:C38)</f>
-        <v>530</v>
+        <v>561</v>
       </c>
       <c r="D39" s="18">
         <f>SUM(D5:D38)</f>
-        <v>430</v>
+        <v>457</v>
       </c>
       <c r="E39" s="18">
         <f t="shared" si="20"/>
-        <v>0.81132075471698117</v>
+        <v>0.81461675579322634</v>
       </c>
       <c r="F39" s="18">
         <f>SUM(F5:F38)</f>
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="G39" s="18">
         <f>SUM(G5:G38)</f>
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="H39" s="18">
         <f t="shared" si="21"/>
-        <v>0.8110236220472441</v>
+        <v>0.82352941176470584</v>
       </c>
       <c r="I39" s="18">
         <f>SUM(I5:I38)</f>
-        <v>403</v>
+        <v>425</v>
       </c>
       <c r="J39" s="18">
         <f>SUM(J5:J38)</f>
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="K39" s="18">
         <f t="shared" si="23"/>
-        <v>0.81141439205955335</v>
+        <v>0.81176470588235294</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -23828,39 +23852,39 @@
       <c r="B41" s="20"/>
       <c r="C41" s="21">
         <f>C39+N39</f>
-        <v>530</v>
+        <v>561</v>
       </c>
       <c r="D41" s="21">
         <f>D39+O39</f>
-        <v>430</v>
+        <v>457</v>
       </c>
       <c r="E41" s="21">
         <f>IF(AND(C41&lt;&gt;"",D41&lt;&gt;""),D41/C41,"")</f>
-        <v>0.81132075471698117</v>
+        <v>0.81461675579322634</v>
       </c>
       <c r="F41" s="21">
         <f>F39+Q39</f>
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="G41" s="21">
         <f>G39+R39</f>
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="H41" s="21">
         <f>IF(AND(F41&lt;&gt;"",G41&lt;&gt;""),G41/F41,"")</f>
-        <v>0.8110236220472441</v>
+        <v>0.82352941176470584</v>
       </c>
       <c r="I41" s="21">
         <f>I39+T39</f>
-        <v>403</v>
+        <v>425</v>
       </c>
       <c r="J41" s="21">
         <f>J39+U39</f>
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="K41" s="21">
         <f>IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),J41/I41,"")</f>
-        <v>0.81141439205955335</v>
+        <v>0.81176470588235294</v>
       </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-08 09:19:41
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14D6165-6442-45A0-BC31-4A6F03DFE6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97F11A4-1FC6-404E-B578-C9775419ECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="307">
   <si>
     <t>英语真题阅读 正确率记录</t>
   </si>
@@ -958,6 +958,10 @@
   </si>
   <si>
     <t>填空题</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>综合篇中三个物理应用题目未做</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1447,33 +1451,21 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1492,6 +1484,27 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1499,15 +1512,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7512,7 +7516,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="62" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="56"/>
@@ -7539,13 +7543,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="59" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="59"/>
+      <c r="B4" s="60"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="61"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8050,13 +8054,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="65" t="s">
+      <c r="A41" s="59" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="58"/>
-      <c r="C41" s="58"/>
-      <c r="D41" s="58"/>
-      <c r="E41" s="59"/>
+      <c r="B41" s="60"/>
+      <c r="C41" s="60"/>
+      <c r="D41" s="60"/>
+      <c r="E41" s="61"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8537,13 +8541,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="65" t="s">
+      <c r="A83" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="58"/>
-      <c r="C83" s="58"/>
-      <c r="D83" s="58"/>
-      <c r="E83" s="59"/>
+      <c r="B83" s="60"/>
+      <c r="C83" s="60"/>
+      <c r="D83" s="60"/>
+      <c r="E83" s="61"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8761,7 +8765,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="63" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="56"/>
@@ -8782,26 +8786,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="68" t="s">
+      <c r="C3" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="71" t="s">
+      <c r="D3" s="60"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="67" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="58"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="70" t="s">
+      <c r="G3" s="60"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="69" t="s">
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="58"/>
-      <c r="N3" s="59"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="61"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9436,7 +9440,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:N112"/>
+  <dimension ref="A1:O112"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -9445,7 +9449,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="73" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="56"/>
@@ -9463,21 +9467,21 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="63" t="s">
+      <c r="C3" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="61" t="s">
+      <c r="D3" s="60"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="70" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="58"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="60" t="s">
+      <c r="G3" s="60"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9515,19 +9519,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="59"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="61"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9626,23 +9630,27 @@
         <f t="shared" si="0"/>
         <v>0.875</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4" t="str">
+      <c r="F8" s="4">
+        <v>33</v>
+      </c>
+      <c r="G8" s="4">
+        <v>27</v>
+      </c>
+      <c r="H8" s="4">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.81818181818181823</v>
       </c>
       <c r="I8" s="4">
         <f t="shared" si="2"/>
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="J8" s="4">
         <f t="shared" si="3"/>
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="K8" s="4">
         <f t="shared" si="4"/>
-        <v>0.875</v>
+        <v>0.84615384615384615</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9844,44 +9852,44 @@
       </c>
       <c r="F15" s="7">
         <f>SUM(F6:F14)</f>
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="G15" s="7">
         <f>SUM(G6:G14)</f>
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="H15" s="7">
         <f t="shared" si="1"/>
-        <v>0.89473684210526316</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="I15" s="7">
         <f>SUM(I6:I14)</f>
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="J15" s="7">
         <f>SUM(J6:J14)</f>
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="4"/>
-        <v>0.88405797101449279</v>
+        <v>0.87134502923976609</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="58"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="58"/>
-      <c r="F17" s="58"/>
-      <c r="G17" s="58"/>
-      <c r="H17" s="58"/>
-      <c r="I17" s="58"/>
-      <c r="J17" s="58"/>
-      <c r="K17" s="59"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="60"/>
+      <c r="J17" s="60"/>
+      <c r="K17" s="61"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10107,19 +10115,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="58"/>
-      <c r="C26" s="58"/>
-      <c r="D26" s="58"/>
-      <c r="E26" s="58"/>
-      <c r="F26" s="58"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="58"/>
-      <c r="J26" s="58"/>
-      <c r="K26" s="59"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="60"/>
+      <c r="G26" s="60"/>
+      <c r="H26" s="60"/>
+      <c r="I26" s="60"/>
+      <c r="J26" s="60"/>
+      <c r="K26" s="61"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10301,7 +10309,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>151</v>
       </c>
@@ -10331,7 +10339,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>152</v>
       </c>
@@ -10361,7 +10369,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>153</v>
       </c>
@@ -10403,7 +10411,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>154</v>
       </c>
@@ -10422,31 +10430,31 @@
       </c>
       <c r="F36" s="10">
         <f>F15+F24+F35</f>
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="G36" s="10">
         <f>G15+G24+G35</f>
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="H36" s="10">
         <f t="shared" si="10"/>
-        <v>0.89473684210526316</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="I36" s="10">
         <f>I15+I24+I35</f>
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="J36" s="10">
         <f>J15+J24+J35</f>
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>0.88405797101449279</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="64" t="s">
+        <v>0.87134502923976609</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="71" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="56"/>
@@ -10463,32 +10471,32 @@
       <c r="M39" s="56"/>
       <c r="N39" s="56"/>
     </row>
-    <row r="40" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="63" t="s">
+      <c r="C41" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="58"/>
-      <c r="E41" s="59"/>
-      <c r="F41" s="61" t="s">
+      <c r="D41" s="60"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="70" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="58"/>
-      <c r="H41" s="59"/>
-      <c r="I41" s="62" t="s">
+      <c r="G41" s="60"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="74" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="58"/>
-      <c r="K41" s="59"/>
-      <c r="L41" s="60" t="s">
+      <c r="J41" s="60"/>
+      <c r="K41" s="61"/>
+      <c r="L41" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="58"/>
-      <c r="N41" s="59"/>
-    </row>
-    <row r="42" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M41" s="60"/>
+      <c r="N41" s="61"/>
+    </row>
+    <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>50</v>
       </c>
@@ -10532,25 +10540,25 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="57" t="s">
+    <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="58"/>
-      <c r="C43" s="58"/>
-      <c r="D43" s="58"/>
-      <c r="E43" s="58"/>
-      <c r="F43" s="58"/>
-      <c r="G43" s="58"/>
-      <c r="H43" s="58"/>
-      <c r="I43" s="58"/>
-      <c r="J43" s="58"/>
-      <c r="K43" s="58"/>
-      <c r="L43" s="58"/>
-      <c r="M43" s="58"/>
-      <c r="N43" s="59"/>
-    </row>
-    <row r="44" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="60"/>
+      <c r="C43" s="60"/>
+      <c r="D43" s="60"/>
+      <c r="E43" s="60"/>
+      <c r="F43" s="60"/>
+      <c r="G43" s="60"/>
+      <c r="H43" s="60"/>
+      <c r="I43" s="60"/>
+      <c r="J43" s="60"/>
+      <c r="K43" s="60"/>
+      <c r="L43" s="60"/>
+      <c r="M43" s="60"/>
+      <c r="N43" s="61"/>
+    </row>
+    <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>128</v>
       </c>
@@ -10601,7 +10609,7 @@
         <v>0.57894736842105265</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>129</v>
       </c>
@@ -10651,7 +10659,7 @@
         <v>0.63157894736842102</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>130</v>
       </c>
@@ -10669,11 +10677,15 @@
         <f t="shared" si="14"/>
         <v>0.76470588235294112</v>
       </c>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4" t="str">
+      <c r="F46" s="4">
+        <v>41</v>
+      </c>
+      <c r="G46" s="4">
+        <v>27</v>
+      </c>
+      <c r="H46" s="4">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.65853658536585369</v>
       </c>
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
@@ -10683,18 +10695,21 @@
       </c>
       <c r="L46" s="4">
         <f t="shared" si="17"/>
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="M46" s="4">
         <f t="shared" si="18"/>
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="N46" s="4">
         <f t="shared" si="19"/>
-        <v>0.76470588235294112</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0.68965517241379315</v>
+      </c>
+      <c r="O46" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>131</v>
       </c>
@@ -10733,7 +10748,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>132</v>
       </c>
@@ -10947,15 +10962,15 @@
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="G53" s="7">
         <f>SUM(G44:G52)</f>
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="H53" s="7">
         <f t="shared" si="15"/>
-        <v>0.6071428571428571</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="I53" s="7">
         <f>SUM(I44:I52)</f>
@@ -10971,35 +10986,35 @@
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.64864864864864868</v>
+        <v>0.65217391304347827</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="57" t="s">
+      <c r="A55" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="58"/>
-      <c r="C55" s="58"/>
-      <c r="D55" s="58"/>
-      <c r="E55" s="58"/>
-      <c r="F55" s="58"/>
-      <c r="G55" s="58"/>
-      <c r="H55" s="58"/>
-      <c r="I55" s="58"/>
-      <c r="J55" s="58"/>
-      <c r="K55" s="58"/>
-      <c r="L55" s="58"/>
-      <c r="M55" s="58"/>
-      <c r="N55" s="59"/>
+      <c r="B55" s="60"/>
+      <c r="C55" s="60"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="60"/>
+      <c r="G55" s="60"/>
+      <c r="H55" s="60"/>
+      <c r="I55" s="60"/>
+      <c r="J55" s="60"/>
+      <c r="K55" s="60"/>
+      <c r="L55" s="60"/>
+      <c r="M55" s="60"/>
+      <c r="N55" s="61"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11291,22 +11306,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="57" t="s">
+      <c r="A64" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="58"/>
-      <c r="C64" s="58"/>
-      <c r="D64" s="58"/>
-      <c r="E64" s="58"/>
-      <c r="F64" s="58"/>
-      <c r="G64" s="58"/>
-      <c r="H64" s="58"/>
-      <c r="I64" s="58"/>
-      <c r="J64" s="58"/>
-      <c r="K64" s="58"/>
-      <c r="L64" s="58"/>
-      <c r="M64" s="58"/>
-      <c r="N64" s="59"/>
+      <c r="B64" s="60"/>
+      <c r="C64" s="60"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="60"/>
+      <c r="F64" s="60"/>
+      <c r="G64" s="60"/>
+      <c r="H64" s="60"/>
+      <c r="I64" s="60"/>
+      <c r="J64" s="60"/>
+      <c r="K64" s="60"/>
+      <c r="L64" s="60"/>
+      <c r="M64" s="60"/>
+      <c r="N64" s="61"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11693,15 +11708,15 @@
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="G74" s="10">
         <f>G53+G62+G73</f>
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="H74" s="10">
         <f t="shared" si="28"/>
-        <v>0.6071428571428571</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="I74" s="10">
         <f>I53+I62+I73</f>
@@ -11717,19 +11732,19 @@
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.64864864864864868</v>
+        <v>0.65217391304347827</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="64" t="s">
+      <c r="A77" s="71" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="56"/>
@@ -11747,21 +11762,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="63" t="s">
+      <c r="C79" s="68" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="58"/>
-      <c r="E79" s="59"/>
-      <c r="F79" s="61" t="s">
+      <c r="D79" s="60"/>
+      <c r="E79" s="61"/>
+      <c r="F79" s="70" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="58"/>
-      <c r="H79" s="59"/>
-      <c r="I79" s="60" t="s">
+      <c r="G79" s="60"/>
+      <c r="H79" s="61"/>
+      <c r="I79" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="58"/>
-      <c r="K79" s="59"/>
+      <c r="J79" s="60"/>
+      <c r="K79" s="61"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11799,19 +11814,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="57" t="s">
+      <c r="A81" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="58"/>
-      <c r="C81" s="58"/>
-      <c r="D81" s="58"/>
-      <c r="E81" s="58"/>
-      <c r="F81" s="58"/>
-      <c r="G81" s="58"/>
-      <c r="H81" s="58"/>
-      <c r="I81" s="58"/>
-      <c r="J81" s="58"/>
-      <c r="K81" s="59"/>
+      <c r="B81" s="60"/>
+      <c r="C81" s="60"/>
+      <c r="D81" s="60"/>
+      <c r="E81" s="60"/>
+      <c r="F81" s="60"/>
+      <c r="G81" s="60"/>
+      <c r="H81" s="60"/>
+      <c r="I81" s="60"/>
+      <c r="J81" s="60"/>
+      <c r="K81" s="61"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -11913,39 +11928,39 @@
       </c>
       <c r="C84" s="4">
         <f t="shared" si="33"/>
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="D84" s="4">
         <f t="shared" si="34"/>
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="E84" s="4">
         <f t="shared" si="35"/>
-        <v>0.875</v>
+        <v>0.84615384615384615</v>
       </c>
       <c r="F84" s="4">
         <f t="shared" si="36"/>
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G84" s="4">
         <f t="shared" si="37"/>
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H84" s="4">
         <f t="shared" si="38"/>
-        <v>0.76470588235294112</v>
+        <v>0.68965517241379315</v>
       </c>
       <c r="I84" s="4">
         <f t="shared" si="39"/>
-        <v>49</v>
+        <v>123</v>
       </c>
       <c r="J84" s="4">
         <f t="shared" si="40"/>
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="K84" s="4">
         <f t="shared" si="41"/>
-        <v>0.83673469387755106</v>
+        <v>0.77235772357723576</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12225,56 +12240,56 @@
       <c r="B91" s="6"/>
       <c r="C91" s="7">
         <f>SUM(C82:C90)</f>
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D91" s="7">
         <f>SUM(D82:D90)</f>
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="E91" s="7">
         <f t="shared" si="35"/>
-        <v>0.88405797101449279</v>
+        <v>0.87134502923976609</v>
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.64864864864864868</v>
+        <v>0.65217391304347827</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>212</v>
+        <v>286</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>170</v>
+        <v>224</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.80188679245283023</v>
+        <v>0.78321678321678323</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="57" t="s">
+      <c r="A93" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="58"/>
-      <c r="C93" s="58"/>
-      <c r="D93" s="58"/>
-      <c r="E93" s="58"/>
-      <c r="F93" s="58"/>
-      <c r="G93" s="58"/>
-      <c r="H93" s="58"/>
-      <c r="I93" s="58"/>
-      <c r="J93" s="58"/>
-      <c r="K93" s="59"/>
+      <c r="B93" s="60"/>
+      <c r="C93" s="60"/>
+      <c r="D93" s="60"/>
+      <c r="E93" s="60"/>
+      <c r="F93" s="60"/>
+      <c r="G93" s="60"/>
+      <c r="H93" s="60"/>
+      <c r="I93" s="60"/>
+      <c r="J93" s="60"/>
+      <c r="K93" s="61"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12590,19 +12605,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="57" t="s">
+      <c r="A102" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="58"/>
-      <c r="C102" s="58"/>
-      <c r="D102" s="58"/>
-      <c r="E102" s="58"/>
-      <c r="F102" s="58"/>
-      <c r="G102" s="58"/>
-      <c r="H102" s="58"/>
-      <c r="I102" s="58"/>
-      <c r="J102" s="58"/>
-      <c r="K102" s="59"/>
+      <c r="B102" s="60"/>
+      <c r="C102" s="60"/>
+      <c r="D102" s="60"/>
+      <c r="E102" s="60"/>
+      <c r="F102" s="60"/>
+      <c r="G102" s="60"/>
+      <c r="H102" s="60"/>
+      <c r="I102" s="60"/>
+      <c r="J102" s="60"/>
+      <c r="K102" s="61"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13013,49 +13028,43 @@
       <c r="B112" s="9"/>
       <c r="C112" s="10">
         <f>C91+C100+C111</f>
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D112" s="10">
         <f>D91+D100+D111</f>
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="E112" s="10">
         <f t="shared" si="51"/>
-        <v>0.88405797101449279</v>
+        <v>0.87134502923976609</v>
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.64864864864864868</v>
+        <v>0.65217391304347827</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>212</v>
+        <v>286</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>170</v>
+        <v>224</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.80188679245283023</v>
+        <v>0.78321678321678323</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13072,6 +13081,12 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13465,7 +13480,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="75" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="56"/>
@@ -13492,32 +13507,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16711,7 +16726,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="73" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="56"/>
@@ -16738,32 +16753,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19603,7 +19618,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="75" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="56"/>
@@ -19630,32 +19645,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21641,7 +21656,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="75" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="56"/>
@@ -21668,32 +21683,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24442,7 +24457,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="56"/>
@@ -24472,35 +24487,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="77" t="s">
+      <c r="B3" s="58" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="56"/>
       <c r="D3" s="56"/>
       <c r="E3" s="56"/>
       <c r="F3" s="56"/>
-      <c r="G3" s="77" t="s">
+      <c r="G3" s="58" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="56"/>
       <c r="I3" s="56"/>
       <c r="J3" s="56"/>
       <c r="K3" s="56"/>
-      <c r="L3" s="77" t="s">
+      <c r="L3" s="58" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="56"/>
       <c r="N3" s="56"/>
       <c r="O3" s="56"/>
       <c r="P3" s="56"/>
-      <c r="Q3" s="77" t="s">
+      <c r="Q3" s="58" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="56"/>
       <c r="S3" s="56"/>
       <c r="T3" s="56"/>
       <c r="U3" s="56"/>
-      <c r="V3" s="76" t="s">
+      <c r="V3" s="57" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="56"/>
@@ -25062,15 +25077,21 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G11" s="48"/>
-      <c r="H11" s="48"/>
+      <c r="G11" s="48">
+        <v>7.7</v>
+      </c>
+      <c r="H11" s="48">
+        <v>19</v>
+      </c>
       <c r="I11" s="48">
         <v>5</v>
       </c>
-      <c r="J11" s="48"/>
-      <c r="K11" s="48" t="str">
+      <c r="J11" s="48">
+        <v>4</v>
+      </c>
+      <c r="K11" s="48">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="L11" s="48"/>
       <c r="M11" s="48"/>
@@ -25098,11 +25119,11 @@
       </c>
       <c r="W11" s="48">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="X11" s="48">
         <f t="shared" si="6"/>
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25644,11 +25665,11 @@
       </c>
       <c r="J21" s="46">
         <f>SUM(J5:J20)</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K21" s="46">
         <f t="shared" si="1"/>
-        <v>0.1125</v>
+        <v>0.16250000000000001</v>
       </c>
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
@@ -25684,11 +25705,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.11874999999999999</v>
+        <v>0.13125000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25718,11 +25739,11 @@
       </c>
       <c r="J23" s="53">
         <f>J21</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K23" s="53">
         <f>IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),J23/I23,"")</f>
-        <v>0.1125</v>
+        <v>0.16250000000000001</v>
       </c>
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
@@ -25758,11 +25779,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.11874999999999999</v>
+        <v>0.13125000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-09 21:08:09
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97F11A4-1FC6-404E-B578-C9775419ECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751AF446-F18F-4D91-A4E6-F94A7C379454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1451,21 +1451,33 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1484,27 +1496,6 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1512,6 +1503,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7516,7 +7516,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="66" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="56"/>
@@ -7543,13 +7543,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="60"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="61"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="59"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8054,13 +8054,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="59" t="s">
+      <c r="A41" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="60"/>
-      <c r="C41" s="60"/>
-      <c r="D41" s="60"/>
-      <c r="E41" s="61"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="59"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8541,13 +8541,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="59" t="s">
+      <c r="A83" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="60"/>
-      <c r="C83" s="60"/>
-      <c r="D83" s="60"/>
-      <c r="E83" s="61"/>
+      <c r="B83" s="58"/>
+      <c r="C83" s="58"/>
+      <c r="D83" s="58"/>
+      <c r="E83" s="59"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8765,7 +8765,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="67" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="56"/>
@@ -8786,26 +8786,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="64" t="s">
+      <c r="C3" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="67" t="s">
+      <c r="D3" s="58"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="71" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="60"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="66" t="s">
+      <c r="G3" s="58"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="70" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="65" t="s">
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="60"/>
-      <c r="N3" s="61"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="59"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9449,7 +9449,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="55" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="56"/>
@@ -9467,21 +9467,21 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="68" t="s">
+      <c r="C3" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="70" t="s">
+      <c r="D3" s="58"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="60"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="72" t="s">
+      <c r="G3" s="58"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9519,19 +9519,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="60"/>
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
-      <c r="I5" s="60"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="61"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
+      <c r="J5" s="58"/>
+      <c r="K5" s="59"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9877,19 +9877,19 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="69" t="s">
+      <c r="A17" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="60"/>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="61"/>
+      <c r="B17" s="58"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="58"/>
+      <c r="K17" s="59"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10115,19 +10115,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="69" t="s">
+      <c r="A26" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="60"/>
-      <c r="H26" s="60"/>
-      <c r="I26" s="60"/>
-      <c r="J26" s="60"/>
-      <c r="K26" s="61"/>
+      <c r="B26" s="58"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="59"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10454,7 +10454,7 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="71" t="s">
+      <c r="A39" s="64" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="56"/>
@@ -10475,26 +10475,26 @@
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="68" t="s">
+      <c r="C41" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="60"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="70" t="s">
+      <c r="D41" s="58"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="60"/>
-      <c r="H41" s="61"/>
-      <c r="I41" s="74" t="s">
+      <c r="G41" s="58"/>
+      <c r="H41" s="59"/>
+      <c r="I41" s="62" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="60"/>
-      <c r="K41" s="61"/>
-      <c r="L41" s="72" t="s">
+      <c r="J41" s="58"/>
+      <c r="K41" s="59"/>
+      <c r="L41" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="60"/>
-      <c r="N41" s="61"/>
+      <c r="M41" s="58"/>
+      <c r="N41" s="59"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10541,22 +10541,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="69" t="s">
+      <c r="A43" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="60"/>
-      <c r="C43" s="60"/>
-      <c r="D43" s="60"/>
-      <c r="E43" s="60"/>
-      <c r="F43" s="60"/>
-      <c r="G43" s="60"/>
-      <c r="H43" s="60"/>
-      <c r="I43" s="60"/>
-      <c r="J43" s="60"/>
-      <c r="K43" s="60"/>
-      <c r="L43" s="60"/>
-      <c r="M43" s="60"/>
-      <c r="N43" s="61"/>
+      <c r="B43" s="58"/>
+      <c r="C43" s="58"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="58"/>
+      <c r="F43" s="58"/>
+      <c r="G43" s="58"/>
+      <c r="H43" s="58"/>
+      <c r="I43" s="58"/>
+      <c r="J43" s="58"/>
+      <c r="K43" s="58"/>
+      <c r="L43" s="58"/>
+      <c r="M43" s="58"/>
+      <c r="N43" s="59"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10999,22 +10999,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="69" t="s">
+      <c r="A55" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="60"/>
-      <c r="C55" s="60"/>
-      <c r="D55" s="60"/>
-      <c r="E55" s="60"/>
-      <c r="F55" s="60"/>
-      <c r="G55" s="60"/>
-      <c r="H55" s="60"/>
-      <c r="I55" s="60"/>
-      <c r="J55" s="60"/>
-      <c r="K55" s="60"/>
-      <c r="L55" s="60"/>
-      <c r="M55" s="60"/>
-      <c r="N55" s="61"/>
+      <c r="B55" s="58"/>
+      <c r="C55" s="58"/>
+      <c r="D55" s="58"/>
+      <c r="E55" s="58"/>
+      <c r="F55" s="58"/>
+      <c r="G55" s="58"/>
+      <c r="H55" s="58"/>
+      <c r="I55" s="58"/>
+      <c r="J55" s="58"/>
+      <c r="K55" s="58"/>
+      <c r="L55" s="58"/>
+      <c r="M55" s="58"/>
+      <c r="N55" s="59"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11306,22 +11306,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="69" t="s">
+      <c r="A64" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="60"/>
-      <c r="C64" s="60"/>
-      <c r="D64" s="60"/>
-      <c r="E64" s="60"/>
-      <c r="F64" s="60"/>
-      <c r="G64" s="60"/>
-      <c r="H64" s="60"/>
-      <c r="I64" s="60"/>
-      <c r="J64" s="60"/>
-      <c r="K64" s="60"/>
-      <c r="L64" s="60"/>
-      <c r="M64" s="60"/>
-      <c r="N64" s="61"/>
+      <c r="B64" s="58"/>
+      <c r="C64" s="58"/>
+      <c r="D64" s="58"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="58"/>
+      <c r="G64" s="58"/>
+      <c r="H64" s="58"/>
+      <c r="I64" s="58"/>
+      <c r="J64" s="58"/>
+      <c r="K64" s="58"/>
+      <c r="L64" s="58"/>
+      <c r="M64" s="58"/>
+      <c r="N64" s="59"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11744,7 +11744,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="71" t="s">
+      <c r="A77" s="64" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="56"/>
@@ -11762,21 +11762,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="68" t="s">
+      <c r="C79" s="63" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="60"/>
-      <c r="E79" s="61"/>
-      <c r="F79" s="70" t="s">
+      <c r="D79" s="58"/>
+      <c r="E79" s="59"/>
+      <c r="F79" s="61" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="60"/>
-      <c r="H79" s="61"/>
-      <c r="I79" s="72" t="s">
+      <c r="G79" s="58"/>
+      <c r="H79" s="59"/>
+      <c r="I79" s="60" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="60"/>
-      <c r="K79" s="61"/>
+      <c r="J79" s="58"/>
+      <c r="K79" s="59"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11814,19 +11814,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="69" t="s">
+      <c r="A81" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="60"/>
-      <c r="C81" s="60"/>
-      <c r="D81" s="60"/>
-      <c r="E81" s="60"/>
-      <c r="F81" s="60"/>
-      <c r="G81" s="60"/>
-      <c r="H81" s="60"/>
-      <c r="I81" s="60"/>
-      <c r="J81" s="60"/>
-      <c r="K81" s="61"/>
+      <c r="B81" s="58"/>
+      <c r="C81" s="58"/>
+      <c r="D81" s="58"/>
+      <c r="E81" s="58"/>
+      <c r="F81" s="58"/>
+      <c r="G81" s="58"/>
+      <c r="H81" s="58"/>
+      <c r="I81" s="58"/>
+      <c r="J81" s="58"/>
+      <c r="K81" s="59"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12277,19 +12277,19 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="69" t="s">
+      <c r="A93" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="60"/>
-      <c r="C93" s="60"/>
-      <c r="D93" s="60"/>
-      <c r="E93" s="60"/>
-      <c r="F93" s="60"/>
-      <c r="G93" s="60"/>
-      <c r="H93" s="60"/>
-      <c r="I93" s="60"/>
-      <c r="J93" s="60"/>
-      <c r="K93" s="61"/>
+      <c r="B93" s="58"/>
+      <c r="C93" s="58"/>
+      <c r="D93" s="58"/>
+      <c r="E93" s="58"/>
+      <c r="F93" s="58"/>
+      <c r="G93" s="58"/>
+      <c r="H93" s="58"/>
+      <c r="I93" s="58"/>
+      <c r="J93" s="58"/>
+      <c r="K93" s="59"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12605,19 +12605,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="69" t="s">
+      <c r="A102" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="60"/>
-      <c r="C102" s="60"/>
-      <c r="D102" s="60"/>
-      <c r="E102" s="60"/>
-      <c r="F102" s="60"/>
-      <c r="G102" s="60"/>
-      <c r="H102" s="60"/>
-      <c r="I102" s="60"/>
-      <c r="J102" s="60"/>
-      <c r="K102" s="61"/>
+      <c r="B102" s="58"/>
+      <c r="C102" s="58"/>
+      <c r="D102" s="58"/>
+      <c r="E102" s="58"/>
+      <c r="F102" s="58"/>
+      <c r="G102" s="58"/>
+      <c r="H102" s="58"/>
+      <c r="I102" s="58"/>
+      <c r="J102" s="58"/>
+      <c r="K102" s="59"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13065,6 +13065,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13081,12 +13087,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13480,7 +13480,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="72" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="56"/>
@@ -13507,32 +13507,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16726,7 +16726,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="55" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="56"/>
@@ -16753,32 +16753,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19618,7 +19618,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="72" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="56"/>
@@ -19645,32 +19645,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21656,7 +21656,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="72" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="56"/>
@@ -21683,32 +21683,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="74" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="59"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24457,7 +24457,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="75" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="56"/>
@@ -24487,35 +24487,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="77" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="56"/>
       <c r="D3" s="56"/>
       <c r="E3" s="56"/>
       <c r="F3" s="56"/>
-      <c r="G3" s="58" t="s">
+      <c r="G3" s="77" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="56"/>
       <c r="I3" s="56"/>
       <c r="J3" s="56"/>
       <c r="K3" s="56"/>
-      <c r="L3" s="58" t="s">
+      <c r="L3" s="77" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="56"/>
       <c r="N3" s="56"/>
       <c r="O3" s="56"/>
       <c r="P3" s="56"/>
-      <c r="Q3" s="58" t="s">
+      <c r="Q3" s="77" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="56"/>
       <c r="S3" s="56"/>
       <c r="T3" s="56"/>
       <c r="U3" s="56"/>
-      <c r="V3" s="57" t="s">
+      <c r="V3" s="76" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="56"/>
@@ -25093,15 +25093,21 @@
         <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="48"/>
+      <c r="L11" s="48">
+        <v>7.8</v>
+      </c>
+      <c r="M11" s="48">
+        <v>12</v>
+      </c>
       <c r="N11" s="48">
         <v>5</v>
       </c>
-      <c r="O11" s="48"/>
-      <c r="P11" s="48" t="str">
+      <c r="O11" s="48">
+        <v>4</v>
+      </c>
+      <c r="P11" s="48">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="Q11" s="48"/>
       <c r="R11" s="48"/>
@@ -25119,11 +25125,11 @@
       </c>
       <c r="W11" s="48">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="X11" s="48">
         <f t="shared" si="6"/>
-        <v>0.45</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25679,11 +25685,11 @@
       </c>
       <c r="O21" s="46">
         <f>SUM(O5:O20)</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="P21" s="46">
         <f t="shared" si="2"/>
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="Q21" s="50"/>
       <c r="R21" s="50"/>
@@ -25705,11 +25711,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.13125000000000001</v>
+        <v>0.14374999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25753,11 +25759,11 @@
       </c>
       <c r="O23" s="53">
         <f>O21</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="P23" s="53">
         <f>IF(AND(N23&lt;&gt;"",O23&lt;&gt;""),O23/N23,"")</f>
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="Q23" s="52"/>
       <c r="R23" s="52"/>
@@ -25779,11 +25785,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.13125000000000001</v>
+        <v>0.14374999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-12 17:05:29
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751AF446-F18F-4D91-A4E6-F94A7C379454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29530367-20BA-495C-9E65-0C9C4DC4BC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -1451,33 +1451,21 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1496,6 +1484,27 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1503,15 +1512,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7516,7 +7516,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="62" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="56"/>
@@ -7543,13 +7543,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="59" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="59"/>
+      <c r="B4" s="60"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="61"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8054,13 +8054,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="65" t="s">
+      <c r="A41" s="59" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="58"/>
-      <c r="C41" s="58"/>
-      <c r="D41" s="58"/>
-      <c r="E41" s="59"/>
+      <c r="B41" s="60"/>
+      <c r="C41" s="60"/>
+      <c r="D41" s="60"/>
+      <c r="E41" s="61"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8541,13 +8541,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="65" t="s">
+      <c r="A83" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="58"/>
-      <c r="C83" s="58"/>
-      <c r="D83" s="58"/>
-      <c r="E83" s="59"/>
+      <c r="B83" s="60"/>
+      <c r="C83" s="60"/>
+      <c r="D83" s="60"/>
+      <c r="E83" s="61"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8765,7 +8765,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="63" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="56"/>
@@ -8786,26 +8786,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="68" t="s">
+      <c r="C3" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="71" t="s">
+      <c r="D3" s="60"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="67" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="58"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="70" t="s">
+      <c r="G3" s="60"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="69" t="s">
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="58"/>
-      <c r="N3" s="59"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="61"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9005,36 +9005,50 @@
       <c r="A8" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34" t="str">
+      <c r="B8" s="34">
+        <v>711</v>
+      </c>
+      <c r="C8" s="34">
+        <v>7</v>
+      </c>
+      <c r="D8" s="34">
+        <v>7</v>
+      </c>
+      <c r="E8" s="34">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34" t="str">
+        <v>1</v>
+      </c>
+      <c r="F8" s="34">
+        <v>8</v>
+      </c>
+      <c r="G8" s="34">
+        <v>8</v>
+      </c>
+      <c r="H8" s="34">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I8" s="34"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34" t="str">
+        <v>1</v>
+      </c>
+      <c r="I8" s="34">
+        <v>19</v>
+      </c>
+      <c r="J8" s="34">
+        <v>13</v>
+      </c>
+      <c r="K8" s="34">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.68421052631578949</v>
       </c>
       <c r="L8" s="34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="M8" s="34">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="34" t="e">
+        <v>28</v>
+      </c>
+      <c r="N8" s="34">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.82352941176470584</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9224,51 +9238,51 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>0.8125</v>
+        <v>0.83636363636363631</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>0.83720930232558144</v>
+        <v>0.86274509803921573</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="J14" s="37">
         <f>SUM(J5:J13)</f>
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="K14" s="37">
         <f t="shared" si="2"/>
-        <v>0.66216216216216217</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.75151515151515147</v>
+        <v>0.76381909547738691</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9279,51 +9293,51 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>0.8125</v>
+        <v>0.83636363636363631</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>0.83720930232558144</v>
+        <v>0.86274509803921573</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="J16" s="40">
         <f>J14</f>
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="K16" s="40">
         <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),J16/I16,"")</f>
-        <v>0.66216216216216217</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.75151515151515147</v>
+        <v>0.76381909547738691</v>
       </c>
     </row>
   </sheetData>
@@ -9449,7 +9463,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="68" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="56"/>
@@ -9467,21 +9481,21 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="63" t="s">
+      <c r="C3" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="61" t="s">
+      <c r="D3" s="60"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="58"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="60" t="s">
+      <c r="G3" s="60"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9519,19 +9533,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="59"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="61"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9877,19 +9891,19 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="58"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="58"/>
-      <c r="F17" s="58"/>
-      <c r="G17" s="58"/>
-      <c r="H17" s="58"/>
-      <c r="I17" s="58"/>
-      <c r="J17" s="58"/>
-      <c r="K17" s="59"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="60"/>
+      <c r="J17" s="60"/>
+      <c r="K17" s="61"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10115,19 +10129,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="58"/>
-      <c r="C26" s="58"/>
-      <c r="D26" s="58"/>
-      <c r="E26" s="58"/>
-      <c r="F26" s="58"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="58"/>
-      <c r="J26" s="58"/>
-      <c r="K26" s="59"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="60"/>
+      <c r="G26" s="60"/>
+      <c r="H26" s="60"/>
+      <c r="I26" s="60"/>
+      <c r="J26" s="60"/>
+      <c r="K26" s="61"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10454,7 +10468,7 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="64" t="s">
+      <c r="A39" s="74" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="56"/>
@@ -10475,26 +10489,26 @@
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="63" t="s">
+      <c r="C41" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="58"/>
-      <c r="E41" s="59"/>
-      <c r="F41" s="61" t="s">
+      <c r="D41" s="60"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="58"/>
-      <c r="H41" s="59"/>
-      <c r="I41" s="62" t="s">
+      <c r="G41" s="60"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="72" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="58"/>
-      <c r="K41" s="59"/>
-      <c r="L41" s="60" t="s">
+      <c r="J41" s="60"/>
+      <c r="K41" s="61"/>
+      <c r="L41" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="58"/>
-      <c r="N41" s="59"/>
+      <c r="M41" s="60"/>
+      <c r="N41" s="61"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10541,22 +10555,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="57" t="s">
+      <c r="A43" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="58"/>
-      <c r="C43" s="58"/>
-      <c r="D43" s="58"/>
-      <c r="E43" s="58"/>
-      <c r="F43" s="58"/>
-      <c r="G43" s="58"/>
-      <c r="H43" s="58"/>
-      <c r="I43" s="58"/>
-      <c r="J43" s="58"/>
-      <c r="K43" s="58"/>
-      <c r="L43" s="58"/>
-      <c r="M43" s="58"/>
-      <c r="N43" s="59"/>
+      <c r="B43" s="60"/>
+      <c r="C43" s="60"/>
+      <c r="D43" s="60"/>
+      <c r="E43" s="60"/>
+      <c r="F43" s="60"/>
+      <c r="G43" s="60"/>
+      <c r="H43" s="60"/>
+      <c r="I43" s="60"/>
+      <c r="J43" s="60"/>
+      <c r="K43" s="60"/>
+      <c r="L43" s="60"/>
+      <c r="M43" s="60"/>
+      <c r="N43" s="61"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10999,22 +11013,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="57" t="s">
+      <c r="A55" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="58"/>
-      <c r="C55" s="58"/>
-      <c r="D55" s="58"/>
-      <c r="E55" s="58"/>
-      <c r="F55" s="58"/>
-      <c r="G55" s="58"/>
-      <c r="H55" s="58"/>
-      <c r="I55" s="58"/>
-      <c r="J55" s="58"/>
-      <c r="K55" s="58"/>
-      <c r="L55" s="58"/>
-      <c r="M55" s="58"/>
-      <c r="N55" s="59"/>
+      <c r="B55" s="60"/>
+      <c r="C55" s="60"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="60"/>
+      <c r="G55" s="60"/>
+      <c r="H55" s="60"/>
+      <c r="I55" s="60"/>
+      <c r="J55" s="60"/>
+      <c r="K55" s="60"/>
+      <c r="L55" s="60"/>
+      <c r="M55" s="60"/>
+      <c r="N55" s="61"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11306,22 +11320,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="57" t="s">
+      <c r="A64" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="58"/>
-      <c r="C64" s="58"/>
-      <c r="D64" s="58"/>
-      <c r="E64" s="58"/>
-      <c r="F64" s="58"/>
-      <c r="G64" s="58"/>
-      <c r="H64" s="58"/>
-      <c r="I64" s="58"/>
-      <c r="J64" s="58"/>
-      <c r="K64" s="58"/>
-      <c r="L64" s="58"/>
-      <c r="M64" s="58"/>
-      <c r="N64" s="59"/>
+      <c r="B64" s="60"/>
+      <c r="C64" s="60"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="60"/>
+      <c r="F64" s="60"/>
+      <c r="G64" s="60"/>
+      <c r="H64" s="60"/>
+      <c r="I64" s="60"/>
+      <c r="J64" s="60"/>
+      <c r="K64" s="60"/>
+      <c r="L64" s="60"/>
+      <c r="M64" s="60"/>
+      <c r="N64" s="61"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11744,7 +11758,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="64" t="s">
+      <c r="A77" s="74" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="56"/>
@@ -11762,21 +11776,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="63" t="s">
+      <c r="C79" s="73" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="58"/>
-      <c r="E79" s="59"/>
-      <c r="F79" s="61" t="s">
+      <c r="D79" s="60"/>
+      <c r="E79" s="61"/>
+      <c r="F79" s="71" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="58"/>
-      <c r="H79" s="59"/>
-      <c r="I79" s="60" t="s">
+      <c r="G79" s="60"/>
+      <c r="H79" s="61"/>
+      <c r="I79" s="70" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="58"/>
-      <c r="K79" s="59"/>
+      <c r="J79" s="60"/>
+      <c r="K79" s="61"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11814,19 +11828,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="57" t="s">
+      <c r="A81" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="58"/>
-      <c r="C81" s="58"/>
-      <c r="D81" s="58"/>
-      <c r="E81" s="58"/>
-      <c r="F81" s="58"/>
-      <c r="G81" s="58"/>
-      <c r="H81" s="58"/>
-      <c r="I81" s="58"/>
-      <c r="J81" s="58"/>
-      <c r="K81" s="59"/>
+      <c r="B81" s="60"/>
+      <c r="C81" s="60"/>
+      <c r="D81" s="60"/>
+      <c r="E81" s="60"/>
+      <c r="F81" s="60"/>
+      <c r="G81" s="60"/>
+      <c r="H81" s="60"/>
+      <c r="I81" s="60"/>
+      <c r="J81" s="60"/>
+      <c r="K81" s="61"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12277,19 +12291,19 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="57" t="s">
+      <c r="A93" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="58"/>
-      <c r="C93" s="58"/>
-      <c r="D93" s="58"/>
-      <c r="E93" s="58"/>
-      <c r="F93" s="58"/>
-      <c r="G93" s="58"/>
-      <c r="H93" s="58"/>
-      <c r="I93" s="58"/>
-      <c r="J93" s="58"/>
-      <c r="K93" s="59"/>
+      <c r="B93" s="60"/>
+      <c r="C93" s="60"/>
+      <c r="D93" s="60"/>
+      <c r="E93" s="60"/>
+      <c r="F93" s="60"/>
+      <c r="G93" s="60"/>
+      <c r="H93" s="60"/>
+      <c r="I93" s="60"/>
+      <c r="J93" s="60"/>
+      <c r="K93" s="61"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12605,19 +12619,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="57" t="s">
+      <c r="A102" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="58"/>
-      <c r="C102" s="58"/>
-      <c r="D102" s="58"/>
-      <c r="E102" s="58"/>
-      <c r="F102" s="58"/>
-      <c r="G102" s="58"/>
-      <c r="H102" s="58"/>
-      <c r="I102" s="58"/>
-      <c r="J102" s="58"/>
-      <c r="K102" s="59"/>
+      <c r="B102" s="60"/>
+      <c r="C102" s="60"/>
+      <c r="D102" s="60"/>
+      <c r="E102" s="60"/>
+      <c r="F102" s="60"/>
+      <c r="G102" s="60"/>
+      <c r="H102" s="60"/>
+      <c r="I102" s="60"/>
+      <c r="J102" s="60"/>
+      <c r="K102" s="61"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13480,7 +13494,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="75" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="56"/>
@@ -13507,32 +13521,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16726,7 +16740,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="68" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="56"/>
@@ -16753,32 +16767,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19618,7 +19632,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="75" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="56"/>
@@ -19645,32 +19659,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21656,7 +21670,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="75" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="56"/>
@@ -21683,32 +21697,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="73" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
+      <c r="S3" s="60"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="60"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24457,7 +24471,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="56"/>
@@ -24487,35 +24501,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="77" t="s">
+      <c r="B3" s="58" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="56"/>
       <c r="D3" s="56"/>
       <c r="E3" s="56"/>
       <c r="F3" s="56"/>
-      <c r="G3" s="77" t="s">
+      <c r="G3" s="58" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="56"/>
       <c r="I3" s="56"/>
       <c r="J3" s="56"/>
       <c r="K3" s="56"/>
-      <c r="L3" s="77" t="s">
+      <c r="L3" s="58" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="56"/>
       <c r="N3" s="56"/>
       <c r="O3" s="56"/>
       <c r="P3" s="56"/>
-      <c r="Q3" s="77" t="s">
+      <c r="Q3" s="58" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="56"/>
       <c r="S3" s="56"/>
       <c r="T3" s="56"/>
       <c r="U3" s="56"/>
-      <c r="V3" s="76" t="s">
+      <c r="V3" s="57" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="56"/>
@@ -25109,15 +25123,21 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q11" s="48"/>
-      <c r="R11" s="48"/>
+      <c r="Q11" s="48">
+        <v>7.9</v>
+      </c>
+      <c r="R11" s="48">
+        <v>19</v>
+      </c>
       <c r="S11" s="48">
         <v>5</v>
       </c>
-      <c r="T11" s="48"/>
-      <c r="U11" s="48" t="str">
+      <c r="T11" s="48">
+        <v>3</v>
+      </c>
+      <c r="U11" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="V11" s="48">
         <f t="shared" si="4"/>
@@ -25125,11 +25145,11 @@
       </c>
       <c r="W11" s="48">
         <f t="shared" si="5"/>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="X11" s="48">
         <f t="shared" si="6"/>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25699,11 +25719,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.13750000000000001</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25711,11 +25731,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.14374999999999999</v>
+        <v>0.15312500000000001</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25773,11 +25793,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>0.1</v>
+        <v>0.13750000000000001</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -25785,11 +25805,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.14374999999999999</v>
+        <v>0.15312500000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-17 15:32:04
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29530367-20BA-495C-9E65-0C9C4DC4BC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BF2F9D-99C9-43EC-AC14-C5851D29F6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="307">
   <si>
     <t>英语真题阅读 正确率记录</t>
   </si>
@@ -1313,7 +1313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1449,6 +1449,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7516,13 +7519,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
     </row>
     <row r="2" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7543,13 +7546,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="60" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="60"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="61"/>
+      <c r="B4" s="61"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="62"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8054,13 +8057,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="59" t="s">
+      <c r="A41" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="60"/>
-      <c r="C41" s="60"/>
-      <c r="D41" s="60"/>
-      <c r="E41" s="61"/>
+      <c r="B41" s="61"/>
+      <c r="C41" s="61"/>
+      <c r="D41" s="61"/>
+      <c r="E41" s="62"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8541,13 +8544,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="59" t="s">
+      <c r="A83" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="60"/>
-      <c r="C83" s="60"/>
-      <c r="D83" s="60"/>
-      <c r="E83" s="61"/>
+      <c r="B83" s="61"/>
+      <c r="C83" s="61"/>
+      <c r="D83" s="61"/>
+      <c r="E83" s="62"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8765,47 +8768,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
     </row>
     <row r="2" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="64" t="s">
+      <c r="C3" s="65" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="67" t="s">
+      <c r="D3" s="61"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="68" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="60"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="66" t="s">
+      <c r="G3" s="61"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="67" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="65" t="s">
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="66" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="60"/>
-      <c r="N3" s="61"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="62"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9055,18 +9058,28 @@
       <c r="A9" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34" t="str">
+      <c r="B9" s="34">
+        <v>716</v>
+      </c>
+      <c r="C9" s="34">
+        <v>16</v>
+      </c>
+      <c r="D9" s="34">
+        <v>13</v>
+      </c>
+      <c r="E9" s="34">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34" t="str">
+        <v>0.8125</v>
+      </c>
+      <c r="F9" s="34">
+        <v>12</v>
+      </c>
+      <c r="G9" s="34">
+        <v>8</v>
+      </c>
+      <c r="H9" s="34">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I9" s="34"/>
       <c r="J9" s="34"/>
@@ -9076,15 +9089,15 @@
       </c>
       <c r="L9" s="34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="M9" s="34">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N9" s="34" t="e">
+        <v>21</v>
+      </c>
+      <c r="N9" s="34">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9238,27 +9251,27 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>0.83636363636363631</v>
+        <v>0.83098591549295775</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>0.86274509803921573</v>
+        <v>0.82539682539682535</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
@@ -9274,15 +9287,15 @@
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>199</v>
+        <v>227</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.76381909547738691</v>
+        <v>0.76211453744493396</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9293,27 +9306,27 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>0.83636363636363631</v>
+        <v>0.83098591549295775</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>0.86274509803921573</v>
+        <v>0.82539682539682535</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
@@ -9329,15 +9342,15 @@
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>199</v>
+        <v>227</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.76381909547738691</v>
+        <v>0.76211453744493396</v>
       </c>
     </row>
   </sheetData>
@@ -9463,39 +9476,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="69" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="73" t="s">
+      <c r="C3" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="71" t="s">
+      <c r="D3" s="61"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="72" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="60"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="70" t="s">
+      <c r="G3" s="61"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9533,19 +9546,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="60"/>
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
-      <c r="I5" s="60"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="61"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="61"/>
+      <c r="K5" s="62"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9891,19 +9904,19 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="69" t="s">
+      <c r="A17" s="70" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="60"/>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="61"/>
+      <c r="B17" s="61"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="62"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10129,19 +10142,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="69" t="s">
+      <c r="A26" s="70" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="60"/>
-      <c r="H26" s="60"/>
-      <c r="I26" s="60"/>
-      <c r="J26" s="60"/>
-      <c r="K26" s="61"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="61"/>
+      <c r="J26" s="61"/>
+      <c r="K26" s="62"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10468,47 +10481,47 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="74" t="s">
+      <c r="A39" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="56"/>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="56"/>
-      <c r="J39" s="56"/>
-      <c r="K39" s="56"/>
-      <c r="L39" s="56"/>
-      <c r="M39" s="56"/>
-      <c r="N39" s="56"/>
+      <c r="B39" s="57"/>
+      <c r="C39" s="57"/>
+      <c r="D39" s="57"/>
+      <c r="E39" s="57"/>
+      <c r="F39" s="57"/>
+      <c r="G39" s="57"/>
+      <c r="H39" s="57"/>
+      <c r="I39" s="57"/>
+      <c r="J39" s="57"/>
+      <c r="K39" s="57"/>
+      <c r="L39" s="57"/>
+      <c r="M39" s="57"/>
+      <c r="N39" s="57"/>
     </row>
     <row r="40" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="73" t="s">
+      <c r="C41" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="60"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="71" t="s">
+      <c r="D41" s="61"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="72" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="60"/>
-      <c r="H41" s="61"/>
-      <c r="I41" s="72" t="s">
+      <c r="G41" s="61"/>
+      <c r="H41" s="62"/>
+      <c r="I41" s="73" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="60"/>
-      <c r="K41" s="61"/>
-      <c r="L41" s="70" t="s">
+      <c r="J41" s="61"/>
+      <c r="K41" s="62"/>
+      <c r="L41" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="60"/>
-      <c r="N41" s="61"/>
+      <c r="M41" s="61"/>
+      <c r="N41" s="62"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10555,22 +10568,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="69" t="s">
+      <c r="A43" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="60"/>
-      <c r="C43" s="60"/>
-      <c r="D43" s="60"/>
-      <c r="E43" s="60"/>
-      <c r="F43" s="60"/>
-      <c r="G43" s="60"/>
-      <c r="H43" s="60"/>
-      <c r="I43" s="60"/>
-      <c r="J43" s="60"/>
-      <c r="K43" s="60"/>
-      <c r="L43" s="60"/>
-      <c r="M43" s="60"/>
-      <c r="N43" s="61"/>
+      <c r="B43" s="61"/>
+      <c r="C43" s="61"/>
+      <c r="D43" s="61"/>
+      <c r="E43" s="61"/>
+      <c r="F43" s="61"/>
+      <c r="G43" s="61"/>
+      <c r="H43" s="61"/>
+      <c r="I43" s="61"/>
+      <c r="J43" s="61"/>
+      <c r="K43" s="61"/>
+      <c r="L43" s="61"/>
+      <c r="M43" s="61"/>
+      <c r="N43" s="62"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -11013,22 +11026,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="69" t="s">
+      <c r="A55" s="70" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="60"/>
-      <c r="C55" s="60"/>
-      <c r="D55" s="60"/>
-      <c r="E55" s="60"/>
-      <c r="F55" s="60"/>
-      <c r="G55" s="60"/>
-      <c r="H55" s="60"/>
-      <c r="I55" s="60"/>
-      <c r="J55" s="60"/>
-      <c r="K55" s="60"/>
-      <c r="L55" s="60"/>
-      <c r="M55" s="60"/>
-      <c r="N55" s="61"/>
+      <c r="B55" s="61"/>
+      <c r="C55" s="61"/>
+      <c r="D55" s="61"/>
+      <c r="E55" s="61"/>
+      <c r="F55" s="61"/>
+      <c r="G55" s="61"/>
+      <c r="H55" s="61"/>
+      <c r="I55" s="61"/>
+      <c r="J55" s="61"/>
+      <c r="K55" s="61"/>
+      <c r="L55" s="61"/>
+      <c r="M55" s="61"/>
+      <c r="N55" s="62"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11320,22 +11333,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="69" t="s">
+      <c r="A64" s="70" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="60"/>
-      <c r="C64" s="60"/>
-      <c r="D64" s="60"/>
-      <c r="E64" s="60"/>
-      <c r="F64" s="60"/>
-      <c r="G64" s="60"/>
-      <c r="H64" s="60"/>
-      <c r="I64" s="60"/>
-      <c r="J64" s="60"/>
-      <c r="K64" s="60"/>
-      <c r="L64" s="60"/>
-      <c r="M64" s="60"/>
-      <c r="N64" s="61"/>
+      <c r="B64" s="61"/>
+      <c r="C64" s="61"/>
+      <c r="D64" s="61"/>
+      <c r="E64" s="61"/>
+      <c r="F64" s="61"/>
+      <c r="G64" s="61"/>
+      <c r="H64" s="61"/>
+      <c r="I64" s="61"/>
+      <c r="J64" s="61"/>
+      <c r="K64" s="61"/>
+      <c r="L64" s="61"/>
+      <c r="M64" s="61"/>
+      <c r="N64" s="62"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11758,39 +11771,39 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="74" t="s">
+      <c r="A77" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="56"/>
-      <c r="C77" s="56"/>
-      <c r="D77" s="56"/>
-      <c r="E77" s="56"/>
-      <c r="F77" s="56"/>
-      <c r="G77" s="56"/>
-      <c r="H77" s="56"/>
-      <c r="I77" s="56"/>
-      <c r="J77" s="56"/>
-      <c r="K77" s="56"/>
+      <c r="B77" s="57"/>
+      <c r="C77" s="57"/>
+      <c r="D77" s="57"/>
+      <c r="E77" s="57"/>
+      <c r="F77" s="57"/>
+      <c r="G77" s="57"/>
+      <c r="H77" s="57"/>
+      <c r="I77" s="57"/>
+      <c r="J77" s="57"/>
+      <c r="K77" s="57"/>
     </row>
     <row r="78" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="73" t="s">
+      <c r="C79" s="74" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="60"/>
-      <c r="E79" s="61"/>
-      <c r="F79" s="71" t="s">
+      <c r="D79" s="61"/>
+      <c r="E79" s="62"/>
+      <c r="F79" s="72" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="60"/>
-      <c r="H79" s="61"/>
-      <c r="I79" s="70" t="s">
+      <c r="G79" s="61"/>
+      <c r="H79" s="62"/>
+      <c r="I79" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="60"/>
-      <c r="K79" s="61"/>
+      <c r="J79" s="61"/>
+      <c r="K79" s="62"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11828,19 +11841,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="69" t="s">
+      <c r="A81" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="60"/>
-      <c r="C81" s="60"/>
-      <c r="D81" s="60"/>
-      <c r="E81" s="60"/>
-      <c r="F81" s="60"/>
-      <c r="G81" s="60"/>
-      <c r="H81" s="60"/>
-      <c r="I81" s="60"/>
-      <c r="J81" s="60"/>
-      <c r="K81" s="61"/>
+      <c r="B81" s="61"/>
+      <c r="C81" s="61"/>
+      <c r="D81" s="61"/>
+      <c r="E81" s="61"/>
+      <c r="F81" s="61"/>
+      <c r="G81" s="61"/>
+      <c r="H81" s="61"/>
+      <c r="I81" s="61"/>
+      <c r="J81" s="61"/>
+      <c r="K81" s="62"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12291,19 +12304,19 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="69" t="s">
+      <c r="A93" s="70" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="60"/>
-      <c r="C93" s="60"/>
-      <c r="D93" s="60"/>
-      <c r="E93" s="60"/>
-      <c r="F93" s="60"/>
-      <c r="G93" s="60"/>
-      <c r="H93" s="60"/>
-      <c r="I93" s="60"/>
-      <c r="J93" s="60"/>
-      <c r="K93" s="61"/>
+      <c r="B93" s="61"/>
+      <c r="C93" s="61"/>
+      <c r="D93" s="61"/>
+      <c r="E93" s="61"/>
+      <c r="F93" s="61"/>
+      <c r="G93" s="61"/>
+      <c r="H93" s="61"/>
+      <c r="I93" s="61"/>
+      <c r="J93" s="61"/>
+      <c r="K93" s="62"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12619,19 +12632,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="69" t="s">
+      <c r="A102" s="70" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="60"/>
-      <c r="C102" s="60"/>
-      <c r="D102" s="60"/>
-      <c r="E102" s="60"/>
-      <c r="F102" s="60"/>
-      <c r="G102" s="60"/>
-      <c r="H102" s="60"/>
-      <c r="I102" s="60"/>
-      <c r="J102" s="60"/>
-      <c r="K102" s="61"/>
+      <c r="B102" s="61"/>
+      <c r="C102" s="61"/>
+      <c r="D102" s="61"/>
+      <c r="E102" s="61"/>
+      <c r="F102" s="61"/>
+      <c r="G102" s="61"/>
+      <c r="H102" s="61"/>
+      <c r="I102" s="61"/>
+      <c r="J102" s="61"/>
+      <c r="K102" s="62"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13494,59 +13507,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="76" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
+      <c r="R1" s="57"/>
+      <c r="S1" s="57"/>
+      <c r="T1" s="57"/>
+      <c r="U1" s="57"/>
+      <c r="V1" s="57"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="78" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="77" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -15810,33 +15823,39 @@
       <c r="B43" s="15">
         <v>506</v>
       </c>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15" t="str">
+      <c r="C43" s="15">
+        <v>23</v>
+      </c>
+      <c r="D43" s="15">
+        <v>17</v>
+      </c>
+      <c r="E43" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15" t="str">
+        <v>0.73913043478260865</v>
+      </c>
+      <c r="F43" s="15">
+        <v>11</v>
+      </c>
+      <c r="G43" s="15">
+        <v>10</v>
+      </c>
+      <c r="H43" s="15">
         <f t="shared" si="11"/>
-        <v/>
+        <v>0.90909090909090906</v>
       </c>
       <c r="I43" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J43" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K43" s="15" t="e">
+        <v>7</v>
+      </c>
+      <c r="K43" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L43" s="44" t="s">
-        <v>209</v>
-      </c>
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="L43" s="44"/>
       <c r="M43" s="15"/>
       <c r="N43" s="15"/>
       <c r="O43" s="15"/>
@@ -15870,33 +15889,39 @@
       <c r="B44" s="15">
         <v>506</v>
       </c>
-      <c r="C44" s="15"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15" t="str">
+      <c r="C44" s="15">
+        <v>16</v>
+      </c>
+      <c r="D44" s="15">
+        <v>13</v>
+      </c>
+      <c r="E44" s="15">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15" t="str">
+        <v>0.8125</v>
+      </c>
+      <c r="F44" s="15">
+        <v>4</v>
+      </c>
+      <c r="G44" s="15">
+        <v>4</v>
+      </c>
+      <c r="H44" s="15">
         <f t="shared" si="11"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I44" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J44" s="15">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K44" s="15" t="e">
+        <v>9</v>
+      </c>
+      <c r="K44" s="15">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L44" s="44" t="s">
-        <v>209</v>
-      </c>
+        <v>0.75</v>
+      </c>
+      <c r="L44" s="44"/>
       <c r="M44" s="15"/>
       <c r="N44" s="15"/>
       <c r="O44" s="15"/>
@@ -15930,39 +15955,39 @@
       <c r="B45" s="17"/>
       <c r="C45" s="18">
         <f>SUM(C5:C44)</f>
-        <v>595</v>
+        <v>634</v>
       </c>
       <c r="D45" s="18">
         <f>SUM(D5:D44)</f>
-        <v>508</v>
+        <v>538</v>
       </c>
       <c r="E45" s="18">
         <f t="shared" si="10"/>
-        <v>0.85378151260504198</v>
+        <v>0.8485804416403786</v>
       </c>
       <c r="F45" s="18">
         <f>SUM(F5:F44)</f>
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="G45" s="18">
         <f>SUM(G5:G44)</f>
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="H45" s="18">
         <f t="shared" si="11"/>
-        <v>0.83040935672514615</v>
+        <v>0.83870967741935487</v>
       </c>
       <c r="I45" s="18">
         <f>SUM(I5:I44)</f>
-        <v>424</v>
+        <v>448</v>
       </c>
       <c r="J45" s="18">
         <f>SUM(J5:J44)</f>
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="K45" s="18">
         <f t="shared" si="13"/>
-        <v>0.8632075471698113</v>
+        <v>0.8526785714285714</v>
       </c>
       <c r="L45" s="17"/>
       <c r="M45" s="17"/>
@@ -16011,39 +16036,39 @@
       <c r="B47" s="20"/>
       <c r="C47" s="21">
         <f>C45+N45</f>
-        <v>595</v>
+        <v>634</v>
       </c>
       <c r="D47" s="21">
         <f>D45+O45</f>
-        <v>508</v>
+        <v>538</v>
       </c>
       <c r="E47" s="21">
         <f>IF(AND(C47&lt;&gt;"",D47&lt;&gt;""),D47/C47,"")</f>
-        <v>0.85378151260504198</v>
+        <v>0.8485804416403786</v>
       </c>
       <c r="F47" s="21">
         <f>F45+Q45</f>
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="G47" s="21">
         <f>G45+R45</f>
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="H47" s="21">
         <f>IF(AND(F47&lt;&gt;"",G47&lt;&gt;""),G47/F47,"")</f>
-        <v>0.83040935672514615</v>
+        <v>0.83870967741935487</v>
       </c>
       <c r="I47" s="21">
         <f>I45+T45</f>
-        <v>424</v>
+        <v>448</v>
       </c>
       <c r="J47" s="21">
         <f>J45+U45</f>
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="K47" s="21">
         <f>IF(AND(I47&lt;&gt;"",J47&lt;&gt;""),J47/I47,"")</f>
-        <v>0.8632075471698113</v>
+        <v>0.8526785714285714</v>
       </c>
       <c r="L47" s="20"/>
       <c r="M47" s="20"/>
@@ -16740,59 +16765,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="69" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
+      <c r="R1" s="57"/>
+      <c r="S1" s="57"/>
+      <c r="T1" s="57"/>
+      <c r="U1" s="57"/>
+      <c r="V1" s="57"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="78" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="77" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19632,59 +19657,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="76" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
+      <c r="R1" s="57"/>
+      <c r="S1" s="57"/>
+      <c r="T1" s="57"/>
+      <c r="U1" s="57"/>
+      <c r="V1" s="57"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="78" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="77" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21670,59 +21695,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="76" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
+      <c r="R1" s="57"/>
+      <c r="S1" s="57"/>
+      <c r="T1" s="57"/>
+      <c r="U1" s="57"/>
+      <c r="V1" s="57"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="78" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="61"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="77" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24471,69 +24496,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
-      <c r="W1" s="56"/>
-      <c r="X1" s="56"/>
+      <c r="A1" s="56" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
+      <c r="R1" s="57"/>
+      <c r="S1" s="57"/>
+      <c r="T1" s="57"/>
+      <c r="U1" s="57"/>
+      <c r="V1" s="57"/>
+      <c r="W1" s="57"/>
+      <c r="X1" s="57"/>
     </row>
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="58" t="s">
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="58" t="s">
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="58" t="s">
+      <c r="M3" s="57"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="57" t="s">
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="56"/>
-      <c r="X3" s="56"/>
+      <c r="W3" s="57"/>
+      <c r="X3" s="57"/>
     </row>
     <row r="4" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
@@ -24622,10 +24647,12 @@
       <c r="D5" s="48">
         <v>5</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48" t="str">
+      <c r="E5" s="48">
+        <v>2</v>
+      </c>
+      <c r="F5" s="48">
         <f t="shared" ref="F5:F21" si="0">IF(AND(D5&lt;&gt;"",E5&lt;&gt;""),E5/D5,"")</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="G5" s="48" t="s">
         <v>14</v>
@@ -24636,10 +24663,12 @@
       <c r="I5" s="48">
         <v>5</v>
       </c>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48" t="str">
+      <c r="J5" s="48">
+        <v>2</v>
+      </c>
+      <c r="K5" s="48">
         <f t="shared" ref="K5:K21" si="1">IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),J5/I5,"")</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="L5" s="48" t="s">
         <v>15</v>
@@ -24650,10 +24679,12 @@
       <c r="N5" s="48">
         <v>5</v>
       </c>
-      <c r="O5" s="48"/>
-      <c r="P5" s="48" t="str">
+      <c r="O5" s="48">
+        <v>3</v>
+      </c>
+      <c r="P5" s="48">
         <f t="shared" ref="P5:P21" si="2">IF(AND(N5&lt;&gt;"",O5&lt;&gt;""),O5/N5,"")</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="Q5" s="48" t="s">
         <v>16</v>
@@ -24664,10 +24695,12 @@
       <c r="S5" s="48">
         <v>5</v>
       </c>
-      <c r="T5" s="48"/>
-      <c r="U5" s="48" t="str">
+      <c r="T5" s="48">
+        <v>1</v>
+      </c>
+      <c r="U5" s="48">
         <f t="shared" ref="U5:U21" si="3">IF(AND(S5&lt;&gt;"",T5&lt;&gt;""),T5/S5,"")</f>
-        <v/>
+        <v>0.2</v>
       </c>
       <c r="V5" s="48">
         <f t="shared" ref="V5:V20" si="4">D5+I5+N5+S5</f>
@@ -24675,11 +24708,11 @@
       </c>
       <c r="W5" s="48">
         <f t="shared" ref="W5:W20" si="5">E5+J5+O5+T5</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="X5" s="48">
         <f t="shared" ref="X5:X21" si="6">IF(AND(V5&lt;&gt;"",W5&lt;&gt;""),W5/V5,"")</f>
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -24695,10 +24728,12 @@
       <c r="D6" s="48">
         <v>5</v>
       </c>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48" t="str">
+      <c r="E6" s="48">
+        <v>4</v>
+      </c>
+      <c r="F6" s="48">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="G6" s="48" t="s">
         <v>19</v>
@@ -24709,10 +24744,12 @@
       <c r="I6" s="48">
         <v>5</v>
       </c>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48" t="str">
+      <c r="J6" s="48">
+        <v>2</v>
+      </c>
+      <c r="K6" s="48">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="L6" s="48" t="s">
         <v>20</v>
@@ -24723,10 +24760,12 @@
       <c r="N6" s="48">
         <v>5</v>
       </c>
-      <c r="O6" s="48"/>
-      <c r="P6" s="48" t="str">
+      <c r="O6" s="48">
+        <v>4</v>
+      </c>
+      <c r="P6" s="48">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="Q6" s="48" t="s">
         <v>21</v>
@@ -24737,10 +24776,12 @@
       <c r="S6" s="48">
         <v>5</v>
       </c>
-      <c r="T6" s="48"/>
-      <c r="U6" s="48" t="str">
+      <c r="T6" s="48">
+        <v>3</v>
+      </c>
+      <c r="U6" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="V6" s="48">
         <f t="shared" si="4"/>
@@ -24748,11 +24789,11 @@
       </c>
       <c r="W6" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="X6" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -24768,10 +24809,12 @@
       <c r="D7" s="48">
         <v>5</v>
       </c>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48" t="str">
+      <c r="E7" s="48">
+        <v>2</v>
+      </c>
+      <c r="F7" s="48">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="G7" s="48" t="s">
         <v>24</v>
@@ -24782,10 +24825,12 @@
       <c r="I7" s="48">
         <v>5</v>
       </c>
-      <c r="J7" s="48"/>
-      <c r="K7" s="48" t="str">
+      <c r="J7" s="48">
+        <v>2</v>
+      </c>
+      <c r="K7" s="48">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="L7" s="48" t="s">
         <v>25</v>
@@ -24796,10 +24841,12 @@
       <c r="N7" s="48">
         <v>5</v>
       </c>
-      <c r="O7" s="48"/>
-      <c r="P7" s="48" t="str">
+      <c r="O7" s="48">
+        <v>5</v>
+      </c>
+      <c r="P7" s="48">
         <f t="shared" si="2"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q7" s="48" t="s">
         <v>26</v>
@@ -24810,10 +24857,12 @@
       <c r="S7" s="48">
         <v>5</v>
       </c>
-      <c r="T7" s="48"/>
-      <c r="U7" s="48" t="str">
+      <c r="T7" s="48">
+        <v>2</v>
+      </c>
+      <c r="U7" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="V7" s="48">
         <f t="shared" si="4"/>
@@ -24821,11 +24870,11 @@
       </c>
       <c r="W7" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="X7" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25156,35 +25205,53 @@
       <c r="A12" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="48"/>
-      <c r="C12" s="48"/>
+      <c r="B12" s="48">
+        <v>7.12</v>
+      </c>
+      <c r="C12" s="48">
+        <v>13</v>
+      </c>
       <c r="D12" s="48">
         <v>5</v>
       </c>
-      <c r="E12" s="48"/>
-      <c r="F12" s="48" t="str">
+      <c r="E12" s="48">
+        <v>4</v>
+      </c>
+      <c r="F12" s="48">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G12" s="48"/>
-      <c r="H12" s="48"/>
+        <v>0.8</v>
+      </c>
+      <c r="G12" s="48">
+        <v>7.13</v>
+      </c>
+      <c r="H12" s="48">
+        <v>10</v>
+      </c>
       <c r="I12" s="48">
         <v>5</v>
       </c>
-      <c r="J12" s="48"/>
-      <c r="K12" s="48" t="str">
+      <c r="J12" s="48">
+        <v>3</v>
+      </c>
+      <c r="K12" s="48">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="L12" s="48"/>
-      <c r="M12" s="48"/>
+        <v>0.6</v>
+      </c>
+      <c r="L12" s="48">
+        <v>7.16</v>
+      </c>
+      <c r="M12" s="48">
+        <v>16</v>
+      </c>
       <c r="N12" s="48">
         <v>5</v>
       </c>
-      <c r="O12" s="48"/>
-      <c r="P12" s="48" t="str">
+      <c r="O12" s="48">
+        <v>4</v>
+      </c>
+      <c r="P12" s="48">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="Q12" s="48"/>
       <c r="R12" s="48"/>
@@ -25202,11 +25269,11 @@
       </c>
       <c r="W12" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="X12" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25228,7 +25295,7 @@
       <c r="I13" s="48">
         <v>5</v>
       </c>
-      <c r="J13" s="48"/>
+      <c r="J13" s="55"/>
       <c r="K13" s="48" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -25677,11 +25744,11 @@
       </c>
       <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" si="0"/>
-        <v>0.1125</v>
+        <v>0.26250000000000001</v>
       </c>
       <c r="G21" s="50"/>
       <c r="H21" s="50"/>
@@ -25691,11 +25758,11 @@
       </c>
       <c r="J21" s="46">
         <f>SUM(J5:J20)</f>
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K21" s="46">
         <f t="shared" si="1"/>
-        <v>0.16250000000000001</v>
+        <v>0.27500000000000002</v>
       </c>
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
@@ -25705,11 +25772,11 @@
       </c>
       <c r="O21" s="46">
         <f>SUM(O5:O20)</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="P21" s="46">
         <f t="shared" si="2"/>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q21" s="50"/>
       <c r="R21" s="50"/>
@@ -25719,11 +25786,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>0.13750000000000001</v>
+        <v>0.21249999999999999</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25731,11 +25798,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.15312500000000001</v>
+        <v>0.28749999999999998</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25751,11 +25818,11 @@
       </c>
       <c r="E23" s="53">
         <f>E21</f>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F23" s="53">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23/D23,"")</f>
-        <v>0.1125</v>
+        <v>0.26250000000000001</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -25765,11 +25832,11 @@
       </c>
       <c r="J23" s="53">
         <f>J21</f>
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K23" s="53">
         <f>IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),J23/I23,"")</f>
-        <v>0.16250000000000001</v>
+        <v>0.27500000000000002</v>
       </c>
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
@@ -25779,11 +25846,11 @@
       </c>
       <c r="O23" s="53">
         <f>O21</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="P23" s="53">
         <f>IF(AND(N23&lt;&gt;"",O23&lt;&gt;""),O23/N23,"")</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q23" s="52"/>
       <c r="R23" s="52"/>
@@ -25793,11 +25860,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>0.13750000000000001</v>
+        <v>0.21249999999999999</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -25805,11 +25872,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.15312500000000001</v>
+        <v>0.28749999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-27 10:34:25
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BF2F9D-99C9-43EC-AC14-C5851D29F6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFEFA7A-C95F-4397-B5A4-280D648E65C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1454,30 +1454,15 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1485,6 +1470,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1515,6 +1506,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7519,7 +7519,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="65" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="57"/>
@@ -7546,13 +7546,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="61"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="62"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="60"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8057,13 +8057,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="60" t="s">
+      <c r="A41" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="61"/>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="62"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8544,13 +8544,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="60" t="s">
+      <c r="A83" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="61"/>
-      <c r="C83" s="61"/>
-      <c r="D83" s="61"/>
-      <c r="E83" s="62"/>
+      <c r="B83" s="59"/>
+      <c r="C83" s="59"/>
+      <c r="D83" s="59"/>
+      <c r="E83" s="60"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8768,7 +8768,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="56" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="57"/>
@@ -8789,26 +8789,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="58" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="61"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="68" t="s">
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="63" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="67" t="s">
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="66" t="s">
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="61" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="61"/>
-      <c r="N3" s="62"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="60"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9081,59 +9081,77 @@
         <f t="shared" si="1"/>
         <v>0.66666666666666663</v>
       </c>
-      <c r="I9" s="34"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34" t="str">
+      <c r="I9" s="34">
+        <v>22</v>
+      </c>
+      <c r="J9" s="34">
+        <v>17</v>
+      </c>
+      <c r="K9" s="34">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.77272727272727271</v>
       </c>
       <c r="L9" s="34">
         <f t="shared" si="3"/>
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="M9" s="34">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="N9" s="34">
         <f t="shared" si="5"/>
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34" t="str">
+      <c r="B10" s="34">
+        <v>718</v>
+      </c>
+      <c r="C10" s="34">
+        <v>12</v>
+      </c>
+      <c r="D10" s="34">
+        <v>12</v>
+      </c>
+      <c r="E10" s="34">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34" t="str">
+        <v>1</v>
+      </c>
+      <c r="F10" s="34">
+        <v>10</v>
+      </c>
+      <c r="G10" s="34">
+        <v>8</v>
+      </c>
+      <c r="H10" s="34">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34" t="str">
+        <v>0.8</v>
+      </c>
+      <c r="I10" s="34">
+        <v>18</v>
+      </c>
+      <c r="J10" s="34">
+        <v>13</v>
+      </c>
+      <c r="K10" s="34">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.72222222222222221</v>
       </c>
       <c r="L10" s="34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="M10" s="34">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N10" s="34" t="e">
+        <v>33</v>
+      </c>
+      <c r="N10" s="34">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.82499999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9251,51 +9269,51 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>0.83098591549295775</v>
+        <v>0.85542168674698793</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>0.82539682539682535</v>
+        <v>0.82191780821917804</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="J14" s="37">
         <f>SUM(J5:J13)</f>
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="K14" s="37">
         <f t="shared" si="2"/>
-        <v>0.66666666666666663</v>
+        <v>0.69172932330827064</v>
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>227</v>
+        <v>289</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>173</v>
+        <v>223</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.76211453744493396</v>
+        <v>0.77162629757785473</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9306,51 +9324,51 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>0.83098591549295775</v>
+        <v>0.85542168674698793</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>0.82539682539682535</v>
+        <v>0.82191780821917804</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="J16" s="40">
         <f>J14</f>
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="K16" s="40">
         <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),J16/I16,"")</f>
-        <v>0.66666666666666663</v>
+        <v>0.69172932330827064</v>
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>227</v>
+        <v>289</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>173</v>
+        <v>223</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.76211453744493396</v>
+        <v>0.77162629757785473</v>
       </c>
     </row>
   </sheetData>
@@ -9476,7 +9494,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="66" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="57"/>
@@ -9494,21 +9512,21 @@
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="74" t="s">
+      <c r="C3" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="61"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="72" t="s">
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="71" t="s">
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9546,19 +9564,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
-      <c r="H5" s="61"/>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
-      <c r="K5" s="62"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9904,19 +9922,19 @@
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="70" t="s">
+      <c r="A17" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="61"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="62"/>
+      <c r="B17" s="59"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="60"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10142,19 +10160,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="70" t="s">
+      <c r="A26" s="67" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="61"/>
-      <c r="C26" s="61"/>
-      <c r="D26" s="61"/>
-      <c r="E26" s="61"/>
-      <c r="F26" s="61"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="61"/>
-      <c r="I26" s="61"/>
-      <c r="J26" s="61"/>
-      <c r="K26" s="62"/>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="60"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10481,7 +10499,7 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="75" t="s">
+      <c r="A39" s="72" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="57"/>
@@ -10502,26 +10520,26 @@
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="74" t="s">
+      <c r="C41" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="61"/>
-      <c r="E41" s="62"/>
-      <c r="F41" s="72" t="s">
+      <c r="D41" s="59"/>
+      <c r="E41" s="60"/>
+      <c r="F41" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="61"/>
-      <c r="H41" s="62"/>
-      <c r="I41" s="73" t="s">
+      <c r="G41" s="59"/>
+      <c r="H41" s="60"/>
+      <c r="I41" s="70" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="61"/>
-      <c r="K41" s="62"/>
-      <c r="L41" s="71" t="s">
+      <c r="J41" s="59"/>
+      <c r="K41" s="60"/>
+      <c r="L41" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="61"/>
-      <c r="N41" s="62"/>
+      <c r="M41" s="59"/>
+      <c r="N41" s="60"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10568,22 +10586,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="70" t="s">
+      <c r="A43" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="61"/>
-      <c r="C43" s="61"/>
-      <c r="D43" s="61"/>
-      <c r="E43" s="61"/>
-      <c r="F43" s="61"/>
-      <c r="G43" s="61"/>
-      <c r="H43" s="61"/>
-      <c r="I43" s="61"/>
-      <c r="J43" s="61"/>
-      <c r="K43" s="61"/>
-      <c r="L43" s="61"/>
-      <c r="M43" s="61"/>
-      <c r="N43" s="62"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
+      <c r="H43" s="59"/>
+      <c r="I43" s="59"/>
+      <c r="J43" s="59"/>
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
+      <c r="M43" s="59"/>
+      <c r="N43" s="60"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -11026,22 +11044,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="70" t="s">
+      <c r="A55" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="61"/>
-      <c r="C55" s="61"/>
-      <c r="D55" s="61"/>
-      <c r="E55" s="61"/>
-      <c r="F55" s="61"/>
-      <c r="G55" s="61"/>
-      <c r="H55" s="61"/>
-      <c r="I55" s="61"/>
-      <c r="J55" s="61"/>
-      <c r="K55" s="61"/>
-      <c r="L55" s="61"/>
-      <c r="M55" s="61"/>
-      <c r="N55" s="62"/>
+      <c r="B55" s="59"/>
+      <c r="C55" s="59"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="59"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="59"/>
+      <c r="K55" s="59"/>
+      <c r="L55" s="59"/>
+      <c r="M55" s="59"/>
+      <c r="N55" s="60"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11333,22 +11351,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="70" t="s">
+      <c r="A64" s="67" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="61"/>
-      <c r="C64" s="61"/>
-      <c r="D64" s="61"/>
-      <c r="E64" s="61"/>
-      <c r="F64" s="61"/>
-      <c r="G64" s="61"/>
-      <c r="H64" s="61"/>
-      <c r="I64" s="61"/>
-      <c r="J64" s="61"/>
-      <c r="K64" s="61"/>
-      <c r="L64" s="61"/>
-      <c r="M64" s="61"/>
-      <c r="N64" s="62"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="59"/>
+      <c r="D64" s="59"/>
+      <c r="E64" s="59"/>
+      <c r="F64" s="59"/>
+      <c r="G64" s="59"/>
+      <c r="H64" s="59"/>
+      <c r="I64" s="59"/>
+      <c r="J64" s="59"/>
+      <c r="K64" s="59"/>
+      <c r="L64" s="59"/>
+      <c r="M64" s="59"/>
+      <c r="N64" s="60"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11771,7 +11789,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="75" t="s">
+      <c r="A77" s="72" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="57"/>
@@ -11789,21 +11807,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="74" t="s">
+      <c r="C79" s="71" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="61"/>
-      <c r="E79" s="62"/>
-      <c r="F79" s="72" t="s">
+      <c r="D79" s="59"/>
+      <c r="E79" s="60"/>
+      <c r="F79" s="69" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="61"/>
-      <c r="H79" s="62"/>
-      <c r="I79" s="71" t="s">
+      <c r="G79" s="59"/>
+      <c r="H79" s="60"/>
+      <c r="I79" s="68" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="61"/>
-      <c r="K79" s="62"/>
+      <c r="J79" s="59"/>
+      <c r="K79" s="60"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11841,19 +11859,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="70" t="s">
+      <c r="A81" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="61"/>
-      <c r="C81" s="61"/>
-      <c r="D81" s="61"/>
-      <c r="E81" s="61"/>
-      <c r="F81" s="61"/>
-      <c r="G81" s="61"/>
-      <c r="H81" s="61"/>
-      <c r="I81" s="61"/>
-      <c r="J81" s="61"/>
-      <c r="K81" s="62"/>
+      <c r="B81" s="59"/>
+      <c r="C81" s="59"/>
+      <c r="D81" s="59"/>
+      <c r="E81" s="59"/>
+      <c r="F81" s="59"/>
+      <c r="G81" s="59"/>
+      <c r="H81" s="59"/>
+      <c r="I81" s="59"/>
+      <c r="J81" s="59"/>
+      <c r="K81" s="60"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12304,19 +12322,19 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="70" t="s">
+      <c r="A93" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="61"/>
-      <c r="C93" s="61"/>
-      <c r="D93" s="61"/>
-      <c r="E93" s="61"/>
-      <c r="F93" s="61"/>
-      <c r="G93" s="61"/>
-      <c r="H93" s="61"/>
-      <c r="I93" s="61"/>
-      <c r="J93" s="61"/>
-      <c r="K93" s="62"/>
+      <c r="B93" s="59"/>
+      <c r="C93" s="59"/>
+      <c r="D93" s="59"/>
+      <c r="E93" s="59"/>
+      <c r="F93" s="59"/>
+      <c r="G93" s="59"/>
+      <c r="H93" s="59"/>
+      <c r="I93" s="59"/>
+      <c r="J93" s="59"/>
+      <c r="K93" s="60"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12632,19 +12650,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="70" t="s">
+      <c r="A102" s="67" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="61"/>
-      <c r="C102" s="61"/>
-      <c r="D102" s="61"/>
-      <c r="E102" s="61"/>
-      <c r="F102" s="61"/>
-      <c r="G102" s="61"/>
-      <c r="H102" s="61"/>
-      <c r="I102" s="61"/>
-      <c r="J102" s="61"/>
-      <c r="K102" s="62"/>
+      <c r="B102" s="59"/>
+      <c r="C102" s="59"/>
+      <c r="D102" s="59"/>
+      <c r="E102" s="59"/>
+      <c r="F102" s="59"/>
+      <c r="G102" s="59"/>
+      <c r="H102" s="59"/>
+      <c r="I102" s="59"/>
+      <c r="J102" s="59"/>
+      <c r="K102" s="60"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13507,7 +13525,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="73" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="57"/>
@@ -13534,32 +13552,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="77" t="s">
+      <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16765,7 +16783,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="66" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="57"/>
@@ -16792,32 +16810,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="77" t="s">
+      <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19657,7 +19675,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="73" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="57"/>
@@ -19684,32 +19702,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="77" t="s">
+      <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21695,7 +21713,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="73" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="57"/>
@@ -21722,32 +21740,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="77" t="s">
+      <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="60"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24496,7 +24514,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="57"/>
@@ -24526,35 +24544,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="78" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="57"/>
       <c r="D3" s="57"/>
       <c r="E3" s="57"/>
       <c r="F3" s="57"/>
-      <c r="G3" s="59" t="s">
+      <c r="G3" s="78" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="57"/>
       <c r="I3" s="57"/>
       <c r="J3" s="57"/>
       <c r="K3" s="57"/>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="78" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="57"/>
       <c r="N3" s="57"/>
       <c r="O3" s="57"/>
       <c r="P3" s="57"/>
-      <c r="Q3" s="59" t="s">
+      <c r="Q3" s="78" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="57"/>
       <c r="S3" s="57"/>
       <c r="T3" s="57"/>
       <c r="U3" s="57"/>
-      <c r="V3" s="58" t="s">
+      <c r="V3" s="77" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="57"/>
@@ -25253,15 +25271,21 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q12" s="48"/>
-      <c r="R12" s="48"/>
+      <c r="Q12" s="48">
+        <v>7.17</v>
+      </c>
+      <c r="R12" s="48">
+        <v>17</v>
+      </c>
       <c r="S12" s="48">
         <v>5</v>
       </c>
-      <c r="T12" s="48"/>
-      <c r="U12" s="48" t="str">
+      <c r="T12" s="48">
+        <v>4</v>
+      </c>
+      <c r="U12" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="V12" s="48">
         <f t="shared" si="4"/>
@@ -25269,26 +25293,32 @@
       </c>
       <c r="W12" s="48">
         <f t="shared" si="5"/>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="X12" s="48">
         <f t="shared" si="6"/>
-        <v>0.55000000000000004</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="48"/>
-      <c r="C13" s="48"/>
+      <c r="B13" s="48">
+        <v>7.18</v>
+      </c>
+      <c r="C13" s="48">
+        <v>16</v>
+      </c>
       <c r="D13" s="48">
         <v>5</v>
       </c>
-      <c r="E13" s="48"/>
-      <c r="F13" s="48" t="str">
+      <c r="E13" s="48">
+        <v>5</v>
+      </c>
+      <c r="F13" s="48">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="G13" s="48"/>
       <c r="H13" s="48"/>
@@ -25326,11 +25356,11 @@
       </c>
       <c r="W13" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X13" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25744,11 +25774,11 @@
       </c>
       <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" si="0"/>
-        <v>0.26250000000000001</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="G21" s="50"/>
       <c r="H21" s="50"/>
@@ -25786,11 +25816,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>0.21249999999999999</v>
+        <v>0.26250000000000001</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25798,11 +25828,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.28749999999999998</v>
+        <v>0.31562499999999999</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25818,11 +25848,11 @@
       </c>
       <c r="E23" s="53">
         <f>E21</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F23" s="53">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23/D23,"")</f>
-        <v>0.26250000000000001</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -25860,11 +25890,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>0.21249999999999999</v>
+        <v>0.26250000000000001</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -25872,11 +25902,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.28749999999999998</v>
+        <v>0.31562499999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-27 14:42:51
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFEFA7A-C95F-4397-B5A4-280D648E65C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A718A7-4489-4697-AF02-A9C6A19A2FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9158,18 +9158,28 @@
       <c r="A11" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34" t="str">
+      <c r="B11" s="34">
+        <v>727</v>
+      </c>
+      <c r="C11" s="34">
+        <v>17</v>
+      </c>
+      <c r="D11" s="34">
+        <v>12</v>
+      </c>
+      <c r="E11" s="34">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34" t="str">
+        <v>0.70588235294117652</v>
+      </c>
+      <c r="F11" s="34">
+        <v>7</v>
+      </c>
+      <c r="G11" s="34">
+        <v>3</v>
+      </c>
+      <c r="H11" s="34">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.42857142857142855</v>
       </c>
       <c r="I11" s="34"/>
       <c r="J11" s="34"/>
@@ -9179,15 +9189,15 @@
       </c>
       <c r="L11" s="34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M11" s="34">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N11" s="34" t="e">
+        <v>15</v>
+      </c>
+      <c r="N11" s="34">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9269,27 +9279,27 @@
       <c r="B14" s="36"/>
       <c r="C14" s="37">
         <f>SUM(C5:C13)</f>
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D14" s="37">
         <f>SUM(D5:D13)</f>
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="E14" s="37">
         <f t="shared" si="0"/>
-        <v>0.85542168674698793</v>
+        <v>0.83</v>
       </c>
       <c r="F14" s="37">
         <f>SUM(F5:F13)</f>
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H14" s="37">
         <f t="shared" si="1"/>
-        <v>0.82191780821917804</v>
+        <v>0.78749999999999998</v>
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
@@ -9305,15 +9315,15 @@
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>289</v>
+        <v>313</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.77162629757785473</v>
+        <v>0.76038338658146964</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9324,27 +9334,27 @@
       <c r="B16" s="39"/>
       <c r="C16" s="40">
         <f>C14</f>
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D16" s="40">
         <f>D14</f>
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="E16" s="40">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),D16/C16,"")</f>
-        <v>0.85542168674698793</v>
+        <v>0.83</v>
       </c>
       <c r="F16" s="40">
         <f>F14</f>
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G16" s="40">
         <f>G14</f>
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H16" s="40">
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),G16/F16,"")</f>
-        <v>0.82191780821917804</v>
+        <v>0.78749999999999998</v>
       </c>
       <c r="I16" s="40">
         <f>I14</f>
@@ -9360,15 +9370,15 @@
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>289</v>
+        <v>313</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.77162629757785473</v>
+        <v>0.76038338658146964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-30 17:54:12
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A718A7-4489-4697-AF02-A9C6A19A2FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88F5DD4-C377-4ED8-9485-23EE13FF263F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="308">
   <si>
     <t>英语真题阅读 正确率记录</t>
   </si>
@@ -962,6 +962,10 @@
   </si>
   <si>
     <t>综合篇中三个物理应用题目未做</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>空间解析几何的内容未完成</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1454,22 +1458,28 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1478,25 +1488,19 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7519,13 +7523,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
     </row>
     <row r="2" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7546,13 +7550,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="64" t="s">
+      <c r="A4" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="58"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8057,13 +8061,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="64" t="s">
+      <c r="A41" s="66" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="59"/>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
+      <c r="B41" s="57"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8544,13 +8548,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="64" t="s">
+      <c r="A83" s="66" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="59"/>
-      <c r="C83" s="59"/>
-      <c r="D83" s="59"/>
-      <c r="E83" s="60"/>
+      <c r="B83" s="57"/>
+      <c r="C83" s="57"/>
+      <c r="D83" s="57"/>
+      <c r="E83" s="58"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8768,47 +8772,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="68" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
     </row>
     <row r="2" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="69" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="63" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="62" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="71" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="61" t="s">
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="59"/>
-      <c r="N3" s="60"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="58"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9181,23 +9185,27 @@
         <f t="shared" si="1"/>
         <v>0.42857142857142855</v>
       </c>
-      <c r="I11" s="34"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34" t="str">
+      <c r="I11" s="34">
+        <v>23</v>
+      </c>
+      <c r="J11" s="34">
+        <v>16</v>
+      </c>
+      <c r="K11" s="34">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.69565217391304346</v>
       </c>
       <c r="L11" s="34">
         <f t="shared" si="3"/>
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="M11" s="34">
         <f t="shared" si="4"/>
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="N11" s="34">
         <f t="shared" si="5"/>
-        <v>0.625</v>
+        <v>0.65957446808510634</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -9303,27 +9311,27 @@
       </c>
       <c r="I14" s="37">
         <f>SUM(I5:I13)</f>
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="J14" s="37">
         <f>SUM(J5:J13)</f>
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="K14" s="37">
         <f t="shared" si="2"/>
-        <v>0.69172932330827064</v>
+        <v>0.69230769230769229</v>
       </c>
       <c r="L14" s="37">
         <f>SUM(L5:L13)</f>
-        <v>313</v>
+        <v>336</v>
       </c>
       <c r="M14" s="37">
         <f>SUM(M5:M13)</f>
-        <v>238</v>
+        <v>254</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="5"/>
-        <v>0.76038338658146964</v>
+        <v>0.75595238095238093</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9358,27 +9366,27 @@
       </c>
       <c r="I16" s="40">
         <f>I14</f>
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="J16" s="40">
         <f>J14</f>
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="K16" s="40">
         <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),J16/I16,"")</f>
-        <v>0.69172932330827064</v>
+        <v>0.69230769230769229</v>
       </c>
       <c r="L16" s="40">
         <f>L14</f>
-        <v>313</v>
+        <v>336</v>
       </c>
       <c r="M16" s="40">
         <f>M14</f>
-        <v>238</v>
+        <v>254</v>
       </c>
       <c r="N16" s="40">
         <f>IF(AND(L16&lt;&gt;"",M16&lt;&gt;""),M16/L16,"")</f>
-        <v>0.76038338658146964</v>
+        <v>0.75595238095238093</v>
       </c>
     </row>
   </sheetData>
@@ -9503,42 +9511,42 @@
     <col min="3" max="14" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+    <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="64" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-    </row>
-    <row r="2" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+    </row>
+    <row r="2" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="69" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="68" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
-    </row>
-    <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
+    </row>
+    <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>50</v>
       </c>
@@ -9573,22 +9581,22 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="67" t="s">
+    <row r="5" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="60"/>
-    </row>
-    <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="58"/>
+    </row>
+    <row r="6" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>128</v>
       </c>
@@ -9628,7 +9636,7 @@
         <v>0.94594594594594594</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>129</v>
       </c>
@@ -9668,7 +9676,7 @@
         <v>0.85507246376811596</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>130</v>
       </c>
@@ -9708,7 +9716,7 @@
         <v>0.84615384615384615</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>131</v>
       </c>
@@ -9738,11 +9746,13 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="4">
+        <v>728</v>
+      </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="str">
@@ -9767,8 +9777,11 @@
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L10" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>133</v>
       </c>
@@ -9798,7 +9811,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>134</v>
       </c>
@@ -9828,37 +9841,47 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4" t="str">
+      <c r="B13" s="4">
+        <v>729</v>
+      </c>
+      <c r="C13" s="4">
+        <v>15</v>
+      </c>
+      <c r="D13" s="4">
+        <v>10</v>
+      </c>
+      <c r="E13" s="4">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4" t="str">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="F13" s="4">
+        <v>20</v>
+      </c>
+      <c r="G13" s="4">
+        <v>18</v>
+      </c>
+      <c r="H13" s="4">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.9</v>
       </c>
       <c r="I13" s="4">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J13" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K13" s="4" t="e">
+        <v>28</v>
+      </c>
+      <c r="K13" s="4">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>136</v>
       </c>
@@ -9888,63 +9911,63 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>137</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7">
         <f>SUM(C6:C14)</f>
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D15" s="7">
         <f>SUM(D6:D14)</f>
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>0.87654320987654322</v>
+        <v>0.84375</v>
       </c>
       <c r="F15" s="7">
         <f>SUM(F6:F14)</f>
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G15" s="7">
         <f>SUM(G6:G14)</f>
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="H15" s="7">
         <f t="shared" si="1"/>
-        <v>0.8666666666666667</v>
+        <v>0.87272727272727268</v>
       </c>
       <c r="I15" s="7">
         <f>SUM(I6:I14)</f>
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="J15" s="7">
         <f>SUM(J6:J14)</f>
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="4"/>
-        <v>0.87134502923976609</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>0.85922330097087374</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="67" t="s">
+      <c r="A17" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="60"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="58"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10170,19 +10193,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="67" t="s">
+      <c r="A26" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="60"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="58"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10473,83 +10496,83 @@
       <c r="B36" s="9"/>
       <c r="C36" s="10">
         <f>C15+C24+C35</f>
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D36" s="10">
         <f>D15+D24+D35</f>
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="E36" s="10">
         <f t="shared" si="9"/>
-        <v>0.87654320987654322</v>
+        <v>0.84375</v>
       </c>
       <c r="F36" s="10">
         <f>F15+F24+F35</f>
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G36" s="10">
         <f>G15+G24+G35</f>
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="H36" s="10">
         <f t="shared" si="10"/>
-        <v>0.8666666666666667</v>
+        <v>0.87272727272727268</v>
       </c>
       <c r="I36" s="10">
         <f>I15+I24+I35</f>
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="J36" s="10">
         <f>J15+J24+J35</f>
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="K36" s="10">
         <f t="shared" si="12"/>
-        <v>0.87134502923976609</v>
+        <v>0.85922330097087374</v>
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="72" t="s">
+      <c r="A39" s="61" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="57"/>
-      <c r="C39" s="57"/>
-      <c r="D39" s="57"/>
-      <c r="E39" s="57"/>
-      <c r="F39" s="57"/>
-      <c r="G39" s="57"/>
-      <c r="H39" s="57"/>
-      <c r="I39" s="57"/>
-      <c r="J39" s="57"/>
-      <c r="K39" s="57"/>
-      <c r="L39" s="57"/>
-      <c r="M39" s="57"/>
-      <c r="N39" s="57"/>
+      <c r="B39" s="62"/>
+      <c r="C39" s="62"/>
+      <c r="D39" s="62"/>
+      <c r="E39" s="62"/>
+      <c r="F39" s="62"/>
+      <c r="G39" s="62"/>
+      <c r="H39" s="62"/>
+      <c r="I39" s="62"/>
+      <c r="J39" s="62"/>
+      <c r="K39" s="62"/>
+      <c r="L39" s="62"/>
+      <c r="M39" s="62"/>
+      <c r="N39" s="62"/>
     </row>
     <row r="40" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="71" t="s">
+      <c r="C41" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="59"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="69" t="s">
+      <c r="D41" s="57"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="59"/>
-      <c r="H41" s="60"/>
-      <c r="I41" s="70" t="s">
+      <c r="G41" s="57"/>
+      <c r="H41" s="58"/>
+      <c r="I41" s="65" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="59"/>
-      <c r="K41" s="60"/>
-      <c r="L41" s="68" t="s">
+      <c r="J41" s="57"/>
+      <c r="K41" s="58"/>
+      <c r="L41" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="59"/>
-      <c r="N41" s="60"/>
+      <c r="M41" s="57"/>
+      <c r="N41" s="58"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10596,22 +10619,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="67" t="s">
+      <c r="A43" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="59"/>
-      <c r="C43" s="59"/>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="59"/>
-      <c r="I43" s="59"/>
-      <c r="J43" s="59"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="60"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="57"/>
+      <c r="J43" s="57"/>
+      <c r="K43" s="57"/>
+      <c r="L43" s="57"/>
+      <c r="M43" s="57"/>
+      <c r="N43" s="58"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10809,7 +10832,7 @@
       </c>
       <c r="B48" s="4">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>728</v>
       </c>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
@@ -10926,13 +10949,17 @@
       </c>
       <c r="B51" s="4">
         <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4" t="str">
+        <v>729</v>
+      </c>
+      <c r="C51" s="4">
+        <v>13</v>
+      </c>
+      <c r="D51" s="4">
+        <v>8</v>
+      </c>
+      <c r="E51" s="4">
         <f t="shared" si="14"/>
-        <v/>
+        <v>0.61538461538461542</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -10948,15 +10975,15 @@
       </c>
       <c r="L51" s="4">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="M51" s="4">
         <f>D51+G51+J51</f>
-        <v>0</v>
-      </c>
-      <c r="N51" s="4" t="e">
+        <v>8</v>
+      </c>
+      <c r="N51" s="4">
         <f t="shared" si="19"/>
-        <v>#DIV/0!</v>
+        <v>0.61538461538461542</v>
       </c>
     </row>
     <row r="52" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -11005,15 +11032,15 @@
       <c r="B53" s="6"/>
       <c r="C53" s="7">
         <f>SUM(C44:C52)</f>
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="D53" s="7">
         <f>SUM(D44:D52)</f>
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E53" s="7">
         <f t="shared" si="14"/>
-        <v>0.73170731707317072</v>
+        <v>0.70370370370370372</v>
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
@@ -11041,35 +11068,35 @@
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.65217391304347827</v>
+        <v>0.6484375</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="67" t="s">
+      <c r="A55" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="59"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="F55" s="59"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="59"/>
-      <c r="I55" s="59"/>
-      <c r="J55" s="59"/>
-      <c r="K55" s="59"/>
-      <c r="L55" s="59"/>
-      <c r="M55" s="59"/>
-      <c r="N55" s="60"/>
+      <c r="B55" s="57"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="57"/>
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="57"/>
+      <c r="I55" s="57"/>
+      <c r="J55" s="57"/>
+      <c r="K55" s="57"/>
+      <c r="L55" s="57"/>
+      <c r="M55" s="57"/>
+      <c r="N55" s="58"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11361,22 +11388,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="67" t="s">
+      <c r="A64" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="59"/>
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-      <c r="F64" s="59"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="59"/>
-      <c r="I64" s="59"/>
-      <c r="J64" s="59"/>
-      <c r="K64" s="59"/>
-      <c r="L64" s="59"/>
-      <c r="M64" s="59"/>
-      <c r="N64" s="60"/>
+      <c r="B64" s="57"/>
+      <c r="C64" s="57"/>
+      <c r="D64" s="57"/>
+      <c r="E64" s="57"/>
+      <c r="F64" s="57"/>
+      <c r="G64" s="57"/>
+      <c r="H64" s="57"/>
+      <c r="I64" s="57"/>
+      <c r="J64" s="57"/>
+      <c r="K64" s="57"/>
+      <c r="L64" s="57"/>
+      <c r="M64" s="57"/>
+      <c r="N64" s="58"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11751,15 +11778,15 @@
       <c r="B74" s="9"/>
       <c r="C74" s="10">
         <f>C53+C62+C73</f>
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="D74" s="10">
         <f>D53+D62+D73</f>
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E74" s="10">
         <f t="shared" si="27"/>
-        <v>0.73170731707317072</v>
+        <v>0.70370370370370372</v>
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
@@ -11787,51 +11814,51 @@
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.65217391304347827</v>
+        <v>0.6484375</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="72" t="s">
+      <c r="A77" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="57"/>
-      <c r="C77" s="57"/>
-      <c r="D77" s="57"/>
-      <c r="E77" s="57"/>
-      <c r="F77" s="57"/>
-      <c r="G77" s="57"/>
-      <c r="H77" s="57"/>
-      <c r="I77" s="57"/>
-      <c r="J77" s="57"/>
-      <c r="K77" s="57"/>
+      <c r="B77" s="62"/>
+      <c r="C77" s="62"/>
+      <c r="D77" s="62"/>
+      <c r="E77" s="62"/>
+      <c r="F77" s="62"/>
+      <c r="G77" s="62"/>
+      <c r="H77" s="62"/>
+      <c r="I77" s="62"/>
+      <c r="J77" s="62"/>
+      <c r="K77" s="62"/>
     </row>
     <row r="78" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="71" t="s">
+      <c r="C79" s="56" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="59"/>
-      <c r="E79" s="60"/>
-      <c r="F79" s="69" t="s">
+      <c r="D79" s="57"/>
+      <c r="E79" s="58"/>
+      <c r="F79" s="60" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="59"/>
-      <c r="H79" s="60"/>
-      <c r="I79" s="68" t="s">
+      <c r="G79" s="57"/>
+      <c r="H79" s="58"/>
+      <c r="I79" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="59"/>
-      <c r="K79" s="60"/>
+      <c r="J79" s="57"/>
+      <c r="K79" s="58"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11869,19 +11896,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="67" t="s">
+      <c r="A81" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="59"/>
-      <c r="C81" s="59"/>
-      <c r="D81" s="59"/>
-      <c r="E81" s="59"/>
-      <c r="F81" s="59"/>
-      <c r="G81" s="59"/>
-      <c r="H81" s="59"/>
-      <c r="I81" s="59"/>
-      <c r="J81" s="59"/>
-      <c r="K81" s="60"/>
+      <c r="B81" s="57"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12069,7 +12096,7 @@
       </c>
       <c r="B86" s="4">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>728</v>
       </c>
       <c r="C86" s="4">
         <f t="shared" si="33"/>
@@ -12204,43 +12231,43 @@
       </c>
       <c r="B89" s="4">
         <f t="shared" si="32"/>
-        <v>0</v>
+        <v>729</v>
       </c>
       <c r="C89" s="4">
         <f t="shared" si="33"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="D89" s="4">
         <f t="shared" si="34"/>
-        <v>0</v>
-      </c>
-      <c r="E89" s="4" t="e">
+        <v>28</v>
+      </c>
+      <c r="E89" s="4">
         <f t="shared" si="35"/>
-        <v>#DIV/0!</v>
+        <v>0.8</v>
       </c>
       <c r="F89" s="4">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G89" s="4">
         <f t="shared" si="37"/>
-        <v>0</v>
-      </c>
-      <c r="H89" s="4" t="e">
+        <v>8</v>
+      </c>
+      <c r="H89" s="4">
         <f t="shared" si="38"/>
-        <v>#DIV/0!</v>
+        <v>0.61538461538461542</v>
       </c>
       <c r="I89" s="4">
         <f t="shared" si="39"/>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="J89" s="4">
         <f t="shared" si="40"/>
-        <v>0</v>
-      </c>
-      <c r="K89" s="4" t="e">
+        <v>36</v>
+      </c>
+      <c r="K89" s="4">
         <f t="shared" si="41"/>
-        <v>#DIV/0!</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12295,56 +12322,56 @@
       <c r="B91" s="6"/>
       <c r="C91" s="7">
         <f>SUM(C82:C90)</f>
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="D91" s="7">
         <f>SUM(D82:D90)</f>
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="E91" s="7">
         <f t="shared" si="35"/>
-        <v>0.87134502923976609</v>
+        <v>0.85922330097087374</v>
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.65217391304347827</v>
+        <v>0.6484375</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>286</v>
+        <v>334</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>224</v>
+        <v>260</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.78321678321678323</v>
+        <v>0.77844311377245512</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="67" t="s">
+      <c r="A93" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="59"/>
-      <c r="C93" s="59"/>
-      <c r="D93" s="59"/>
-      <c r="E93" s="59"/>
-      <c r="F93" s="59"/>
-      <c r="G93" s="59"/>
-      <c r="H93" s="59"/>
-      <c r="I93" s="59"/>
-      <c r="J93" s="59"/>
-      <c r="K93" s="60"/>
+      <c r="B93" s="57"/>
+      <c r="C93" s="57"/>
+      <c r="D93" s="57"/>
+      <c r="E93" s="57"/>
+      <c r="F93" s="57"/>
+      <c r="G93" s="57"/>
+      <c r="H93" s="57"/>
+      <c r="I93" s="57"/>
+      <c r="J93" s="57"/>
+      <c r="K93" s="58"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12660,19 +12687,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="67" t="s">
+      <c r="A102" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="59"/>
-      <c r="C102" s="59"/>
-      <c r="D102" s="59"/>
-      <c r="E102" s="59"/>
-      <c r="F102" s="59"/>
-      <c r="G102" s="59"/>
-      <c r="H102" s="59"/>
-      <c r="I102" s="59"/>
-      <c r="J102" s="59"/>
-      <c r="K102" s="60"/>
+      <c r="B102" s="57"/>
+      <c r="C102" s="57"/>
+      <c r="D102" s="57"/>
+      <c r="E102" s="57"/>
+      <c r="F102" s="57"/>
+      <c r="G102" s="57"/>
+      <c r="H102" s="57"/>
+      <c r="I102" s="57"/>
+      <c r="J102" s="57"/>
+      <c r="K102" s="58"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13083,49 +13110,43 @@
       <c r="B112" s="9"/>
       <c r="C112" s="10">
         <f>C91+C100+C111</f>
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="D112" s="10">
         <f>D91+D100+D111</f>
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="E112" s="10">
         <f t="shared" si="51"/>
-        <v>0.87134502923976609</v>
+        <v>0.85922330097087374</v>
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.65217391304347827</v>
+        <v>0.6484375</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>286</v>
+        <v>334</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>224</v>
+        <v>260</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.78321678321678323</v>
+        <v>0.77844311377245512</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13142,6 +13163,12 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13538,56 +13565,56 @@
       <c r="A1" s="73" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16793,59 +16820,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="64" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19688,56 +19715,56 @@
       <c r="A1" s="73" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21726,56 +21753,56 @@
       <c r="A1" s="73" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="11"/>
       <c r="M3" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59"/>
-      <c r="U3" s="59"/>
-      <c r="V3" s="60"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24527,29 +24554,29 @@
       <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="57"/>
-      <c r="W1" s="57"/>
-      <c r="X1" s="57"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
     </row>
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -24557,36 +24584,36 @@
       <c r="B3" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
       <c r="G3" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="62"/>
       <c r="Q3" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
+      <c r="R3" s="62"/>
+      <c r="S3" s="62"/>
+      <c r="T3" s="62"/>
+      <c r="U3" s="62"/>
       <c r="V3" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="57"/>
-      <c r="X3" s="57"/>
+      <c r="W3" s="62"/>
+      <c r="X3" s="62"/>
     </row>
     <row r="4" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">

</xml_diff>

<commit_message>
vault backup: 2026-08-01 17:04:37
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88F5DD4-C377-4ED8-9485-23EE13FF263F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9B2180-C601-42F6-8AF0-2C176D92EFDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="张宇1000题" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="310">
   <si>
     <t>英语真题阅读 正确率记录</t>
   </si>
@@ -966,6 +966,14 @@
   </si>
   <si>
     <t>空间解析几何的内容未完成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7.30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7.31</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1317,7 +1325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1458,28 +1466,34 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -7523,13 +7537,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
     </row>
     <row r="2" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7550,13 +7564,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="58"/>
+      <c r="B4" s="61"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="62"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8061,13 +8075,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="66" t="s">
+      <c r="A41" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="57"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="B41" s="61"/>
+      <c r="C41" s="61"/>
+      <c r="D41" s="61"/>
+      <c r="E41" s="62"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8548,13 +8562,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="57"/>
-      <c r="C83" s="57"/>
-      <c r="D83" s="57"/>
-      <c r="E83" s="58"/>
+      <c r="B83" s="61"/>
+      <c r="C83" s="61"/>
+      <c r="D83" s="61"/>
+      <c r="E83" s="62"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8772,47 +8786,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="70" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
     </row>
     <row r="2" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="69" t="s">
+      <c r="C3" s="71" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="72" t="s">
+      <c r="D3" s="61"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="74" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="71" t="s">
+      <c r="G3" s="61"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="73" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="70" t="s">
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="58"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="62"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9512,39 +9526,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
     </row>
     <row r="2" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="56" t="s">
+      <c r="C3" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60" t="s">
+      <c r="D3" s="61"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="62"/>
       <c r="I3" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9582,19 +9596,19 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="59" t="s">
+      <c r="A5" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="58"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="61"/>
+      <c r="K5" s="62"/>
     </row>
     <row r="6" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9955,19 +9969,19 @@
     </row>
     <row r="16" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="59" t="s">
+      <c r="A17" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="57"/>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="58"/>
+      <c r="B17" s="61"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="62"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10193,19 +10207,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="59" t="s">
+      <c r="A26" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="57"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="58"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="61"/>
+      <c r="J26" s="61"/>
+      <c r="K26" s="62"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10532,47 +10546,47 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="61" t="s">
+      <c r="A39" s="67" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="62"/>
-      <c r="C39" s="62"/>
-      <c r="D39" s="62"/>
-      <c r="E39" s="62"/>
-      <c r="F39" s="62"/>
-      <c r="G39" s="62"/>
-      <c r="H39" s="62"/>
-      <c r="I39" s="62"/>
-      <c r="J39" s="62"/>
-      <c r="K39" s="62"/>
-      <c r="L39" s="62"/>
-      <c r="M39" s="62"/>
-      <c r="N39" s="62"/>
+      <c r="B39" s="59"/>
+      <c r="C39" s="59"/>
+      <c r="D39" s="59"/>
+      <c r="E39" s="59"/>
+      <c r="F39" s="59"/>
+      <c r="G39" s="59"/>
+      <c r="H39" s="59"/>
+      <c r="I39" s="59"/>
+      <c r="J39" s="59"/>
+      <c r="K39" s="59"/>
+      <c r="L39" s="59"/>
+      <c r="M39" s="59"/>
+      <c r="N39" s="59"/>
     </row>
     <row r="40" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="56" t="s">
+      <c r="C41" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
-      <c r="F41" s="60" t="s">
+      <c r="D41" s="61"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="57"/>
-      <c r="H41" s="58"/>
+      <c r="G41" s="61"/>
+      <c r="H41" s="62"/>
       <c r="I41" s="65" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="57"/>
-      <c r="K41" s="58"/>
+      <c r="J41" s="61"/>
+      <c r="K41" s="62"/>
       <c r="L41" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="57"/>
-      <c r="N41" s="58"/>
+      <c r="M41" s="61"/>
+      <c r="N41" s="62"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10619,22 +10633,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="59" t="s">
+      <c r="A43" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="57"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="57"/>
-      <c r="N43" s="58"/>
+      <c r="B43" s="61"/>
+      <c r="C43" s="61"/>
+      <c r="D43" s="61"/>
+      <c r="E43" s="61"/>
+      <c r="F43" s="61"/>
+      <c r="G43" s="61"/>
+      <c r="H43" s="61"/>
+      <c r="I43" s="61"/>
+      <c r="J43" s="61"/>
+      <c r="K43" s="61"/>
+      <c r="L43" s="61"/>
+      <c r="M43" s="61"/>
+      <c r="N43" s="62"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -10961,29 +10975,37 @@
         <f t="shared" si="14"/>
         <v>0.61538461538461542</v>
       </c>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4" t="str">
+      <c r="F51" s="4">
+        <v>17</v>
+      </c>
+      <c r="G51" s="4">
+        <v>15</v>
+      </c>
+      <c r="H51" s="4">
         <f>IF(AND(F51&lt;&gt;"",G51&lt;&gt;""),G51/F51,"")</f>
-        <v/>
-      </c>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4" t="str">
+        <v>0.88235294117647056</v>
+      </c>
+      <c r="I51" s="4">
+        <v>2</v>
+      </c>
+      <c r="J51" s="4">
+        <v>1</v>
+      </c>
+      <c r="K51" s="4">
         <f t="shared" si="16"/>
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="L51" s="4">
         <f t="shared" si="17"/>
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="M51" s="4">
         <f>D51+G51+J51</f>
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="N51" s="4">
         <f t="shared" si="19"/>
-        <v>0.61538461538461542</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="52" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -11044,59 +11066,59 @@
       </c>
       <c r="F53" s="7">
         <f>SUM(F44:F52)</f>
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="G53" s="7">
         <f>SUM(G44:G52)</f>
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="H53" s="7">
         <f t="shared" si="15"/>
-        <v>0.6376811594202898</v>
+        <v>0.68604651162790697</v>
       </c>
       <c r="I53" s="7">
         <f>SUM(I44:I52)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J53" s="7">
         <f>SUM(J44:J52)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K53" s="7">
         <f t="shared" si="16"/>
-        <v>0.2</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="L53" s="7">
         <f>SUM(L44:L52)</f>
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="M53" s="7">
         <f>SUM(M44:M52)</f>
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="N53" s="7">
         <f t="shared" si="19"/>
-        <v>0.6484375</v>
+        <v>0.67346938775510201</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="59" t="s">
+      <c r="A55" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="57"/>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="57"/>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
-      <c r="I55" s="57"/>
-      <c r="J55" s="57"/>
-      <c r="K55" s="57"/>
-      <c r="L55" s="57"/>
-      <c r="M55" s="57"/>
-      <c r="N55" s="58"/>
+      <c r="B55" s="61"/>
+      <c r="C55" s="61"/>
+      <c r="D55" s="61"/>
+      <c r="E55" s="61"/>
+      <c r="F55" s="61"/>
+      <c r="G55" s="61"/>
+      <c r="H55" s="61"/>
+      <c r="I55" s="61"/>
+      <c r="J55" s="61"/>
+      <c r="K55" s="61"/>
+      <c r="L55" s="61"/>
+      <c r="M55" s="61"/>
+      <c r="N55" s="62"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11388,22 +11410,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="59" t="s">
+      <c r="A64" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="57"/>
-      <c r="H64" s="57"/>
-      <c r="I64" s="57"/>
-      <c r="J64" s="57"/>
-      <c r="K64" s="57"/>
-      <c r="L64" s="57"/>
-      <c r="M64" s="57"/>
-      <c r="N64" s="58"/>
+      <c r="B64" s="61"/>
+      <c r="C64" s="61"/>
+      <c r="D64" s="61"/>
+      <c r="E64" s="61"/>
+      <c r="F64" s="61"/>
+      <c r="G64" s="61"/>
+      <c r="H64" s="61"/>
+      <c r="I64" s="61"/>
+      <c r="J64" s="61"/>
+      <c r="K64" s="61"/>
+      <c r="L64" s="61"/>
+      <c r="M64" s="61"/>
+      <c r="N64" s="62"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11790,75 +11812,75 @@
       </c>
       <c r="F74" s="10">
         <f>F53+F62+F73</f>
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="G74" s="10">
         <f>G53+G62+G73</f>
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="H74" s="10">
         <f t="shared" si="28"/>
-        <v>0.6376811594202898</v>
+        <v>0.68604651162790697</v>
       </c>
       <c r="I74" s="10">
         <f>I53+I62+I73</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J74" s="10">
         <f>J53+J62+J73</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74" s="10">
         <f t="shared" si="29"/>
-        <v>0.2</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="L74" s="10">
         <f>L53+L62+L73</f>
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="M74" s="10">
         <f>M53+M62+M73</f>
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="N74" s="10">
         <f t="shared" si="31"/>
-        <v>0.6484375</v>
+        <v>0.67346938775510201</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="61" t="s">
+      <c r="A77" s="67" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="62"/>
-      <c r="C77" s="62"/>
-      <c r="D77" s="62"/>
-      <c r="E77" s="62"/>
-      <c r="F77" s="62"/>
-      <c r="G77" s="62"/>
-      <c r="H77" s="62"/>
-      <c r="I77" s="62"/>
-      <c r="J77" s="62"/>
-      <c r="K77" s="62"/>
+      <c r="B77" s="59"/>
+      <c r="C77" s="59"/>
+      <c r="D77" s="59"/>
+      <c r="E77" s="59"/>
+      <c r="F77" s="59"/>
+      <c r="G77" s="59"/>
+      <c r="H77" s="59"/>
+      <c r="I77" s="59"/>
+      <c r="J77" s="59"/>
+      <c r="K77" s="59"/>
     </row>
     <row r="78" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="56" t="s">
+      <c r="C79" s="66" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="57"/>
-      <c r="E79" s="58"/>
-      <c r="F79" s="60" t="s">
+      <c r="D79" s="61"/>
+      <c r="E79" s="62"/>
+      <c r="F79" s="64" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="57"/>
-      <c r="H79" s="58"/>
+      <c r="G79" s="61"/>
+      <c r="H79" s="62"/>
       <c r="I79" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="57"/>
-      <c r="K79" s="58"/>
+      <c r="J79" s="61"/>
+      <c r="K79" s="62"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11896,19 +11918,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="59" t="s">
+      <c r="A81" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="57"/>
-      <c r="C81" s="57"/>
-      <c r="D81" s="57"/>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="57"/>
-      <c r="J81" s="57"/>
-      <c r="K81" s="58"/>
+      <c r="B81" s="61"/>
+      <c r="C81" s="61"/>
+      <c r="D81" s="61"/>
+      <c r="E81" s="61"/>
+      <c r="F81" s="61"/>
+      <c r="G81" s="61"/>
+      <c r="H81" s="61"/>
+      <c r="I81" s="61"/>
+      <c r="J81" s="61"/>
+      <c r="K81" s="62"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12247,27 +12269,27 @@
       </c>
       <c r="F89" s="4">
         <f t="shared" si="36"/>
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G89" s="4">
         <f t="shared" si="37"/>
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="H89" s="4">
         <f t="shared" si="38"/>
-        <v>0.61538461538461542</v>
+        <v>0.75</v>
       </c>
       <c r="I89" s="4">
         <f t="shared" si="39"/>
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="J89" s="4">
         <f t="shared" si="40"/>
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="K89" s="4">
         <f t="shared" si="41"/>
-        <v>0.75</v>
+        <v>0.77611940298507465</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -12334,44 +12356,44 @@
       </c>
       <c r="F91" s="7">
         <f>SUM(F82:F90)</f>
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="G91" s="7">
         <f>SUM(G82:G90)</f>
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="H91" s="7">
         <f t="shared" si="38"/>
-        <v>0.6484375</v>
+        <v>0.67346938775510201</v>
       </c>
       <c r="I91" s="7">
         <f>SUM(I82:I90)</f>
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="J91" s="7">
         <f>SUM(J82:J90)</f>
-        <v>260</v>
+        <v>276</v>
       </c>
       <c r="K91" s="7">
         <f t="shared" si="41"/>
-        <v>0.77844311377245512</v>
+        <v>0.78186968838526916</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="59" t="s">
+      <c r="A93" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="57"/>
-      <c r="C93" s="57"/>
-      <c r="D93" s="57"/>
-      <c r="E93" s="57"/>
-      <c r="F93" s="57"/>
-      <c r="G93" s="57"/>
-      <c r="H93" s="57"/>
-      <c r="I93" s="57"/>
-      <c r="J93" s="57"/>
-      <c r="K93" s="58"/>
+      <c r="B93" s="61"/>
+      <c r="C93" s="61"/>
+      <c r="D93" s="61"/>
+      <c r="E93" s="61"/>
+      <c r="F93" s="61"/>
+      <c r="G93" s="61"/>
+      <c r="H93" s="61"/>
+      <c r="I93" s="61"/>
+      <c r="J93" s="61"/>
+      <c r="K93" s="62"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12687,19 +12709,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="59" t="s">
+      <c r="A102" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="57"/>
-      <c r="C102" s="57"/>
-      <c r="D102" s="57"/>
-      <c r="E102" s="57"/>
-      <c r="F102" s="57"/>
-      <c r="G102" s="57"/>
-      <c r="H102" s="57"/>
-      <c r="I102" s="57"/>
-      <c r="J102" s="57"/>
-      <c r="K102" s="58"/>
+      <c r="B102" s="61"/>
+      <c r="C102" s="61"/>
+      <c r="D102" s="61"/>
+      <c r="E102" s="61"/>
+      <c r="F102" s="61"/>
+      <c r="G102" s="61"/>
+      <c r="H102" s="61"/>
+      <c r="I102" s="61"/>
+      <c r="J102" s="61"/>
+      <c r="K102" s="62"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13122,31 +13144,37 @@
       </c>
       <c r="F112" s="10">
         <f>F91+F100+F111</f>
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="G112" s="10">
         <f>G91+G100+G111</f>
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="H112" s="10">
         <f t="shared" si="53"/>
-        <v>0.6484375</v>
+        <v>0.67346938775510201</v>
       </c>
       <c r="I112" s="10">
         <f>I91+I100+I111</f>
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="J112" s="10">
         <f>J91+J100+J111</f>
-        <v>260</v>
+        <v>276</v>
       </c>
       <c r="K112" s="10">
         <f t="shared" si="55"/>
-        <v>0.77844311377245512</v>
+        <v>0.78186968838526916</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13163,12 +13191,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13562,59 +13584,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="75" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="59"/>
+      <c r="V1" s="59"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="74" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16820,59 +16842,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="58" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="59"/>
+      <c r="V1" s="59"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="74" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19712,59 +19734,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="75" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="59"/>
+      <c r="V1" s="59"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="74" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21750,59 +21772,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="75" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="59"/>
+      <c r="V1" s="59"/>
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="74" t="s">
+      <c r="M3" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="58"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="61"/>
+      <c r="Q3" s="61"/>
+      <c r="R3" s="61"/>
+      <c r="S3" s="61"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="62"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24551,69 +24573,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
+      <c r="A1" s="78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="59"/>
+      <c r="V1" s="59"/>
+      <c r="W1" s="59"/>
+      <c r="X1" s="59"/>
     </row>
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="78" t="s">
+      <c r="B3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="78" t="s">
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="78" t="s">
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="62"/>
-      <c r="N3" s="62"/>
-      <c r="O3" s="62"/>
-      <c r="P3" s="62"/>
-      <c r="Q3" s="78" t="s">
+      <c r="M3" s="59"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="62"/>
-      <c r="S3" s="62"/>
-      <c r="T3" s="62"/>
-      <c r="U3" s="62"/>
-      <c r="V3" s="77" t="s">
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="62"/>
-      <c r="X3" s="62"/>
+      <c r="W3" s="59"/>
+      <c r="X3" s="59"/>
     </row>
     <row r="4" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
@@ -24693,7 +24715,7 @@
       <c r="A5" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="56" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="48">
@@ -24709,7 +24731,7 @@
         <f t="shared" ref="F5:F21" si="0">IF(AND(D5&lt;&gt;"",E5&lt;&gt;""),E5/D5,"")</f>
         <v>0.4</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="56" t="s">
         <v>14</v>
       </c>
       <c r="H5" s="48">
@@ -24725,7 +24747,7 @@
         <f t="shared" ref="K5:K21" si="1">IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),J5/I5,"")</f>
         <v>0.4</v>
       </c>
-      <c r="L5" s="48" t="s">
+      <c r="L5" s="56" t="s">
         <v>15</v>
       </c>
       <c r="M5" s="48">
@@ -24741,7 +24763,7 @@
         <f t="shared" ref="P5:P21" si="2">IF(AND(N5&lt;&gt;"",O5&lt;&gt;""),O5/N5,"")</f>
         <v>0.6</v>
       </c>
-      <c r="Q5" s="48" t="s">
+      <c r="Q5" s="56" t="s">
         <v>16</v>
       </c>
       <c r="R5" s="48">
@@ -24774,7 +24796,7 @@
       <c r="A6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="56" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="48">
@@ -24790,7 +24812,7 @@
         <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
-      <c r="G6" s="48" t="s">
+      <c r="G6" s="56" t="s">
         <v>19</v>
       </c>
       <c r="H6" s="48">
@@ -24806,7 +24828,7 @@
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
-      <c r="L6" s="48" t="s">
+      <c r="L6" s="56" t="s">
         <v>20</v>
       </c>
       <c r="M6" s="48">
@@ -24822,7 +24844,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q6" s="48" t="s">
+      <c r="Q6" s="56" t="s">
         <v>21</v>
       </c>
       <c r="R6" s="48">
@@ -24855,7 +24877,7 @@
       <c r="A7" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="56" t="s">
         <v>23</v>
       </c>
       <c r="C7" s="48">
@@ -24871,7 +24893,7 @@
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="G7" s="48" t="s">
+      <c r="G7" s="56" t="s">
         <v>24</v>
       </c>
       <c r="H7" s="48">
@@ -24887,7 +24909,7 @@
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="56" t="s">
         <v>25</v>
       </c>
       <c r="M7" s="48">
@@ -24903,7 +24925,7 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="Q7" s="48" t="s">
+      <c r="Q7" s="56" t="s">
         <v>26</v>
       </c>
       <c r="R7" s="48">
@@ -24936,7 +24958,7 @@
       <c r="A8" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="56" t="s">
         <v>28</v>
       </c>
       <c r="C8" s="48">
@@ -24952,7 +24974,7 @@
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="G8" s="48" t="s">
+      <c r="G8" s="56" t="s">
         <v>29</v>
       </c>
       <c r="H8" s="48">
@@ -24968,7 +24990,7 @@
         <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="L8" s="48" t="s">
+      <c r="L8" s="56" t="s">
         <v>30</v>
       </c>
       <c r="M8" s="48">
@@ -24984,7 +25006,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q8" s="48" t="s">
+      <c r="Q8" s="56" t="s">
         <v>31</v>
       </c>
       <c r="R8" s="48">
@@ -25017,7 +25039,7 @@
       <c r="A9" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="56" t="s">
         <v>33</v>
       </c>
       <c r="C9" s="48">
@@ -25033,7 +25055,7 @@
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="G9" s="48" t="s">
+      <c r="G9" s="56" t="s">
         <v>34</v>
       </c>
       <c r="H9" s="48">
@@ -25049,7 +25071,7 @@
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
-      <c r="L9" s="48" t="s">
+      <c r="L9" s="56" t="s">
         <v>35</v>
       </c>
       <c r="M9" s="48">
@@ -25065,7 +25087,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q9" s="48">
+      <c r="Q9" s="56">
         <v>6.21</v>
       </c>
       <c r="R9" s="48">
@@ -25098,7 +25120,7 @@
       <c r="A10" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="48">
+      <c r="B10" s="56">
         <v>6.23</v>
       </c>
       <c r="C10" s="48">
@@ -25114,7 +25136,7 @@
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="G10" s="48">
+      <c r="G10" s="56">
         <v>6.25</v>
       </c>
       <c r="H10" s="48">
@@ -25130,7 +25152,7 @@
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="L10" s="48">
+      <c r="L10" s="56">
         <v>6.28</v>
       </c>
       <c r="M10" s="48">
@@ -25146,7 +25168,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q10" s="48">
+      <c r="Q10" s="56">
         <v>7.2</v>
       </c>
       <c r="R10" s="48">
@@ -25179,7 +25201,7 @@
       <c r="A11" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="56">
         <v>7.4</v>
       </c>
       <c r="C11" s="48">
@@ -25195,7 +25217,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G11" s="48">
+      <c r="G11" s="56">
         <v>7.7</v>
       </c>
       <c r="H11" s="48">
@@ -25211,7 +25233,7 @@
         <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="L11" s="48">
+      <c r="L11" s="56">
         <v>7.8</v>
       </c>
       <c r="M11" s="48">
@@ -25227,7 +25249,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q11" s="48">
+      <c r="Q11" s="56">
         <v>7.9</v>
       </c>
       <c r="R11" s="48">
@@ -25260,7 +25282,7 @@
       <c r="A12" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="48">
+      <c r="B12" s="56">
         <v>7.12</v>
       </c>
       <c r="C12" s="48">
@@ -25276,7 +25298,7 @@
         <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
-      <c r="G12" s="48">
+      <c r="G12" s="56">
         <v>7.13</v>
       </c>
       <c r="H12" s="48">
@@ -25292,7 +25314,7 @@
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="L12" s="48">
+      <c r="L12" s="56">
         <v>7.16</v>
       </c>
       <c r="M12" s="48">
@@ -25308,7 +25330,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="Q12" s="48">
+      <c r="Q12" s="56">
         <v>7.17</v>
       </c>
       <c r="R12" s="48">
@@ -25341,7 +25363,7 @@
       <c r="A13" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="48">
+      <c r="B13" s="56">
         <v>7.18</v>
       </c>
       <c r="C13" s="48">
@@ -25357,27 +25379,39 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G13" s="48"/>
-      <c r="H13" s="48"/>
+      <c r="G13" s="57" t="s">
+        <v>308</v>
+      </c>
+      <c r="H13" s="48">
+        <v>20</v>
+      </c>
       <c r="I13" s="48">
         <v>5</v>
       </c>
-      <c r="J13" s="55"/>
-      <c r="K13" s="48" t="str">
+      <c r="J13" s="55">
+        <v>2</v>
+      </c>
+      <c r="K13" s="48">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="L13" s="48"/>
-      <c r="M13" s="48"/>
+        <v>0.4</v>
+      </c>
+      <c r="L13" s="57" t="s">
+        <v>309</v>
+      </c>
+      <c r="M13" s="48">
+        <v>14</v>
+      </c>
       <c r="N13" s="48">
         <v>5</v>
       </c>
-      <c r="O13" s="48"/>
-      <c r="P13" s="48" t="str">
+      <c r="O13" s="48">
+        <v>5</v>
+      </c>
+      <c r="P13" s="48">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q13" s="48"/>
+        <v>1</v>
+      </c>
+      <c r="Q13" s="56"/>
       <c r="R13" s="48"/>
       <c r="S13" s="48">
         <v>5</v>
@@ -25393,18 +25427,18 @@
       </c>
       <c r="W13" s="48">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="X13" s="48">
         <f t="shared" si="6"/>
-        <v>0.25</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="48"/>
+      <c r="B14" s="56"/>
       <c r="C14" s="48"/>
       <c r="D14" s="48">
         <v>5</v>
@@ -25414,7 +25448,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G14" s="48"/>
+      <c r="G14" s="56"/>
       <c r="H14" s="48"/>
       <c r="I14" s="48">
         <v>5</v>
@@ -25424,7 +25458,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L14" s="48"/>
+      <c r="L14" s="56"/>
       <c r="M14" s="48"/>
       <c r="N14" s="48">
         <v>5</v>
@@ -25434,7 +25468,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q14" s="48"/>
+      <c r="Q14" s="56"/>
       <c r="R14" s="48"/>
       <c r="S14" s="48">
         <v>5</v>
@@ -25461,7 +25495,7 @@
       <c r="A15" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="56"/>
       <c r="C15" s="48"/>
       <c r="D15" s="48">
         <v>5</v>
@@ -25471,7 +25505,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G15" s="48"/>
+      <c r="G15" s="56"/>
       <c r="H15" s="48"/>
       <c r="I15" s="48">
         <v>5</v>
@@ -25481,7 +25515,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L15" s="48"/>
+      <c r="L15" s="56"/>
       <c r="M15" s="48"/>
       <c r="N15" s="48">
         <v>5</v>
@@ -25491,7 +25525,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q15" s="48"/>
+      <c r="Q15" s="56"/>
       <c r="R15" s="48"/>
       <c r="S15" s="48">
         <v>5</v>
@@ -25518,7 +25552,7 @@
       <c r="A16" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="48"/>
+      <c r="B16" s="56"/>
       <c r="C16" s="48"/>
       <c r="D16" s="48">
         <v>5</v>
@@ -25528,7 +25562,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G16" s="48"/>
+      <c r="G16" s="56"/>
       <c r="H16" s="48"/>
       <c r="I16" s="48">
         <v>5</v>
@@ -25538,7 +25572,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L16" s="48"/>
+      <c r="L16" s="56"/>
       <c r="M16" s="48"/>
       <c r="N16" s="48">
         <v>5</v>
@@ -25548,7 +25582,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q16" s="48"/>
+      <c r="Q16" s="56"/>
       <c r="R16" s="48"/>
       <c r="S16" s="48">
         <v>5</v>
@@ -25575,7 +25609,7 @@
       <c r="A17" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="48"/>
+      <c r="B17" s="56"/>
       <c r="C17" s="48"/>
       <c r="D17" s="48">
         <v>5</v>
@@ -25585,7 +25619,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G17" s="48"/>
+      <c r="G17" s="56"/>
       <c r="H17" s="48"/>
       <c r="I17" s="48">
         <v>5</v>
@@ -25595,7 +25629,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L17" s="48"/>
+      <c r="L17" s="56"/>
       <c r="M17" s="48"/>
       <c r="N17" s="48">
         <v>5</v>
@@ -25605,7 +25639,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q17" s="48"/>
+      <c r="Q17" s="56"/>
       <c r="R17" s="48"/>
       <c r="S17" s="48">
         <v>5</v>
@@ -25632,7 +25666,7 @@
       <c r="A18" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="48"/>
+      <c r="B18" s="56"/>
       <c r="C18" s="48"/>
       <c r="D18" s="48">
         <v>5</v>
@@ -25642,7 +25676,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G18" s="48"/>
+      <c r="G18" s="56"/>
       <c r="H18" s="48"/>
       <c r="I18" s="48">
         <v>5</v>
@@ -25652,7 +25686,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L18" s="48"/>
+      <c r="L18" s="56"/>
       <c r="M18" s="48"/>
       <c r="N18" s="48">
         <v>5</v>
@@ -25662,7 +25696,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q18" s="48"/>
+      <c r="Q18" s="56"/>
       <c r="R18" s="48"/>
       <c r="S18" s="48">
         <v>5</v>
@@ -25689,7 +25723,7 @@
       <c r="A19" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="48"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="48"/>
       <c r="D19" s="48">
         <v>5</v>
@@ -25699,7 +25733,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G19" s="48"/>
+      <c r="G19" s="56"/>
       <c r="H19" s="48"/>
       <c r="I19" s="48">
         <v>5</v>
@@ -25709,7 +25743,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L19" s="48"/>
+      <c r="L19" s="56"/>
       <c r="M19" s="48"/>
       <c r="N19" s="48">
         <v>5</v>
@@ -25719,7 +25753,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q19" s="48"/>
+      <c r="Q19" s="56"/>
       <c r="R19" s="48"/>
       <c r="S19" s="48">
         <v>5</v>
@@ -25746,7 +25780,7 @@
       <c r="A20" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="56"/>
       <c r="C20" s="48"/>
       <c r="D20" s="48">
         <v>5</v>
@@ -25756,7 +25790,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G20" s="48"/>
+      <c r="G20" s="56"/>
       <c r="H20" s="48"/>
       <c r="I20" s="48">
         <v>5</v>
@@ -25766,7 +25800,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L20" s="48"/>
+      <c r="L20" s="56"/>
       <c r="M20" s="48"/>
       <c r="N20" s="48">
         <v>5</v>
@@ -25776,7 +25810,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q20" s="48"/>
+      <c r="Q20" s="56"/>
       <c r="R20" s="48"/>
       <c r="S20" s="48">
         <v>5</v>
@@ -25825,11 +25859,11 @@
       </c>
       <c r="J21" s="46">
         <f>SUM(J5:J20)</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K21" s="46">
         <f t="shared" si="1"/>
-        <v>0.27500000000000002</v>
+        <v>0.3</v>
       </c>
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
@@ -25839,11 +25873,11 @@
       </c>
       <c r="O21" s="46">
         <f>SUM(O5:O20)</f>
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="P21" s="46">
         <f t="shared" si="2"/>
-        <v>0.4</v>
+        <v>0.46250000000000002</v>
       </c>
       <c r="Q21" s="50"/>
       <c r="R21" s="50"/>
@@ -25865,11 +25899,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.31562499999999999</v>
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25899,11 +25933,11 @@
       </c>
       <c r="J23" s="53">
         <f>J21</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K23" s="53">
         <f>IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),J23/I23,"")</f>
-        <v>0.27500000000000002</v>
+        <v>0.3</v>
       </c>
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
@@ -25913,11 +25947,11 @@
       </c>
       <c r="O23" s="53">
         <f>O21</f>
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="P23" s="53">
         <f>IF(AND(N23&lt;&gt;"",O23&lt;&gt;""),O23/N23,"")</f>
-        <v>0.4</v>
+        <v>0.46250000000000002</v>
       </c>
       <c r="Q23" s="52"/>
       <c r="R23" s="52"/>
@@ -25939,11 +25973,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.31562499999999999</v>
+        <v>0.33750000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-08-04 19:55:19
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9B2180-C601-42F6-8AF0-2C176D92EFDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2682CACF-456B-4C7C-8F9A-41296C77CB6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="313">
   <si>
     <t>英语真题阅读 正确率记录</t>
   </si>
@@ -974,6 +974,18 @@
   </si>
   <si>
     <t>7.31</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6.4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1472,33 +1484,21 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1517,6 +1517,27 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1524,15 +1545,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7537,7 +7549,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="65" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="59"/>
@@ -7564,13 +7576,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="61"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="62"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="64"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
@@ -8075,13 +8087,13 @@
     </row>
     <row r="40" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="68" t="s">
+      <c r="A41" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="61"/>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="62"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="64"/>
     </row>
     <row r="42" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
@@ -8562,13 +8574,13 @@
     </row>
     <row r="82" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="68" t="s">
+      <c r="A83" s="62" t="s">
         <v>106</v>
       </c>
-      <c r="B83" s="61"/>
-      <c r="C83" s="61"/>
-      <c r="D83" s="61"/>
-      <c r="E83" s="62"/>
+      <c r="B83" s="63"/>
+      <c r="C83" s="63"/>
+      <c r="D83" s="63"/>
+      <c r="E83" s="64"/>
     </row>
     <row r="84" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -8786,7 +8798,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="66" t="s">
         <v>114</v>
       </c>
       <c r="B1" s="59"/>
@@ -8807,26 +8819,26 @@
     <row r="3" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="61"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="74" t="s">
+      <c r="D3" s="63"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="70" t="s">
         <v>305</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="73" t="s">
+      <c r="G3" s="63"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="69" t="s">
         <v>116</v>
       </c>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="72" t="s">
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="61"/>
-      <c r="N3" s="62"/>
+      <c r="M3" s="63"/>
+      <c r="N3" s="64"/>
     </row>
     <row r="4" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
@@ -9526,7 +9538,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="76" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="59"/>
@@ -9544,21 +9556,21 @@
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="66" t="s">
+      <c r="C3" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="61"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="64" t="s">
+      <c r="D3" s="63"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="63" t="s">
+      <c r="G3" s="63"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -9596,19 +9608,19 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="72" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
-      <c r="H5" s="61"/>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
-      <c r="K5" s="62"/>
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9969,19 +9981,19 @@
     </row>
     <row r="16" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="60" t="s">
+      <c r="A17" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="61"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="62"/>
+      <c r="B17" s="63"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
+      <c r="I17" s="63"/>
+      <c r="J17" s="63"/>
+      <c r="K17" s="64"/>
     </row>
     <row r="18" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -10207,19 +10219,19 @@
     </row>
     <row r="25" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="60" t="s">
+      <c r="A26" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="61"/>
-      <c r="C26" s="61"/>
-      <c r="D26" s="61"/>
-      <c r="E26" s="61"/>
-      <c r="F26" s="61"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="61"/>
-      <c r="I26" s="61"/>
-      <c r="J26" s="61"/>
-      <c r="K26" s="62"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
+      <c r="E26" s="63"/>
+      <c r="F26" s="63"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63"/>
+      <c r="I26" s="63"/>
+      <c r="J26" s="63"/>
+      <c r="K26" s="64"/>
     </row>
     <row r="27" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -10546,7 +10558,7 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="67" t="s">
+      <c r="A39" s="74" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="59"/>
@@ -10567,26 +10579,26 @@
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="66" t="s">
+      <c r="C41" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="61"/>
-      <c r="E41" s="62"/>
-      <c r="F41" s="64" t="s">
+      <c r="D41" s="63"/>
+      <c r="E41" s="64"/>
+      <c r="F41" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="61"/>
-      <c r="H41" s="62"/>
-      <c r="I41" s="65" t="s">
+      <c r="G41" s="63"/>
+      <c r="H41" s="64"/>
+      <c r="I41" s="77" t="s">
         <v>156</v>
       </c>
-      <c r="J41" s="61"/>
-      <c r="K41" s="62"/>
-      <c r="L41" s="63" t="s">
+      <c r="J41" s="63"/>
+      <c r="K41" s="64"/>
+      <c r="L41" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="M41" s="61"/>
-      <c r="N41" s="62"/>
+      <c r="M41" s="63"/>
+      <c r="N41" s="64"/>
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -10633,22 +10645,22 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="60" t="s">
+      <c r="A43" s="72" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="61"/>
-      <c r="C43" s="61"/>
-      <c r="D43" s="61"/>
-      <c r="E43" s="61"/>
-      <c r="F43" s="61"/>
-      <c r="G43" s="61"/>
-      <c r="H43" s="61"/>
-      <c r="I43" s="61"/>
-      <c r="J43" s="61"/>
-      <c r="K43" s="61"/>
-      <c r="L43" s="61"/>
-      <c r="M43" s="61"/>
-      <c r="N43" s="62"/>
+      <c r="B43" s="63"/>
+      <c r="C43" s="63"/>
+      <c r="D43" s="63"/>
+      <c r="E43" s="63"/>
+      <c r="F43" s="63"/>
+      <c r="G43" s="63"/>
+      <c r="H43" s="63"/>
+      <c r="I43" s="63"/>
+      <c r="J43" s="63"/>
+      <c r="K43" s="63"/>
+      <c r="L43" s="63"/>
+      <c r="M43" s="63"/>
+      <c r="N43" s="64"/>
     </row>
     <row r="44" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -11103,22 +11115,22 @@
     </row>
     <row r="54" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="60" t="s">
+      <c r="A55" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="61"/>
-      <c r="C55" s="61"/>
-      <c r="D55" s="61"/>
-      <c r="E55" s="61"/>
-      <c r="F55" s="61"/>
-      <c r="G55" s="61"/>
-      <c r="H55" s="61"/>
-      <c r="I55" s="61"/>
-      <c r="J55" s="61"/>
-      <c r="K55" s="61"/>
-      <c r="L55" s="61"/>
-      <c r="M55" s="61"/>
-      <c r="N55" s="62"/>
+      <c r="B55" s="63"/>
+      <c r="C55" s="63"/>
+      <c r="D55" s="63"/>
+      <c r="E55" s="63"/>
+      <c r="F55" s="63"/>
+      <c r="G55" s="63"/>
+      <c r="H55" s="63"/>
+      <c r="I55" s="63"/>
+      <c r="J55" s="63"/>
+      <c r="K55" s="63"/>
+      <c r="L55" s="63"/>
+      <c r="M55" s="63"/>
+      <c r="N55" s="64"/>
     </row>
     <row r="56" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -11410,22 +11422,22 @@
     </row>
     <row r="63" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="60" t="s">
+      <c r="A64" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="B64" s="61"/>
-      <c r="C64" s="61"/>
-      <c r="D64" s="61"/>
-      <c r="E64" s="61"/>
-      <c r="F64" s="61"/>
-      <c r="G64" s="61"/>
-      <c r="H64" s="61"/>
-      <c r="I64" s="61"/>
-      <c r="J64" s="61"/>
-      <c r="K64" s="61"/>
-      <c r="L64" s="61"/>
-      <c r="M64" s="61"/>
-      <c r="N64" s="62"/>
+      <c r="B64" s="63"/>
+      <c r="C64" s="63"/>
+      <c r="D64" s="63"/>
+      <c r="E64" s="63"/>
+      <c r="F64" s="63"/>
+      <c r="G64" s="63"/>
+      <c r="H64" s="63"/>
+      <c r="I64" s="63"/>
+      <c r="J64" s="63"/>
+      <c r="K64" s="63"/>
+      <c r="L64" s="63"/>
+      <c r="M64" s="63"/>
+      <c r="N64" s="64"/>
     </row>
     <row r="65" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -11848,7 +11860,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="67" t="s">
+      <c r="A77" s="74" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="59"/>
@@ -11866,21 +11878,21 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="66" t="s">
+      <c r="C79" s="71" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="61"/>
-      <c r="E79" s="62"/>
-      <c r="F79" s="64" t="s">
+      <c r="D79" s="63"/>
+      <c r="E79" s="64"/>
+      <c r="F79" s="73" t="s">
         <v>155</v>
       </c>
-      <c r="G79" s="61"/>
-      <c r="H79" s="62"/>
-      <c r="I79" s="63" t="s">
+      <c r="G79" s="63"/>
+      <c r="H79" s="64"/>
+      <c r="I79" s="75" t="s">
         <v>113</v>
       </c>
-      <c r="J79" s="61"/>
-      <c r="K79" s="62"/>
+      <c r="J79" s="63"/>
+      <c r="K79" s="64"/>
     </row>
     <row r="80" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -11918,19 +11930,19 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="60" t="s">
+      <c r="A81" s="72" t="s">
         <v>53</v>
       </c>
-      <c r="B81" s="61"/>
-      <c r="C81" s="61"/>
-      <c r="D81" s="61"/>
-      <c r="E81" s="61"/>
-      <c r="F81" s="61"/>
-      <c r="G81" s="61"/>
-      <c r="H81" s="61"/>
-      <c r="I81" s="61"/>
-      <c r="J81" s="61"/>
-      <c r="K81" s="62"/>
+      <c r="B81" s="63"/>
+      <c r="C81" s="63"/>
+      <c r="D81" s="63"/>
+      <c r="E81" s="63"/>
+      <c r="F81" s="63"/>
+      <c r="G81" s="63"/>
+      <c r="H81" s="63"/>
+      <c r="I81" s="63"/>
+      <c r="J81" s="63"/>
+      <c r="K81" s="64"/>
     </row>
     <row r="82" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
@@ -12381,19 +12393,19 @@
     </row>
     <row r="92" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="60" t="s">
+      <c r="A93" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="B93" s="61"/>
-      <c r="C93" s="61"/>
-      <c r="D93" s="61"/>
-      <c r="E93" s="61"/>
-      <c r="F93" s="61"/>
-      <c r="G93" s="61"/>
-      <c r="H93" s="61"/>
-      <c r="I93" s="61"/>
-      <c r="J93" s="61"/>
-      <c r="K93" s="62"/>
+      <c r="B93" s="63"/>
+      <c r="C93" s="63"/>
+      <c r="D93" s="63"/>
+      <c r="E93" s="63"/>
+      <c r="F93" s="63"/>
+      <c r="G93" s="63"/>
+      <c r="H93" s="63"/>
+      <c r="I93" s="63"/>
+      <c r="J93" s="63"/>
+      <c r="K93" s="64"/>
     </row>
     <row r="94" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
@@ -12709,19 +12721,19 @@
     </row>
     <row r="101" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="60" t="s">
+      <c r="A102" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="B102" s="61"/>
-      <c r="C102" s="61"/>
-      <c r="D102" s="61"/>
-      <c r="E102" s="61"/>
-      <c r="F102" s="61"/>
-      <c r="G102" s="61"/>
-      <c r="H102" s="61"/>
-      <c r="I102" s="61"/>
-      <c r="J102" s="61"/>
-      <c r="K102" s="62"/>
+      <c r="B102" s="63"/>
+      <c r="C102" s="63"/>
+      <c r="D102" s="63"/>
+      <c r="E102" s="63"/>
+      <c r="F102" s="63"/>
+      <c r="G102" s="63"/>
+      <c r="H102" s="63"/>
+      <c r="I102" s="63"/>
+      <c r="J102" s="63"/>
+      <c r="K102" s="64"/>
     </row>
     <row r="103" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
@@ -13169,12 +13181,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13191,6 +13197,12 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -13584,7 +13596,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>159</v>
       </c>
       <c r="B1" s="59"/>
@@ -13611,32 +13623,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="80" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="79" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="63"/>
+      <c r="O3" s="63"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="63"/>
+      <c r="R3" s="63"/>
+      <c r="S3" s="63"/>
+      <c r="T3" s="63"/>
+      <c r="U3" s="63"/>
+      <c r="V3" s="64"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -16842,7 +16854,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="76" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="59"/>
@@ -16869,32 +16881,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="80" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="79" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="63"/>
+      <c r="O3" s="63"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="63"/>
+      <c r="R3" s="63"/>
+      <c r="S3" s="63"/>
+      <c r="T3" s="63"/>
+      <c r="U3" s="63"/>
+      <c r="V3" s="64"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -19734,7 +19746,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="59"/>
@@ -19761,32 +19773,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="80" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="79" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="63"/>
+      <c r="O3" s="63"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="63"/>
+      <c r="R3" s="63"/>
+      <c r="S3" s="63"/>
+      <c r="T3" s="63"/>
+      <c r="U3" s="63"/>
+      <c r="V3" s="64"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -21772,7 +21784,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>270</v>
       </c>
       <c r="B1" s="59"/>
@@ -21799,32 +21811,32 @@
     </row>
     <row r="2" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77" t="s">
+      <c r="A3" s="80" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
       <c r="L3" s="11"/>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="79" t="s">
         <v>161</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="62"/>
+      <c r="N3" s="63"/>
+      <c r="O3" s="63"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="63"/>
+      <c r="R3" s="63"/>
+      <c r="S3" s="63"/>
+      <c r="T3" s="63"/>
+      <c r="U3" s="63"/>
+      <c r="V3" s="64"/>
     </row>
     <row r="4" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -24573,7 +24585,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="58" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="59"/>
@@ -24603,35 +24615,35 @@
     <row r="2" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="61" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="59"/>
       <c r="D3" s="59"/>
       <c r="E3" s="59"/>
       <c r="F3" s="59"/>
-      <c r="G3" s="80" t="s">
+      <c r="G3" s="61" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="59"/>
       <c r="I3" s="59"/>
       <c r="J3" s="59"/>
       <c r="K3" s="59"/>
-      <c r="L3" s="80" t="s">
+      <c r="L3" s="61" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="59"/>
       <c r="N3" s="59"/>
       <c r="O3" s="59"/>
       <c r="P3" s="59"/>
-      <c r="Q3" s="80" t="s">
+      <c r="Q3" s="61" t="s">
         <v>4</v>
       </c>
       <c r="R3" s="59"/>
       <c r="S3" s="59"/>
       <c r="T3" s="59"/>
       <c r="U3" s="59"/>
-      <c r="V3" s="79" t="s">
+      <c r="V3" s="60" t="s">
         <v>5</v>
       </c>
       <c r="W3" s="59"/>
@@ -25411,15 +25423,21 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="Q13" s="56"/>
-      <c r="R13" s="48"/>
+      <c r="Q13" s="57" t="s">
+        <v>310</v>
+      </c>
+      <c r="R13" s="48">
+        <v>23</v>
+      </c>
       <c r="S13" s="48">
         <v>5</v>
       </c>
-      <c r="T13" s="48"/>
-      <c r="U13" s="48" t="str">
+      <c r="T13" s="48">
+        <v>3</v>
+      </c>
+      <c r="U13" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="V13" s="48">
         <f t="shared" si="4"/>
@@ -25427,36 +25445,48 @@
       </c>
       <c r="W13" s="48">
         <f t="shared" si="5"/>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="X13" s="48">
         <f t="shared" si="6"/>
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="48"/>
+      <c r="B14" s="57" t="s">
+        <v>311</v>
+      </c>
+      <c r="C14" s="48">
+        <v>13</v>
+      </c>
       <c r="D14" s="48">
         <v>5</v>
       </c>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48" t="str">
+      <c r="E14" s="48">
+        <v>4</v>
+      </c>
+      <c r="F14" s="48">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G14" s="56"/>
-      <c r="H14" s="48"/>
+        <v>0.8</v>
+      </c>
+      <c r="G14" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="H14" s="48">
+        <v>23</v>
+      </c>
       <c r="I14" s="48">
         <v>5</v>
       </c>
-      <c r="J14" s="48"/>
-      <c r="K14" s="48" t="str">
+      <c r="J14" s="48">
+        <v>3</v>
+      </c>
+      <c r="K14" s="48">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="L14" s="56"/>
       <c r="M14" s="48"/>
@@ -25484,11 +25514,11 @@
       </c>
       <c r="W14" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="X14" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25845,11 +25875,11 @@
       </c>
       <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" si="0"/>
-        <v>0.32500000000000001</v>
+        <v>0.375</v>
       </c>
       <c r="G21" s="50"/>
       <c r="H21" s="50"/>
@@ -25859,11 +25889,11 @@
       </c>
       <c r="J21" s="46">
         <f>SUM(J5:J20)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K21" s="46">
         <f t="shared" si="1"/>
-        <v>0.3</v>
+        <v>0.33750000000000002</v>
       </c>
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
@@ -25887,11 +25917,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>0.26250000000000001</v>
+        <v>0.3</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25899,11 +25929,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.33750000000000002</v>
+        <v>0.36875000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25919,11 +25949,11 @@
       </c>
       <c r="E23" s="53">
         <f>E21</f>
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F23" s="53">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23/D23,"")</f>
-        <v>0.32500000000000001</v>
+        <v>0.375</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -25933,11 +25963,11 @@
       </c>
       <c r="J23" s="53">
         <f>J21</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K23" s="53">
         <f>IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),J23/I23,"")</f>
-        <v>0.3</v>
+        <v>0.33750000000000002</v>
       </c>
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
@@ -25961,11 +25991,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>0.26250000000000001</v>
+        <v>0.3</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -25973,11 +26003,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.33750000000000002</v>
+        <v>0.36875000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-08-10 19:50:13
</commit_message>
<xml_diff>
--- a/习题册.xlsx
+++ b/习题册.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\34406\Documents\Obsidian Vault\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2682CACF-456B-4C7C-8F9A-41296C77CB6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357FFD9E-00FD-4488-8A60-7048DF03A398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="317">
   <si>
     <t>英语真题阅读 正确率记录</t>
   </si>
@@ -985,7 +985,23 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>6.4</t>
+    <t>8.4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1517,25 +1533,25 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9538,7 +9554,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="71" t="s">
         <v>126</v>
       </c>
       <c r="B1" s="59"/>
@@ -9556,17 +9572,17 @@
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="76" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="63"/>
       <c r="E3" s="64"/>
-      <c r="F3" s="73" t="s">
+      <c r="F3" s="74" t="s">
         <v>106</v>
       </c>
       <c r="G3" s="63"/>
       <c r="H3" s="64"/>
-      <c r="I3" s="75" t="s">
+      <c r="I3" s="73" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="63"/>
@@ -10558,7 +10574,7 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="74" t="s">
+      <c r="A39" s="77" t="s">
         <v>155</v>
       </c>
       <c r="B39" s="59"/>
@@ -10579,22 +10595,22 @@
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="71" t="s">
+      <c r="C41" s="76" t="s">
         <v>52</v>
       </c>
       <c r="D41" s="63"/>
       <c r="E41" s="64"/>
-      <c r="F41" s="73" t="s">
+      <c r="F41" s="74" t="s">
         <v>106</v>
       </c>
       <c r="G41" s="63"/>
       <c r="H41" s="64"/>
-      <c r="I41" s="77" t="s">
+      <c r="I41" s="75" t="s">
         <v>156</v>
       </c>
       <c r="J41" s="63"/>
       <c r="K41" s="64"/>
-      <c r="L41" s="75" t="s">
+      <c r="L41" s="73" t="s">
         <v>47</v>
       </c>
       <c r="M41" s="63"/>
@@ -11860,7 +11876,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="74" t="s">
+      <c r="A77" s="77" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="59"/>
@@ -11878,17 +11894,17 @@
     <row r="79" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="71" t="s">
+      <c r="C79" s="76" t="s">
         <v>158</v>
       </c>
       <c r="D79" s="63"/>
       <c r="E79" s="64"/>
-      <c r="F79" s="73" t="s">
+      <c r="F79" s="74" t="s">
         <v>155</v>
       </c>
       <c r="G79" s="63"/>
       <c r="H79" s="64"/>
-      <c r="I79" s="75" t="s">
+      <c r="I79" s="73" t="s">
         <v>113</v>
       </c>
       <c r="J79" s="63"/>
@@ -13181,6 +13197,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A93:K93"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="L41:N41"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A81:K81"/>
     <mergeCell ref="A55:N55"/>
@@ -13197,12 +13219,6 @@
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A77:K77"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="F79:H79"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="L41:N41"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E6:E15">
@@ -16854,7 +16870,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="71" t="s">
         <v>211</v>
       </c>
       <c r="B1" s="59"/>
@@ -25488,25 +25504,37 @@
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="L14" s="56"/>
-      <c r="M14" s="48"/>
+      <c r="L14" s="57" t="s">
+        <v>313</v>
+      </c>
+      <c r="M14" s="48">
+        <v>14</v>
+      </c>
       <c r="N14" s="48">
         <v>5</v>
       </c>
-      <c r="O14" s="48"/>
-      <c r="P14" s="48" t="str">
+      <c r="O14" s="48">
+        <v>4</v>
+      </c>
+      <c r="P14" s="48">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q14" s="56"/>
-      <c r="R14" s="48"/>
+        <v>0.8</v>
+      </c>
+      <c r="Q14" s="57" t="s">
+        <v>314</v>
+      </c>
+      <c r="R14" s="48">
+        <v>22</v>
+      </c>
       <c r="S14" s="48">
         <v>5</v>
       </c>
-      <c r="T14" s="48"/>
-      <c r="U14" s="48" t="str">
+      <c r="T14" s="48">
+        <v>5</v>
+      </c>
+      <c r="U14" s="48">
         <f t="shared" si="3"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="V14" s="48">
         <f t="shared" si="4"/>
@@ -25514,36 +25542,48 @@
       </c>
       <c r="W14" s="48">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="X14" s="48">
         <f t="shared" si="6"/>
-        <v>0.35</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="56"/>
-      <c r="C15" s="48"/>
+      <c r="B15" s="57" t="s">
+        <v>315</v>
+      </c>
+      <c r="C15" s="48">
+        <v>21</v>
+      </c>
       <c r="D15" s="48">
         <v>5</v>
       </c>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48" t="str">
+      <c r="E15" s="48">
+        <v>4</v>
+      </c>
+      <c r="F15" s="48">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G15" s="56"/>
-      <c r="H15" s="48"/>
+        <v>0.8</v>
+      </c>
+      <c r="G15" s="57" t="s">
+        <v>316</v>
+      </c>
+      <c r="H15" s="48">
+        <v>17</v>
+      </c>
       <c r="I15" s="48">
         <v>5</v>
       </c>
-      <c r="J15" s="48"/>
-      <c r="K15" s="48" t="str">
+      <c r="J15" s="48">
+        <v>5</v>
+      </c>
+      <c r="K15" s="48">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="L15" s="56"/>
       <c r="M15" s="48"/>
@@ -25571,11 +25611,11 @@
       </c>
       <c r="W15" s="48">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="X15" s="48">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25">
@@ -25875,11 +25915,11 @@
       </c>
       <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" si="0"/>
-        <v>0.375</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="G21" s="50"/>
       <c r="H21" s="50"/>
@@ -25889,11 +25929,11 @@
       </c>
       <c r="J21" s="46">
         <f>SUM(J5:J20)</f>
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="K21" s="46">
         <f t="shared" si="1"/>
-        <v>0.33750000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
@@ -25903,11 +25943,11 @@
       </c>
       <c r="O21" s="46">
         <f>SUM(O5:O20)</f>
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="P21" s="46">
         <f t="shared" si="2"/>
-        <v>0.46250000000000002</v>
+        <v>0.51249999999999996</v>
       </c>
       <c r="Q21" s="50"/>
       <c r="R21" s="50"/>
@@ -25917,11 +25957,11 @@
       </c>
       <c r="T21" s="46">
         <f>SUM(T5:T20)</f>
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="U21" s="46">
         <f t="shared" si="3"/>
-        <v>0.3</v>
+        <v>0.36249999999999999</v>
       </c>
       <c r="V21" s="46">
         <f>SUM(V5:V20)</f>
@@ -25929,11 +25969,11 @@
       </c>
       <c r="W21" s="46">
         <f>SUM(W5:W20)</f>
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="X21" s="46">
         <f t="shared" si="6"/>
-        <v>0.36875000000000002</v>
+        <v>0.42499999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25949,11 +25989,11 @@
       </c>
       <c r="E23" s="53">
         <f>E21</f>
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F23" s="53">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23/D23,"")</f>
-        <v>0.375</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -25963,11 +26003,11 @@
       </c>
       <c r="J23" s="53">
         <f>J21</f>
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="K23" s="53">
         <f>IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),J23/I23,"")</f>
-        <v>0.33750000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
@@ -25977,11 +26017,11 @@
       </c>
       <c r="O23" s="53">
         <f>O21</f>
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="P23" s="53">
         <f>IF(AND(N23&lt;&gt;"",O23&lt;&gt;""),O23/N23,"")</f>
-        <v>0.46250000000000002</v>
+        <v>0.51249999999999996</v>
       </c>
       <c r="Q23" s="52"/>
       <c r="R23" s="52"/>
@@ -25991,11 +26031,11 @@
       </c>
       <c r="T23" s="53">
         <f>T21</f>
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="U23" s="53">
         <f>IF(AND(S23&lt;&gt;"",T23&lt;&gt;""),T23/S23,"")</f>
-        <v>0.3</v>
+        <v>0.36249999999999999</v>
       </c>
       <c r="V23" s="53">
         <f>V21</f>
@@ -26003,11 +26043,11 @@
       </c>
       <c r="W23" s="53">
         <f>W21</f>
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="X23" s="53">
         <f>IF(AND(V23&lt;&gt;"",W23&lt;&gt;""),W23/V23,"")</f>
-        <v>0.36875000000000002</v>
+        <v>0.42499999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>